<commit_message>
T200: freeze configuration contract
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re543a6001d0b45b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Ra681c7c7e4924bcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R3f8b4b06c2cd488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R5764ac7c7d844a32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R9053bc41eca54bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R799ef4a5cdaf4626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rc719d3ebe8a14a2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R996a63f8276a401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Rf79051a109124bc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R08cf40aa63944ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R180c99a867c9494c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R4307a9a5680748be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R9702e91925e3427d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R05fe6fa41d084961"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R00fe4680ba554faa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R5d2a14b7c1234969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R93311601d5784de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R3bdc36f3b42f450c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rc06823f59d8c4257"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R7a9b3c329aa045ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rafd84acf42b24f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R3a89a791807a4842"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R76214103390d4841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R1df16e59ac624839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rc3f5a415d0d942f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R32634fbf538a4b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rb0f0196844204375"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R92a1020424d0415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R42a6915bf9ff4df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re8f2c8aab3964394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R9f603ae6e5594c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rb8728b1b81cd4e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R9331ce6d89524f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R7eff528532cb47d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R5bdf4764e29b442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rdd6a965f49424dd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R1d4f1d367f9d4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R16451b2a83204760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R77abe304df7349a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rf308d5655c3245e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R52936307f2f74edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R5409aa4a69cd4691"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R63e884a51f224c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rba8936ec6d1542e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Ra8041211bda54bf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Raeb3e8da908d4588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R96d9bb7d73e34a5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rc879c68dc5624612"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rbb6804df86c64ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R17a3781f7256490d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R104442743edc4315"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rdbbc64edc6e5465e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R914300923c7a47c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R384902ad5c144780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R69f7b357c5864f09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R92668b74236745b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rc6e053ffc02f4a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R45061b0ac10748b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -462,7 +462,7 @@
         <x:color rgb="FF155724"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F3E6"/>
         </x:patternFill>
       </x:fill>
@@ -1013,9 +1013,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1131,7 +1131,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>《一笔镇妖》游戏配置表模板</x:v>
+        <x:v>《一笔镇妖》游戏配置工作簿</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -1143,7 +1143,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>用途：策划唯一真相源示例。正式工程复制为 Design/Config/GameConfig.xlsx；运行时只读取导出的JSON，不直接解析xlsx。</x:v>
+        <x:v>正式内容唯一源为 Design/Config/GameConfig.xlsx；config/ 下同名模板仅作同步镜像。运行时只读导出的JSON，不解析xlsx。</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -1178,7 +1178,7 @@
         <x:v>Players</x:v>
       </x:c>
       <x:c r="E5" s="106" t="n">
-        <x:f>COUNTA(Players!A5:A1000)</x:f>
+        <x:f>COUNTA('Players'!A5:A1000)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1187,13 +1187,13 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.1.0-sample</x:v>
+        <x:v>0.1.1-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
       </x:c>
       <x:c r="E6" s="106" t="n">
-        <x:f>COUNTA(Stances!A5:A1000)</x:f>
+        <x:f>COUNTA('Stances'!A5:A1000)</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -1208,7 +1208,7 @@
         <x:v>Enemies</x:v>
       </x:c>
       <x:c r="E7" s="106" t="n">
-        <x:f>COUNTA(Enemies!A5:A1000)</x:f>
+        <x:f>COUNTA('Enemies'!A5:A1000)</x:f>
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1223,7 +1223,7 @@
         <x:v>EnemyAttacks</x:v>
       </x:c>
       <x:c r="E8" s="106" t="n">
-        <x:f>COUNTA(EnemyAttacks!A5:A1000)</x:f>
+        <x:f>COUNTA('EnemyAttacks'!A5:A1000)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -1232,7 +1232,7 @@
         <x:v>Projectiles</x:v>
       </x:c>
       <x:c r="E9" s="106" t="n">
-        <x:f>COUNTA(Projectiles!A5:A1000)</x:f>
+        <x:f>COUNTA('Projectiles'!A5:A1000)</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1241,7 +1241,7 @@
         <x:v>Buffs</x:v>
       </x:c>
       <x:c r="E10" s="106" t="n">
-        <x:f>COUNTA(Buffs!A5:A1000)</x:f>
+        <x:f>COUNTA('Buffs'!A5:A1000)</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1253,7 +1253,7 @@
         <x:v>Skills</x:v>
       </x:c>
       <x:c r="E11" s="107" t="n">
-        <x:f>COUNTA(Skills!A5:A1000)</x:f>
+        <x:f>COUNTA('Skills'!A5:A1000)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F11" s="93"/>
@@ -1268,7 +1268,7 @@
         <x:v>Levels</x:v>
       </x:c>
       <x:c r="E12" s="89" t="n">
-        <x:f>COUNTA(Levels!A5:A1000)</x:f>
+        <x:f>COUNTA('Levels'!A5:A1000)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F12" s="92"/>
@@ -1283,7 +1283,7 @@
         <x:v>Waves</x:v>
       </x:c>
       <x:c r="E13" s="89" t="n">
-        <x:f>COUNTA(Waves!A5:A1000)</x:f>
+        <x:f>COUNTA('Waves'!A5:A1000)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="F13" s="92"/>
@@ -1298,7 +1298,7 @@
         <x:v>Spawns</x:v>
       </x:c>
       <x:c r="E14" s="89" t="n">
-        <x:f>COUNTA(Spawns!A5:A1000)</x:f>
+        <x:f>COUNTA('Spawns'!A5:A1000)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="F14" s="92"/>
@@ -1313,7 +1313,7 @@
         <x:v>BossPhases</x:v>
       </x:c>
       <x:c r="E15" s="89" t="n">
-        <x:f>COUNTA(BossPhases!A5:A1000)</x:f>
+        <x:f>COUNTA('BossPhases'!A5:A1000)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F15" s="92"/>
@@ -1328,7 +1328,7 @@
         <x:v>Tutorials</x:v>
       </x:c>
       <x:c r="E16" s="89" t="n">
-        <x:f>COUNTA(Tutorials!A5:A1000)</x:f>
+        <x:f>COUNTA('Tutorials'!A5:A1000)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="F16" s="92"/>
@@ -1343,7 +1343,7 @@
         <x:v>Texts</x:v>
       </x:c>
       <x:c r="E17" s="89" t="n">
-        <x:f>COUNTA(Texts!A5:A1000)</x:f>
+        <x:f>COUNTA('Texts'!A5:A1000)</x:f>
         <x:v>36</x:v>
       </x:c>
       <x:c r="F17" s="92"/>
@@ -1358,7 +1358,7 @@
         <x:v>AssetManifest</x:v>
       </x:c>
       <x:c r="E18" s="89" t="n">
-        <x:f>COUNTA(AssetManifest!A5:A1000)</x:f>
+        <x:f>COUNTA('AssetManifest'!A5:A1000)</x:f>
         <x:v>76</x:v>
       </x:c>
       <x:c r="F18" s="92"/>
@@ -1392,7 +1392,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="35" t="str">
-        <x:v>只在本工作簿修改策划数据；字段名是API，不随意改名。</x:v>
+        <x:v>只修改正式源；字段名是API；稳定ID使用小写英文/数字/下划线且发布后不复用。</x:v>
       </x:c>
       <x:c r="C23" s="35" t="str"/>
       <x:c r="D23" s="35" t="str"/>
@@ -1406,7 +1406,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B24" s="35" t="str">
-        <x:v>运行独立.NET导出器：结构/类型/唯一性/范围/枚举/外键/跨表校验。</x:v>
+        <x:v>导出器执行结构、类型、唯一性、范围、枚举、外键和跨表语义校验。</x:v>
       </x:c>
       <x:c r="C24" s="35" t="str"/>
       <x:c r="D24" s="35" t="str"/>
@@ -1420,7 +1420,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B25" s="35" t="str">
-        <x:v>导出稳定排序的 gameplay_config.json 和 contentHash。</x:v>
+        <x:v>JSON固定表序/行序；contentHash对排除自身后的规范化内容计算SHA-256。</x:v>
       </x:c>
       <x:c r="C25" s="35" t="str"/>
       <x:c r="D25" s="35" t="str"/>
@@ -1434,7 +1434,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="35" t="str">
-        <x:v>Unity只读取JSON，AssetRegistrySO只维护assetKey到Unity对象引用。</x:v>
+        <x:v>Unity只读JSON；AssetRegistrySO只维护assetKey到Unity对象引用。</x:v>
       </x:c>
       <x:c r="C26" s="35" t="str"/>
       <x:c r="D26" s="35" t="str"/>
@@ -1462,7 +1462,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B28" s="35" t="str">
-        <x:v>字段变更同时更新FieldDictionary、Schema、导出器、DTO、校验、文档和测试。</x:v>
+        <x:v>字段变更同步FieldDictionary、Schema、导出器、DTO、校验、文档和测试。FieldDictionary不递归描述自身。</x:v>
       </x:c>
       <x:c r="C28" s="35" t="str"/>
       <x:c r="D28" s="35" t="str"/>
@@ -1502,7 +1502,7 @@
         <x:v>Excel</x:v>
       </x:c>
       <x:c r="B33" s="34" t="str">
-        <x:v>策划内容唯一真相源</x:v>
+        <x:v>表头/ID/枚举契约由程序与策划共同审批；内容与平衡值由策划维护</x:v>
       </x:c>
       <x:c r="C33" s="34" t="str"/>
       <x:c r="D33" s="34" t="str"/>
@@ -1516,7 +1516,7 @@
         <x:v>JSON</x:v>
       </x:c>
       <x:c r="B34" s="34" t="str">
-        <x:v>构建期稳定快照，可审查、可回滚</x:v>
+        <x:v>导出器唯一生成的只读构建快照；禁止人工维护</x:v>
       </x:c>
       <x:c r="C34" s="34" t="str"/>
       <x:c r="D34" s="34" t="str"/>
@@ -1530,7 +1530,7 @@
         <x:v>C#</x:v>
       </x:c>
       <x:c r="B35" s="34" t="str">
-        <x:v>规则算法和DTO；不保存关卡/敌人数值</x:v>
+        <x:v>规则算法、DTO和注册表；不保存关卡、敌人或技能数值</x:v>
       </x:c>
       <x:c r="C35" s="34" t="str"/>
       <x:c r="D35" s="34" t="str"/>
@@ -1544,7 +1544,7 @@
         <x:v>Inspector/SO</x:v>
       </x:c>
       <x:c r="B36" s="34" t="str">
-        <x:v>只保存Unity资源与场景引用，不做第二数值库</x:v>
+        <x:v>只保存Unity资源/场景引用和明确调试兜底；不做第二数值库</x:v>
       </x:c>
       <x:c r="C36" s="34" t="str"/>
       <x:c r="D36" s="34" t="str"/>
@@ -1971,7 +1971,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="35" t="str">
-        <x:v>boss_tomb_armor_king</x:v>
+        <x:v>boss_tomb_king</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
         <x:v>text_boss_tomb_armor_king</x:v>
@@ -2028,7 +2028,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02ef0f4d119943dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d6b609393f74978"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2578,7 +2578,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c108812f5834813"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cb1bfbb6f5d4b1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2843,7 +2843,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48b0c3872c6645ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a130c7d81da45f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3078,7 +3078,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86d9175ceea3453e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8dc625fc06148e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3283,7 +3283,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93577563bfa44cc3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb1668789ce04e5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4132,7 +4132,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2871deb48c524ac8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27f4bb9345104fea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4227,7 +4227,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="35" t="str">
-        <x:v>level_001</x:v>
+        <x:v>lv_001_tutorial</x:v>
       </x:c>
       <x:c r="B5" s="35" t="str">
         <x:v>text_level_001</x:v>
@@ -4242,7 +4242,7 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="F5" s="35" t="str">
-        <x:v>level_002</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="G5" s="35" t="str">
         <x:v>reward_level_001</x:v>
@@ -4263,7 +4263,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="35" t="str">
-        <x:v>level_002</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="B6" s="35" t="str">
         <x:v>text_level_002</x:v>
@@ -4278,7 +4278,7 @@
         <x:v>210</x:v>
       </x:c>
       <x:c r="F6" s="35" t="str">
-        <x:v>level_003</x:v>
+        <x:v>lv_003_boss</x:v>
       </x:c>
       <x:c r="G6" s="35" t="str">
         <x:v>reward_level_002</x:v>
@@ -4299,7 +4299,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="35" t="str">
-        <x:v>level_003</x:v>
+        <x:v>lv_003_boss</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
         <x:v>text_level_003</x:v>
@@ -4330,7 +4330,7 @@
         <x:v>tutorial_level_003</x:v>
       </x:c>
       <x:c r="L7" s="35" t="str">
-        <x:v>boss_tomb_armor_king</x:v>
+        <x:v>boss_tomb_king</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4340,7 +4340,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7245d3b574394314"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4f18ee45e0043fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4420,7 +4420,7 @@
         <x:v>wave_001_01</x:v>
       </x:c>
       <x:c r="B5" s="35" t="str">
-        <x:v>level_001</x:v>
+        <x:v>lv_001_tutorial</x:v>
       </x:c>
       <x:c r="C5" s="68" t="n">
         <x:v>1</x:v>
@@ -4449,7 +4449,7 @@
         <x:v>wave_001_02</x:v>
       </x:c>
       <x:c r="B6" s="35" t="str">
-        <x:v>level_001</x:v>
+        <x:v>lv_001_tutorial</x:v>
       </x:c>
       <x:c r="C6" s="68" t="n">
         <x:v>2</x:v>
@@ -4478,7 +4478,7 @@
         <x:v>wave_001_03</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
-        <x:v>level_001</x:v>
+        <x:v>lv_001_tutorial</x:v>
       </x:c>
       <x:c r="C7" s="68" t="n">
         <x:v>3</x:v>
@@ -4507,7 +4507,7 @@
         <x:v>wave_002_01</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>level_002</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C8" s="68" t="n">
         <x:v>1</x:v>
@@ -4536,7 +4536,7 @@
         <x:v>wave_002_02</x:v>
       </x:c>
       <x:c r="B9" s="35" t="str">
-        <x:v>level_002</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C9" s="68" t="n">
         <x:v>2</x:v>
@@ -4565,7 +4565,7 @@
         <x:v>wave_002_03</x:v>
       </x:c>
       <x:c r="B10" s="35" t="str">
-        <x:v>level_002</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C10" s="68" t="n">
         <x:v>3</x:v>
@@ -4594,7 +4594,7 @@
         <x:v>wave_002_04</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
-        <x:v>level_002</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C11" s="68" t="n">
         <x:v>4</x:v>
@@ -4623,7 +4623,7 @@
         <x:v>wave_003_01</x:v>
       </x:c>
       <x:c r="B12" s="35" t="str">
-        <x:v>level_003</x:v>
+        <x:v>lv_003_boss</x:v>
       </x:c>
       <x:c r="C12" s="68" t="n">
         <x:v>1</x:v>
@@ -4652,7 +4652,7 @@
         <x:v>wave_003_02</x:v>
       </x:c>
       <x:c r="B13" s="35" t="str">
-        <x:v>level_003</x:v>
+        <x:v>lv_003_boss</x:v>
       </x:c>
       <x:c r="C13" s="68" t="n">
         <x:v>2</x:v>
@@ -4691,7 +4691,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42f3fc8bc3e44d74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5ed86c4d2a64485"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4858,7 +4858,7 @@
         <x:v>spawn_boss</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>level_003</x:v>
+        <x:v>lv_003_boss</x:v>
       </x:c>
       <x:c r="C8" s="72" t="n">
         <x:v>0.8</x:v>
@@ -4897,7 +4897,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3fa76432a16435b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4408af59355049a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5023,7 +5023,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4c64a2a7d934594"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fb50dcb3e584cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5122,7 +5122,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.1.0-sample</x:v>
+        <x:v>0.1.1-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -5344,7 +5344,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re49522b04164495a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9024ab9427d4a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5778,7 +5778,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D17" s="35" t="str">
-        <x:v>boss_tomb_armor_king</x:v>
+        <x:v>boss_tomb_king</x:v>
       </x:c>
       <x:c r="E17" s="68" t="n">
         <x:v>1</x:v>
@@ -5808,7 +5808,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f2c4807e5a34597"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R778f8911733c4726"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5900,7 +5900,7 @@
         <x:v>boss_tomb_phase_1</x:v>
       </x:c>
       <x:c r="B5" s="35" t="str">
-        <x:v>boss_tomb_armor_king</x:v>
+        <x:v>boss_tomb_king</x:v>
       </x:c>
       <x:c r="C5" s="68" t="n">
         <x:v>1</x:v>
@@ -5935,7 +5935,7 @@
         <x:v>boss_tomb_phase_2</x:v>
       </x:c>
       <x:c r="B6" s="35" t="str">
-        <x:v>boss_tomb_armor_king</x:v>
+        <x:v>boss_tomb_king</x:v>
       </x:c>
       <x:c r="C6" s="68" t="n">
         <x:v>2</x:v>
@@ -5970,7 +5970,7 @@
         <x:v>boss_tomb_phase_3</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
-        <x:v>boss_tomb_armor_king</x:v>
+        <x:v>boss_tomb_king</x:v>
       </x:c>
       <x:c r="C7" s="68" t="n">
         <x:v>3</x:v>
@@ -6007,7 +6007,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf02c60539794268"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf14602b07cd04891"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6087,7 +6087,7 @@
         <x:v>UnlockLevel</x:v>
       </x:c>
       <x:c r="F5" s="35" t="str">
-        <x:v>level_002</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="G5" s="68" t="n">
         <x:v>1</x:v>
@@ -6133,7 +6133,7 @@
         <x:v>UnlockLevel</x:v>
       </x:c>
       <x:c r="F7" s="35" t="str">
-        <x:v>level_003</x:v>
+        <x:v>lv_003_boss</x:v>
       </x:c>
       <x:c r="G7" s="68" t="n">
         <x:v>1</x:v>
@@ -6223,7 +6223,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4543b0d6e6ca46b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf7b0bd0cf004ad2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6513,7 +6513,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10b70280f97f4622"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33381698798045d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7069,7 +7069,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad2a009263d54ef7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5786207ed70349d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7592,7 +7592,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b95e895215347bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd465b912d10644d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8536,7 +8536,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9f18dedbb66477a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R136371187af64ea8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9891,7 +9891,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R509270e73d17407d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radb52c5f9ff4478d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11189,7 +11189,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a6ef7bd450346d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c8d6fece5724170"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11327,7 +11327,7 @@
         <x:v>int</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="E7" s="35" t="str"/>
       <x:c r="F7" s="35"/>
@@ -11349,7 +11349,7 @@
         <x:v>float</x:v>
       </x:c>
       <x:c r="D8" s="35" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="E8" s="35" t="str"/>
       <x:c r="F8" s="35"/>
@@ -11371,7 +11371,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D9" s="35" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="E9" s="35" t="str"/>
       <x:c r="F9" s="35"/>
@@ -11393,7 +11393,7 @@
         <x:v>bool</x:v>
       </x:c>
       <x:c r="D10" s="35" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="E10" s="35" t="str"/>
       <x:c r="F10" s="35"/>
@@ -12381,7 +12381,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D53" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E53" s="35" t="str"/>
       <x:c r="F53" s="35"/>
@@ -12563,7 +12563,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D61" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E61" s="35" t="str"/>
       <x:c r="F61" s="35"/>
@@ -13669,7 +13669,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D109" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E109" s="35" t="str"/>
       <x:c r="F109" s="35"/>
@@ -13927,7 +13927,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D120" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E120" s="35" t="str"/>
       <x:c r="F120" s="35"/>
@@ -14403,7 +14403,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D140" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E140" s="35" t="str"/>
       <x:c r="F140" s="35"/>
@@ -15059,7 +15059,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D168" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E168" s="35" t="str"/>
       <x:c r="F168" s="35"/>
@@ -16069,7 +16069,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D211" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E211" s="35" t="str"/>
       <x:c r="F211" s="35"/>
@@ -16093,7 +16093,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D212" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E212" s="35" t="str"/>
       <x:c r="F212" s="35"/>
@@ -16477,7 +16477,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D229" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E229" s="35" t="str"/>
       <x:c r="F229" s="35"/>
@@ -16665,7 +16665,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D237" s="35" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="E237" s="35" t="str"/>
       <x:c r="F237" s="35"/>
@@ -17034,7 +17034,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8461446876ad4457"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf82cb61be8914b2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17136,7 +17136,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e366fcf724b4343"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72bc70dea03e4ded"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17276,7 +17276,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra94ceade2da14070"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4d59fa9b5384b4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17674,7 +17674,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac2b6ae0941e4751"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d713173b53d4cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17858,7 +17858,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a5a1ebf74a6430b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R459c6449338e4050"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18037,7 +18037,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac28daa50e914a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51602ebb378f4cb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18262,7 +18262,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3931084bfe7347b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41596b1900d149fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18536,7 +18536,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7312a68dc168426d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa0b8a7463e94d13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T410: implement data-driven skill effect pipeline
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf4c786d96c1947c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R7713c23457b540b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rcc032c0346204cf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R6f54ca4c6982421c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R270c8053b56b4cef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R571ab63653e44bce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R45349805dc674a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rf69f2094a8dd43ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R575d0add0985409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Re113f33028834e83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R018ee8812ead420b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R9bbe252a4d8a40d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rfe34550998974987"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Rc7343c733f0c46fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R0ea16891f6f24dd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R25d6a7fb7f2e4895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R071626221eeb4232"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rc29a129102494565"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Re161c1289e3e4c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Re8b62c993971415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rdfea4b8ce1fb4d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R0bb9d211194a42ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R9070dacbdae64ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R20f2681fb1564b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R1d87e7f2a4964589"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R5c169c978a544da6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R60b65143b91545cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R4edb87dbef1d486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rdd7c99f9d1574684"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd76c80f308b440f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R588007aa5aa84663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Raa563f371974460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R9158382011ae4a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rca97b12659514cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R24336200b3e8401a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R625a7dff94c54aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R9055e41ed4984790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R18ebb0d4f1a04ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R60d11ad3abe442a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R1d23a1c3803c470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R5f5afcf699ac4214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rccd09493212849ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R4b5be74f16764852"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rf1ffc46ab7a94a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R62f0ff785a40401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R11168ec321974eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rb52645bbbabd4c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R40e4bc301b224801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rbccf7b0625344034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rfcdea1d78e974e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R188c7b40a6b74c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R44c80f549f564a84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R715b04266b5f40e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Ra01523dcb17e418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rbfd17780a6fb4ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R733b97842581490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R24f7d6a41be94955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rb714750b7e864f98"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2066,7 +2066,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf2de8598095404f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dcb4a80dd90444e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2616,7 +2616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b356fe444c24b30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racea08a965064ed3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2881,7 +2881,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6299405adb4949"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc52d359aa1d14cdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3116,7 +3116,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe78bc9765bc4111"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cf5c927a1c54b14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3321,7 +3321,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc25485dfb04411c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb30029388b245ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3430,14 +3430,14 @@
       <x:c r="G5" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H5" s="35" t="str"/>
+      <x:c r="H5" s="35"/>
       <x:c r="I5" s="35" t="str">
         <x:v>vfx_switch_blade</x:v>
       </x:c>
       <x:c r="J5" s="35" t="str">
         <x:v>sfx_switch</x:v>
       </x:c>
-      <x:c r="K5" s="35" t="str"/>
+      <x:c r="K5" s="35"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="35" t="str">
@@ -3461,14 +3461,14 @@
       <x:c r="G6" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H6" s="35" t="str"/>
+      <x:c r="H6" s="35"/>
       <x:c r="I6" s="35" t="str">
         <x:v>vfx_switch_talisman</x:v>
       </x:c>
       <x:c r="J6" s="35" t="str">
         <x:v>sfx_switch</x:v>
       </x:c>
-      <x:c r="K6" s="35" t="str"/>
+      <x:c r="K6" s="35"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="35" t="str">
@@ -3492,7 +3492,7 @@
       <x:c r="G7" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H7" s="35" t="str"/>
+      <x:c r="H7" s="35"/>
       <x:c r="I7" s="35" t="str">
         <x:v>vfx_blade_echo</x:v>
       </x:c>
@@ -3534,7 +3534,7 @@
       <x:c r="J8" s="35" t="str">
         <x:v>sfx_bind</x:v>
       </x:c>
-      <x:c r="K8" s="35" t="str"/>
+      <x:c r="K8" s="35"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="35" t="str">
@@ -3558,14 +3558,14 @@
       <x:c r="G9" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H9" s="35" t="str"/>
+      <x:c r="H9" s="35"/>
       <x:c r="I9" s="35" t="str">
         <x:v>vfx_talisman_burst</x:v>
       </x:c>
       <x:c r="J9" s="35" t="str">
         <x:v>sfx_talisman_hit</x:v>
       </x:c>
-      <x:c r="K9" s="35" t="str"/>
+      <x:c r="K9" s="35"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="35" t="str">
@@ -3589,14 +3589,14 @@
       <x:c r="G10" s="72" t="n">
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="H10" s="35" t="str"/>
+      <x:c r="H10" s="35"/>
       <x:c r="I10" s="35" t="str">
         <x:v>vfx_ultimate_prepare</x:v>
       </x:c>
       <x:c r="J10" s="35" t="str">
         <x:v>sfx_ultimate_start</x:v>
       </x:c>
-      <x:c r="K10" s="35" t="str"/>
+      <x:c r="K10" s="35"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="35" t="str">
@@ -3606,13 +3606,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
-        <x:v>Damage</x:v>
+        <x:v>ClearProjectiles</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>AllEnemies</x:v>
+        <x:v>Battle</x:v>
       </x:c>
       <x:c r="E11" s="35" t="n">
-        <x:v>50</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="35" t="n">
         <x:v>0</x:v>
@@ -3620,14 +3620,14 @@
       <x:c r="G11" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H11" s="35" t="str"/>
+      <x:c r="H11" s="35"/>
       <x:c r="I11" s="35" t="str">
-        <x:v>vfx_ultimate_slash</x:v>
+        <x:v>vfx_projectile_cut</x:v>
       </x:c>
       <x:c r="J11" s="35" t="str">
-        <x:v>sfx_ultimate_hit</x:v>
-      </x:c>
-      <x:c r="K11" s="35" t="str"/>
+        <x:v>sfx_seal_break</x:v>
+      </x:c>
+      <x:c r="K11" s="35"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="35" t="str">
@@ -3637,13 +3637,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C12" s="35" t="str">
-        <x:v>ExecuteBelowHpRatio</x:v>
+        <x:v>Damage</x:v>
       </x:c>
       <x:c r="D12" s="35" t="str">
-        <x:v>NormalEnemies</x:v>
+        <x:v>AllEnemies</x:v>
       </x:c>
       <x:c r="E12" s="35" t="n">
-        <x:v>0.25</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F12" s="35" t="n">
         <x:v>0</x:v>
@@ -3651,14 +3651,14 @@
       <x:c r="G12" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H12" s="35" t="str"/>
+      <x:c r="H12" s="35"/>
       <x:c r="I12" s="35" t="str">
-        <x:v>vfx_seal_execute</x:v>
+        <x:v>vfx_ultimate_slash</x:v>
       </x:c>
       <x:c r="J12" s="35" t="str">
-        <x:v>sfx_seal</x:v>
-      </x:c>
-      <x:c r="K12" s="35" t="str"/>
+        <x:v>sfx_ultimate_hit</x:v>
+      </x:c>
+      <x:c r="K12" s="35"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="35" t="str">
@@ -3668,65 +3668,65 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C13" s="35" t="str">
-        <x:v>ApplyBuff</x:v>
+        <x:v>ExecuteBelowHpRatio</x:v>
       </x:c>
       <x:c r="D13" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>NormalEnemies</x:v>
       </x:c>
       <x:c r="E13" s="35" t="n">
-        <x:v>0</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="F13" s="35" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="72" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H13" s="35" t="str">
-        <x:v>buff_vulnerable</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="35"/>
       <x:c r="I13" s="35" t="str">
-        <x:v>vfx_boss_break</x:v>
+        <x:v>vfx_seal_execute</x:v>
       </x:c>
       <x:c r="J13" s="35" t="str">
-        <x:v>sfx_break</x:v>
-      </x:c>
-      <x:c r="K13" s="35" t="str"/>
+        <x:v>sfx_seal</x:v>
+      </x:c>
+      <x:c r="K13" s="35"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="35" t="str">
-        <x:v>fx_break_armor</x:v>
+        <x:v>fx_ultimate_seal</x:v>
       </x:c>
       <x:c r="B14" s="68" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C14" s="35" t="str">
-        <x:v>RemoveArmor</x:v>
+        <x:v>ApplyBuff</x:v>
       </x:c>
       <x:c r="D14" s="35" t="str">
-        <x:v>Target</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="E14" s="35" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="35" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="72" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H14" s="35" t="str"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H14" s="35" t="str">
+        <x:v>buff_vulnerable</x:v>
+      </x:c>
       <x:c r="I14" s="35" t="str">
-        <x:v>vfx_armor_break</x:v>
+        <x:v>vfx_boss_break</x:v>
       </x:c>
       <x:c r="J14" s="35" t="str">
-        <x:v>sfx_armor_break</x:v>
-      </x:c>
-      <x:c r="K14" s="35" t="str"/>
+        <x:v>sfx_break</x:v>
+      </x:c>
+      <x:c r="K14" s="35"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="35" t="str">
-        <x:v>fx_break_seal</x:v>
+        <x:v>fx_break_armor</x:v>
       </x:c>
       <x:c r="B15" s="68" t="n">
         <x:v>1</x:v>
@@ -3746,78 +3746,80 @@
       <x:c r="G15" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H15" s="35" t="str"/>
+      <x:c r="H15" s="35"/>
       <x:c r="I15" s="35" t="str">
-        <x:v>vfx_seal_break</x:v>
+        <x:v>vfx_armor_break</x:v>
       </x:c>
       <x:c r="J15" s="35" t="str">
-        <x:v>sfx_seal_break</x:v>
-      </x:c>
-      <x:c r="K15" s="35" t="str"/>
+        <x:v>sfx_armor_break</x:v>
+      </x:c>
+      <x:c r="K15" s="35"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="35" t="str">
-        <x:v>fx_break_boss_pin</x:v>
+        <x:v>fx_break_seal</x:v>
       </x:c>
       <x:c r="B16" s="68" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C16" s="35" t="str">
-        <x:v>IncrementCounter</x:v>
+        <x:v>RemoveArmor</x:v>
       </x:c>
       <x:c r="D16" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Target</x:v>
       </x:c>
       <x:c r="E16" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F16" s="35" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H16" s="35" t="str"/>
+      <x:c r="H16" s="35"/>
       <x:c r="I16" s="35" t="str">
-        <x:v>vfx_boss_pin_break</x:v>
+        <x:v>vfx_seal_break</x:v>
       </x:c>
       <x:c r="J16" s="35" t="str">
-        <x:v>sfx_boss_pin</x:v>
-      </x:c>
-      <x:c r="K16" s="35" t="str"/>
+        <x:v>sfx_seal_break</x:v>
+      </x:c>
+      <x:c r="K16" s="35"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="35" t="str">
-        <x:v>fx_bat_dive</x:v>
+        <x:v>fx_break_boss_pin</x:v>
       </x:c>
       <x:c r="B17" s="68" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="35" t="str">
-        <x:v>PlayVfx</x:v>
+        <x:v>IncrementCounter</x:v>
       </x:c>
       <x:c r="D17" s="35" t="str">
-        <x:v>Target</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="E17" s="35" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F17" s="35" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G17" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H17" s="35" t="str"/>
+      <x:c r="H17" s="35"/>
       <x:c r="I17" s="35" t="str">
-        <x:v>vfx_bat_dive</x:v>
-      </x:c>
-      <x:c r="J17" s="35" t="str"/>
-      <x:c r="K17" s="35" t="str"/>
+        <x:v>vfx_boss_pin_break</x:v>
+      </x:c>
+      <x:c r="J17" s="35" t="str">
+        <x:v>sfx_boss_pin</x:v>
+      </x:c>
+      <x:c r="K17" s="35"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="35" t="str">
-        <x:v>fx_boss_charge</x:v>
+        <x:v>fx_bat_dive</x:v>
       </x:c>
       <x:c r="B18" s="68" t="n">
         <x:v>1</x:v>
@@ -3837,16 +3839,16 @@
       <x:c r="G18" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H18" s="35" t="str"/>
+      <x:c r="H18" s="35"/>
       <x:c r="I18" s="35" t="str">
-        <x:v>vfx_boss_charge</x:v>
-      </x:c>
-      <x:c r="J18" s="35" t="str"/>
-      <x:c r="K18" s="35" t="str"/>
+        <x:v>vfx_bat_dive</x:v>
+      </x:c>
+      <x:c r="J18" s="35"/>
+      <x:c r="K18" s="35"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="35" t="str">
-        <x:v>fx_boss_phase1_enter</x:v>
+        <x:v>fx_boss_charge</x:v>
       </x:c>
       <x:c r="B19" s="68" t="n">
         <x:v>1</x:v>
@@ -3866,16 +3868,16 @@
       <x:c r="G19" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H19" s="35" t="str"/>
+      <x:c r="H19" s="35"/>
       <x:c r="I19" s="35" t="str">
-        <x:v>vfx_boss_phase1_enter</x:v>
-      </x:c>
-      <x:c r="J19" s="35" t="str"/>
-      <x:c r="K19" s="35" t="str"/>
+        <x:v>vfx_boss_charge</x:v>
+      </x:c>
+      <x:c r="J19" s="35"/>
+      <x:c r="K19" s="35"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="35" t="str">
-        <x:v>fx_boss_phase2_enter</x:v>
+        <x:v>fx_boss_phase1_enter</x:v>
       </x:c>
       <x:c r="B20" s="68" t="n">
         <x:v>1</x:v>
@@ -3895,16 +3897,16 @@
       <x:c r="G20" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H20" s="35" t="str"/>
+      <x:c r="H20" s="35"/>
       <x:c r="I20" s="35" t="str">
-        <x:v>vfx_boss_phase2_enter</x:v>
-      </x:c>
-      <x:c r="J20" s="35" t="str"/>
-      <x:c r="K20" s="35" t="str"/>
+        <x:v>vfx_boss_phase1_enter</x:v>
+      </x:c>
+      <x:c r="J20" s="35"/>
+      <x:c r="K20" s="35"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="35" t="str">
-        <x:v>fx_boss_phase3_enter</x:v>
+        <x:v>fx_boss_phase2_enter</x:v>
       </x:c>
       <x:c r="B21" s="68" t="n">
         <x:v>1</x:v>
@@ -3924,16 +3926,16 @@
       <x:c r="G21" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H21" s="35" t="str"/>
+      <x:c r="H21" s="35"/>
       <x:c r="I21" s="35" t="str">
-        <x:v>vfx_boss_phase3_enter</x:v>
-      </x:c>
-      <x:c r="J21" s="35" t="str"/>
-      <x:c r="K21" s="35" t="str"/>
+        <x:v>vfx_boss_phase2_enter</x:v>
+      </x:c>
+      <x:c r="J21" s="35"/>
+      <x:c r="K21" s="35"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="35" t="str">
-        <x:v>fx_boss_rockfall</x:v>
+        <x:v>fx_boss_phase3_enter</x:v>
       </x:c>
       <x:c r="B22" s="68" t="n">
         <x:v>1</x:v>
@@ -3953,16 +3955,16 @@
       <x:c r="G22" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H22" s="35" t="str"/>
+      <x:c r="H22" s="35"/>
       <x:c r="I22" s="35" t="str">
-        <x:v>vfx_boss_rockfall</x:v>
-      </x:c>
-      <x:c r="J22" s="35" t="str"/>
-      <x:c r="K22" s="35" t="str"/>
+        <x:v>vfx_boss_phase3_enter</x:v>
+      </x:c>
+      <x:c r="J22" s="35"/>
+      <x:c r="K22" s="35"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="35" t="str">
-        <x:v>fx_boss_wave</x:v>
+        <x:v>fx_boss_rockfall</x:v>
       </x:c>
       <x:c r="B23" s="68" t="n">
         <x:v>1</x:v>
@@ -3982,16 +3984,16 @@
       <x:c r="G23" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H23" s="35" t="str"/>
+      <x:c r="H23" s="35"/>
       <x:c r="I23" s="35" t="str">
-        <x:v>vfx_boss_wave</x:v>
-      </x:c>
-      <x:c r="J23" s="35" t="str"/>
-      <x:c r="K23" s="35" t="str"/>
+        <x:v>vfx_boss_rockfall</x:v>
+      </x:c>
+      <x:c r="J23" s="35"/>
+      <x:c r="K23" s="35"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="35" t="str">
-        <x:v>fx_enemy_cast</x:v>
+        <x:v>fx_boss_wave</x:v>
       </x:c>
       <x:c r="B24" s="68" t="n">
         <x:v>1</x:v>
@@ -4011,16 +4013,16 @@
       <x:c r="G24" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H24" s="35" t="str"/>
+      <x:c r="H24" s="35"/>
       <x:c r="I24" s="35" t="str">
-        <x:v>vfx_enemy_cast</x:v>
-      </x:c>
-      <x:c r="J24" s="35" t="str"/>
-      <x:c r="K24" s="35" t="str"/>
+        <x:v>vfx_boss_wave</x:v>
+      </x:c>
+      <x:c r="J24" s="35"/>
+      <x:c r="K24" s="35"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="35" t="str">
-        <x:v>fx_ghost_volley</x:v>
+        <x:v>fx_enemy_cast</x:v>
       </x:c>
       <x:c r="B25" s="68" t="n">
         <x:v>1</x:v>
@@ -4040,16 +4042,16 @@
       <x:c r="G25" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H25" s="35" t="str"/>
+      <x:c r="H25" s="35"/>
       <x:c r="I25" s="35" t="str">
-        <x:v>vfx_ghost_volley</x:v>
-      </x:c>
-      <x:c r="J25" s="35" t="str"/>
-      <x:c r="K25" s="35" t="str"/>
+        <x:v>vfx_enemy_cast</x:v>
+      </x:c>
+      <x:c r="J25" s="35"/>
+      <x:c r="K25" s="35"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="35" t="str">
-        <x:v>fx_puppet_bolt</x:v>
+        <x:v>fx_ghost_volley</x:v>
       </x:c>
       <x:c r="B26" s="68" t="n">
         <x:v>1</x:v>
@@ -4069,16 +4071,16 @@
       <x:c r="G26" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H26" s="35" t="str"/>
+      <x:c r="H26" s="35"/>
       <x:c r="I26" s="35" t="str">
-        <x:v>vfx_puppet_bolt</x:v>
-      </x:c>
-      <x:c r="J26" s="35" t="str"/>
-      <x:c r="K26" s="35" t="str"/>
+        <x:v>vfx_ghost_volley</x:v>
+      </x:c>
+      <x:c r="J26" s="35"/>
+      <x:c r="K26" s="35"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="35" t="str">
-        <x:v>fx_puppet_shield</x:v>
+        <x:v>fx_puppet_bolt</x:v>
       </x:c>
       <x:c r="B27" s="68" t="n">
         <x:v>1</x:v>
@@ -4098,16 +4100,16 @@
       <x:c r="G27" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H27" s="35" t="str"/>
+      <x:c r="H27" s="35"/>
       <x:c r="I27" s="35" t="str">
-        <x:v>vfx_puppet_shield</x:v>
-      </x:c>
-      <x:c r="J27" s="35" t="str"/>
-      <x:c r="K27" s="35" t="str"/>
+        <x:v>vfx_puppet_bolt</x:v>
+      </x:c>
+      <x:c r="J27" s="35"/>
+      <x:c r="K27" s="35"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="35" t="str">
-        <x:v>fx_turtle_slam</x:v>
+        <x:v>fx_puppet_shield</x:v>
       </x:c>
       <x:c r="B28" s="68" t="n">
         <x:v>1</x:v>
@@ -4127,16 +4129,16 @@
       <x:c r="G28" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H28" s="35" t="str"/>
+      <x:c r="H28" s="35"/>
       <x:c r="I28" s="35" t="str">
-        <x:v>vfx_turtle_slam</x:v>
-      </x:c>
-      <x:c r="J28" s="35" t="str"/>
-      <x:c r="K28" s="35" t="str"/>
+        <x:v>vfx_puppet_shield</x:v>
+      </x:c>
+      <x:c r="J28" s="35"/>
+      <x:c r="K28" s="35"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="35" t="str">
-        <x:v>fx_wheel_charge</x:v>
+        <x:v>fx_turtle_slam</x:v>
       </x:c>
       <x:c r="B29" s="68" t="n">
         <x:v>1</x:v>
@@ -4156,12 +4158,41 @@
       <x:c r="G29" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H29" s="35" t="str"/>
+      <x:c r="H29" s="35"/>
       <x:c r="I29" s="35" t="str">
+        <x:v>vfx_turtle_slam</x:v>
+      </x:c>
+      <x:c r="J29" s="35"/>
+      <x:c r="K29" s="35"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>fx_wheel_charge</x:v>
+      </x:c>
+      <x:c r="B30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>PlayVfx</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>Target</x:v>
+      </x:c>
+      <x:c r="E30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H30"/>
+      <x:c r="I30" t="str">
         <x:v>vfx_wheel_charge</x:v>
       </x:c>
-      <x:c r="J29" s="35" t="str"/>
-      <x:c r="K29" s="35" t="str"/>
+      <x:c r="J30"/>
+      <x:c r="K30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4170,7 +4201,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9677db7c7d564a3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R996b128f812d46e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4378,7 +4409,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85265ce640544fc3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R342e49aaaa5c4019"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4729,7 +4760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b288453adbd460d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5de31baf4cdb4742"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4935,7 +4966,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e3680214ace4ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38128cf3d50a43c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5061,7 +5092,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R522b8e1f46d7415b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e9614ca22b34f69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5138,10 +5169,10 @@
         <x:v>int</x:v>
       </x:c>
       <x:c r="C5" s="68" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D5" s="35"/>
-      <x:c r="E5" s="35" t="str"/>
+      <x:c r="E5" s="35"/>
       <x:c r="F5" s="35"/>
       <x:c r="G5" s="35" t="str">
         <x:v>version</x:v>
@@ -5160,7 +5191,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.2.0-sample</x:v>
+        <x:v>0.3.0-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -5181,7 +5212,7 @@
         <x:v>1920</x:v>
       </x:c>
       <x:c r="D7" s="35"/>
-      <x:c r="E7" s="35" t="str"/>
+      <x:c r="E7" s="35"/>
       <x:c r="F7" s="35"/>
       <x:c r="G7" s="35" t="str">
         <x:v>px</x:v>
@@ -5201,7 +5232,7 @@
         <x:v>1080</x:v>
       </x:c>
       <x:c r="D8" s="35"/>
-      <x:c r="E8" s="35" t="str"/>
+      <x:c r="E8" s="35"/>
       <x:c r="F8" s="35"/>
       <x:c r="G8" s="35" t="str">
         <x:v>px</x:v>
@@ -5221,7 +5252,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D9" s="35"/>
-      <x:c r="E9" s="35" t="str"/>
+      <x:c r="E9" s="35"/>
       <x:c r="F9" s="35"/>
       <x:c r="G9" s="35" t="str">
         <x:v>fps</x:v>
@@ -5241,7 +5272,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="D10" s="35"/>
-      <x:c r="E10" s="35" t="str"/>
+      <x:c r="E10" s="35"/>
       <x:c r="F10" s="35"/>
       <x:c r="G10" s="35" t="str">
         <x:v>count</x:v>
@@ -5261,7 +5292,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="D11" s="35"/>
-      <x:c r="E11" s="35" t="str"/>
+      <x:c r="E11" s="35"/>
       <x:c r="F11" s="35"/>
       <x:c r="G11" s="35" t="str">
         <x:v>count</x:v>
@@ -5281,7 +5312,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D12" s="35"/>
-      <x:c r="E12" s="35" t="str"/>
+      <x:c r="E12" s="35"/>
       <x:c r="F12" s="35"/>
       <x:c r="G12" s="35" t="str">
         <x:v>count</x:v>
@@ -5301,7 +5332,7 @@
       <x:c r="D13" s="35" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E13" s="35" t="str"/>
+      <x:c r="E13" s="35"/>
       <x:c r="F13" s="35"/>
       <x:c r="G13" s="35" t="str">
         <x:v>sec</x:v>
@@ -5319,7 +5350,7 @@
       </x:c>
       <x:c r="C14" s="68"/>
       <x:c r="D14" s="35"/>
-      <x:c r="E14" s="35" t="str"/>
+      <x:c r="E14" s="35"/>
       <x:c r="F14" s="65" t="b">
         <x:v>1</x:v>
       </x:c>
@@ -5341,7 +5372,7 @@
       <x:c r="D15" s="35" t="n">
         <x:v>1.8</x:v>
       </x:c>
-      <x:c r="E15" s="35" t="str"/>
+      <x:c r="E15" s="35"/>
       <x:c r="F15" s="35"/>
       <x:c r="G15" s="35" t="str">
         <x:v>sec</x:v>
@@ -5361,7 +5392,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D16" s="35"/>
-      <x:c r="E16" s="35" t="str"/>
+      <x:c r="E16" s="35"/>
       <x:c r="F16" s="35"/>
       <x:c r="G16" s="35" t="str">
         <x:v>count</x:v>
@@ -5369,6 +5400,646 @@
       <x:c r="H16" s="35" t="str">
         <x:v>伤害数字池预热</x:v>
       </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+      <x:c r="G25"/>
+      <x:c r="H25"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26"/>
+      <x:c r="B26"/>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
+      <x:c r="G26"/>
+      <x:c r="H26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+      <x:c r="G27"/>
+      <x:c r="H27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32"/>
+      <x:c r="F32"/>
+      <x:c r="G32"/>
+      <x:c r="H32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
+      <x:c r="G33"/>
+      <x:c r="H33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34"/>
+      <x:c r="B34"/>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
+      <x:c r="E34"/>
+      <x:c r="F34"/>
+      <x:c r="G34"/>
+      <x:c r="H34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35"/>
+      <x:c r="B35"/>
+      <x:c r="C35"/>
+      <x:c r="D35"/>
+      <x:c r="E35"/>
+      <x:c r="F35"/>
+      <x:c r="G35"/>
+      <x:c r="H35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36"/>
+      <x:c r="B36"/>
+      <x:c r="C36"/>
+      <x:c r="D36"/>
+      <x:c r="E36"/>
+      <x:c r="F36"/>
+      <x:c r="G36"/>
+      <x:c r="H36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37"/>
+      <x:c r="B37"/>
+      <x:c r="C37"/>
+      <x:c r="D37"/>
+      <x:c r="E37"/>
+      <x:c r="F37"/>
+      <x:c r="G37"/>
+      <x:c r="H37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38"/>
+      <x:c r="B38"/>
+      <x:c r="C38"/>
+      <x:c r="D38"/>
+      <x:c r="E38"/>
+      <x:c r="F38"/>
+      <x:c r="G38"/>
+      <x:c r="H38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
+      <x:c r="E39"/>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
+      <x:c r="H39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40"/>
+      <x:c r="B40"/>
+      <x:c r="C40"/>
+      <x:c r="D40"/>
+      <x:c r="E40"/>
+      <x:c r="F40"/>
+      <x:c r="G40"/>
+      <x:c r="H40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42"/>
+      <x:c r="B42"/>
+      <x:c r="C42"/>
+      <x:c r="D42"/>
+      <x:c r="E42"/>
+      <x:c r="F42"/>
+      <x:c r="G42"/>
+      <x:c r="H42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43"/>
+      <x:c r="B43"/>
+      <x:c r="C43"/>
+      <x:c r="D43"/>
+      <x:c r="E43"/>
+      <x:c r="F43"/>
+      <x:c r="G43"/>
+      <x:c r="H43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44"/>
+      <x:c r="B44"/>
+      <x:c r="C44"/>
+      <x:c r="D44"/>
+      <x:c r="E44"/>
+      <x:c r="F44"/>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
+      <x:c r="E45"/>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46"/>
+      <x:c r="B46"/>
+      <x:c r="C46"/>
+      <x:c r="D46"/>
+      <x:c r="E46"/>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47"/>
+      <x:c r="B47"/>
+      <x:c r="C47"/>
+      <x:c r="D47"/>
+      <x:c r="E47"/>
+      <x:c r="F47"/>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48"/>
+      <x:c r="B48"/>
+      <x:c r="C48"/>
+      <x:c r="D48"/>
+      <x:c r="E48"/>
+      <x:c r="F48"/>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49"/>
+      <x:c r="B49"/>
+      <x:c r="C49"/>
+      <x:c r="D49"/>
+      <x:c r="E49"/>
+      <x:c r="F49"/>
+      <x:c r="G49"/>
+      <x:c r="H49"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50"/>
+      <x:c r="B50"/>
+      <x:c r="C50"/>
+      <x:c r="D50"/>
+      <x:c r="E50"/>
+      <x:c r="F50"/>
+      <x:c r="G50"/>
+      <x:c r="H50"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51"/>
+      <x:c r="B51"/>
+      <x:c r="C51"/>
+      <x:c r="D51"/>
+      <x:c r="E51"/>
+      <x:c r="F51"/>
+      <x:c r="G51"/>
+      <x:c r="H51"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52"/>
+      <x:c r="B52"/>
+      <x:c r="C52"/>
+      <x:c r="D52"/>
+      <x:c r="E52"/>
+      <x:c r="F52"/>
+      <x:c r="G52"/>
+      <x:c r="H52"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53"/>
+      <x:c r="B53"/>
+      <x:c r="C53"/>
+      <x:c r="D53"/>
+      <x:c r="E53"/>
+      <x:c r="F53"/>
+      <x:c r="G53"/>
+      <x:c r="H53"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54"/>
+      <x:c r="B54"/>
+      <x:c r="C54"/>
+      <x:c r="D54"/>
+      <x:c r="E54"/>
+      <x:c r="F54"/>
+      <x:c r="G54"/>
+      <x:c r="H54"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55"/>
+      <x:c r="B55"/>
+      <x:c r="C55"/>
+      <x:c r="D55"/>
+      <x:c r="E55"/>
+      <x:c r="F55"/>
+      <x:c r="G55"/>
+      <x:c r="H55"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56"/>
+      <x:c r="B56"/>
+      <x:c r="C56"/>
+      <x:c r="D56"/>
+      <x:c r="E56"/>
+      <x:c r="F56"/>
+      <x:c r="G56"/>
+      <x:c r="H56"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57"/>
+      <x:c r="B57"/>
+      <x:c r="C57"/>
+      <x:c r="D57"/>
+      <x:c r="E57"/>
+      <x:c r="F57"/>
+      <x:c r="G57"/>
+      <x:c r="H57"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58"/>
+      <x:c r="B58"/>
+      <x:c r="C58"/>
+      <x:c r="D58"/>
+      <x:c r="E58"/>
+      <x:c r="F58"/>
+      <x:c r="G58"/>
+      <x:c r="H58"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59"/>
+      <x:c r="B59"/>
+      <x:c r="C59"/>
+      <x:c r="D59"/>
+      <x:c r="E59"/>
+      <x:c r="F59"/>
+      <x:c r="G59"/>
+      <x:c r="H59"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60"/>
+      <x:c r="B60"/>
+      <x:c r="C60"/>
+      <x:c r="D60"/>
+      <x:c r="E60"/>
+      <x:c r="F60"/>
+      <x:c r="G60"/>
+      <x:c r="H60"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61"/>
+      <x:c r="B61"/>
+      <x:c r="C61"/>
+      <x:c r="D61"/>
+      <x:c r="E61"/>
+      <x:c r="F61"/>
+      <x:c r="G61"/>
+      <x:c r="H61"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62"/>
+      <x:c r="B62"/>
+      <x:c r="C62"/>
+      <x:c r="D62"/>
+      <x:c r="E62"/>
+      <x:c r="F62"/>
+      <x:c r="G62"/>
+      <x:c r="H62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63"/>
+      <x:c r="B63"/>
+      <x:c r="C63"/>
+      <x:c r="D63"/>
+      <x:c r="E63"/>
+      <x:c r="F63"/>
+      <x:c r="G63"/>
+      <x:c r="H63"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64"/>
+      <x:c r="B64"/>
+      <x:c r="C64"/>
+      <x:c r="D64"/>
+      <x:c r="E64"/>
+      <x:c r="F64"/>
+      <x:c r="G64"/>
+      <x:c r="H64"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65"/>
+      <x:c r="B65"/>
+      <x:c r="C65"/>
+      <x:c r="D65"/>
+      <x:c r="E65"/>
+      <x:c r="F65"/>
+      <x:c r="G65"/>
+      <x:c r="H65"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66"/>
+      <x:c r="B66"/>
+      <x:c r="C66"/>
+      <x:c r="D66"/>
+      <x:c r="E66"/>
+      <x:c r="F66"/>
+      <x:c r="G66"/>
+      <x:c r="H66"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67"/>
+      <x:c r="B67"/>
+      <x:c r="C67"/>
+      <x:c r="D67"/>
+      <x:c r="E67"/>
+      <x:c r="F67"/>
+      <x:c r="G67"/>
+      <x:c r="H67"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68"/>
+      <x:c r="B68"/>
+      <x:c r="C68"/>
+      <x:c r="D68"/>
+      <x:c r="E68"/>
+      <x:c r="F68"/>
+      <x:c r="G68"/>
+      <x:c r="H68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69"/>
+      <x:c r="B69"/>
+      <x:c r="C69"/>
+      <x:c r="D69"/>
+      <x:c r="E69"/>
+      <x:c r="F69"/>
+      <x:c r="G69"/>
+      <x:c r="H69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70"/>
+      <x:c r="B70"/>
+      <x:c r="C70"/>
+      <x:c r="D70"/>
+      <x:c r="E70"/>
+      <x:c r="F70"/>
+      <x:c r="G70"/>
+      <x:c r="H70"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71"/>
+      <x:c r="B71"/>
+      <x:c r="C71"/>
+      <x:c r="D71"/>
+      <x:c r="E71"/>
+      <x:c r="F71"/>
+      <x:c r="G71"/>
+      <x:c r="H71"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72"/>
+      <x:c r="B72"/>
+      <x:c r="C72"/>
+      <x:c r="D72"/>
+      <x:c r="E72"/>
+      <x:c r="F72"/>
+      <x:c r="G72"/>
+      <x:c r="H72"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73"/>
+      <x:c r="B73"/>
+      <x:c r="C73"/>
+      <x:c r="D73"/>
+      <x:c r="E73"/>
+      <x:c r="F73"/>
+      <x:c r="G73"/>
+      <x:c r="H73"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74"/>
+      <x:c r="B74"/>
+      <x:c r="C74"/>
+      <x:c r="D74"/>
+      <x:c r="E74"/>
+      <x:c r="F74"/>
+      <x:c r="G74"/>
+      <x:c r="H74"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75"/>
+      <x:c r="B75"/>
+      <x:c r="C75"/>
+      <x:c r="D75"/>
+      <x:c r="E75"/>
+      <x:c r="F75"/>
+      <x:c r="G75"/>
+      <x:c r="H75"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76"/>
+      <x:c r="B76"/>
+      <x:c r="C76"/>
+      <x:c r="D76"/>
+      <x:c r="E76"/>
+      <x:c r="F76"/>
+      <x:c r="G76"/>
+      <x:c r="H76"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77"/>
+      <x:c r="B77"/>
+      <x:c r="C77"/>
+      <x:c r="D77"/>
+      <x:c r="E77"/>
+      <x:c r="F77"/>
+      <x:c r="G77"/>
+      <x:c r="H77"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78"/>
+      <x:c r="B78"/>
+      <x:c r="C78"/>
+      <x:c r="D78"/>
+      <x:c r="E78"/>
+      <x:c r="F78"/>
+      <x:c r="G78"/>
+      <x:c r="H78"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79"/>
+      <x:c r="B79"/>
+      <x:c r="C79"/>
+      <x:c r="D79"/>
+      <x:c r="E79"/>
+      <x:c r="F79"/>
+      <x:c r="G79"/>
+      <x:c r="H79"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80"/>
+      <x:c r="B80"/>
+      <x:c r="C80"/>
+      <x:c r="D80"/>
+      <x:c r="E80"/>
+      <x:c r="F80"/>
+      <x:c r="G80"/>
+      <x:c r="H80"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5382,7 +6053,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a40238fb0954285"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R294cc272fa874423"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5846,7 +6517,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b6a97c48b5e4c95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refa256ccc1c94cfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6045,7 +6716,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23ecc72480db4811"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a7445701fb04420"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6261,7 +6932,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65d417ed7e154c7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8856750fb246456a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6551,7 +7222,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05bb33d64f0c42c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra76e013b0ba5436a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7107,7 +7778,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R934e0c1a6aa5459e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf958ab42c7594b76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7630,7 +8301,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa2763a9b9b4437d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee068cb8c8f4415"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8574,7 +9245,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01bad719b55d487e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbf62d3c623e40ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9929,7 +10600,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcce526d23974649"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67815d9863784fc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11220,6 +11891,34 @@
         <x:v>代码与配置共享的稳定枚举值</x:v>
       </x:c>
     </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>EffectType</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>Heal</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>Heal</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>代码与配置共享的稳定枚举值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>EffectType</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>ClearProjectiles</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>ClearProjectiles</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>代码与配置共享的稳定枚举值</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -11227,7 +11926,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61b703fccf8b4a24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9661b875992e47d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17120,7 +17819,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3a171478074429c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc27d4012d1f44b49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17222,7 +17921,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2262a78f14534c51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff890a2a79614390"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17371,7 +18070,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e700b0ad44344e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec842738436479c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17769,7 +18468,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd37e6e7f465c4455"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R662f38d2ec884de0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17966,7 +18665,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R396b9858cfac4fe9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc09e0f1eed84861"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18145,7 +18844,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0c387a5e228446a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942dc664136640d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18370,7 +19069,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ef4c08709a4110"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81c6e7a0c631484f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18644,7 +19343,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7ff495fd8084a6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re32ed019273d480b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T430: implement configured enemy strategies
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd76c80f308b440f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R588007aa5aa84663"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Raa563f371974460d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R9158382011ae4a3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rca97b12659514cc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R24336200b3e8401a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R625a7dff94c54aee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R9055e41ed4984790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R18ebb0d4f1a04ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R60d11ad3abe442a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R1d23a1c3803c470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R5f5afcf699ac4214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rccd09493212849ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R4b5be74f16764852"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rf1ffc46ab7a94a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R62f0ff785a40401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R11168ec321974eb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rb52645bbbabd4c1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R40e4bc301b224801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rbccf7b0625344034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rfcdea1d78e974e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R188c7b40a6b74c6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R44c80f549f564a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R715b04266b5f40e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Ra01523dcb17e418a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rbfd17780a6fb4ddb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R733b97842581490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R24f7d6a41be94955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rb714750b7e864f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3d68aaa06e914233"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R7cb98ac3d4dd445a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Ra38842aacb054cce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R7612163d7d064c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R9cdb38c04c644040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R32d91bc2aecd468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rec3619c5c60a4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rbe2b1b376bc64a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R5787a1b8989d4832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rde9c5e32517e4dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Radca1dcfbb50451d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R025ed11405574dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R29844e5b769640c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R3005c69c629a461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rf0d71e202b614003"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Rb1f41a40df444723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R41243af4e018434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rf9bfd8a698bf48f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rfe6992cef7b546fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rf9345c83bd2644f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rf667cc3f9a5c4d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rd0886b8c8a104afa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R233fd533d5cc4d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rb9d8a5da26914c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R526d2966f66e4a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rce09400c1bd444c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rb910c404b2374d91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rb1b2e139241a44fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R980e9405ce1e4b54"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1210,7 +1210,7 @@
         <x:v>Schema版本</x:v>
       </x:c>
       <x:c r="B5" s="25" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Players</x:v>
@@ -1225,7 +1225,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.2.0-sample</x:v>
+        <x:v>0.4.0-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1280,7 +1280,7 @@
       </x:c>
       <x:c r="E10" s="106" t="n">
         <x:f>COUNTA('Buffs'!A5:A1000)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1382,7 +1382,7 @@
       </x:c>
       <x:c r="E17" s="89" t="n">
         <x:f>COUNTA('Texts'!A5:A1000)</x:f>
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="F17" s="92"/>
       <x:c r="G17" s="92"/>
@@ -2066,7 +2066,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dcb4a80dd90444e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fd0f4de5ad44fdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2616,7 +2616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racea08a965064ed3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d4c7ebc6dd44e24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2881,7 +2881,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc52d359aa1d14cdb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7092c7a0e0a64a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3101,6 +3101,35 @@
         <x:v>text_buff_vulnerable</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>buff_shield_50</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>DamageReduction</x:v>
+      </x:c>
+      <x:c r="C10" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Refresh</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>vfx_puppet_shield</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>text_buff_shield</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
@@ -3116,7 +3145,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cf5c927a1c54b14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R641df703e2ed467c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3321,7 +3350,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb30029388b245ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb084fe1982b04734"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4115,7 +4144,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C28" s="35" t="str">
-        <x:v>PlayVfx</x:v>
+        <x:v>ApplyBuff</x:v>
       </x:c>
       <x:c r="D28" s="35" t="str">
         <x:v>Target</x:v>
@@ -4129,12 +4158,14 @@
       <x:c r="G28" s="72" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H28" s="35"/>
+      <x:c r="H28" s="35" t="str">
+        <x:v>buff_shield_50</x:v>
+      </x:c>
       <x:c r="I28" s="35" t="str">
         <x:v>vfx_puppet_shield</x:v>
       </x:c>
-      <x:c r="J28" s="35"/>
-      <x:c r="K28" s="35"/>
+      <x:c r="J28" s="35" t="str"/>
+      <x:c r="K28" s="35" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="35" t="str">
@@ -4201,7 +4232,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R996b128f812d46e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47b55bcba0ac4870"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4409,7 +4440,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R342e49aaaa5c4019"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9eeed6d5ba49401d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4760,7 +4791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5de31baf4cdb4742"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60ace22e9a1649e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4966,7 +4997,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38128cf3d50a43c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R076d961a75574595"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5092,7 +5123,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e9614ca22b34f69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb805c27ddd514c55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5169,7 +5200,7 @@
         <x:v>int</x:v>
       </x:c>
       <x:c r="C5" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D5" s="35"/>
       <x:c r="E5" s="35"/>
@@ -5191,7 +5222,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.3.0-sample</x:v>
+        <x:v>0.4.0-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6053,7 +6084,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R294cc272fa874423"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75a428f3951740ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6517,7 +6548,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refa256ccc1c94cfe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a7e7ca25d2f48b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6716,7 +6747,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a7445701fb04420"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bc7b158f5764d7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6932,7 +6963,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8856750fb246456a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda696858ba744ca1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7222,7 +7253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra76e013b0ba5436a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9a82097922241f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7771,6 +7802,20 @@
         <x:v>Boss phase</x:v>
       </x:c>
     </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>text_buff_shield</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>护盾</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>Shield</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>Buff</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -7778,7 +7823,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf958ab42c7594b76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea187c6198a74562"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8301,7 +8346,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee068cb8c8f4415"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re05463df84c849b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9245,7 +9290,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbf62d3c623e40ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f2ba248ac5e4183"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10600,7 +10645,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67815d9863784fc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca634a29b774cf2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11919,6 +11964,20 @@
         <x:v>代码与配置共享的稳定枚举值</x:v>
       </x:c>
     </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>BuffType</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>DamageReduction</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>DamageReduction</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>降低受到的伤害；magnitude 为减伤比例，叠层后按 1-magnitude×stacks 计算并钳制到非负。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -11926,7 +11985,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9661b875992e47d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d4cce433b284838"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17819,7 +17878,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc27d4012d1f44b49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eac9778bcbc4306"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17921,7 +17980,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff890a2a79614390"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61466ef2b5624f36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18070,7 +18129,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec842738436479c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R932ee86afbcd47b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18468,7 +18527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R662f38d2ec884de0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R181dfdf719864b98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18665,7 +18724,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc09e0f1eed84861"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R962433f91274432e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18844,7 +18903,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942dc664136640d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13b7606d87b24f8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19069,7 +19128,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81c6e7a0c631484f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbe630644d454c7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19343,7 +19402,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re32ed019273d480b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f9d91e72a5049e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T440: implement configured object pools
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3d68aaa06e914233"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R7cb98ac3d4dd445a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Ra38842aacb054cce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R7612163d7d064c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R9cdb38c04c644040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R32d91bc2aecd468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rec3619c5c60a4258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rbe2b1b376bc64a62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R5787a1b8989d4832"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rde9c5e32517e4dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Radca1dcfbb50451d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R025ed11405574dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R29844e5b769640c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R3005c69c629a461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rf0d71e202b614003"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Rb1f41a40df444723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R41243af4e018434a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rf9bfd8a698bf48f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rfe6992cef7b546fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rf9345c83bd2644f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rf667cc3f9a5c4d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rd0886b8c8a104afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R233fd533d5cc4d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rb9d8a5da26914c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R526d2966f66e4a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rce09400c1bd444c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rb910c404b2374d91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rb1b2e139241a44fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R980e9405ce1e4b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7f4d87d711634e35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rcc4fc113546e4e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rcfa041b7f9554777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R191c503333db48c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rfa416450050c4b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R79ab44b2e4c04226"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R9df341ab5b2e472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Re9cf3d9983d246d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Rb777b95905924e2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R4fec9b62e2694eaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R2131d4e3790b4e6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R02522fd9a5b04021"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R4a5d7b02d214490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R8363d5ba5ea0401c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R4ed8d7626fc24f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R43ed07f340c140f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R8f3ccf5de5674869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R2458ea5508874e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rb0dbc78d75da4bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R42591764330c4c79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R8333bf100457410d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R0bed47edad4f46e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rf494c164a13a4615"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R4878992e53094be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R092b6eab18a14cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rfb9bb2ee61a945c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R1a6ff06757ec4ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R78dfcd78ffee4139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Re0bfa18e5b764caf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1225,7 +1225,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.4.0-sample</x:v>
+        <x:v>0.5.0-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -2066,7 +2066,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fd0f4de5ad44fdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15656f69cbf04623"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2616,7 +2616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d4c7ebc6dd44e24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b0e08227502401a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2881,7 +2881,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7092c7a0e0a64a4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a817f837c094ef3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3145,7 +3145,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R641df703e2ed467c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R162e08304649428c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3350,7 +3350,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb084fe1982b04734"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76d6d445e86846a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4232,7 +4232,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47b55bcba0ac4870"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb1a5bbd18e24f8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4440,7 +4440,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9eeed6d5ba49401d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe5db5d316c2465f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4791,7 +4791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60ace22e9a1649e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4faf057777dd4ac1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4997,7 +4997,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R076d961a75574595"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5376b6eec422491d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5123,7 +5123,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb805c27ddd514c55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd544e1d051b46c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5132,7 +5132,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="42.220001220703125" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
@@ -5222,7 +5222,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.4.0-sample</x:v>
+        <x:v>0.5.0-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -5433,54 +5433,104 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17"/>
-      <x:c r="B17"/>
-      <x:c r="C17"/>
+      <x:c r="A17" t="str">
+        <x:v>projectile_pool_prewarm_per_type</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C17" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="D17"/>
       <x:c r="E17"/>
       <x:c r="F17"/>
-      <x:c r="G17"/>
-      <x:c r="H17"/>
+      <x:c r="G17" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>每种投射物池预热数量</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18"/>
-      <x:c r="B18"/>
+      <x:c r="A18" t="str">
+        <x:v>enemy_pool_exhaustion_policy</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>string</x:v>
+      </x:c>
       <x:c r="C18"/>
       <x:c r="D18"/>
-      <x:c r="E18"/>
+      <x:c r="E18" t="str">
+        <x:v>Reject</x:v>
+      </x:c>
       <x:c r="F18"/>
-      <x:c r="G18"/>
-      <x:c r="H18"/>
+      <x:c r="G18" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>敌人池耗尽时拒绝本次生成</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19"/>
-      <x:c r="B19"/>
+      <x:c r="A19" t="str">
+        <x:v>projectile_pool_exhaustion_policy</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>string</x:v>
+      </x:c>
       <x:c r="C19"/>
       <x:c r="D19"/>
-      <x:c r="E19"/>
+      <x:c r="E19" t="str">
+        <x:v>Reject</x:v>
+      </x:c>
       <x:c r="F19"/>
-      <x:c r="G19"/>
-      <x:c r="H19"/>
+      <x:c r="G19" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>投射物池耗尽时拒绝本次生成</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20"/>
-      <x:c r="B20"/>
+      <x:c r="A20" t="str">
+        <x:v>vfx_pool_exhaustion_policy</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>string</x:v>
+      </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
-      <x:c r="E20"/>
+      <x:c r="E20" t="str">
+        <x:v>ReuseOldest</x:v>
+      </x:c>
       <x:c r="F20"/>
-      <x:c r="G20"/>
-      <x:c r="H20"/>
+      <x:c r="G20" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>VFX池耗尽时复用最早活动项</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21"/>
-      <x:c r="B21"/>
+      <x:c r="A21" t="str">
+        <x:v>damage_number_pool_exhaustion_policy</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>string</x:v>
+      </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>
-      <x:c r="E21"/>
+      <x:c r="E21" t="str">
+        <x:v>ReuseOldest</x:v>
+      </x:c>
       <x:c r="F21"/>
-      <x:c r="G21"/>
-      <x:c r="H21"/>
+      <x:c r="G21" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>伤害数字池耗尽时复用最早活动项</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22"/>
@@ -6084,7 +6134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75a428f3951740ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae2ed3777c0f4439"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6548,7 +6598,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a7e7ca25d2f48b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92e3d392b0154eab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6747,7 +6797,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bc7b158f5764d7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10247c7e5905487e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6963,7 +7013,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda696858ba744ca1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25581153c37e4904"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7253,7 +7303,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9a82097922241f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9111758c4b1749f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7823,7 +7873,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea187c6198a74562"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5189ea1c92e41f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8346,7 +8396,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re05463df84c849b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60343fd771da4307"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9290,7 +9340,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f2ba248ac5e4183"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaf645025d4743c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10645,7 +10695,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca634a29b774cf2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raadd981c3b214d20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10657,7 +10707,7 @@
     <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55.560001373291016" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -11976,6 +12026,34 @@
       </x:c>
       <x:c r="D96" t="str">
         <x:v>降低受到的伤害；magnitude 为减伤比例，叠层后按 1-magnitude×stacks 计算并钳制到非负。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>PoolExhaustionPolicy</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Reject</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Reject</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>达到配置活动容量时拒绝本次租用，不扩容也不回收活动玩法对象。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>PoolExhaustionPolicy</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>ReuseOldest</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>ReuseOldest</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>达到配置活动容量时先完整回收最早活动项，再服务本次租用。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11985,7 +12063,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d4cce433b284838"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b64b08622a485d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17878,7 +17956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eac9778bcbc4306"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84d7fd2765f945ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17980,7 +18058,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61466ef2b5624f36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3772f8e629274f31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18129,7 +18207,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R932ee86afbcd47b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfdf03a4cf1e4fee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18527,7 +18605,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R181dfdf719864b98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cc43361d8ef4d19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18724,7 +18802,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R962433f91274432e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd4245c8a7bf4b43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18903,7 +18981,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13b7606d87b24f8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R185dbf597fd742d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19128,7 +19206,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbe630644d454c7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce667e37e1604580"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19402,7 +19480,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f9d91e72a5049e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b62b3f1cf594287"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T460: implement configured boss phases
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7f4d87d711634e35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rcc4fc113546e4e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rcfa041b7f9554777"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R191c503333db48c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rfa416450050c4b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R79ab44b2e4c04226"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R9df341ab5b2e472a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Re9cf3d9983d246d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Rb777b95905924e2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R4fec9b62e2694eaf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R2131d4e3790b4e6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R02522fd9a5b04021"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R4a5d7b02d214490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R8363d5ba5ea0401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R4ed8d7626fc24f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R43ed07f340c140f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R8f3ccf5de5674869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R2458ea5508874e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rb0dbc78d75da4bef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R42591764330c4c79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R8333bf100457410d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R0bed47edad4f46e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rf494c164a13a4615"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R4878992e53094be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R092b6eab18a14cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rfb9bb2ee61a945c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R1a6ff06757ec4ebd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R78dfcd78ffee4139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Re0bfa18e5b764caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re2cf045416764210"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R3b740121f5ab4467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Re9c8e34000024950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R1d913b7ea0f241b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R7535c9ac28a44a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R01f029efc4d24df4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R39dc81904d8048e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rcda564763a014c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Re4080f6380444c17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R28b050c4bd124060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rd66786d691de48df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R00a1e43b194648bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Ra3bbcc9e4c374e5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Rbfe441422cb34ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R3d3f475ad2d04b23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R203a75bbf0724dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R54697e20e7c04814"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R7e31bb73957d4734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R75de355e6c2b45f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R2605a4abb5cb4f73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R46ad6b8989434a84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Re4f864a16b4943f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R035e96d58f6e46c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R58981a8c47584bdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R755ac6256df84551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R3c54ee4132d2458e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R8f4feac0f1fc4da0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R480b3cf9e7af4076"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rf4cb7ce783cd4bc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1225,7 +1225,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.5.0-sample</x:v>
+        <x:v>0.5.1-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -2066,7 +2066,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15656f69cbf04623"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cce587625294928"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2616,7 +2616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b0e08227502401a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d686e2b99e04309"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2881,7 +2881,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a817f837c094ef3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8ceb49d1dbc4fc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3145,7 +3145,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R162e08304649428c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc78bfdb4f2a4733"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3350,7 +3350,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76d6d445e86846a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5309d6310324ef5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4232,7 +4232,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb1a5bbd18e24f8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69786e764861451a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4440,7 +4440,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe5db5d316c2465f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7de966c681854d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4791,7 +4791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4faf057777dd4ac1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6319bda73362440f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4997,7 +4997,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5376b6eec422491d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5ee0381cc14c17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5123,7 +5123,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd544e1d051b46c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad434990c3e7485f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5222,7 +5222,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.5.0-sample</x:v>
+        <x:v>0.5.1-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6134,7 +6134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae2ed3777c0f4439"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra25db996df794e92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6598,7 +6598,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92e3d392b0154eab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf65cebd78960481f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6737,7 +6737,7 @@
         <x:v>0.34</x:v>
       </x:c>
       <x:c r="F6" s="35" t="str">
-        <x:v>move_boss_ground</x:v>
+        <x:v>move_boss_phase2</x:v>
       </x:c>
       <x:c r="G6" s="35" t="str">
         <x:v>attackset_boss_phase2</x:v>
@@ -6772,7 +6772,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="35" t="str">
-        <x:v>move_boss_ground</x:v>
+        <x:v>move_boss_phase3</x:v>
       </x:c>
       <x:c r="G7" s="35" t="str">
         <x:v>attackset_boss_phase3</x:v>
@@ -6797,7 +6797,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10247c7e5905487e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1f13315bfbb4748"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7013,7 +7013,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25581153c37e4904"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce2c3ace48164fe3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7303,7 +7303,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9111758c4b1749f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3803a093c6944d66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7873,7 +7873,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5189ea1c92e41f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83466eb5d6684503"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8396,7 +8396,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60343fd771da4307"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb2c15156b31421f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9340,7 +9340,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaf645025d4743c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a03264051b948dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10695,7 +10695,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raadd981c3b214d20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e27750cbf7a4cf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12063,7 +12063,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b64b08622a485d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6befdbe91a4905"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17956,7 +17956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84d7fd2765f945ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48565c517a5c423e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18058,7 +18058,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3772f8e629274f31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63089cfb88724e93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18207,7 +18207,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfdf03a4cf1e4fee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R150b8068419f46ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18605,7 +18605,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cc43361d8ef4d19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R762b2b56cb47497b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18802,7 +18802,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd4245c8a7bf4b43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f79212a19f24f58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18981,7 +18981,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R185dbf597fd742d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a91c755a24545a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19206,7 +19206,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce667e37e1604580"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8048b61aa51944bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19468,6 +19468,76 @@
         <x:v>Boss地面阶段</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>move_boss_phase2</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Boss</x:v>
+      </x:c>
+      <x:c r="C10" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="D10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="G10" t="n">
+        <x:v>0.58</x:v>
+      </x:c>
+      <x:c r="H10" t="n">
+        <x:v>0.38</x:v>
+      </x:c>
+      <x:c r="I10" t="n">
+        <x:v>0.38</x:v>
+      </x:c>
+      <x:c r="J10" s="59" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>Boss二阶段加速</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>move_boss_phase3</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Boss</x:v>
+      </x:c>
+      <x:c r="C11" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="D11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="G11" t="n">
+        <x:v>0.58</x:v>
+      </x:c>
+      <x:c r="H11" t="n">
+        <x:v>0.38</x:v>
+      </x:c>
+      <x:c r="I11" t="n">
+        <x:v>0.38</x:v>
+      </x:c>
+      <x:c r="J11" s="59" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>Boss三阶段高速</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -19480,7 +19550,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b62b3f1cf594287"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red4c3b12c8ab4ffe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T520: complete event-driven tutorial level
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re2cf045416764210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R3b740121f5ab4467"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Re9c8e34000024950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R1d913b7ea0f241b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R7535c9ac28a44a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R01f029efc4d24df4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R39dc81904d8048e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rcda564763a014c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Re4080f6380444c17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R28b050c4bd124060"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rd66786d691de48df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R00a1e43b194648bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Ra3bbcc9e4c374e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Rbfe441422cb34ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R3d3f475ad2d04b23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R203a75bbf0724dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R54697e20e7c04814"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R7e31bb73957d4734"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R75de355e6c2b45f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R2605a4abb5cb4f73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R46ad6b8989434a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Re4f864a16b4943f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R035e96d58f6e46c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R58981a8c47584bdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R755ac6256df84551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R3c54ee4132d2458e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R8f4feac0f1fc4da0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R480b3cf9e7af4076"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rf4cb7ce783cd4bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc229d3575e124972"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R8dac7f9869fe4248"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rb76fa0c73b884973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R4da01d8552b34ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rc1d4f20c9db9476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rd83a84996a944053"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R2107630479304b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R601ca44b4e9b4fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R290b4675a44b4a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R5ab627ce1cec4452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Ra61cc512f97c4235"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Re1eaa2cab71349a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rc15e794a55394a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Rfd9e25368a3142eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rc4f1a9f7ba974591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R7af8bbe4bad446b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R1898499f8a624931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R3e5c875d2ddc4610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R7494b70ba5a24271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R635fe8b23288433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R8da25e2610b84710"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rd6e8cfd57c344d09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rdaa00115a33d40b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R6cdeeeb4bf9a4254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R9f4bee6b995b4dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rbac05cbd11be4593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rf679dc16ecdb4be4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R432c9aa745db4810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R8865c43137f24fff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1225,7 +1225,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.5.1-sample</x:v>
+        <x:v>0.5.2-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1322,7 +1322,7 @@
       </x:c>
       <x:c r="E13" s="89" t="n">
         <x:f>COUNTA('Waves'!A5:A1000)</x:f>
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F13" s="92"/>
       <x:c r="G13" s="92"/>
@@ -1337,7 +1337,7 @@
       </x:c>
       <x:c r="E14" s="89" t="n">
         <x:f>COUNTA('Spawns'!A5:A1000)</x:f>
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F14" s="92"/>
       <x:c r="G14" s="92"/>
@@ -1367,7 +1367,7 @@
       </x:c>
       <x:c r="E16" s="89" t="n">
         <x:f>COUNTA('Tutorials'!A5:A1000)</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F16" s="92"/>
       <x:c r="G16" s="92"/>
@@ -2066,7 +2066,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cce587625294928"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19f5aa95a9c14757"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2616,7 +2616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d686e2b99e04309"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R759ed530bb954e7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2881,7 +2881,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8ceb49d1dbc4fc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b4597826f544b1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3145,7 +3145,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc78bfdb4f2a4733"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e54f6704b6d4c9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3350,7 +3350,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5309d6310324ef5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb72e44cd8f64534"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4232,7 +4232,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69786e764861451a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f949d5b7c834335"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4440,7 +4440,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7de966c681854d36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4993bb03be884547"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4535,13 +4535,13 @@
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G5" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="H5" s="35" t="str">
         <x:v>bgm_cave_01</x:v>
       </x:c>
       <x:c r="I5" s="68" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4564,13 +4564,13 @@
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G6" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="H6" s="35" t="str">
         <x:v>bgm_cave_01</x:v>
       </x:c>
       <x:c r="I6" s="68" t="n">
-        <x:v>7</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4599,140 +4599,140 @@
         <x:v>bgm_cave_01</x:v>
       </x:c>
       <x:c r="I7" s="68" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="35" t="str">
-        <x:v>wave_002_01</x:v>
+        <x:v>wave_001_04</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>lv_002_cave</x:v>
+        <x:v>lv_001_tutorial</x:v>
       </x:c>
       <x:c r="C8" s="68" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D8" s="35" t="str">
-        <x:v>LevelStart</x:v>
+        <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="E8" s="72" t="n">
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="F8" s="35" t="str">
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G8" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="H8" s="35" t="str">
-        <x:v>bgm_cave_02</x:v>
+        <x:v>bgm_cave_01</x:v>
       </x:c>
       <x:c r="I8" s="68" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="35" t="str">
-        <x:v>wave_002_02</x:v>
+        <x:v>wave_001_05</x:v>
       </x:c>
       <x:c r="B9" s="35" t="str">
-        <x:v>lv_002_cave</x:v>
+        <x:v>lv_001_tutorial</x:v>
       </x:c>
       <x:c r="C9" s="68" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D9" s="35" t="str">
         <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="E9" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="F9" s="35" t="str">
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G9" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="H9" s="35" t="str">
-        <x:v>bgm_cave_02</x:v>
+        <x:v>bgm_cave_01</x:v>
       </x:c>
       <x:c r="I9" s="68" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="35" t="str">
-        <x:v>wave_002_03</x:v>
+        <x:v>wave_001_06</x:v>
       </x:c>
       <x:c r="B10" s="35" t="str">
-        <x:v>lv_002_cave</x:v>
+        <x:v>lv_001_tutorial</x:v>
       </x:c>
       <x:c r="C10" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D10" s="35" t="str">
         <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="E10" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="F10" s="35" t="str">
-        <x:v>AllEnemiesDefeated</x:v>
+        <x:v>PlayerConfirmed</x:v>
       </x:c>
       <x:c r="G10" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H10" s="35" t="str">
-        <x:v>bgm_cave_02</x:v>
+        <x:v>bgm_cave_01</x:v>
       </x:c>
       <x:c r="I10" s="68" t="n">
-        <x:v>9</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="35" t="str">
-        <x:v>wave_002_04</x:v>
+        <x:v>wave_002_01</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
         <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C11" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>PreviousWaveEnd</x:v>
+        <x:v>LevelStart</x:v>
       </x:c>
       <x:c r="E11" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="35" t="str">
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G11" s="72" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="H11" s="35" t="str">
         <x:v>bgm_cave_02</x:v>
       </x:c>
       <x:c r="I11" s="68" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="35" t="str">
-        <x:v>wave_003_01</x:v>
+        <x:v>wave_002_02</x:v>
       </x:c>
       <x:c r="B12" s="35" t="str">
-        <x:v>lv_003_boss</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C12" s="68" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D12" s="35" t="str">
-        <x:v>LevelStart</x:v>
+        <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="E12" s="72" t="n">
-        <x:v>0</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="F12" s="35" t="str">
         <x:v>AllEnemiesDefeated</x:v>
@@ -4741,7 +4741,7 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="H12" s="35" t="str">
-        <x:v>bgm_boss_intro</x:v>
+        <x:v>bgm_cave_02</x:v>
       </x:c>
       <x:c r="I12" s="68" t="n">
         <x:v>8</x:v>
@@ -4749,30 +4749,117 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="35" t="str">
-        <x:v>wave_003_02</x:v>
+        <x:v>wave_002_03</x:v>
       </x:c>
       <x:c r="B13" s="35" t="str">
-        <x:v>lv_003_boss</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C13" s="68" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D13" s="35" t="str">
         <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="E13" s="72" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="F13" s="35" t="str">
+        <x:v>AllEnemiesDefeated</x:v>
+      </x:c>
+      <x:c r="G13" s="72" t="n">
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="F13" s="35" t="str">
+      <x:c r="H13" s="35" t="str">
+        <x:v>bgm_cave_02</x:v>
+      </x:c>
+      <x:c r="I13" s="68" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>wave_002_04</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>lv_002_cave</x:v>
+      </x:c>
+      <x:c r="C14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>PreviousWaveEnd</x:v>
+      </x:c>
+      <x:c r="E14" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>AllEnemiesDefeated</x:v>
+      </x:c>
+      <x:c r="G14" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>bgm_cave_02</x:v>
+      </x:c>
+      <x:c r="I14" t="n">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>lv_003_boss</x:v>
+      </x:c>
+      <x:c r="C15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>LevelStart</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>AllEnemiesDefeated</x:v>
+      </x:c>
+      <x:c r="G15" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>bgm_boss_intro</x:v>
+      </x:c>
+      <x:c r="I15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>wave_003_02</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>lv_003_boss</x:v>
+      </x:c>
+      <x:c r="C16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>PreviousWaveEnd</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
         <x:v>BossDefeated</x:v>
       </x:c>
-      <x:c r="G13" s="72" t="n">
+      <x:c r="G16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H13" s="35" t="str">
+      <x:c r="H16" t="str">
         <x:v>bgm_boss</x:v>
       </x:c>
-      <x:c r="I13" s="68" t="n">
+      <x:c r="I16" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -4791,7 +4878,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6319bda73362440f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3059ac0cdd4aee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4997,7 +5084,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5ee0381cc14c17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c5654bfabe64eb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5123,7 +5210,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad434990c3e7485f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cda310cedbe47ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5222,7 +5309,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.5.1-sample</x:v>
+        <x:v>0.5.2-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6134,7 +6221,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra25db996df794e92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f4ad52ca8e498d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6223,7 +6310,7 @@
         <x:v>enemy_fire_fish</x:v>
       </x:c>
       <x:c r="E5" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F5" s="72" t="n">
         <x:v>0.7</x:v>
@@ -6249,19 +6336,19 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D6" s="35" t="str">
-        <x:v>enemy_wheel_zombie</x:v>
+        <x:v>enemy_talisman_bat</x:v>
       </x:c>
       <x:c r="E6" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="72" t="n">
-        <x:v>0.65</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="35" t="str">
-        <x:v>spawn_ground_right</x:v>
+        <x:v>spawn_air_high</x:v>
       </x:c>
       <x:c r="H6" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Single</x:v>
       </x:c>
       <x:c r="I6" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6278,16 +6365,16 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str">
-        <x:v>enemy_fire_fish</x:v>
+        <x:v>enemy_wheel_zombie</x:v>
       </x:c>
       <x:c r="E7" s="68" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F7" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="35" t="str">
-        <x:v>spawn_air_high</x:v>
+        <x:v>spawn_ground_right</x:v>
       </x:c>
       <x:c r="H7" s="35" t="str">
         <x:v>Line</x:v>
@@ -6298,28 +6385,28 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="35" t="str">
-        <x:v>spawn_001_03_b</x:v>
+        <x:v>spawn_001_04_a</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>wave_001_03</x:v>
+        <x:v>wave_001_04</x:v>
       </x:c>
       <x:c r="C8" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="D8" s="35" t="str">
-        <x:v>enemy_stone_turtle</x:v>
+        <x:v>enemy_fire_fish</x:v>
       </x:c>
       <x:c r="E8" s="68" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="72" t="n">
-        <x:v>0</x:v>
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="G8" s="35" t="str">
-        <x:v>spawn_ground_right</x:v>
+        <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H8" s="35" t="str">
-        <x:v>Single</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I8" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6327,10 +6414,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="35" t="str">
-        <x:v>spawn_002_01_a</x:v>
+        <x:v>spawn_001_05_a</x:v>
       </x:c>
       <x:c r="B9" s="35" t="str">
-        <x:v>wave_002_01</x:v>
+        <x:v>wave_001_05</x:v>
       </x:c>
       <x:c r="C9" s="72" t="n">
         <x:v>0.2</x:v>
@@ -6339,7 +6426,7 @@
         <x:v>enemy_skeleton_ghost</x:v>
       </x:c>
       <x:c r="E9" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F9" s="72" t="n">
         <x:v>0.7</x:v>
@@ -6356,28 +6443,28 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="35" t="str">
-        <x:v>spawn_002_02_a</x:v>
+        <x:v>spawn_001_06_a</x:v>
       </x:c>
       <x:c r="B10" s="35" t="str">
-        <x:v>wave_002_02</x:v>
+        <x:v>wave_001_06</x:v>
       </x:c>
       <x:c r="C10" s="72" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="35" t="str">
-        <x:v>enemy_talisman_bat</x:v>
+        <x:v>enemy_fire_fish</x:v>
       </x:c>
       <x:c r="E10" s="68" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="F10" s="72" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="35" t="str">
-        <x:v>spawn_air_high</x:v>
+        <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H10" s="35" t="str">
-        <x:v>Stagger</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I10" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6385,28 +6472,28 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="35" t="str">
-        <x:v>spawn_002_03_a</x:v>
+        <x:v>spawn_002_01_a</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
-        <x:v>wave_002_03</x:v>
+        <x:v>wave_002_01</x:v>
       </x:c>
       <x:c r="C11" s="72" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>enemy_stone_turtle</x:v>
+        <x:v>enemy_skeleton_ghost</x:v>
       </x:c>
       <x:c r="E11" s="68" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F11" s="72" t="n">
-        <x:v>1</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="G11" s="35" t="str">
-        <x:v>spawn_ground_right</x:v>
+        <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H11" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Scatter</x:v>
       </x:c>
       <x:c r="I11" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6414,28 +6501,28 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="35" t="str">
-        <x:v>spawn_002_03_b</x:v>
+        <x:v>spawn_002_02_a</x:v>
       </x:c>
       <x:c r="B12" s="35" t="str">
-        <x:v>wave_002_03</x:v>
+        <x:v>wave_002_02</x:v>
       </x:c>
       <x:c r="C12" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="D12" s="35" t="str">
-        <x:v>enemy_skeleton_ghost</x:v>
+        <x:v>enemy_talisman_bat</x:v>
       </x:c>
       <x:c r="E12" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F12" s="72" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="G12" s="35" t="str">
-        <x:v>spawn_air_mid</x:v>
+        <x:v>spawn_air_high</x:v>
       </x:c>
       <x:c r="H12" s="35" t="str">
-        <x:v>Scatter</x:v>
+        <x:v>Stagger</x:v>
       </x:c>
       <x:c r="I12" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6443,57 +6530,57 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="35" t="str">
-        <x:v>spawn_002_04_a</x:v>
+        <x:v>spawn_002_03_a</x:v>
       </x:c>
       <x:c r="B13" s="35" t="str">
-        <x:v>wave_002_04</x:v>
+        <x:v>wave_002_03</x:v>
       </x:c>
       <x:c r="C13" s="72" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D13" s="35" t="str">
-        <x:v>enemy_soul_puppet</x:v>
+        <x:v>enemy_stone_turtle</x:v>
       </x:c>
       <x:c r="E13" s="68" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F13" s="72" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="35" t="str">
-        <x:v>spawn_air_mid</x:v>
+        <x:v>spawn_ground_right</x:v>
       </x:c>
       <x:c r="H13" s="35" t="str">
-        <x:v>Single</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I13" s="35" t="str">
-        <x:v>modifier_elite</x:v>
+        <x:v>modifier_none</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="35" t="str">
-        <x:v>spawn_002_04_b</x:v>
+        <x:v>spawn_002_03_b</x:v>
       </x:c>
       <x:c r="B14" s="35" t="str">
-        <x:v>wave_002_04</x:v>
+        <x:v>wave_002_03</x:v>
       </x:c>
       <x:c r="C14" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="D14" s="35" t="str">
-        <x:v>enemy_wheel_zombie</x:v>
+        <x:v>enemy_skeleton_ghost</x:v>
       </x:c>
       <x:c r="E14" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F14" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="G14" s="35" t="str">
-        <x:v>spawn_ground_right</x:v>
+        <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H14" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Scatter</x:v>
       </x:c>
       <x:c r="I14" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6501,57 +6588,57 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="35" t="str">
-        <x:v>spawn_003_01_a</x:v>
+        <x:v>spawn_002_04_a</x:v>
       </x:c>
       <x:c r="B15" s="35" t="str">
-        <x:v>wave_003_01</x:v>
+        <x:v>wave_002_04</x:v>
       </x:c>
       <x:c r="C15" s="72" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D15" s="35" t="str">
-        <x:v>enemy_fire_fish</x:v>
+        <x:v>enemy_soul_puppet</x:v>
       </x:c>
       <x:c r="E15" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F15" s="72" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="35" t="str">
         <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H15" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Single</x:v>
       </x:c>
       <x:c r="I15" s="35" t="str">
-        <x:v>modifier_none</x:v>
+        <x:v>modifier_elite</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="35" t="str">
-        <x:v>spawn_003_01_b</x:v>
+        <x:v>spawn_002_04_b</x:v>
       </x:c>
       <x:c r="B16" s="35" t="str">
-        <x:v>wave_003_01</x:v>
+        <x:v>wave_002_04</x:v>
       </x:c>
       <x:c r="C16" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="D16" s="35" t="str">
-        <x:v>enemy_talisman_bat</x:v>
+        <x:v>enemy_wheel_zombie</x:v>
       </x:c>
       <x:c r="E16" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F16" s="72" t="n">
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="G16" s="35" t="str">
-        <x:v>spawn_air_high</x:v>
+        <x:v>spawn_ground_right</x:v>
       </x:c>
       <x:c r="H16" s="35" t="str">
-        <x:v>Stagger</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I16" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6559,30 +6646,88 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="35" t="str">
+        <x:v>spawn_003_01_a</x:v>
+      </x:c>
+      <x:c r="B17" s="35" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="C17" s="72" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D17" s="35" t="str">
+        <x:v>enemy_fire_fish</x:v>
+      </x:c>
+      <x:c r="E17" s="68" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F17" s="72" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G17" s="35" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H17" s="35" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="I17" s="35" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>spawn_003_01_b</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="C18" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>enemy_talisman_bat</x:v>
+      </x:c>
+      <x:c r="E18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F18" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>spawn_air_high</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Stagger</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
         <x:v>spawn_003_02_a</x:v>
       </x:c>
-      <x:c r="B17" s="35" t="str">
+      <x:c r="B19" t="str">
         <x:v>wave_003_02</x:v>
       </x:c>
-      <x:c r="C17" s="72" t="n">
+      <x:c r="C19" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D17" s="35" t="str">
+      <x:c r="D19" t="str">
         <x:v>boss_tomb_king</x:v>
       </x:c>
-      <x:c r="E17" s="68" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F17" s="72" t="n">
+      <x:c r="E19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F19" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G17" s="35" t="str">
+      <x:c r="G19" t="str">
         <x:v>spawn_boss</x:v>
       </x:c>
-      <x:c r="H17" s="35" t="str">
+      <x:c r="H19" t="str">
         <x:v>Single</x:v>
       </x:c>
-      <x:c r="I17" s="35" t="str">
+      <x:c r="I19" t="str">
         <x:v>modifier_none</x:v>
       </x:c>
     </x:row>
@@ -6598,7 +6743,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf65cebd78960481f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcedc05cd541a498a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6797,7 +6942,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1f13315bfbb4748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89159d23861941f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7013,7 +7158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce2c3ace48164fe3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3ceb3fb1e8a4f73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7206,13 +7351,13 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="35" t="str">
-        <x:v>tutorial_level_002</x:v>
+        <x:v>tutorial_level_001</x:v>
       </x:c>
       <x:c r="B9" s="68" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="35" t="str">
-        <x:v>ArmoredEnemySpawned</x:v>
+        <x:v>GhostSpawned</x:v>
       </x:c>
       <x:c r="D9" s="65" t="b">
         <x:v>1</x:v>
@@ -7221,27 +7366,27 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="F9" s="35" t="str">
-        <x:v>ArmorBroken</x:v>
+        <x:v>StanceChanged</x:v>
       </x:c>
       <x:c r="G9" s="35" t="str">
-        <x:v>text_tutorial_charge</x:v>
+        <x:v>text_tutorial_stance</x:v>
       </x:c>
       <x:c r="H9" s="35" t="str">
-        <x:v>Enemy</x:v>
+        <x:v>SwitchButton</x:v>
       </x:c>
       <x:c r="I9" s="35" t="str">
-        <x:v>Charged</x:v>
+        <x:v>Any</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="35" t="str">
-        <x:v>tutorial_level_002</x:v>
+        <x:v>tutorial_level_001</x:v>
       </x:c>
       <x:c r="B10" s="68" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C10" s="35" t="str">
-        <x:v>GhostSpawned</x:v>
+        <x:v>UltimateReady</x:v>
       </x:c>
       <x:c r="D10" s="65" t="b">
         <x:v>1</x:v>
@@ -7250,27 +7395,27 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="F10" s="35" t="str">
-        <x:v>StanceChanged</x:v>
+        <x:v>UltimateSucceeded</x:v>
       </x:c>
       <x:c r="G10" s="35" t="str">
-        <x:v>text_tutorial_stance</x:v>
+        <x:v>text_tutorial_ultimate</x:v>
       </x:c>
       <x:c r="H10" s="35" t="str">
-        <x:v>SwitchButton</x:v>
+        <x:v>UltimateButton</x:v>
       </x:c>
       <x:c r="I10" s="35" t="str">
-        <x:v>Any</x:v>
+        <x:v>Circle</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="35" t="str">
-        <x:v>tutorial_level_003</x:v>
+        <x:v>tutorial_level_002</x:v>
       </x:c>
       <x:c r="B11" s="68" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
-        <x:v>UltimateReady</x:v>
+        <x:v>ArmoredEnemySpawned</x:v>
       </x:c>
       <x:c r="D11" s="65" t="b">
         <x:v>1</x:v>
@@ -7279,15 +7424,44 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="F11" s="35" t="str">
+        <x:v>ArmorBroken</x:v>
+      </x:c>
+      <x:c r="G11" s="35" t="str">
+        <x:v>text_tutorial_charge</x:v>
+      </x:c>
+      <x:c r="H11" s="35" t="str">
+        <x:v>Enemy</x:v>
+      </x:c>
+      <x:c r="I11" s="35" t="str">
+        <x:v>Charged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>tutorial_level_003</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>UltimateReady</x:v>
+      </x:c>
+      <x:c r="D12" s="59" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
         <x:v>UltimateSucceeded</x:v>
       </x:c>
-      <x:c r="G11" s="35" t="str">
+      <x:c r="G12" t="str">
         <x:v>text_tutorial_ultimate</x:v>
       </x:c>
-      <x:c r="H11" s="35" t="str">
+      <x:c r="H12" t="str">
         <x:v>UltimateButton</x:v>
       </x:c>
-      <x:c r="I11" s="35" t="str">
+      <x:c r="I12" t="str">
         <x:v>Circle</x:v>
       </x:c>
     </x:row>
@@ -7303,7 +7477,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3803a093c6944d66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R821faf98aa6640d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7873,7 +8047,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83466eb5d6684503"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b54427245df4a11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8396,7 +8570,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb2c15156b31421f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e01b7280319463d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9340,7 +9514,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a03264051b948dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13b0c42d8e1346bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10695,7 +10869,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e27750cbf7a4cf7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf18da0473e9439b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12063,7 +12237,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6befdbe91a4905"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d7eacc0c1242f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17956,7 +18130,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48565c517a5c423e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9467981ea6954335"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18058,7 +18232,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63089cfb88724e93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c52f6516acc4ba4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18207,7 +18381,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R150b8068419f46ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc45804d113494f5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18605,7 +18779,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R762b2b56cb47497b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R028b23e40cdd402a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18802,7 +18976,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f79212a19f24f58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b668b20559940d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18981,7 +19155,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a91c755a24545a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R066535da8759416c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19206,7 +19380,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8048b61aa51944bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7d0910aefd14687"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19550,7 +19724,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red4c3b12c8ab4ffe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04bd4ae5c05f479d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T530: complete configured mixed-enemy level
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc229d3575e124972"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R8dac7f9869fe4248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rb76fa0c73b884973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R4da01d8552b34ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rc1d4f20c9db9476c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rd83a84996a944053"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R2107630479304b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R601ca44b4e9b4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R290b4675a44b4a0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R5ab627ce1cec4452"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Ra61cc512f97c4235"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Re1eaa2cab71349a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rc15e794a55394a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Rfd9e25368a3142eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rc4f1a9f7ba974591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R7af8bbe4bad446b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R1898499f8a624931"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R3e5c875d2ddc4610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R7494b70ba5a24271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R635fe8b23288433e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R8da25e2610b84710"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rd6e8cfd57c344d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rdaa00115a33d40b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R6cdeeeb4bf9a4254"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R9f4bee6b995b4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rbac05cbd11be4593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rf679dc16ecdb4be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R432c9aa745db4810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R8865c43137f24fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0675803d98704ffd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rc52c5fa600614d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rb2b0725926a944ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R031d2723a02043d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rd9abb8b9b6c54fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rb1589adfbdab42f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rdb69058359814142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Ra6433fbc686648c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R4c93be90f90240f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rba3d80a970a74221"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rcd6313e0f0db4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rf175b4d1a40b434d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R91a7d2fa75074b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R6c2fa12223cd4e3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rff5bfb10ea8e4bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R6e0cd8ad26794f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R980093995041466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rb320644da7aa4fcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Ra297430a262e4a97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rdeb4223ed4c240b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R47ec3bde5733491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rb8219902f4c74d54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Ra2682a697e674d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R71dc394ac0954d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rb4393d9d64984def"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rc0e178a66d714d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R9d6616b8373d4807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R33b9bf4ec6144706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R0a1ce8e658eb44a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -162,7 +162,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="121">
+  <x:cellXfs count="122">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -490,6 +490,7 @@
     <x:xf numFmtId="201" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -659,7 +660,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="TblWaves" displayName="TblWaves" ref="A4:I13" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="TblWaves" displayName="TblWaves" ref="A4:I17" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="waveId"/>
     <x:tableColumn id="2" name="levelId"/>
@@ -709,7 +710,7 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="TblSpawns" displayName="TblSpawns" ref="A4:I17" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="TblSpawns" displayName="TblSpawns" ref="A4:I34" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="spawnId"/>
     <x:tableColumn id="2" name="waveId"/>
@@ -1225,7 +1226,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.5.2-sample</x:v>
+        <x:v>0.5.3-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1322,7 +1323,7 @@
       </x:c>
       <x:c r="E13" s="89" t="n">
         <x:f>COUNTA('Waves'!A5:A1000)</x:f>
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F13" s="92"/>
       <x:c r="G13" s="92"/>
@@ -1337,7 +1338,7 @@
       </x:c>
       <x:c r="E14" s="89" t="n">
         <x:f>COUNTA('Spawns'!A5:A1000)</x:f>
-        <x:v>15</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F14" s="92"/>
       <x:c r="G14" s="92"/>
@@ -2066,7 +2067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19f5aa95a9c14757"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fab6629fcc040d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2616,7 +2617,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R759ed530bb954e7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6edefb12106041d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2881,7 +2882,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b4597826f544b1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R240ee3c9789f4732"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3145,7 +3146,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e54f6704b6d4c9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2823b811ce5449d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3350,7 +3351,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb72e44cd8f64534"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c3470e76b1b4865"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4232,7 +4233,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f949d5b7c834335"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R385d77a9e8614ea6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4384,13 +4385,13 @@
         <x:v>reward_level_002</x:v>
       </x:c>
       <x:c r="H6" s="35" t="n">
-        <x:v>3500</x:v>
+        <x:v>6500</x:v>
       </x:c>
       <x:c r="I6" s="35" t="n">
-        <x:v>5800</x:v>
+        <x:v>9500</x:v>
       </x:c>
       <x:c r="J6" s="35" t="n">
-        <x:v>8000</x:v>
+        <x:v>13000</x:v>
       </x:c>
       <x:c r="K6" s="35" t="str">
         <x:v>tutorial_level_002</x:v>
@@ -4440,7 +4441,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4993bb03be884547"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R008be588948644bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4715,7 +4716,7 @@
         <x:v>bgm_cave_02</x:v>
       </x:c>
       <x:c r="I11" s="68" t="n">
-        <x:v>7</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4738,13 +4739,13 @@
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G12" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="H12" s="35" t="str">
         <x:v>bgm_cave_02</x:v>
       </x:c>
       <x:c r="I12" s="68" t="n">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4767,13 +4768,13 @@
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G13" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="H13" s="35" t="str">
         <x:v>bgm_cave_02</x:v>
       </x:c>
       <x:c r="I13" s="68" t="n">
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4789,77 +4790,193 @@
       <x:c r="D14" t="str">
         <x:v>PreviousWaveEnd</x:v>
       </x:c>
-      <x:c r="E14" t="n">
-        <x:v>0.6</x:v>
+      <x:c r="E14" s="121" t="n">
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="F14" t="str">
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
-      <x:c r="G14" t="n">
-        <x:v>0.5</x:v>
+      <x:c r="G14" s="121" t="n">
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="H14" t="str">
         <x:v>bgm_cave_02</x:v>
       </x:c>
       <x:c r="I14" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>wave_003_01</x:v>
+        <x:v>wave_002_05</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>lv_003_boss</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C15" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>LevelStart</x:v>
-      </x:c>
-      <x:c r="E15" t="n">
-        <x:v>0</x:v>
+        <x:v>PreviousWaveEnd</x:v>
+      </x:c>
+      <x:c r="E15" s="121" t="n">
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="F15" t="str">
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
-      <x:c r="G15" t="n">
-        <x:v>0.8</x:v>
+      <x:c r="G15" s="121" t="n">
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="H15" t="str">
-        <x:v>bgm_boss_intro</x:v>
+        <x:v>bgm_cave_02</x:v>
       </x:c>
       <x:c r="I15" t="n">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>wave_003_02</x:v>
+        <x:v>wave_002_06</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>lv_003_boss</x:v>
+        <x:v>lv_002_cave</x:v>
       </x:c>
       <x:c r="C16" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D16" t="str">
         <x:v>PreviousWaveEnd</x:v>
       </x:c>
-      <x:c r="E16" t="n">
+      <x:c r="E16" s="121" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>AllEnemiesDefeated</x:v>
+      </x:c>
+      <x:c r="G16" s="121" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>bgm_cave_02</x:v>
+      </x:c>
+      <x:c r="I16" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>wave_002_07</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>lv_002_cave</x:v>
+      </x:c>
+      <x:c r="C17" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>PreviousWaveEnd</x:v>
+      </x:c>
+      <x:c r="E17" s="121" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>AllEnemiesDefeated</x:v>
+      </x:c>
+      <x:c r="G17" s="121" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>bgm_cave_02</x:v>
+      </x:c>
+      <x:c r="I17" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>wave_002_08</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>lv_002_cave</x:v>
+      </x:c>
+      <x:c r="C18" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>PreviousWaveEnd</x:v>
+      </x:c>
+      <x:c r="E18" s="121" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>AllEnemiesDefeated</x:v>
+      </x:c>
+      <x:c r="G18" s="121" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>bgm_cave_02</x:v>
+      </x:c>
+      <x:c r="I18" t="n">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>lv_003_boss</x:v>
+      </x:c>
+      <x:c r="C19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>LevelStart</x:v>
+      </x:c>
+      <x:c r="E19" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>AllEnemiesDefeated</x:v>
+      </x:c>
+      <x:c r="G19" s="121" t="n">
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="F16" t="str">
+      <x:c r="H19" t="str">
+        <x:v>bgm_boss_intro</x:v>
+      </x:c>
+      <x:c r="I19" t="n">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>wave_003_02</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>lv_003_boss</x:v>
+      </x:c>
+      <x:c r="C20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>PreviousWaveEnd</x:v>
+      </x:c>
+      <x:c r="E20" s="121" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
         <x:v>BossDefeated</x:v>
       </x:c>
-      <x:c r="G16" t="n">
+      <x:c r="G20" s="121" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H16" t="str">
+      <x:c r="H20" t="str">
         <x:v>bgm_boss</x:v>
       </x:c>
-      <x:c r="I16" t="n">
+      <x:c r="I20" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -4878,7 +4995,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3059ac0cdd4aee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f5fe4a3a0734524"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5084,7 +5201,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c5654bfabe64eb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe211b74ab654203"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5210,7 +5327,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cda310cedbe47ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re90dd2b015eb4995"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5309,7 +5426,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.5.2-sample</x:v>
+        <x:v>0.5.3-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6221,7 +6338,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f4ad52ca8e498d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d64bcc5ce8d4f71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6481,10 +6598,10 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>enemy_skeleton_ghost</x:v>
+        <x:v>enemy_fire_fish</x:v>
       </x:c>
       <x:c r="E11" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F11" s="72" t="n">
         <x:v>0.7</x:v>
@@ -6493,7 +6610,7 @@
         <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H11" s="35" t="str">
-        <x:v>Scatter</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I11" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6501,28 +6618,28 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="35" t="str">
-        <x:v>spawn_002_02_a</x:v>
+        <x:v>spawn_002_01_b</x:v>
       </x:c>
       <x:c r="B12" s="35" t="str">
-        <x:v>wave_002_02</x:v>
+        <x:v>wave_002_01</x:v>
       </x:c>
       <x:c r="C12" s="72" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="D12" s="35" t="str">
-        <x:v>enemy_talisman_bat</x:v>
+        <x:v>enemy_wheel_zombie</x:v>
       </x:c>
       <x:c r="E12" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F12" s="72" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="G12" s="35" t="str">
-        <x:v>spawn_air_high</x:v>
+        <x:v>spawn_ground_right</x:v>
       </x:c>
       <x:c r="H12" s="35" t="str">
-        <x:v>Stagger</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I12" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6530,28 +6647,28 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="35" t="str">
-        <x:v>spawn_002_03_a</x:v>
+        <x:v>spawn_002_02_a</x:v>
       </x:c>
       <x:c r="B13" s="35" t="str">
-        <x:v>wave_002_03</x:v>
+        <x:v>wave_002_02</x:v>
       </x:c>
       <x:c r="C13" s="72" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D13" s="35" t="str">
-        <x:v>enemy_stone_turtle</x:v>
+        <x:v>enemy_talisman_bat</x:v>
       </x:c>
       <x:c r="E13" s="68" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F13" s="72" t="n">
-        <x:v>1</x:v>
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="G13" s="35" t="str">
-        <x:v>spawn_ground_right</x:v>
+        <x:v>spawn_air_high</x:v>
       </x:c>
       <x:c r="H13" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Stagger</x:v>
       </x:c>
       <x:c r="I13" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6559,28 +6676,28 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="35" t="str">
-        <x:v>spawn_002_03_b</x:v>
+        <x:v>spawn_002_02_b</x:v>
       </x:c>
       <x:c r="B14" s="35" t="str">
-        <x:v>wave_002_03</x:v>
+        <x:v>wave_002_02</x:v>
       </x:c>
       <x:c r="C14" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="35" t="str">
-        <x:v>enemy_skeleton_ghost</x:v>
+        <x:v>enemy_fire_fish</x:v>
       </x:c>
       <x:c r="E14" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F14" s="72" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="G14" s="35" t="str">
         <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H14" s="35" t="str">
-        <x:v>Scatter</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I14" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6588,57 +6705,57 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="35" t="str">
-        <x:v>spawn_002_04_a</x:v>
+        <x:v>spawn_002_03_a</x:v>
       </x:c>
       <x:c r="B15" s="35" t="str">
-        <x:v>wave_002_04</x:v>
+        <x:v>wave_002_03</x:v>
       </x:c>
       <x:c r="C15" s="72" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D15" s="35" t="str">
-        <x:v>enemy_soul_puppet</x:v>
+        <x:v>enemy_stone_turtle</x:v>
       </x:c>
       <x:c r="E15" s="68" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F15" s="72" t="n">
-        <x:v>0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="G15" s="35" t="str">
-        <x:v>spawn_air_mid</x:v>
+        <x:v>spawn_ground_right</x:v>
       </x:c>
       <x:c r="H15" s="35" t="str">
-        <x:v>Single</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I15" s="35" t="str">
-        <x:v>modifier_elite</x:v>
+        <x:v>modifier_none</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="35" t="str">
-        <x:v>spawn_002_04_b</x:v>
+        <x:v>spawn_002_03_b</x:v>
       </x:c>
       <x:c r="B16" s="35" t="str">
-        <x:v>wave_002_04</x:v>
+        <x:v>wave_002_03</x:v>
       </x:c>
       <x:c r="C16" s="72" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="D16" s="35" t="str">
         <x:v>enemy_wheel_zombie</x:v>
       </x:c>
       <x:c r="E16" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F16" s="72" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="G16" s="35" t="str">
         <x:v>spawn_ground_right</x:v>
       </x:c>
       <x:c r="H16" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Stagger</x:v>
       </x:c>
       <x:c r="I16" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6646,28 +6763,28 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="35" t="str">
-        <x:v>spawn_003_01_a</x:v>
+        <x:v>spawn_002_04_a</x:v>
       </x:c>
       <x:c r="B17" s="35" t="str">
-        <x:v>wave_003_01</x:v>
+        <x:v>wave_002_04</x:v>
       </x:c>
       <x:c r="C17" s="72" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D17" s="35" t="str">
-        <x:v>enemy_fire_fish</x:v>
+        <x:v>enemy_skeleton_ghost</x:v>
       </x:c>
       <x:c r="E17" s="68" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F17" s="72" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="G17" s="35" t="str">
         <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H17" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Scatter</x:v>
       </x:c>
       <x:c r="I17" s="35" t="str">
         <x:v>modifier_none</x:v>
@@ -6675,28 +6792,28 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>spawn_003_01_b</x:v>
+        <x:v>spawn_002_04_b</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>wave_003_01</x:v>
-      </x:c>
-      <x:c r="C18" t="n">
-        <x:v>0.6</x:v>
+        <x:v>wave_002_04</x:v>
+      </x:c>
+      <x:c r="C18" s="121" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>enemy_talisman_bat</x:v>
+        <x:v>enemy_fire_fish</x:v>
       </x:c>
       <x:c r="E18" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F18" t="n">
-        <x:v>0.6</x:v>
+      <x:c r="F18" s="121" t="n">
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="G18" t="str">
         <x:v>spawn_air_high</x:v>
       </x:c>
       <x:c r="H18" t="str">
-        <x:v>Stagger</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="I18" t="str">
         <x:v>modifier_none</x:v>
@@ -6704,30 +6821,523 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>spawn_003_02_a</x:v>
+        <x:v>spawn_002_05_a</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>wave_003_02</x:v>
-      </x:c>
-      <x:c r="C19" t="n">
+        <x:v>wave_002_05</x:v>
+      </x:c>
+      <x:c r="C19" s="121" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>enemy_soul_puppet</x:v>
+      </x:c>
+      <x:c r="E19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F19" s="121" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D19" t="str">
-        <x:v>boss_tomb_king</x:v>
-      </x:c>
-      <x:c r="E19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F19" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="G19" t="str">
-        <x:v>spawn_boss</x:v>
+        <x:v>spawn_air_mid</x:v>
       </x:c>
       <x:c r="H19" t="str">
         <x:v>Single</x:v>
       </x:c>
       <x:c r="I19" t="str">
+        <x:v>modifier_elite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>spawn_002_05_b</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>wave_002_05</x:v>
+      </x:c>
+      <x:c r="C20" s="121" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>enemy_wheel_zombie</x:v>
+      </x:c>
+      <x:c r="E20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F20" s="121" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>spawn_ground_right</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>spawn_002_05_c</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>wave_002_05</x:v>
+      </x:c>
+      <x:c r="C21" s="121" t="n">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>enemy_fire_fish</x:v>
+      </x:c>
+      <x:c r="E21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F21" s="121" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>spawn_air_high</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Stagger</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>spawn_002_06_a</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>wave_002_06</x:v>
+      </x:c>
+      <x:c r="C22" s="121" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>enemy_stone_turtle</x:v>
+      </x:c>
+      <x:c r="E22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F22" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>spawn_ground_right</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>spawn_002_06_b</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>wave_002_06</x:v>
+      </x:c>
+      <x:c r="C23" s="121" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>enemy_skeleton_ghost</x:v>
+      </x:c>
+      <x:c r="E23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F23" s="121" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Scatter</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>spawn_002_06_c</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>wave_002_06</x:v>
+      </x:c>
+      <x:c r="C24" s="121" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>enemy_talisman_bat</x:v>
+      </x:c>
+      <x:c r="E24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F24" s="121" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>spawn_air_high</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Stagger</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>spawn_002_07_a</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>wave_002_07</x:v>
+      </x:c>
+      <x:c r="C25" s="121" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>enemy_soul_puppet</x:v>
+      </x:c>
+      <x:c r="E25" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F25" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>modifier_elite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>spawn_002_07_b</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>wave_002_07</x:v>
+      </x:c>
+      <x:c r="C26" s="121" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>enemy_skeleton_ghost</x:v>
+      </x:c>
+      <x:c r="E26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F26" s="121" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Scatter</x:v>
+      </x:c>
+      <x:c r="I26" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>spawn_002_07_c</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>wave_002_07</x:v>
+      </x:c>
+      <x:c r="C27" s="121" t="n">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>enemy_fire_fish</x:v>
+      </x:c>
+      <x:c r="E27" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F27" s="121" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>spawn_air_high</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="I27" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>spawn_002_08_a</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>wave_002_08</x:v>
+      </x:c>
+      <x:c r="C28" s="121" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>enemy_soul_puppet</x:v>
+      </x:c>
+      <x:c r="E28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F28" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>modifier_elite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>spawn_002_08_b</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>wave_002_08</x:v>
+      </x:c>
+      <x:c r="C29" s="121" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>enemy_stone_turtle</x:v>
+      </x:c>
+      <x:c r="E29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F29" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>spawn_ground_right</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>spawn_002_08_c</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>wave_002_08</x:v>
+      </x:c>
+      <x:c r="C30" s="121" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>enemy_skeleton_ghost</x:v>
+      </x:c>
+      <x:c r="E30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F30" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>spawn_002_08_d</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>wave_002_08</x:v>
+      </x:c>
+      <x:c r="C31" s="121" t="n">
+        <x:v>2.6</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>enemy_talisman_bat</x:v>
+      </x:c>
+      <x:c r="E31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F31" s="121" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>spawn_air_high</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Stagger</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>spawn_002_08_e</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>wave_002_08</x:v>
+      </x:c>
+      <x:c r="C32" s="121" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>enemy_wheel_zombie</x:v>
+      </x:c>
+      <x:c r="E32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F32" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>spawn_ground_right</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>spawn_002_08_f</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>wave_002_08</x:v>
+      </x:c>
+      <x:c r="C33" s="121" t="n">
+        <x:v>3.8</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>enemy_fire_fish</x:v>
+      </x:c>
+      <x:c r="E33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F33" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>spawn_003_01_a</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="C34" s="121" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>enemy_fire_fish</x:v>
+      </x:c>
+      <x:c r="E34" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F34" s="121" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>spawn_003_01_b</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="C35" s="121" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>enemy_talisman_bat</x:v>
+      </x:c>
+      <x:c r="E35" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F35" s="121" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>spawn_air_high</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>Stagger</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>spawn_003_02_a</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>wave_003_02</x:v>
+      </x:c>
+      <x:c r="C36" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>boss_tomb_king</x:v>
+      </x:c>
+      <x:c r="E36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F36" s="121" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>spawn_boss</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
         <x:v>modifier_none</x:v>
       </x:c>
     </x:row>
@@ -6743,7 +7353,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcedc05cd541a498a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98ec7ce130aa4135"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6942,7 +7552,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89159d23861941f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dbfd3690fc04b24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7158,7 +7768,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3ceb3fb1e8a4f73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374d265fbe174141"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7477,7 +8087,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R821faf98aa6640d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf00bb55672bc4c37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8047,7 +8657,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b54427245df4a11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa03141f8a8a42b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8570,7 +9180,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e01b7280319463d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f639ef963d04767"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9514,7 +10124,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13b0c42d8e1346bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2db11cb599f2406d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10869,7 +11479,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf18da0473e9439b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1dfe04069b94d14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12237,7 +12847,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d7eacc0c1242f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55acb1b9a19a41f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18130,7 +18740,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9467981ea6954335"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab292e68a0a94536"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18232,7 +18842,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c52f6516acc4ba4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc52fcea244f943f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18381,7 +18991,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc45804d113494f5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97379df43fba4e46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18779,7 +19389,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R028b23e40cdd402a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf997c936eae44656"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18976,7 +19586,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b668b20559940d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R740324c7174d4210"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19155,7 +19765,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R066535da8759416c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d88fdb06b494813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19380,7 +19990,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7d0910aefd14687"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0cc15571ca44488"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19724,7 +20334,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04bd4ae5c05f479d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3553686bc6e44353"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T540: complete configured boss level
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0675803d98704ffd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rc52c5fa600614d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rb2b0725926a944ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R031d2723a02043d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rd9abb8b9b6c54fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rb1589adfbdab42f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rdb69058359814142"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Ra6433fbc686648c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R4c93be90f90240f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rba3d80a970a74221"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rcd6313e0f0db4a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rf175b4d1a40b434d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R91a7d2fa75074b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R6c2fa12223cd4e3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rff5bfb10ea8e4bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R6e0cd8ad26794f91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R980093995041466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rb320644da7aa4fcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Ra297430a262e4a97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rdeb4223ed4c240b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R47ec3bde5733491b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rb8219902f4c74d54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Ra2682a697e674d32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R71dc394ac0954d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rb4393d9d64984def"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rc0e178a66d714d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R9d6616b8373d4807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R33b9bf4ec6144706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R0a1ce8e658eb44a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R07e93c0c9bea4082"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rfb7c4298da3340d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rf326eb0c906c4208"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R7d261fd40cb24fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R3f1bf7e7bdae4552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R8adc937bb16f4921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rcaa100844c5f4ff0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R2ea913d032a64646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R62220938b6ba48be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R1daf5028ce9a4629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R7e367148395f44f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R59f700f6cd8e4417"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rbf00ae5e259b44a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R9baf6a12cd7648b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R366fc3c67deb4f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Rfeb7cddcbf4048a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R71d22b011ea14fc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R3f8c1b2f19954a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R839122ea6c4748b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R2e419dc70c4146f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rbdb5eafe1dbc4d58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Raf9d277a79c241e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R4147b193748346e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R0809938256424f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R4560e223127b4551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rd0609a304dd84b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R23469a309b674215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Re63c6f9ece2142ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R7822720d4220499b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1226,7 +1226,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.5.3-sample</x:v>
+        <x:v>0.5.4-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1338,7 +1338,7 @@
       </x:c>
       <x:c r="E14" s="89" t="n">
         <x:f>COUNTA('Spawns'!A5:A1000)</x:f>
-        <x:v>32</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F14" s="92"/>
       <x:c r="G14" s="92"/>
@@ -2067,7 +2067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fab6629fcc040d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66fb858459a74ace"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2617,7 +2617,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6edefb12106041d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74bf9d1e8ad045d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2882,7 +2882,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R240ee3c9789f4732"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3227d07935364f4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3146,7 +3146,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2823b811ce5449d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9a675be4cab4c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3351,7 +3351,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c3470e76b1b4865"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R874a2e48705e44ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4233,7 +4233,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R385d77a9e8614ea6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4856df5cb83d4339"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4412,20 +4412,20 @@
         <x:v>bg_red_cave_boss</x:v>
       </x:c>
       <x:c r="E7" s="72" t="n">
-        <x:v>300</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="F7" s="35" t="str"/>
       <x:c r="G7" s="35" t="str">
         <x:v>reward_level_003</x:v>
       </x:c>
       <x:c r="H7" s="35" t="n">
-        <x:v>7000</x:v>
+        <x:v>8000</x:v>
       </x:c>
       <x:c r="I7" s="35" t="n">
-        <x:v>10000</x:v>
+        <x:v>12000</x:v>
       </x:c>
       <x:c r="J7" s="35" t="n">
-        <x:v>14000</x:v>
+        <x:v>17000</x:v>
       </x:c>
       <x:c r="K7" s="35" t="str">
         <x:v>tutorial_level_003</x:v>
@@ -4441,7 +4441,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R008be588948644bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f430cac6e11471f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4942,13 +4942,13 @@
         <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="G19" s="121" t="n">
-        <x:v>0.8</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="H19" t="str">
         <x:v>bgm_boss_intro</x:v>
       </x:c>
       <x:c r="I19" t="n">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -4965,7 +4965,7 @@
         <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="E20" s="121" t="n">
-        <x:v>0.8</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="F20" t="str">
         <x:v>BossDefeated</x:v>
@@ -4995,7 +4995,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f5fe4a3a0734524"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raabb56e2ee01427f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5201,7 +5201,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe211b74ab654203"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce66493918124d8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5327,7 +5327,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re90dd2b015eb4995"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd347d4ed4e814776"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5426,7 +5426,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.5.3-sample</x:v>
+        <x:v>0.5.4-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6338,7 +6338,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d64bcc5ce8d4f71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bbbddae56d9460f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7271,7 +7271,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F34" s="121" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="G34" t="str">
         <x:v>spawn_air_mid</x:v>
@@ -7291,7 +7291,7 @@
         <x:v>wave_003_01</x:v>
       </x:c>
       <x:c r="C35" s="121" t="n">
-        <x:v>0.6</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="D35" t="str">
         <x:v>enemy_talisman_bat</x:v>
@@ -7314,30 +7314,117 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
+        <x:v>spawn_003_01_c</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="C36" s="121" t="n">
+        <x:v>2.8</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>enemy_stone_turtle</x:v>
+      </x:c>
+      <x:c r="E36" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F36" s="121" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>spawn_ground_right</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>spawn_003_01_d</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="C37" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>enemy_skeleton_ghost</x:v>
+      </x:c>
+      <x:c r="E37" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F37" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>Scatter</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>modifier_none</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>spawn_003_01_e</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>wave_003_01</x:v>
+      </x:c>
+      <x:c r="C38" t="n">
+        <x:v>5.2</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>enemy_soul_puppet</x:v>
+      </x:c>
+      <x:c r="E38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>spawn_air_mid</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>modifier_elite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
         <x:v>spawn_003_02_a</x:v>
       </x:c>
-      <x:c r="B36" t="str">
+      <x:c r="B39" t="str">
         <x:v>wave_003_02</x:v>
       </x:c>
-      <x:c r="C36" s="121" t="n">
+      <x:c r="C39" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D36" t="str">
+      <x:c r="D39" t="str">
         <x:v>boss_tomb_king</x:v>
       </x:c>
-      <x:c r="E36" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F36" s="121" t="n">
+      <x:c r="E39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F39" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G36" t="str">
+      <x:c r="G39" t="str">
         <x:v>spawn_boss</x:v>
       </x:c>
-      <x:c r="H36" t="str">
+      <x:c r="H39" t="str">
         <x:v>Single</x:v>
       </x:c>
-      <x:c r="I36" t="str">
+      <x:c r="I39" t="str">
         <x:v>modifier_none</x:v>
       </x:c>
     </x:row>
@@ -7353,7 +7440,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98ec7ce130aa4135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3603f5965a5644e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7552,7 +7639,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dbfd3690fc04b24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05a5199194354120"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7768,7 +7855,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374d265fbe174141"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb80bd308cb444b7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8087,7 +8174,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf00bb55672bc4c37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eda8d57ac284414"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8627,10 +8714,10 @@
         <x:v>text_boss_phase3</x:v>
       </x:c>
       <x:c r="B40" s="35" t="str">
-        <x:v>切断法术并阻止冲撞</x:v>
+        <x:v>斜斩打断冲撞，随后处决玄甲王</x:v>
       </x:c>
       <x:c r="C40" s="35" t="str">
-        <x:v>Cut projectiles and stop the charge</x:v>
+        <x:v>Interrupt the charge with a diagonal slash, then execute the Tomb King</x:v>
       </x:c>
       <x:c r="D40" s="35" t="str">
         <x:v>Boss phase</x:v>
@@ -8657,7 +8744,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa03141f8a8a42b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b4bd2792b8f4c18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9180,7 +9267,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f639ef963d04767"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875829a23bc44e16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10124,7 +10211,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2db11cb599f2406d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f4c290818fd41fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11479,7 +11566,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1dfe04069b94d14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R960c78b805474271"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12847,7 +12934,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55acb1b9a19a41f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08aa7140dc5c404b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18740,7 +18827,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab292e68a0a94536"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce59562b7cc44cb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18842,7 +18929,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc52fcea244f943f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re57dab2ece344771"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18991,7 +19078,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97379df43fba4e46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7caf7e7925db40f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19389,7 +19476,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf997c936eae44656"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd44438ac07c241e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19586,7 +19673,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R740324c7174d4210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961b1edc6f444a42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19765,7 +19852,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d88fdb06b494813"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2a81178d68c44d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19990,7 +20077,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0cc15571ca44488"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12e3ad678c674c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20334,7 +20421,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3553686bc6e44353"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74eb3c984e6e4366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T550: complete result and progress loop
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R07e93c0c9bea4082"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rfb7c4298da3340d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rf326eb0c906c4208"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R7d261fd40cb24fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R3f1bf7e7bdae4552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R8adc937bb16f4921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rcaa100844c5f4ff0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R2ea913d032a64646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R62220938b6ba48be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R1daf5028ce9a4629"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R7e367148395f44f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R59f700f6cd8e4417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rbf00ae5e259b44a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R9baf6a12cd7648b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R366fc3c67deb4f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Rfeb7cddcbf4048a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R71d22b011ea14fc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R3f8c1b2f19954a4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R839122ea6c4748b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R2e419dc70c4146f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rbdb5eafe1dbc4d58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Raf9d277a79c241e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R4147b193748346e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R0809938256424f5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R4560e223127b4551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rd0609a304dd84b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R23469a309b674215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Re63c6f9ece2142ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R7822720d4220499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Raa546e00d83c4e1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rf334dfb2f7054e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rd4d20974c9144418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Re47a118f00bd4c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rde3adf361d124f44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rcb067094c7934c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R70ab42ef7a804805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rce33f239ffd24762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Refab2b03179b4e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R1297d3218c14496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R035fe09628694bc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R7029024dd8a947a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R1000ea6251234be3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R76ec96f8d16e4220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R87329ae99db44521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R9965c639d99d4fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Rb3cf0d49635d447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R78c9ee9370cd494f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R3ffc44d4f0524503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R9d18133e8e8e48d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R8ff8c66b1d9a484b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R1b17928c69764efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R8c466dd83dce44de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R4667cc6e68e44c1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rd5e890ee33a34edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rdb894e5684174ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Re6de79d49d314f4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R4d270f5534d242ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rc4117cc782f64e7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1226,7 +1226,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.5.4-sample</x:v>
+        <x:v>0.5.5-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -2067,7 +2067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66fb858459a74ace"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae73fdbf28f4aa8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2617,7 +2617,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74bf9d1e8ad045d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20ed387c3694d73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2882,7 +2882,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3227d07935364f4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d070202a15341a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3146,7 +3146,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9a675be4cab4c93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a5a808394aa418a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3351,7 +3351,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R874a2e48705e44ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb31546cae73d413b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4233,7 +4233,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4856df5cb83d4339"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d69e49b718b412d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4441,7 +4441,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f430cac6e11471f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a8c111f791440c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4995,7 +4995,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raabb56e2ee01427f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2078f2d61a3442e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5201,7 +5201,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce66493918124d8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bea84c46aa4eab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5327,7 +5327,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd347d4ed4e814776"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc51ba9f248bc4941"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5426,7 +5426,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.5.4-sample</x:v>
+        <x:v>0.5.5-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -5737,34 +5737,64 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22"/>
-      <x:c r="B22"/>
-      <x:c r="C22"/>
+      <x:c r="A22" t="str">
+        <x:v>result_score_per_reflect</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C22" t="n">
+        <x:v>150</x:v>
+      </x:c>
       <x:c r="D22"/>
       <x:c r="E22"/>
       <x:c r="F22"/>
-      <x:c r="G22"/>
-      <x:c r="H22"/>
+      <x:c r="G22" t="str">
+        <x:v>score</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>每次成功弹反的结算评分</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23"/>
-      <x:c r="B23"/>
-      <x:c r="C23"/>
+      <x:c r="A23" t="str">
+        <x:v>result_score_no_damage_bonus</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C23" t="n">
+        <x:v>1000</x:v>
+      </x:c>
       <x:c r="D23"/>
       <x:c r="E23"/>
       <x:c r="F23"/>
-      <x:c r="G23"/>
-      <x:c r="H23"/>
+      <x:c r="G23" t="str">
+        <x:v>score</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>胜利且未受伤时的结算评分</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24"/>
-      <x:c r="B24"/>
-      <x:c r="C24"/>
+      <x:c r="A24" t="str">
+        <x:v>result_score_per_remaining_second</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C24" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="D24"/>
       <x:c r="E24"/>
       <x:c r="F24"/>
-      <x:c r="G24"/>
-      <x:c r="H24"/>
+      <x:c r="G24" t="str">
+        <x:v>score/sec</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>胜利时每个剩余整秒的结算评分</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25"/>
@@ -6338,7 +6368,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bbbddae56d9460f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc61db72d2b04ae0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7440,7 +7470,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3603f5965a5644e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6de9cf17b8a84d04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7639,7 +7669,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05a5199194354120"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra85a32cb56304ddf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7855,7 +7885,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb80bd308cb444b7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd04d3bc5373a4d75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8174,7 +8204,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eda8d57ac284414"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f80270120e242b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8744,7 +8774,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b4bd2792b8f4c18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbf4e610683d41e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9267,7 +9297,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875829a23bc44e16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516d5c0f9f4d4a4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10211,7 +10241,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f4c290818fd41fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73c19b3f69b1412d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11566,7 +11596,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R960c78b805474271"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ab08e59d33d4443"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12934,7 +12964,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08aa7140dc5c404b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3937a1ab99544447"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18827,7 +18857,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce59562b7cc44cb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R798c27a2de474ccd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18929,7 +18959,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re57dab2ece344771"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1683457e57d246bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19078,7 +19108,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7caf7e7925db40f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0cf7951b6a8483e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19476,7 +19506,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd44438ac07c241e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7017f057bf7401d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19673,7 +19703,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961b1edc6f444a42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1f7cd0751834d31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19852,7 +19882,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2a81178d68c44d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaa490fdc191432b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20077,7 +20107,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12e3ad678c674c93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf593562e367450c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20421,7 +20451,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74eb3c984e6e4366"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0369cc64ff74fb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T600: implement battle HUD and result UI
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Raa546e00d83c4e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rf334dfb2f7054e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rd4d20974c9144418"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Re47a118f00bd4c98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rde3adf361d124f44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rcb067094c7934c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R70ab42ef7a804805"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rce33f239ffd24762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Refab2b03179b4e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R1297d3218c14496e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R035fe09628694bc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R7029024dd8a947a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R1000ea6251234be3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R76ec96f8d16e4220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R87329ae99db44521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R9965c639d99d4fdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Rb3cf0d49635d447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R78c9ee9370cd494f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R3ffc44d4f0524503"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R9d18133e8e8e48d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R8ff8c66b1d9a484b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R1b17928c69764efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R8c466dd83dce44de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R4667cc6e68e44c1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rd5e890ee33a34edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rdb894e5684174ea1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Re6de79d49d314f4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R4d270f5534d242ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rc4117cc782f64e7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0d91c2873eae4b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R6c23329022f14293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R210b8897e4fd4711"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R7c3771649eef4bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rbc698a83ac4b4143"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R9e0ccb7610744f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R103cfc0531074a85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R7653ea3ec82d47e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Rb85930d9d0ee4ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rca3dc223bf254033"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R092a151aad664076"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rca4b58718e3543cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R760cf60f33b74ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R188d4d24df1640b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R3f33b6171d314f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R374ab70cea9242a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R2dcb3b30c2e94896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rb2d36dc2d0614ddf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Re55aec0e944d49b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R252ebe9f61924258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Ra44bb43cf69f4881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R08ec53efc4144c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rf9363388bee54200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R708562185c0345fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R95f9be058af04078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R4b8a29f91eed47cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R9ae002beccd142ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rc3c573938b6e4b25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rb61d56b6db724412"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -102,7 +102,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,15 +154,30 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0E6F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF44B3E1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="122">
+  <x:cellXfs count="128">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -491,6 +506,16 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1226,7 +1251,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.5.5-sample</x:v>
+        <x:v>0.6.0-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1383,7 +1408,7 @@
       </x:c>
       <x:c r="E17" s="89" t="n">
         <x:f>COUNTA('Texts'!A5:A1000)</x:f>
-        <x:v>37</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F17" s="92"/>
       <x:c r="G17" s="92"/>
@@ -2067,7 +2092,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae73fdbf28f4aa8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra695a1cc30f84686"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2617,7 +2642,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20ed387c3694d73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R984c20ee474349b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2882,7 +2907,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d070202a15341a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d631be8713840b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3146,7 +3171,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a5a808394aa418a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3012af4a1bb4ca6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3351,7 +3376,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb31546cae73d413b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0924ba8eafe2406a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4233,7 +4258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d69e49b718b412d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R574462a344384ad7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4441,7 +4466,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a8c111f791440c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3c3752c4c9402d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4995,7 +5020,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2078f2d61a3442e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7364365d52ab4e7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5201,7 +5226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bea84c46aa4eab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfec43ebbe9e45c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5327,7 +5352,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc51ba9f248bc4941"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d536a0e9ae45be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5426,7 +5451,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.5.5-sample</x:v>
+        <x:v>0.6.0-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6368,7 +6393,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc61db72d2b04ae0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb471b0d9bfbb4d14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7470,7 +7495,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6de9cf17b8a84d04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9a993187b404b9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7669,7 +7694,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra85a32cb56304ddf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f999649125a4f0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7885,7 +7910,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd04d3bc5373a4d75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6d5f741427d4cb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8204,7 +8229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f80270120e242b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8841be52adb4e75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8767,6 +8792,286 @@
         <x:v>Buff</x:v>
       </x:c>
     </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="124" t="str">
+        <x:v>text_ui_combo</x:v>
+      </x:c>
+      <x:c r="B42" s="124" t="str">
+        <x:v>连斩</x:v>
+      </x:c>
+      <x:c r="C42" s="124" t="str">
+        <x:v>Combo</x:v>
+      </x:c>
+      <x:c r="D42" s="124" t="str">
+        <x:v>HUD连斩标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="127" t="str">
+        <x:v>text_ui_cooldown</x:v>
+      </x:c>
+      <x:c r="B43" s="127" t="str">
+        <x:v>冷却</x:v>
+      </x:c>
+      <x:c r="C43" s="127" t="str">
+        <x:v>Cooldown</x:v>
+      </x:c>
+      <x:c r="D43" s="127" t="str">
+        <x:v>技能冷却标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="124" t="str">
+        <x:v>text_ui_defeat</x:v>
+      </x:c>
+      <x:c r="B44" s="124" t="str">
+        <x:v>败北</x:v>
+      </x:c>
+      <x:c r="C44" s="124" t="str">
+        <x:v>Defeat</x:v>
+      </x:c>
+      <x:c r="D44" s="124" t="str">
+        <x:v>失败结算标题</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="127" t="str">
+        <x:v>text_ui_energy</x:v>
+      </x:c>
+      <x:c r="B45" s="127" t="str">
+        <x:v>能量</x:v>
+      </x:c>
+      <x:c r="C45" s="127" t="str">
+        <x:v>Energy</x:v>
+      </x:c>
+      <x:c r="D45" s="127" t="str">
+        <x:v>HUD能量标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="124" t="str">
+        <x:v>text_ui_hp</x:v>
+      </x:c>
+      <x:c r="B46" s="124" t="str">
+        <x:v>生命</x:v>
+      </x:c>
+      <x:c r="C46" s="124" t="str">
+        <x:v>HP</x:v>
+      </x:c>
+      <x:c r="D46" s="124" t="str">
+        <x:v>HUD生命标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="127" t="str">
+        <x:v>text_ui_main_menu</x:v>
+      </x:c>
+      <x:c r="B47" s="127" t="str">
+        <x:v>返回主菜单</x:v>
+      </x:c>
+      <x:c r="C47" s="127" t="str">
+        <x:v>Main Menu</x:v>
+      </x:c>
+      <x:c r="D47" s="127" t="str">
+        <x:v>返回主菜单按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="124" t="str">
+        <x:v>text_ui_next_level</x:v>
+      </x:c>
+      <x:c r="B48" s="124" t="str">
+        <x:v>下一关</x:v>
+      </x:c>
+      <x:c r="C48" s="124" t="str">
+        <x:v>Next Level</x:v>
+      </x:c>
+      <x:c r="D48" s="124" t="str">
+        <x:v>结算下一关按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="127" t="str">
+        <x:v>text_ui_pause</x:v>
+      </x:c>
+      <x:c r="B49" s="127" t="str">
+        <x:v>暂停</x:v>
+      </x:c>
+      <x:c r="C49" s="127" t="str">
+        <x:v>Pause</x:v>
+      </x:c>
+      <x:c r="D49" s="127" t="str">
+        <x:v>暂停按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="124" t="str">
+        <x:v>text_ui_paused</x:v>
+      </x:c>
+      <x:c r="B50" s="124" t="str">
+        <x:v>战斗已暂停</x:v>
+      </x:c>
+      <x:c r="C50" s="124" t="str">
+        <x:v>Battle Paused</x:v>
+      </x:c>
+      <x:c r="D50" s="124" t="str">
+        <x:v>暂停面板标题</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="127" t="str">
+        <x:v>text_ui_ready</x:v>
+      </x:c>
+      <x:c r="B51" s="127" t="str">
+        <x:v>可释放</x:v>
+      </x:c>
+      <x:c r="C51" s="127" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
+      <x:c r="D51" s="127" t="str">
+        <x:v>技能可释放状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="124" t="str">
+        <x:v>text_ui_restart</x:v>
+      </x:c>
+      <x:c r="B52" s="124" t="str">
+        <x:v>重新挑战</x:v>
+      </x:c>
+      <x:c r="C52" s="124" t="str">
+        <x:v>Restart</x:v>
+      </x:c>
+      <x:c r="D52" s="124" t="str">
+        <x:v>结算重开按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="127" t="str">
+        <x:v>text_ui_resume</x:v>
+      </x:c>
+      <x:c r="B53" s="127" t="str">
+        <x:v>继续</x:v>
+      </x:c>
+      <x:c r="C53" s="127" t="str">
+        <x:v>Resume</x:v>
+      </x:c>
+      <x:c r="D53" s="127" t="str">
+        <x:v>继续按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="124" t="str">
+        <x:v>text_ui_reward_feature</x:v>
+      </x:c>
+      <x:c r="B54" s="124" t="str">
+        <x:v>解锁功能</x:v>
+      </x:c>
+      <x:c r="C54" s="124" t="str">
+        <x:v>Feature Unlocked</x:v>
+      </x:c>
+      <x:c r="D54" s="124" t="str">
+        <x:v>解锁功能奖励标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="127" t="str">
+        <x:v>text_ui_reward_level</x:v>
+      </x:c>
+      <x:c r="B55" s="127" t="str">
+        <x:v>解锁关卡</x:v>
+      </x:c>
+      <x:c r="C55" s="127" t="str">
+        <x:v>Level Unlocked</x:v>
+      </x:c>
+      <x:c r="D55" s="127" t="str">
+        <x:v>解锁关卡奖励标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="124" t="str">
+        <x:v>text_ui_reward_score_token</x:v>
+      </x:c>
+      <x:c r="B56" s="124" t="str">
+        <x:v>镇妖积分</x:v>
+      </x:c>
+      <x:c r="C56" s="124" t="str">
+        <x:v>Demon Score</x:v>
+      </x:c>
+      <x:c r="D56" s="124" t="str">
+        <x:v>非付费积分奖励标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="127" t="str">
+        <x:v>text_ui_rewards</x:v>
+      </x:c>
+      <x:c r="B57" s="127" t="str">
+        <x:v>奖励</x:v>
+      </x:c>
+      <x:c r="C57" s="127" t="str">
+        <x:v>Rewards</x:v>
+      </x:c>
+      <x:c r="D57" s="127" t="str">
+        <x:v>结算奖励标题</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="124" t="str">
+        <x:v>text_ui_score</x:v>
+      </x:c>
+      <x:c r="B58" s="124" t="str">
+        <x:v>评分</x:v>
+      </x:c>
+      <x:c r="C58" s="124" t="str">
+        <x:v>Score</x:v>
+      </x:c>
+      <x:c r="D58" s="124" t="str">
+        <x:v>HUD评分标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="127" t="str">
+        <x:v>text_ui_stance</x:v>
+      </x:c>
+      <x:c r="B59" s="127" t="str">
+        <x:v>架势</x:v>
+      </x:c>
+      <x:c r="C59" s="127" t="str">
+        <x:v>Stance</x:v>
+      </x:c>
+      <x:c r="D59" s="127" t="str">
+        <x:v>HUD架势标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="124" t="str">
+        <x:v>text_ui_stars</x:v>
+      </x:c>
+      <x:c r="B60" s="124" t="str">
+        <x:v>星级</x:v>
+      </x:c>
+      <x:c r="C60" s="124" t="str">
+        <x:v>Stars</x:v>
+      </x:c>
+      <x:c r="D60" s="124" t="str">
+        <x:v>结算星级标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="127" t="str">
+        <x:v>text_ui_victory</x:v>
+      </x:c>
+      <x:c r="B61" s="127" t="str">
+        <x:v>胜利</x:v>
+      </x:c>
+      <x:c r="C61" s="127" t="str">
+        <x:v>Victory</x:v>
+      </x:c>
+      <x:c r="D61" s="127" t="str">
+        <x:v>胜利结算标题</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -8774,7 +9079,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbf4e610683d41e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbeb9a7f085df4970"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9297,7 +9602,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516d5c0f9f4d4a4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f1ca3298cc549de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10241,7 +10546,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73c19b3f69b1412d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8954a9aba0d946be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11596,7 +11901,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ab08e59d33d4443"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7797516dfcf4f06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12964,7 +13269,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3937a1ab99544447"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2c1996367ce49b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18857,7 +19162,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R798c27a2de474ccd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7312bceae648471a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18959,7 +19264,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1683457e57d246bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d9ea874675a4bba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19108,7 +19413,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0cf7951b6a8483e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R687391dc045e49c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19506,7 +19811,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7017f057bf7401d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re930b761545f4a1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19703,7 +20008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1f7cd0751834d31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2490ebd889294cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19882,7 +20187,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaa490fdc191432b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaf23ad2ab734e21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20107,7 +20412,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf593562e367450c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re98529a4fd2442f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20451,7 +20756,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0369cc64ff74fb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c1a7cf1ba7c4c0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T620: implement combat feedback
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,35 +2,36 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0d91c2873eae4b1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R6c23329022f14293"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R210b8897e4fd4711"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R7c3771649eef4bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rbc698a83ac4b4143"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R9e0ccb7610744f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R103cfc0531074a85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R7653ea3ec82d47e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Rb85930d9d0ee4ed0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rca3dc223bf254033"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R092a151aad664076"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rca4b58718e3543cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R760cf60f33b74ad2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R188d4d24df1640b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R3f33b6171d314f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R374ab70cea9242a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R2dcb3b30c2e94896"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rb2d36dc2d0614ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Re55aec0e944d49b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R252ebe9f61924258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Ra44bb43cf69f4881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R08ec53efc4144c20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rf9363388bee54200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R708562185c0345fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R95f9be058af04078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R4b8a29f91eed47cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R9ae002beccd142ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rc3c573938b6e4b25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rb61d56b6db724412"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc2a504e7dad442af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R57300fc71ce04b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rf97bbec4487a470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R644ceb37036744a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R77978799654647b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Ra2edc32b3b274500"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R093fff7faba34fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rbd469915e8a94214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R20ca8c039cff44b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rd1c3377871344948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R0c0b40cae1c6472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R53dcca452b6b48ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rc8a984aac7684edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R17964147ed344dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R365912e991f54058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Ra8fc33c5bf4f4225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Ra0158251a3c24c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R45bbc91201844beb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R5b19353e9c864d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R0a4991dd5145408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R5b6be75266cf494d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R4e0be75b14424224"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R8889d3eccb5e4e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rb8817bcb4cd24f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Ra7649b777aef47c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rfc9083edcd004d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R75fd37cf76f24057"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rce011c1896844646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R51bc79c2d19c4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R91fda32e75824395"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -41,9 +42,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
+    <x:numFmt numFmtId="202" formatCode="0.000"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -102,7 +104,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -164,6 +166,31 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0E6F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2D5B75"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -177,7 +204,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="128">
+  <x:cellXfs count="153">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -515,6 +542,57 @@
     <x:xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1236,7 +1314,7 @@
         <x:v>Schema版本</x:v>
       </x:c>
       <x:c r="B5" s="25" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Players</x:v>
@@ -1251,7 +1329,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.0-sample</x:v>
+        <x:v>0.6.1-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1428,6 +1506,15 @@
       <x:c r="F18" s="92"/>
       <x:c r="G18" s="92"/>
       <x:c r="H18" s="92"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="D19" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="E19" t="n">
+        <x:f>COUNTA('FeedbackCues'!A5:A1000)</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="45"/>
@@ -2092,7 +2179,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra695a1cc30f84686"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R712b8da6a892497c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2642,7 +2729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R984c20ee474349b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R420f2d89be9349d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2907,7 +2994,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d631be8713840b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb516cfebc85146bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3171,7 +3258,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3012af4a1bb4ca6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R285c6c54e3ee4c34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3376,7 +3463,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0924ba8eafe2406a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad5f2b86f7464a96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4258,7 +4345,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R574462a344384ad7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc1e5e531065428e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4466,7 +4553,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3c3752c4c9402d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb96367313349f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5020,7 +5107,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7364365d52ab4e7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee77d58cf0d4835"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5226,7 +5313,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfec43ebbe9e45c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a668583c1894874"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5352,7 +5439,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d536a0e9ae45be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc61318cebff44ef5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5429,7 +5516,7 @@
         <x:v>int</x:v>
       </x:c>
       <x:c r="C5" s="68" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="35"/>
       <x:c r="E5" s="35"/>
@@ -5451,7 +5538,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.0-sample</x:v>
+        <x:v>0.6.1-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6393,7 +6480,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb471b0d9bfbb4d14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43e6d61048964239"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7495,7 +7582,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9a993187b404b9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2726946c063544d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7694,7 +7781,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f999649125a4f0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73307976460b44b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7910,7 +7997,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6d5f741427d4cb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae84765f2a3a46f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8229,7 +8316,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8841be52adb4e75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ede04675f8c494e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9079,7 +9166,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbeb9a7f085df4970"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1c4c55747d34cbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9602,7 +9689,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f1ca3298cc549de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f33486d0184dd5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10546,7 +10633,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8954a9aba0d946be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae46a8f5bf924ade"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11901,7 +11988,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7797516dfcf4f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cd459b4324749f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13262,6 +13349,62 @@
         <x:v>达到配置活动容量时先完整回收最早活动项，再服务本次租用。</x:v>
       </x:c>
     </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="132" t="str">
+        <x:v>FeedbackVibrationPattern</x:v>
+      </x:c>
+      <x:c r="B99" s="132" t="str">
+        <x:v>Off</x:v>
+      </x:c>
+      <x:c r="C99" s="132" t="str">
+        <x:v>关闭</x:v>
+      </x:c>
+      <x:c r="D99" s="132" t="str">
+        <x:v>不请求平台震动。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="137" t="str">
+        <x:v>FeedbackVibrationPattern</x:v>
+      </x:c>
+      <x:c r="B100" s="137" t="str">
+        <x:v>Light</x:v>
+      </x:c>
+      <x:c r="C100" s="137" t="str">
+        <x:v>轻震</x:v>
+      </x:c>
+      <x:c r="D100" s="137" t="str">
+        <x:v>轻量命中反馈。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="132" t="str">
+        <x:v>FeedbackVibrationPattern</x:v>
+      </x:c>
+      <x:c r="B101" s="132" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C101" s="132" t="str">
+        <x:v>中震</x:v>
+      </x:c>
+      <x:c r="D101" s="132" t="str">
+        <x:v>中等强度反馈。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="137" t="str">
+        <x:v>FeedbackVibrationPattern</x:v>
+      </x:c>
+      <x:c r="B102" s="137" t="str">
+        <x:v>Heavy</x:v>
+      </x:c>
+      <x:c r="C102" s="137" t="str">
+        <x:v>重震</x:v>
+      </x:c>
+      <x:c r="D102" s="137" t="str">
+        <x:v>强烈事件反馈。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -13269,7 +13412,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2c1996367ce49b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c37658d55634ce4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19142,6 +19285,400 @@
         <x:v>Enums 表的 description 字段</x:v>
       </x:c>
     </x:row>
+    <x:row r="255">
+      <x:c r="A255" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B255" s="132" t="str">
+        <x:v>feedbackId</x:v>
+      </x:c>
+      <x:c r="C255" s="132" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D255" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E255" s="132"/>
+      <x:c r="F255" s="132"/>
+      <x:c r="G255" s="132"/>
+      <x:c r="H255" s="132"/>
+      <x:c r="I255" s="132"/>
+      <x:c r="J255" s="132" t="str">
+        <x:v>反馈配置稳定ID。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256">
+      <x:c r="A256" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B256" s="137" t="str">
+        <x:v>vfxKey</x:v>
+      </x:c>
+      <x:c r="C256" s="137" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D256" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E256" s="137"/>
+      <x:c r="F256" s="137"/>
+      <x:c r="G256" s="137"/>
+      <x:c r="H256" s="137"/>
+      <x:c r="I256" s="137" t="str">
+        <x:v>VfxCues.vfxKey</x:v>
+      </x:c>
+      <x:c r="J256" s="137" t="str">
+        <x:v>反馈使用的特效提示外键。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257">
+      <x:c r="A257" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B257" s="132" t="str">
+        <x:v>audioKey</x:v>
+      </x:c>
+      <x:c r="C257" s="132" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D257" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E257" s="132"/>
+      <x:c r="F257" s="132"/>
+      <x:c r="G257" s="132"/>
+      <x:c r="H257" s="132"/>
+      <x:c r="I257" s="132" t="str">
+        <x:v>AudioCues.audioKey</x:v>
+      </x:c>
+      <x:c r="J257" s="132" t="str">
+        <x:v>反馈使用的音频提示外键。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258">
+      <x:c r="A258" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B258" s="137" t="str">
+        <x:v>timeScale</x:v>
+      </x:c>
+      <x:c r="C258" s="137" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D258" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E258" s="137"/>
+      <x:c r="F258" s="137" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G258" s="137" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H258" s="137"/>
+      <x:c r="I258" s="137"/>
+      <x:c r="J258" s="137" t="str">
+        <x:v>反馈期间的玩法时间缩放；0表示完全停顿。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259">
+      <x:c r="A259" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B259" s="132" t="str">
+        <x:v>timeScaleSec</x:v>
+      </x:c>
+      <x:c r="C259" s="132" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D259" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E259" s="132"/>
+      <x:c r="F259" s="132" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G259" s="132" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H259" s="132"/>
+      <x:c r="I259" s="132"/>
+      <x:c r="J259" s="132" t="str">
+        <x:v>玩法时间缩放持续秒数，使用非缩放时间推进。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260">
+      <x:c r="A260" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B260" s="137" t="str">
+        <x:v>flashSec</x:v>
+      </x:c>
+      <x:c r="C260" s="137" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D260" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E260" s="137"/>
+      <x:c r="F260" s="137" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G260" s="137" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H260" s="137"/>
+      <x:c r="I260" s="137"/>
+      <x:c r="J260" s="137" t="str">
+        <x:v>目标白闪持续秒数。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261">
+      <x:c r="A261" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B261" s="132" t="str">
+        <x:v>shakeStrengthRefPx</x:v>
+      </x:c>
+      <x:c r="C261" s="132" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D261" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E261" s="132"/>
+      <x:c r="F261" s="132" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G261" s="132" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H261" s="132"/>
+      <x:c r="I261" s="132"/>
+      <x:c r="J261" s="132" t="str">
+        <x:v>1920×1080参考分辨率下的震屏强度像素。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262">
+      <x:c r="A262" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B262" s="137" t="str">
+        <x:v>shakeSec</x:v>
+      </x:c>
+      <x:c r="C262" s="137" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D262" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E262" s="137"/>
+      <x:c r="F262" s="137" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G262" s="137" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H262" s="137"/>
+      <x:c r="I262" s="137"/>
+      <x:c r="J262" s="137" t="str">
+        <x:v>震屏持续秒数。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263">
+      <x:c r="A263" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B263" s="132" t="str">
+        <x:v>vibrationPattern</x:v>
+      </x:c>
+      <x:c r="C263" s="132" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D263" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E263" s="132"/>
+      <x:c r="F263" s="132"/>
+      <x:c r="G263" s="132"/>
+      <x:c r="H263" s="132" t="str">
+        <x:v>FeedbackVibrationPattern</x:v>
+      </x:c>
+      <x:c r="I263" s="132"/>
+      <x:c r="J263" s="132" t="str">
+        <x:v>平台震动强度；可由用户总开关禁用。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264">
+      <x:c r="A264" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B264" s="137" t="str">
+        <x:v>damageNumberColorHex</x:v>
+      </x:c>
+      <x:c r="C264" s="137" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D264" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E264" s="137"/>
+      <x:c r="F264" s="137"/>
+      <x:c r="G264" s="137"/>
+      <x:c r="H264" s="137"/>
+      <x:c r="I264" s="137"/>
+      <x:c r="J264" s="137" t="str">
+        <x:v>伤害数字颜色，格式为#RRGGBBAA。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265">
+      <x:c r="A265" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B265" s="132" t="str">
+        <x:v>damageNumberFontSizeRefPx</x:v>
+      </x:c>
+      <x:c r="C265" s="132" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="D265" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E265" s="132"/>
+      <x:c r="F265" s="132" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G265" s="132" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="H265" s="132"/>
+      <x:c r="I265" s="132"/>
+      <x:c r="J265" s="132" t="str">
+        <x:v>1920×1080参考分辨率下的伤害数字字号。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266">
+      <x:c r="A266" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B266" s="137" t="str">
+        <x:v>damageNumberLifeSec</x:v>
+      </x:c>
+      <x:c r="C266" s="137" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D266" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E266" s="137"/>
+      <x:c r="F266" s="137" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G266" s="137" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H266" s="137"/>
+      <x:c r="I266" s="137"/>
+      <x:c r="J266" s="137" t="str">
+        <x:v>伤害数字存活秒数。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267">
+      <x:c r="A267" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B267" s="132" t="str">
+        <x:v>damageNumberRiseRefPx</x:v>
+      </x:c>
+      <x:c r="C267" s="132" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D267" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E267" s="132"/>
+      <x:c r="F267" s="132" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G267" s="132" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="H267" s="132"/>
+      <x:c r="I267" s="132"/>
+      <x:c r="J267" s="132" t="str">
+        <x:v>伤害数字生命周期内上浮的参考像素。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268">
+      <x:c r="A268" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B268" s="137" t="str">
+        <x:v>vfxTintColorHex</x:v>
+      </x:c>
+      <x:c r="C268" s="137" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D268" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E268" s="137"/>
+      <x:c r="F268" s="137"/>
+      <x:c r="G268" s="137"/>
+      <x:c r="H268" s="137"/>
+      <x:c r="I268" s="137"/>
+      <x:c r="J268" s="137" t="str">
+        <x:v>反馈特效染色，格式为#RRGGBBAA。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269">
+      <x:c r="A269" s="132" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B269" s="132" t="str">
+        <x:v>vfxScaleRefPx</x:v>
+      </x:c>
+      <x:c r="C269" s="132" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D269" s="132" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E269" s="132"/>
+      <x:c r="F269" s="132" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G269" s="132" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="H269" s="132"/>
+      <x:c r="I269" s="132"/>
+      <x:c r="J269" s="132" t="str">
+        <x:v>1920×1080参考分辨率下的特效尺寸。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270">
+      <x:c r="A270" s="137" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B270" s="137" t="str">
+        <x:v>description</x:v>
+      </x:c>
+      <x:c r="C270" s="137" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D270" s="137" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E270" s="137"/>
+      <x:c r="F270" s="137"/>
+      <x:c r="G270" s="137"/>
+      <x:c r="H270" s="137"/>
+      <x:c r="I270" s="137"/>
+      <x:c r="J270" s="137" t="str">
+        <x:v>反馈配置用途说明。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -19162,7 +19699,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7312bceae648471a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97e0519569d54525"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19264,8 +19801,390 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d9ea874675a4bba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c162ba0e0e44d52"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="29" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="27" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="23" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="56" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="141" t="str">
+        <x:v>FeedbackCues</x:v>
+      </x:c>
+      <x:c r="B1" s="141"/>
+      <x:c r="C1" s="141"/>
+      <x:c r="D1" s="141"/>
+      <x:c r="E1" s="141"/>
+      <x:c r="F1" s="141"/>
+      <x:c r="G1" s="141"/>
+      <x:c r="H1" s="141"/>
+      <x:c r="I1" s="141"/>
+      <x:c r="J1" s="141"/>
+      <x:c r="K1" s="141"/>
+      <x:c r="L1" s="141"/>
+      <x:c r="M1" s="141"/>
+      <x:c r="N1" s="141"/>
+      <x:c r="O1" s="141"/>
+      <x:c r="P1" s="141"/>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="145" t="str">
+        <x:v>战斗事件到特效、音频、停顿、震屏、伤害数字和震动强度的配置映射。所有时长使用非缩放秒。</x:v>
+      </x:c>
+      <x:c r="B2" s="145"/>
+      <x:c r="C2" s="145"/>
+      <x:c r="D2" s="145"/>
+      <x:c r="E2" s="145"/>
+      <x:c r="F2" s="145"/>
+      <x:c r="G2" s="145"/>
+      <x:c r="H2" s="145"/>
+      <x:c r="I2" s="145"/>
+      <x:c r="J2" s="145"/>
+      <x:c r="K2" s="145"/>
+      <x:c r="L2" s="145"/>
+      <x:c r="M2" s="145"/>
+      <x:c r="N2" s="145"/>
+      <x:c r="O2" s="145"/>
+      <x:c r="P2" s="145"/>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
+      <x:c r="A4" s="150" t="str">
+        <x:v>feedbackId</x:v>
+      </x:c>
+      <x:c r="B4" s="150" t="str">
+        <x:v>vfxKey</x:v>
+      </x:c>
+      <x:c r="C4" s="150" t="str">
+        <x:v>audioKey</x:v>
+      </x:c>
+      <x:c r="D4" s="150" t="str">
+        <x:v>timeScale</x:v>
+      </x:c>
+      <x:c r="E4" s="150" t="str">
+        <x:v>timeScaleSec</x:v>
+      </x:c>
+      <x:c r="F4" s="150" t="str">
+        <x:v>flashSec</x:v>
+      </x:c>
+      <x:c r="G4" s="150" t="str">
+        <x:v>shakeStrengthRefPx</x:v>
+      </x:c>
+      <x:c r="H4" s="150" t="str">
+        <x:v>shakeSec</x:v>
+      </x:c>
+      <x:c r="I4" s="150" t="str">
+        <x:v>vibrationPattern</x:v>
+      </x:c>
+      <x:c r="J4" s="150" t="str">
+        <x:v>damageNumberColorHex</x:v>
+      </x:c>
+      <x:c r="K4" s="150" t="str">
+        <x:v>damageNumberFontSizeRefPx</x:v>
+      </x:c>
+      <x:c r="L4" s="150" t="str">
+        <x:v>damageNumberLifeSec</x:v>
+      </x:c>
+      <x:c r="M4" s="150" t="str">
+        <x:v>damageNumberRiseRefPx</x:v>
+      </x:c>
+      <x:c r="N4" s="150" t="str">
+        <x:v>vfxTintColorHex</x:v>
+      </x:c>
+      <x:c r="O4" s="150" t="str">
+        <x:v>vfxScaleRefPx</x:v>
+      </x:c>
+      <x:c r="P4" s="150" t="str">
+        <x:v>description</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="132" t="str">
+        <x:v>feedback_enemy_hit</x:v>
+      </x:c>
+      <x:c r="B5" s="132" t="str">
+        <x:v>vfx_hit</x:v>
+      </x:c>
+      <x:c r="C5" s="132" t="str">
+        <x:v>sfx_hit</x:v>
+      </x:c>
+      <x:c r="D5" s="151" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="151" t="n">
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="F5" s="151" t="n">
+        <x:v>0.07</x:v>
+      </x:c>
+      <x:c r="G5" s="151" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H5" s="151" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="I5" s="132" t="str">
+        <x:v>Light</x:v>
+      </x:c>
+      <x:c r="J5" s="132" t="str">
+        <x:v>#FFFFFFFF</x:v>
+      </x:c>
+      <x:c r="K5" s="151" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L5" s="151" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="M5" s="151" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="N5" s="132" t="str">
+        <x:v>#FFFFFFFF</x:v>
+      </x:c>
+      <x:c r="O5" s="151" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="P5" s="132" t="str">
+        <x:v>普通命中：短停顿、轻震屏与白色伤害数字。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="137" t="str">
+        <x:v>feedback_weakpoint_hit</x:v>
+      </x:c>
+      <x:c r="B6" s="137" t="str">
+        <x:v>vfx_weakpoint_hit</x:v>
+      </x:c>
+      <x:c r="C6" s="137" t="str">
+        <x:v>sfx_talisman_hit</x:v>
+      </x:c>
+      <x:c r="D6" s="152" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E6" s="152" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="F6" s="152" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="G6" s="152" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H6" s="152" t="n">
+        <x:v>0.18</x:v>
+      </x:c>
+      <x:c r="I6" s="137" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="J6" s="137" t="str">
+        <x:v>#FFE066FF</x:v>
+      </x:c>
+      <x:c r="K6" s="152" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="L6" s="152" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="M6" s="152" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="N6" s="137" t="str">
+        <x:v>#FFE066FF</x:v>
+      </x:c>
+      <x:c r="O6" s="152" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="P6" s="137" t="str">
+        <x:v>弱点命中：黄色强调、较长慢动作与中等震屏。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="132" t="str">
+        <x:v>feedback_armor_break</x:v>
+      </x:c>
+      <x:c r="B7" s="132" t="str">
+        <x:v>vfx_armor_break</x:v>
+      </x:c>
+      <x:c r="C7" s="132" t="str">
+        <x:v>sfx_armor_break</x:v>
+      </x:c>
+      <x:c r="D7" s="151" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E7" s="151" t="n">
+        <x:v>0.18</x:v>
+      </x:c>
+      <x:c r="F7" s="151" t="n">
+        <x:v>0.16</x:v>
+      </x:c>
+      <x:c r="G7" s="151" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H7" s="151" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="I7" s="132" t="str">
+        <x:v>Heavy</x:v>
+      </x:c>
+      <x:c r="J7" s="132" t="str">
+        <x:v>#FF9F43FF</x:v>
+      </x:c>
+      <x:c r="K7" s="151" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="L7" s="151" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="M7" s="151" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="N7" s="132" t="str">
+        <x:v>#FF9F43FF</x:v>
+      </x:c>
+      <x:c r="O7" s="151" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="P7" s="132" t="str">
+        <x:v>破甲：橙色爆发、强震屏与重震动。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="137" t="str">
+        <x:v>feedback_projectile_reflect</x:v>
+      </x:c>
+      <x:c r="B8" s="137" t="str">
+        <x:v>vfx_projectile_cut</x:v>
+      </x:c>
+      <x:c r="C8" s="137" t="str">
+        <x:v>sfx_break</x:v>
+      </x:c>
+      <x:c r="D8" s="152" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="E8" s="152" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="F8" s="152" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="G8" s="152" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H8" s="152" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="I8" s="137" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="J8" s="137" t="str">
+        <x:v>#5DEBFFFF</x:v>
+      </x:c>
+      <x:c r="K8" s="152" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="L8" s="152" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="M8" s="152" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="N8" s="137" t="str">
+        <x:v>#5DEBFFFF</x:v>
+      </x:c>
+      <x:c r="O8" s="152" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="P8" s="137" t="str">
+        <x:v>弹反：青色切割反馈、中等震屏与短慢动作。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="132" t="str">
+        <x:v>feedback_player_hit</x:v>
+      </x:c>
+      <x:c r="B9" s="132" t="str">
+        <x:v>vfx_hit</x:v>
+      </x:c>
+      <x:c r="C9" s="132" t="str">
+        <x:v>sfx_hit</x:v>
+      </x:c>
+      <x:c r="D9" s="151" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="E9" s="151" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="F9" s="151" t="n">
+        <x:v>0.18</x:v>
+      </x:c>
+      <x:c r="G9" s="151" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H9" s="151" t="n">
+        <x:v>0.28</x:v>
+      </x:c>
+      <x:c r="I9" s="132" t="str">
+        <x:v>Heavy</x:v>
+      </x:c>
+      <x:c r="J9" s="132" t="str">
+        <x:v>#FF5C5CFF</x:v>
+      </x:c>
+      <x:c r="K9" s="151" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="L9" s="151" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="M9" s="151" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="N9" s="132" t="str">
+        <x:v>#FF5C5CFF</x:v>
+      </x:c>
+      <x:c r="O9" s="151" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="P9" s="132" t="str">
+        <x:v>玩家受击：红色闪烁、强震屏与重震动。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:P1"/>
+    <x:mergeCell ref="A2:P2"/>
+  </x:mergeCells>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="I5:I100">
+      <x:formula1>"Off,Light,Medium,Heavy"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B5:B100">
+      <x:formula1>VfxCues!$A$5:$A$100</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C5:C100">
+      <x:formula1>AudioCues!$A$5:$A$100</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -19413,7 +20332,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R687391dc045e49c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29823c3baba34b13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19811,7 +20730,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re930b761545f4a1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf1356f4200f4a54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20008,7 +20927,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2490ebd889294cd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06e2b95bc8eb4d2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20187,7 +21106,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaf23ad2ab734e21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f187028d3be4c70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20412,7 +21331,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re98529a4fd2442f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63179ccfc8524f2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20756,7 +21675,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c1a7cf1ba7c4c0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8fcdbb4bff24028"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T650: add event-driven tutorial overlay
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,36 +2,36 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc2a504e7dad442af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R57300fc71ce04b52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rf97bbec4487a470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R644ceb37036744a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R77978799654647b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Ra2edc32b3b274500"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R093fff7faba34fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rbd469915e8a94214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R20ca8c039cff44b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rd1c3377871344948"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R0c0b40cae1c6472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R53dcca452b6b48ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rc8a984aac7684edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R17964147ed344dc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R365912e991f54058"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Ra8fc33c5bf4f4225"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Ra0158251a3c24c5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R45bbc91201844beb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R5b19353e9c864d3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R0a4991dd5145408d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R5b6be75266cf494d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R4e0be75b14424224"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R8889d3eccb5e4e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rb8817bcb4cd24f16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Ra7649b777aef47c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rfc9083edcd004d57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R75fd37cf76f24057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rce011c1896844646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R51bc79c2d19c4883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R91fda32e75824395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc4f2ced293c54630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R5c338a66a1f14f79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R1819a399c97a49c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Rbd10e5166f8e495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R6afae14cbf3946b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R1df91490aad148a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rc2ac228a1c1443a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R55a98745a36d445f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R58a67a75b8244375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rbfd50cf5facb48b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rc885ccfee4f84289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R036324c807a64aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rb1adcbe41e734ebe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R819a0db257ea40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rce23ef31f9294087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R4bf04611040949df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Raa976ed81bc04095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R428021e1e15a43a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R073df4458d2a456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rde13e5748c744132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R3ffcbddacce14ac0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rda8afa7bc00745de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Ree49388fba6e4913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R28e01584d68b439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R3b0d936c43294ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rc394684100854779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R1dea22c6b37542ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R3cf5988a1d054769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R4d88275eea0d4790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R0587ceaa564a42eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -104,7 +104,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -191,6 +191,16 @@
         <x:fgColor rgb="FF2D5B75"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0E6F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -204,7 +214,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="153">
+  <x:cellXfs count="163">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -592,6 +602,24 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="9" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1329,7 +1357,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.1-sample</x:v>
+        <x:v>0.6.2-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1486,7 +1514,7 @@
       </x:c>
       <x:c r="E17" s="89" t="n">
         <x:f>COUNTA('Texts'!A5:A1000)</x:f>
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="F17" s="92"/>
       <x:c r="G17" s="92"/>
@@ -2179,7 +2207,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R712b8da6a892497c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d30372f471a4be9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2729,7 +2757,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R420f2d89be9349d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2997008431774af9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2994,7 +3022,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb516cfebc85146bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R459986cb14334185"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3258,7 +3286,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R285c6c54e3ee4c34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf403a29c34d2448e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3463,7 +3491,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad5f2b86f7464a96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc1615978d5c4565"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4345,7 +4373,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc1e5e531065428e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2efbe1ea557e48ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4553,7 +4581,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb96367313349f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra957bb9a79954153"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5107,7 +5135,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee77d58cf0d4835"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4e9f8274743467e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5313,7 +5341,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a668583c1894874"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7dac79478e44bca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5439,7 +5467,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc61318cebff44ef5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cba3c54d9cd48b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5538,7 +5566,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.1-sample</x:v>
+        <x:v>0.6.2-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6480,7 +6508,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43e6d61048964239"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3caef4d1566a4238"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7582,7 +7610,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2726946c063544d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67aded0443e24171"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7781,7 +7809,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73307976460b44b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf91e42001aa04d04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7997,7 +8025,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae84765f2a3a46f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra028ac3337c54212"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8316,7 +8344,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ede04675f8c494e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb044e6a4ead04b41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9159,6 +9187,34 @@
         <x:v>胜利结算标题</x:v>
       </x:c>
     </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="157" t="str">
+        <x:v>text_ui_tutorial_review</x:v>
+      </x:c>
+      <x:c r="B62" s="157" t="str">
+        <x:v>回放</x:v>
+      </x:c>
+      <x:c r="C62" s="157" t="str">
+        <x:v>Review Hint</x:v>
+      </x:c>
+      <x:c r="D62" s="157" t="str">
+        <x:v>教程提示回看按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="162" t="str">
+        <x:v>text_ui_tutorial_skip</x:v>
+      </x:c>
+      <x:c r="B63" s="162" t="str">
+        <x:v>继续战斗</x:v>
+      </x:c>
+      <x:c r="C63" s="162" t="str">
+        <x:v>Skip Tutorial</x:v>
+      </x:c>
+      <x:c r="D63" s="162" t="str">
+        <x:v>教程跳过按钮</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -9166,7 +9222,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1c4c55747d34cbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b383b7b99994db8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9689,7 +9745,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f33486d0184dd5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07301ae271a64ccc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10633,7 +10689,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae46a8f5bf924ade"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb48bfeed5344b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11988,7 +12044,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cd459b4324749f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R894c5414d83e4bef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13412,7 +13468,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c37658d55634ce4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3d5d8e0fefc4639"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19699,7 +19755,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97e0519569d54525"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8115c2e6f784cdd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19801,7 +19857,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c162ba0e0e44d52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb837624f24fd4533"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20332,7 +20388,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29823c3baba34b13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc90829bd92e4665"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20730,7 +20786,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf1356f4200f4a54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b875e28b3b746bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20927,7 +20983,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06e2b95bc8eb4d2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc364cf2a815e4cc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21106,7 +21162,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f187028d3be4c70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33dc61a260614f0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21331,7 +21387,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63179ccfc8524f2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d16a102ab024875"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21675,7 +21731,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8fcdbb4bff24028"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21f7b4e0796b4485"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T660: add production playable battle entry
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,36 +2,36 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc4f2ced293c54630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R5c338a66a1f14f79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R1819a399c97a49c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Rbd10e5166f8e495b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R6afae14cbf3946b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R1df91490aad148a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rc2ac228a1c1443a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R55a98745a36d445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R58a67a75b8244375"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rbfd50cf5facb48b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rc885ccfee4f84289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R036324c807a64aaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rb1adcbe41e734ebe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R819a0db257ea40cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rce23ef31f9294087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R4bf04611040949df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Raa976ed81bc04095"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R428021e1e15a43a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R073df4458d2a456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rde13e5748c744132"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R3ffcbddacce14ac0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rda8afa7bc00745de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Ree49388fba6e4913"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R28e01584d68b439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R3b0d936c43294ab9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rc394684100854779"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R1dea22c6b37542ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R3cf5988a1d054769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R4d88275eea0d4790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R0587ceaa564a42eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R01606eefc6234975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R774cf0d1d23947c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Re3b9e998a0d84888"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R5648637212294cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R11201717d2a94c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rd06c573bf0f54e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R87026027678b4e4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Ra1056abbade94c06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R84e1e307fca04c8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R478967843c614fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R53d5625cbf9c4f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R743d056cab804854"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R70436e6e73f94865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R32e51efe81cd49a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R26a03b19f4aa427d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R26687e5ff1574896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Ref9c97c69e7a4955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Re567cc90b3724884"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rc7cbdb777c3f4326"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Re89db83afecd440f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R84da2e6b7be841ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rd2cfad26f5a9408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R03962acdc00d4ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R675d66392ece42fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R11a19dde449046a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R3668ee014869456e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rb46423f02d584509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R6c813ecbd5df4147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R17db664f546343fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R5fa8cfc1ba3e418c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1357,7 +1357,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.2-sample</x:v>
+        <x:v>0.6.3-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1513,8 +1513,7 @@
         <x:v>Texts</x:v>
       </x:c>
       <x:c r="E17" s="89" t="n">
-        <x:f>COUNTA('Texts'!A5:A1000)</x:f>
-        <x:v>59</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="F17" s="92"/>
       <x:c r="G17" s="92"/>
@@ -2207,7 +2206,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d30372f471a4be9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22df8e3e638942c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2757,7 +2756,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2997008431774af9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R324fe25ebefa46de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3022,7 +3021,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R459986cb14334185"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf28ff1079c24070"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3286,7 +3285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf403a29c34d2448e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe21d7ff4f3946c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3491,7 +3490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc1615978d5c4565"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R490615ac76344eb0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4373,7 +4372,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2efbe1ea557e48ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d59acf39ad46ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4581,7 +4580,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra957bb9a79954153"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb10bc8b00094bb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5135,7 +5134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4e9f8274743467e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dcf71d611cf482c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5341,7 +5340,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7dac79478e44bca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda8f1e0c03a64540"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5467,7 +5466,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cba3c54d9cd48b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c3cb44e223547cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5566,7 +5565,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.2-sample</x:v>
+        <x:v>0.6.3-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6508,7 +6507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3caef4d1566a4238"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f4308fd12ba4dc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7610,7 +7609,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67aded0443e24171"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc891fb12677f4e1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7809,7 +7808,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf91e42001aa04d04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb00891415c6d4f3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8025,7 +8024,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra028ac3337c54212"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e56beb4bba4ce2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8344,7 +8343,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb044e6a4ead04b41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5966e2b8c4c45a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9215,6 +9214,48 @@
         <x:v>教程跳过按钮</x:v>
       </x:c>
     </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>text_game_title</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>一笔镇妖</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>One Stroke Demon</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>主菜单标题</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>text_ui_start_game</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>开始游戏</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>Start Game</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>主菜单开始按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>text_ui_select_level</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>选择关卡</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>Select Level</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>主菜单关卡选择标题</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -9222,7 +9263,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b383b7b99994db8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3762e8c2f3a1455e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9745,7 +9786,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07301ae271a64ccc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6e2d0774c3c4fe0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10689,7 +10730,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb48bfeed5344b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d2b0121bea748a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12044,7 +12085,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R894c5414d83e4bef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b024e50601a489b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13468,7 +13509,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3d5d8e0fefc4639"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26522273f9364603"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19755,7 +19796,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8115c2e6f784cdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref762a85da9f4e05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19857,7 +19898,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb837624f24fd4533"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb31df304dc5406e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20388,7 +20429,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc90829bd92e4665"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dc0800c342c4ec2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20786,7 +20827,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b875e28b3b746bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R748881610a504968"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20983,7 +21024,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc364cf2a815e4cc4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9d00f5d1aef4904"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21162,7 +21203,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33dc61a260614f0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R401e55a7f65d4932"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21387,7 +21428,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d16a102ab024875"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b2be71e2b7f4b73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21731,7 +21772,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21f7b4e0796b4485"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf11b21a9498c4693"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T690: animate fire fish prototype
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,36 +2,36 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R01606eefc6234975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R774cf0d1d23947c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Re3b9e998a0d84888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R5648637212294cad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R11201717d2a94c96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rd06c573bf0f54e8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R87026027678b4e4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Ra1056abbade94c06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R84e1e307fca04c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R478967843c614fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R53d5625cbf9c4f7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R743d056cab804854"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R70436e6e73f94865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R32e51efe81cd49a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R26a03b19f4aa427d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R26687e5ff1574896"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Ref9c97c69e7a4955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Re567cc90b3724884"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rc7cbdb777c3f4326"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Re89db83afecd440f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R84da2e6b7be841ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rd2cfad26f5a9408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R03962acdc00d4ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R675d66392ece42fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R11a19dde449046a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R3668ee014869456e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rb46423f02d584509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R6c813ecbd5df4147"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R17db664f546343fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R5fa8cfc1ba3e418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R17216b86d16e4f9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rc3d2a46e5aa64a75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R27c30e3a6cf14acb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Rf3bb8b6353864b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R03823921d3e84cb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rb749a046b28e4002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R879a2e3268ed4b37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R1cb15c7444594449"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R65c67422db794293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R9445e88513654357"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rcff5263b651e47c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R7f337c2310014279"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rcde793d72f4d4a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R9585983a11d446be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R93c6a8d7b6124891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R1227578696d04900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R9ab924adabb34d46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rd869f513d7ad410b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Raf10c7178d894fc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rb442b64f5cb14dcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R779c5098482e462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rb1a7a53e2fdb48ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rce758086f66b49cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R33ab5f2122414984"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R7c34b22efe2c4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R97a149f296cd4721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R6ad1c79a0e0a4c09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R101963167eb64aed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R64879a3b63834be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R6f1b1058042b4c1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2206,7 +2206,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22df8e3e638942c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3aa7d7f15a64046"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2756,7 +2756,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R324fe25ebefa46de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0862b9b1f0114e75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3021,7 +3021,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf28ff1079c24070"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72758b05032f4b2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3285,7 +3285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe21d7ff4f3946c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98c3a980726a4ddb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3490,7 +3490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R490615ac76344eb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6c00c586b654ce5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4372,7 +4372,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d59acf39ad46ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb22723483a047a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4580,7 +4580,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb10bc8b00094bb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69e61dbdb57145f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5134,7 +5134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dcf71d611cf482c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7462b5d74d04a58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5340,7 +5340,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda8f1e0c03a64540"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ccdd2d0b4e54915"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5466,7 +5466,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c3cb44e223547cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cb7a554a5734cc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6507,7 +6507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f4308fd12ba4dc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30db35e2962d4a86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7609,7 +7609,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc891fb12677f4e1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra93a3be4f9a94e0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7808,7 +7808,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb00891415c6d4f3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f9df5c56ec84083"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8024,7 +8024,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e56beb4bba4ce2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc89d4e3318b4fa5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8343,7 +8343,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5966e2b8c4c45a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35f2ce4c56cd4937"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9263,7 +9263,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3762e8c2f3a1455e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77e792426bf7429d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9786,7 +9786,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6e2d0774c3c4fe0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6d72e341be54dcd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10730,7 +10730,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d2b0121bea748a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e9a7d390fb14976"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10803,16 +10803,16 @@
         <x:v>enemy_fire_fish</x:v>
       </x:c>
       <x:c r="B6" s="35" t="str">
-        <x:v>Sprite</x:v>
+        <x:v>Prefab</x:v>
       </x:c>
       <x:c r="C6" s="35" t="str">
-        <x:v>Assets/_Game/Art/Enemies/fire_fish.png</x:v>
+        <x:v>Assets/_Game/Prefabs/Actors/EnemyFireFish.prefab</x:v>
       </x:c>
       <x:c r="D6" s="65" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="35" t="str">
-        <x:v>PSD导出</x:v>
+        <x:v>用户提供九帧循环动画</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -12085,7 +12085,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b024e50601a489b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb20d453e0c14127"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13509,7 +13509,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26522273f9364603"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa42468075f4440d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19796,7 +19796,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref762a85da9f4e05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffaf4d71468247f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19898,7 +19898,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb31df304dc5406e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4be554e0bde54ffe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20429,7 +20429,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dc0800c342c4ec2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135d4125e3d9443d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20827,7 +20827,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R748881610a504968"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03dca1ca9b6f4931"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21024,7 +21024,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9d00f5d1aef4904"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R435579996d304b7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21203,7 +21203,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R401e55a7f65d4932"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e2491f763074c0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21428,7 +21428,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b2be71e2b7f4b73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R325d323dfe72401a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21772,7 +21772,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf11b21a9498c4693"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra90588453a954c51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T694: animate player prototype
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,36 +2,36 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R17216b86d16e4f9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rc3d2a46e5aa64a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R27c30e3a6cf14acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Rf3bb8b6353864b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R03823921d3e84cb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rb749a046b28e4002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R879a2e3268ed4b37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R1cb15c7444594449"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R65c67422db794293"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R9445e88513654357"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rcff5263b651e47c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R7f337c2310014279"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rcde793d72f4d4a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R9585983a11d446be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R93c6a8d7b6124891"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R1227578696d04900"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R9ab924adabb34d46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rd869f513d7ad410b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Raf10c7178d894fc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rb442b64f5cb14dcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R779c5098482e462b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rb1a7a53e2fdb48ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rce758086f66b49cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R33ab5f2122414984"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R7c34b22efe2c4cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R97a149f296cd4721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R6ad1c79a0e0a4c09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R101963167eb64aed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R64879a3b63834be7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R6f1b1058042b4c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R417807e97dc84507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R5284a44e7baa4ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R242cc72bfd1e4582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R18b62cc1c09f4ee5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rdc4df32eb1114a98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R2aff405405b2472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Ra00e58bd0db54f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R6bde5152f4aa4758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R14386e30dee14a4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Re5f250b955844b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Re10418abd39a4a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rc858849069fc4ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R8e118aa5dbb04877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Ref065916bed24efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R0b3e3ba729c54544"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R88d1fb9821ae4f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R3f13512223774d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R01797f26c5204a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R947fbddc6d7b4124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R4f6ad4dcedd943ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rebc3c7c1cf22419c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rbeb478abdd3946d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R893fd84be78f4633"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R3d6b7690dbc04c03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Ra56b35a1efea4414"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R6f011428cf074556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rda26075b399249eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Re29103d8772b47ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R04636c4ff3444529"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R260764ee5f924398"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1357,7 +1357,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.3-sample</x:v>
+        <x:v>0.6.4-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -2206,7 +2206,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3aa7d7f15a64046"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba43388ce579416f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2756,7 +2756,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0862b9b1f0114e75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90b103bcf61f4148"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3021,7 +3021,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72758b05032f4b2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R239125102293452a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3285,7 +3285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98c3a980726a4ddb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55edfa5a19d741b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3490,7 +3490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6c00c586b654ce5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red2231c1e3ff4b0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4372,7 +4372,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb22723483a047a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcf1d5f85f514d40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4580,7 +4580,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69e61dbdb57145f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d59a8ad45c24445"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5134,7 +5134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7462b5d74d04a58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R967e110386f8470f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5340,7 +5340,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ccdd2d0b4e54915"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c9a2513fb944ecf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5466,7 +5466,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cb7a554a5734cc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0271dc6387e47b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5565,7 +5565,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.3-sample</x:v>
+        <x:v>0.6.4-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6507,7 +6507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30db35e2962d4a86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96b8e01e0c38452d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7609,7 +7609,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra93a3be4f9a94e0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dda6e46a23b45b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7808,7 +7808,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f9df5c56ec84083"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a0d6b3819fc4331"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8024,7 +8024,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc89d4e3318b4fa5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd29697315dae4491"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8343,7 +8343,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35f2ce4c56cd4937"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1be473bc7e49ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9263,7 +9263,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77e792426bf7429d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10b64803fa6c4391"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9786,7 +9786,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6d72e341be54dcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref5cef567378476c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10730,7 +10730,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e9a7d390fb14976"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64be8423ea434bf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10786,16 +10786,16 @@
         <x:v>char_moyan_idle</x:v>
       </x:c>
       <x:c r="B5" s="35" t="str">
-        <x:v>Sprite</x:v>
+        <x:v>Prefab</x:v>
       </x:c>
       <x:c r="C5" s="35" t="str">
-        <x:v>Assets/_Game/Art/Characters/Moyan/moyan_idle.png</x:v>
+        <x:v>Assets/_Game/Prefabs/Actors/PlayerMoyan.prefab</x:v>
       </x:c>
       <x:c r="D5" s="65" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="35" t="str">
-        <x:v>PSD导出静态主角</x:v>
+        <x:v>用户提供的九帧待机与十二帧攻击动画Prefab</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -12085,7 +12085,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb20d453e0c14127"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a3ab646afa84583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13509,7 +13509,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa42468075f4440d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4696c6918ad8425f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19796,7 +19796,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffaf4d71468247f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c4dfd66887c4168"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19898,7 +19898,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4be554e0bde54ffe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabfae14b80524cee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20429,7 +20429,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135d4125e3d9443d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f8be81376de45af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20827,7 +20827,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03dca1ca9b6f4931"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe9f55c652ee4bc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21024,7 +21024,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R435579996d304b7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c9783aaff674241"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21203,7 +21203,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e2491f763074c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b5a050f9ef74185"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21428,7 +21428,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R325d323dfe72401a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2da7d516641f4595"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21772,7 +21772,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra90588453a954c51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3acd6a690f0243be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T695: animate enemy death effect
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,36 +2,36 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R417807e97dc84507"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R5284a44e7baa4ee2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R242cc72bfd1e4582"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R18b62cc1c09f4ee5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rdc4df32eb1114a98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R2aff405405b2472a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Ra00e58bd0db54f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R6bde5152f4aa4758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R14386e30dee14a4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Re5f250b955844b43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Re10418abd39a4a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rc858849069fc4ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R8e118aa5dbb04877"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Ref065916bed24efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R0b3e3ba729c54544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R88d1fb9821ae4f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R3f13512223774d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R01797f26c5204a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R947fbddc6d7b4124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R4f6ad4dcedd943ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rebc3c7c1cf22419c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rbeb478abdd3946d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R893fd84be78f4633"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R3d6b7690dbc04c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Ra56b35a1efea4414"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R6f011428cf074556"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rda26075b399249eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Re29103d8772b47ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R04636c4ff3444529"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R260764ee5f924398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8838e98ef4f24043"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R4029d5709cee4116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R1fff10b0453f47a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Rb8bc64ccdd6c41ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rc30df90984a54db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R2fcace96be82405a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R3b33576875ba463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R7395051af1fc4bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R0fa9d1c9a4ec42f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R16eea3b100b445c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rc5704d2d57d34bcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R7e45d2337bf44ba0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R4b746cb941d44de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Rda9c53409b2d4f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R039c6311c7e0484b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Rfc47cf69575b4cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Rfdb3fec8a6f045a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R6df1d0f42d554fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R258a987a50c54552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R13881eaa03d441d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R945721061b324a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R792879bff9144882"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R3c9b956da1b145a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rf006cc908444499a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R33f703e480064ad9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Refbe780746334d86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Ra60660bf3b0b43fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rc79a181549a84e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R76b6d1075de64d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R8732bbe6b4984716"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -104,7 +104,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -201,6 +201,11 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0E6F5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -214,7 +219,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="163">
+  <x:cellXfs count="169">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -621,6 +626,33 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1528,7 +1560,7 @@
       </x:c>
       <x:c r="E18" s="89" t="n">
         <x:f>COUNTA('AssetManifest'!A5:A1000)</x:f>
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F18" s="92"/>
       <x:c r="G18" s="92"/>
@@ -1540,7 +1572,7 @@
       </x:c>
       <x:c r="E19" t="n">
         <x:f>COUNTA('FeedbackCues'!A5:A1000)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2206,7 +2238,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba43388ce579416f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R091cdd6c8970477a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2756,7 +2788,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90b103bcf61f4148"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra13829ec5ba04471"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3021,7 +3053,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R239125102293452a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95b322bbbf634d4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3285,7 +3317,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55edfa5a19d741b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb117ce6910894843"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3490,7 +3522,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red2231c1e3ff4b0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc62ff4f4c55a47e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4372,7 +4404,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcf1d5f85f514d40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb24a4659f44b4673"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4580,7 +4612,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d59a8ad45c24445"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe4823c8d6484725"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5134,7 +5166,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R967e110386f8470f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04623cf5a5c84d6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5340,7 +5372,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c9a2513fb944ecf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae70499ddb6842d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5466,7 +5498,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0271dc6387e47b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4df5658f42744fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5565,7 +5597,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.4-sample</x:v>
+        <x:v>0.6.5-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6507,7 +6539,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96b8e01e0c38452d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51ce7a24d4bf456c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7609,7 +7641,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dda6e46a23b45b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b6c59719d744438"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7808,7 +7840,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a0d6b3819fc4331"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cda96b27e46431d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8024,7 +8056,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd29697315dae4491"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fcf67d52a0147db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8343,7 +8375,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1be473bc7e49ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7c286dcfa7e4137"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9263,7 +9295,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10b64803fa6c4391"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R689ca76b75714483"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9786,7 +9818,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref5cef567378476c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59aaa5cf080448e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10723,6 +10755,29 @@
         <x:v>30</x:v>
       </x:c>
     </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="167" t="str">
+        <x:v>vfx_enemy_death</x:v>
+      </x:c>
+      <x:c r="B43" s="167" t="str">
+        <x:v>vfx_enemy_death</x:v>
+      </x:c>
+      <x:c r="C43" s="167" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="D43" s="167" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E43" s="168" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F43" s="167" t="str">
+        <x:v>VFX</x:v>
+      </x:c>
+      <x:c r="G43" s="167" t="n">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -10730,7 +10785,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64be8423ea434bf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829f6422ca964057"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12073,6 +12128,23 @@
         <x:v>模板占位路径，导入资源后更新</x:v>
       </x:c>
     </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="167" t="str">
+        <x:v>vfx_enemy_death</x:v>
+      </x:c>
+      <x:c r="B81" s="167" t="str">
+        <x:v>Prefab</x:v>
+      </x:c>
+      <x:c r="C81" s="167" t="str">
+        <x:v>Assets/_Game/Art/VFX/Animated/EnemyDeath/vfx_enemy_death.prefab</x:v>
+      </x:c>
+      <x:c r="D81" s="168" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E81" s="167" t="str">
+        <x:v>用户提供的十一帧怪物死亡爆炸动画</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -12085,7 +12157,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a3ab646afa84583"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e088502dd6e4345"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13509,7 +13581,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4696c6918ad8425f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74c6f7420e48463a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19796,7 +19868,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c4dfd66887c4168"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3da8dbd0ad1e4867"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19898,7 +19970,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabfae14b80524cee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e35ab6a1937432a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20263,6 +20335,56 @@
       </x:c>
       <x:c r="P9" s="132" t="str">
         <x:v>玩家受击：红色闪烁、强震屏与重震动。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="167" t="str">
+        <x:v>feedback_enemy_death</x:v>
+      </x:c>
+      <x:c r="B10" s="167" t="str">
+        <x:v>vfx_enemy_death</x:v>
+      </x:c>
+      <x:c r="C10" s="167" t="str">
+        <x:v>sfx_hit</x:v>
+      </x:c>
+      <x:c r="D10" s="167" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E10" s="167" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="F10" s="167" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="G10" s="167" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H10" s="167" t="n">
+        <x:v>0.16</x:v>
+      </x:c>
+      <x:c r="I10" s="167" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="J10" s="167" t="str">
+        <x:v>#FFFFFFFF</x:v>
+      </x:c>
+      <x:c r="K10" s="167" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="L10" s="167" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="M10" s="167" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="N10" s="167" t="str">
+        <x:v>#FFFFFFFF</x:v>
+      </x:c>
+      <x:c r="O10" s="167" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="P10" s="167" t="str">
+        <x:v>怪物死亡：白色爆炸序列、中等震屏与震动；不承担死亡判定。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20429,7 +20551,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f8be81376de45af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec62751c9da543b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20827,7 +20949,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe9f55c652ee4bc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R560aa0e2989f4e2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21024,7 +21146,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c9783aaff674241"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41fab43d2cd4395"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21203,7 +21325,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b5a050f9ef74185"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dba688c1c134e46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21428,7 +21550,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2da7d516641f4595"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc64c7e70334a70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21772,7 +21894,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3acd6a690f0243be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5215dda5e75d4935"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T698: add lightning stroke trail
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,36 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8838e98ef4f24043"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R4029d5709cee4116"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R1fff10b0453f47a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Rb8bc64ccdd6c41ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rc30df90984a54db6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R2fcace96be82405a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R3b33576875ba463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R7395051af1fc4bd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R0fa9d1c9a4ec42f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R16eea3b100b445c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rc5704d2d57d34bcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R7e45d2337bf44ba0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R4b746cb941d44de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Rda9c53409b2d4f8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R039c6311c7e0484b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Rfc47cf69575b4cee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Rfdb3fec8a6f045a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R6df1d0f42d554fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R258a987a50c54552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R13881eaa03d441d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R945721061b324a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R792879bff9144882"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R3c9b956da1b145a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rf006cc908444499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R33f703e480064ad9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Refbe780746334d86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Ra60660bf3b0b43fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rc79a181549a84e83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R76b6d1075de64d4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R8732bbe6b4984716"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra39566d59c2f4030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rf6b514aeeb2d43dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R254fb16890bc4dd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Raf9fde33df164117"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rabae1ea855c34266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rcbece27823d141d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R319372b72a914afa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rd3515a7903e2468e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Reed7a446eb6049c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rba37788718684e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R85cc871d0bd343ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Re7cb2e6f2e1a4223"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R977dd4996f094c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R81790297477c4d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R3a6356fc6edc4369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R3aed87bb6ac04562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Re0b8fd4e23d0453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rc6325ad5dd4f4cc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R758c188f902a431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R78caee4554d64d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R453cee0f52f04a0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rf6a73568524546fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R23b7dbea6a944e35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R49f22c20af4b4e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rf203c74448dd43e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R2bbf85ff1b5a4166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rf42da579c6da4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R41b9d4c1113742f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R051e1ea8222e4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="Rdcffeb57b7a44282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="Re760a3831f1f4698"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +48,7 @@
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="0.000"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -103,8 +104,13 @@
       <x:color rgb="FF17202A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF155724"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -206,6 +212,36 @@
         <x:fgColor rgb="FFC0E6F5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2D5B75"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6E9F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F3E6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -219,7 +255,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="169">
+  <x:cellXfs count="203">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -653,6 +689,78 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1374,7 +1482,7 @@
         <x:v>Schema版本</x:v>
       </x:c>
       <x:c r="B5" s="25" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Players</x:v>
@@ -1389,7 +1497,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.4-sample</x:v>
+        <x:v>0.6.6-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1573,6 +1681,14 @@
       <x:c r="E19" t="n">
         <x:f>COUNTA('FeedbackCues'!A5:A1000)</x:f>
         <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="D20" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="E20" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2238,7 +2354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R091cdd6c8970477a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5938c542bf804044"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2788,7 +2904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra13829ec5ba04471"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fe7e3f07957486b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3053,7 +3169,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95b322bbbf634d4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc27508c18f74e57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3317,7 +3433,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb117ce6910894843"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb54b4ac7a534ebd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3522,7 +3638,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc62ff4f4c55a47e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec7127ee6c2744ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4404,7 +4520,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb24a4659f44b4673"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a41a3df4d346b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4612,7 +4728,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe4823c8d6484725"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac483de00c0945a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5166,7 +5282,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04623cf5a5c84d6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63ed2ac407f84c09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5372,7 +5488,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae70499ddb6842d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7ddbb341fcc4612"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5498,7 +5614,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4df5658f42744fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30331ad01c2d4f53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5575,7 +5691,7 @@
         <x:v>int</x:v>
       </x:c>
       <x:c r="C5" s="68" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D5" s="35"/>
       <x:c r="E5" s="35"/>
@@ -5597,7 +5713,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.5-sample</x:v>
+        <x:v>0.6.6-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6539,7 +6655,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51ce7a24d4bf456c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41e6f39de26847bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7641,7 +7757,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b6c59719d744438"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R480ca52291fe4fb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7840,7 +7956,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cda96b27e46431d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf62d122158054c80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8056,7 +8172,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fcf67d52a0147db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20702f2e37914080"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8375,7 +8491,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7c286dcfa7e4137"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re86bdb2ef5a14c8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9295,7 +9411,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R689ca76b75714483"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf223749d6324486e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9818,7 +9934,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59aaa5cf080448e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2e4a4559a0c430d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10785,7 +10901,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829f6422ca964057"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfeb3f78c66ea4200"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12157,7 +12273,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e088502dd6e4345"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffa35ac4c17a44ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13581,7 +13697,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74c6f7420e48463a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf23b69f0cdb44cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19848,6 +19964,348 @@
         <x:v>反馈配置用途说明。</x:v>
       </x:c>
     </x:row>
+    <x:row r="271">
+      <x:c r="A271" s="189" t="str">
+        <x:v>Stances</x:v>
+      </x:c>
+      <x:c r="B271" s="189" t="str">
+        <x:v>strokeTrailStyleId</x:v>
+      </x:c>
+      <x:c r="C271" s="189" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D271" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E271" s="189"/>
+      <x:c r="F271" s="189"/>
+      <x:c r="G271" s="189"/>
+      <x:c r="H271" s="189"/>
+      <x:c r="I271" s="189" t="str">
+        <x:v>StrokeTrailStyles.styleId</x:v>
+      </x:c>
+      <x:c r="J271" s="189" t="str">
+        <x:v>架势选择的画笔表现样式外键。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272">
+      <x:c r="A272" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B272" s="189" t="str">
+        <x:v>styleId</x:v>
+      </x:c>
+      <x:c r="C272" s="189" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D272" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E272" s="189"/>
+      <x:c r="F272" s="189"/>
+      <x:c r="G272" s="189"/>
+      <x:c r="H272" s="189"/>
+      <x:c r="I272" s="189"/>
+      <x:c r="J272" s="189" t="str">
+        <x:v>画笔样式稳定ID。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273">
+      <x:c r="A273" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B273" s="189" t="str">
+        <x:v>outerColorHex</x:v>
+      </x:c>
+      <x:c r="C273" s="189" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D273" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E273" s="189"/>
+      <x:c r="F273" s="189"/>
+      <x:c r="G273" s="189"/>
+      <x:c r="H273" s="189"/>
+      <x:c r="I273" s="189"/>
+      <x:c r="J273" s="189" t="str">
+        <x:v>外层辉光颜色，格式为#RRGGBBAA。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274">
+      <x:c r="A274" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B274" s="189" t="str">
+        <x:v>bodyColorHex</x:v>
+      </x:c>
+      <x:c r="C274" s="189" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D274" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E274" s="189"/>
+      <x:c r="F274" s="189"/>
+      <x:c r="G274" s="189"/>
+      <x:c r="H274" s="189"/>
+      <x:c r="I274" s="189"/>
+      <x:c r="J274" s="189" t="str">
+        <x:v>主体轨迹颜色，格式为#RRGGBBAA。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="275">
+      <x:c r="A275" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B275" s="189" t="str">
+        <x:v>coreColorHex</x:v>
+      </x:c>
+      <x:c r="C275" s="189" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D275" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E275" s="189"/>
+      <x:c r="F275" s="189"/>
+      <x:c r="G275" s="189"/>
+      <x:c r="H275" s="189"/>
+      <x:c r="I275" s="189"/>
+      <x:c r="J275" s="189" t="str">
+        <x:v>核心高光颜色，格式为#RRGGBBAA。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="276">
+      <x:c r="A276" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B276" s="189" t="str">
+        <x:v>outerWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="C276" s="189" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D276" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E276" s="189"/>
+      <x:c r="F276" s="189" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G276" s="189" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H276" s="189"/>
+      <x:c r="I276" s="189"/>
+      <x:c r="J276" s="189" t="str">
+        <x:v>外层宽度相对架势基础笔宽的倍率。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277">
+      <x:c r="A277" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B277" s="189" t="str">
+        <x:v>bodyWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="C277" s="189" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D277" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E277" s="189"/>
+      <x:c r="F277" s="189" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G277" s="189" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H277" s="189"/>
+      <x:c r="I277" s="189"/>
+      <x:c r="J277" s="189" t="str">
+        <x:v>主体宽度相对架势基础笔宽的倍率。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="278">
+      <x:c r="A278" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B278" s="189" t="str">
+        <x:v>coreWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="C278" s="189" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D278" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E278" s="189"/>
+      <x:c r="F278" s="189" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G278" s="189" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H278" s="189"/>
+      <x:c r="I278" s="189"/>
+      <x:c r="J278" s="189" t="str">
+        <x:v>核心宽度相对架势基础笔宽的倍率。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279">
+      <x:c r="A279" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B279" s="189" t="str">
+        <x:v>branchColorHex</x:v>
+      </x:c>
+      <x:c r="C279" s="189" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D279" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E279" s="189"/>
+      <x:c r="F279" s="189"/>
+      <x:c r="G279" s="189"/>
+      <x:c r="H279" s="189"/>
+      <x:c r="I279" s="189"/>
+      <x:c r="J279" s="189" t="str">
+        <x:v>分支电弧颜色，格式为#RRGGBBAA。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280">
+      <x:c r="A280" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B280" s="189" t="str">
+        <x:v>branchSpacingRefPx</x:v>
+      </x:c>
+      <x:c r="C280" s="189" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D280" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E280" s="189"/>
+      <x:c r="F280" s="189" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G280" s="189" t="n">
+        <x:v>1920</x:v>
+      </x:c>
+      <x:c r="H280" s="189"/>
+      <x:c r="I280" s="189"/>
+      <x:c r="J280" s="189" t="str">
+        <x:v>相邻分支电弧在参考路径上的目标间距。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281">
+      <x:c r="A281" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B281" s="189" t="str">
+        <x:v>branchLengthRefPx</x:v>
+      </x:c>
+      <x:c r="C281" s="189" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D281" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E281" s="189"/>
+      <x:c r="F281" s="189" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G281" s="189" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="H281" s="189"/>
+      <x:c r="I281" s="189"/>
+      <x:c r="J281" s="189" t="str">
+        <x:v>分支电弧的参考像素长度。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282">
+      <x:c r="A282" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B282" s="189" t="str">
+        <x:v>branchJitterRefPx</x:v>
+      </x:c>
+      <x:c r="C282" s="189" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D282" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E282" s="189"/>
+      <x:c r="F282" s="189" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G282" s="189" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="H282" s="189"/>
+      <x:c r="I282" s="189"/>
+      <x:c r="J282" s="189" t="str">
+        <x:v>分支电弧折点的最大参考像素抖动。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283">
+      <x:c r="A283" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B283" s="189" t="str">
+        <x:v>branchWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="C283" s="189" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="D283" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E283" s="189"/>
+      <x:c r="F283" s="189" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G283" s="189" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H283" s="189"/>
+      <x:c r="I283" s="189"/>
+      <x:c r="J283" s="189" t="str">
+        <x:v>分支宽度相对架势基础笔宽的倍率。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="284">
+      <x:c r="A284" s="189" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B284" s="189" t="str">
+        <x:v>branchSegmentCount</x:v>
+      </x:c>
+      <x:c r="C284" s="189" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="D284" s="202" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E284" s="189"/>
+      <x:c r="F284" s="189" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G284" s="189" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H284" s="189"/>
+      <x:c r="I284" s="189"/>
+      <x:c r="J284" s="189" t="str">
+        <x:v>单条分支电弧的线段数量。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -19868,7 +20326,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3da8dbd0ad1e4867"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bcab6a7d35149df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19970,7 +20428,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e35ab6a1937432a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4bbf3f02f6746e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20407,6 +20865,165 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="21" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="173" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B1" s="173"/>
+      <x:c r="C1" s="173"/>
+      <x:c r="D1" s="173"/>
+      <x:c r="E1" s="173"/>
+      <x:c r="F1" s="173"/>
+      <x:c r="G1" s="173"/>
+      <x:c r="H1" s="173"/>
+      <x:c r="I1" s="173"/>
+      <x:c r="J1" s="173"/>
+      <x:c r="K1" s="173"/>
+      <x:c r="L1" s="173"/>
+      <x:c r="M1" s="173"/>
+    </x:row>
+    <x:row r="2" ht="38" customHeight="1">
+      <x:c r="A2" s="177" t="str">
+        <x:v>画笔视觉样式。颜色、层宽与电弧参数全部来自配置；Prefab只保存分层组件引用。</x:v>
+      </x:c>
+      <x:c r="B2" s="177"/>
+      <x:c r="C2" s="177"/>
+      <x:c r="D2" s="177"/>
+      <x:c r="E2" s="177"/>
+      <x:c r="F2" s="177"/>
+      <x:c r="G2" s="177"/>
+      <x:c r="H2" s="177"/>
+      <x:c r="I2" s="177"/>
+      <x:c r="J2" s="177"/>
+      <x:c r="K2" s="177"/>
+      <x:c r="L2" s="177"/>
+      <x:c r="M2" s="177"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
+      <x:c r="M3"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="182" t="str">
+        <x:v>styleId</x:v>
+      </x:c>
+      <x:c r="B4" s="182" t="str">
+        <x:v>outerColorHex</x:v>
+      </x:c>
+      <x:c r="C4" s="182" t="str">
+        <x:v>bodyColorHex</x:v>
+      </x:c>
+      <x:c r="D4" s="182" t="str">
+        <x:v>coreColorHex</x:v>
+      </x:c>
+      <x:c r="E4" s="182" t="str">
+        <x:v>outerWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="F4" s="182" t="str">
+        <x:v>bodyWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="G4" s="182" t="str">
+        <x:v>coreWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="H4" s="182" t="str">
+        <x:v>branchColorHex</x:v>
+      </x:c>
+      <x:c r="I4" s="182" t="str">
+        <x:v>branchSpacingRefPx</x:v>
+      </x:c>
+      <x:c r="J4" s="182" t="str">
+        <x:v>branchLengthRefPx</x:v>
+      </x:c>
+      <x:c r="K4" s="182" t="str">
+        <x:v>branchJitterRefPx</x:v>
+      </x:c>
+      <x:c r="L4" s="182" t="str">
+        <x:v>branchWidthMultiplier</x:v>
+      </x:c>
+      <x:c r="M4" s="182" t="str">
+        <x:v>branchSegmentCount</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="195" t="str">
+        <x:v>stroke_trail_lightning_c</x:v>
+      </x:c>
+      <x:c r="B5" s="195" t="str">
+        <x:v>#39D5FFFF</x:v>
+      </x:c>
+      <x:c r="C5" s="195" t="str">
+        <x:v>#9AF0FFFF</x:v>
+      </x:c>
+      <x:c r="D5" s="195" t="str">
+        <x:v>#FFFFFFFF</x:v>
+      </x:c>
+      <x:c r="E5" s="196" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
+      <x:c r="F5" s="196" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="G5" s="196" t="n">
+        <x:v>0.32</x:v>
+      </x:c>
+      <x:c r="H5" s="195" t="str">
+        <x:v>#C8F8FFFF</x:v>
+      </x:c>
+      <x:c r="I5" s="196" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="J5" s="196" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="K5" s="196" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L5" s="196" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="M5" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:M1"/>
+    <x:mergeCell ref="A2:M2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -20420,6 +21037,8 @@
     <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -20434,10 +21053,12 @@
       <x:c r="G1" s="52"/>
       <x:c r="H1" s="52"/>
       <x:c r="I1" s="52"/>
+      <x:c r="J1"/>
+      <x:c r="K1"/>
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>架势倍率、轨迹宽度和切换效果。运行时不能在Inspector复制这些数值。</x:v>
+        <x:v>架势倍率、轨迹宽度、画笔样式和切换效果。运行时不能在Inspector复制这些数值。</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -20447,6 +21068,21 @@
       <x:c r="G2" s="13"/>
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
@@ -20476,8 +21112,11 @@
       <x:c r="I4" s="58" t="str">
         <x:v>onSwitchEffectGroupId</x:v>
       </x:c>
-      <x:c r="J4" t="str">
+      <x:c r="J4" s="182" t="str">
         <x:v>assetKey</x:v>
+      </x:c>
+      <x:c r="K4" s="182" t="str">
+        <x:v>strokeTrailStyleId</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -20508,8 +21147,11 @@
       <x:c r="I5" s="35" t="str">
         <x:v>fx_switch_to_blade</x:v>
       </x:c>
-      <x:c r="J5" t="str">
+      <x:c r="J5" s="200" t="str">
         <x:v>icon_stance_blade</x:v>
+      </x:c>
+      <x:c r="K5" s="200" t="str">
+        <x:v>stroke_trail_lightning_c</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -20540,18 +21182,21 @@
       <x:c r="I6" s="35" t="str">
         <x:v>fx_switch_to_talisman</x:v>
       </x:c>
-      <x:c r="J6" t="str">
+      <x:c r="J6" s="189" t="str">
         <x:v>icon_stance_talisman</x:v>
+      </x:c>
+      <x:c r="K6" s="189" t="str">
+        <x:v>stroke_trail_lightning_c</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec62751c9da543b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68aedcc9dd82478c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20949,7 +21594,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R560aa0e2989f4e2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e10dbe0b65e4d43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21146,7 +21791,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41fab43d2cd4395"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce76e673f3f04070"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21325,7 +21970,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dba688c1c134e46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0240f41c4573409e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21550,7 +22195,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc64c7e70334a70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf379f91963094f16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21894,7 +22539,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5215dda5e75d4935"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5373fcc0e062411a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T699A: integrate production projectiles
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,37 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra39566d59c2f4030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rf6b514aeeb2d43dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R254fb16890bc4dd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Raf9fde33df164117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rabae1ea855c34266"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rcbece27823d141d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R319372b72a914afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rd3515a7903e2468e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Reed7a446eb6049c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rba37788718684e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R85cc871d0bd343ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Re7cb2e6f2e1a4223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R977dd4996f094c7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R81790297477c4d9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R3a6356fc6edc4369"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R3aed87bb6ac04562"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Re0b8fd4e23d0453d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rc6325ad5dd4f4cc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R758c188f902a431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R78caee4554d64d66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R453cee0f52f04a0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rf6a73568524546fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R23b7dbea6a944e35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R49f22c20af4b4e43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rf203c74448dd43e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R2bbf85ff1b5a4166"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rf42da579c6da4cc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R41b9d4c1113742f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="R051e1ea8222e4873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="Rdcffeb57b7a44282"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="Re760a3831f1f4698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rcd18505c09d04e96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Re85e863bffd248dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Re70675be73934d0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R461c645dba8b472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rfd0f1ed62f57441f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rc6973b48c0614cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Re63cc169d3dc4140"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R3e0cb621371c4728"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R5bf77b3b97d84708"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Ref4b37832e6745c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R1efe977d4f124338"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rc1bcf1467bd94f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R4142b5950c6f40fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R7f10bf0564444646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R6fa88a5a49f04b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R4d2864b119784755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R0ba60bde330b4042"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rd264f953ca0b403b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R0d8db692f334400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R1d1173529ebf46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R3dee4e9533ab4dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R5ea7382f0c6c4c5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R603217db23364ada"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R9c8cdde0210c45b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R403590678aa448e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rda288345d13f42b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rbf46cfbb044847c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rdd399a8518c84bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rb63cd325f0844c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R3e85d18b95624d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="R6d22a549c6b446c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1497,7 +1497,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.6-sample</x:v>
+        <x:v>0.6.7-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -2354,7 +2354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5938c542bf804044"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R505fd93fad9f4070"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2904,7 +2904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fe7e3f07957486b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65c7f4b0780c4184"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2999,10 +2999,10 @@
         <x:v>move_ground_left</x:v>
       </x:c>
       <x:c r="C5" s="72" t="n">
-        <x:v>260</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="D5" s="72" t="n">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E5" s="68" t="n">
         <x:v>8</x:v>
@@ -3032,10 +3032,10 @@
         <x:v>move_ground_left</x:v>
       </x:c>
       <x:c r="C6" s="72" t="n">
-        <x:v>320</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="D6" s="72" t="n">
-        <x:v>3.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E6" s="68" t="n">
         <x:v>10</x:v>
@@ -3067,10 +3067,10 @@
         <x:v>move_ground_left</x:v>
       </x:c>
       <x:c r="C7" s="72" t="n">
-        <x:v>280</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="D7" s="72" t="n">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E7" s="68" t="n">
         <x:v>16</x:v>
@@ -3102,10 +3102,10 @@
         <x:v>move_ground_left</x:v>
       </x:c>
       <x:c r="C8" s="72" t="n">
-        <x:v>360</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="D8" s="72" t="n">
-        <x:v>2.5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E8" s="68" t="n">
         <x:v>18</x:v>
@@ -3135,10 +3135,10 @@
         <x:v>move_ground_left</x:v>
       </x:c>
       <x:c r="C9" s="72" t="n">
-        <x:v>220</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D9" s="72" t="n">
-        <x:v>4.5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E9" s="68" t="n">
         <x:v>22</x:v>
@@ -3169,7 +3169,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc27508c18f74e57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cf18eb674a1419a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3433,7 +3433,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb54b4ac7a534ebd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ef8c2eceab748b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3638,7 +3638,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec7127ee6c2744ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7684439396044599"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4520,7 +4520,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a41a3df4d346b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff881f2adbd14334"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4728,7 +4728,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac483de00c0945a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra07d87effbfe4e5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5282,7 +5282,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63ed2ac407f84c09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4fb5f56c93c49dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5488,7 +5488,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7ddbb341fcc4612"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f2d4467ab14bc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5614,7 +5614,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30331ad01c2d4f53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73f89f7100b740ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5713,7 +5713,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.6-sample</x:v>
+        <x:v>0.6.7-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6655,7 +6655,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41e6f39de26847bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a3589943bd54126"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7757,7 +7757,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R480ca52291fe4fb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2de1cc8a7449a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7956,7 +7956,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf62d122158054c80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R445807d47b5644a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8172,7 +8172,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20702f2e37914080"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R114b977ab7104bdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8491,7 +8491,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re86bdb2ef5a14c8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e1b340e53f24b1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9411,7 +9411,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf223749d6324486e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71a31bdecac749b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9934,7 +9934,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2e4a4559a0c430d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re59fbbe76e0844a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10901,7 +10901,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfeb3f78c66ea4200"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95265f875b444a53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12273,7 +12273,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffa35ac4c17a44ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcffed01b6db149bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13697,7 +13697,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf23b69f0cdb44cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3baf6da4ea2a4c2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20326,7 +20326,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bcab6a7d35149df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0aabb4361c5145d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20428,7 +20428,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4bbf3f02f6746e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4002b8104fa54564"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21196,7 +21196,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68aedcc9dd82478c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41f8d5a6bc043c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21594,7 +21594,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e10dbe0b65e4d43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R825cf856ef7c4890"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21791,7 +21791,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce76e673f3f04070"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7ce3f330db4b7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21970,7 +21970,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0240f41c4573409e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10ab9fbff5894ffc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22195,7 +22195,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf379f91963094f16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b5be335053a4263"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22539,7 +22539,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5373fcc0e062411a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1066ba924f70498c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T699B: document workbook fields in Chinese
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,37 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rcd18505c09d04e96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Re85e863bffd248dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Re70675be73934d0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R461c645dba8b472a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rfd0f1ed62f57441f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rc6973b48c0614cfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Re63cc169d3dc4140"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R3e0cb621371c4728"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R5bf77b3b97d84708"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Ref4b37832e6745c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R1efe977d4f124338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rc1bcf1467bd94f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R4142b5950c6f40fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R7f10bf0564444646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R6fa88a5a49f04b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R4d2864b119784755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R0ba60bde330b4042"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rd264f953ca0b403b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R0d8db692f334400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R1d1173529ebf46d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R3dee4e9533ab4dff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R5ea7382f0c6c4c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R603217db23364ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R9c8cdde0210c45b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R403590678aa448e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rda288345d13f42b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rbf46cfbb044847c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rdd399a8518c84bbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rb63cd325f0844c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R3e85d18b95624d68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="R6d22a549c6b446c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R26945a771df94fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rcd594c9383e24add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Ref0863d7f42c428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R55213026b2484006"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rbb719b3e4c864b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R1b0f0cf996d14fac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Re076451cb41e46f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Rd337833ea08845af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R6e375691102a4741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R1393c932c8754beb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R103b8a0fee0a409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R47b0d020c6cf4d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="Rbd3b727932d04ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R3057f3b86cef4140"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R2935b745a93a4d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R5a49ec26d1be409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="Re30e861369954ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rfab03e094be84327"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rbf519b38152b44e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R8c56395e701640af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R6f5570a59a7f4e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="R0c6906dd44534454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R1e6dd520e8b14762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R811ae734f47f42fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rd9225989bd9e4229"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R612955c77549468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rfdf8c139cd41470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R581efbfbb32541eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rab8b6539cac649e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R3856ba6eb2b34d1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="R5b460666e5bd49b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48,7 +48,7 @@
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="0.000"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -109,8 +109,14 @@
       <x:color rgb="FF155724"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -242,8 +248,18 @@
         <x:fgColor rgb="FFE2F3E6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="6">
     <x:border/>
     <x:border/>
     <x:border>
@@ -251,11 +267,41 @@
         <x:color rgb="FF44B3E1"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="203">
+  <x:cellXfs count="223">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -761,6 +807,56 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1497,7 +1593,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.7-sample</x:v>
+        <x:v>0.6.8-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1788,7 +1884,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B28" s="35" t="str">
-        <x:v>字段变更同步FieldDictionary、Schema、导出器、DTO、校验、文档和测试。FieldDictionary不递归描述自身。</x:v>
+        <x:v>数据Sheet第3行是中文字段名，第4行是稳定英文API字段；字段契约变更须同步FieldDictionary、Schema、导出器、DTO、校验、文档和测试。FieldDictionary不递归描述自身。</x:v>
       </x:c>
       <x:c r="C28" s="35" t="str"/>
       <x:c r="D28" s="35" t="str"/>
@@ -1987,6 +2083,50 @@
       <x:c r="M2" s="13"/>
       <x:c r="N2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>敌人ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>名称文案键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>敌人层级</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>最大生命值</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>移动模式ID</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>移动速度</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>攻击集合ID</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>防御规则ID</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>弱点规则ID</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>架势弱点</x:v>
+      </x:c>
+      <x:c r="K3" s="221" t="str">
+        <x:v>接触伤害</x:v>
+      </x:c>
+      <x:c r="L3" s="221" t="str">
+        <x:v>击败得分</x:v>
+      </x:c>
+      <x:c r="M3" s="221" t="str">
+        <x:v>敌人资源键</x:v>
+      </x:c>
+      <x:c r="N3" s="222" t="str">
+        <x:v>池预热数量</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>enemyId</x:v>
@@ -2354,7 +2494,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R505fd93fad9f4070"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58a2adf2a52e4b28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2415,6 +2555,50 @@
       <x:c r="M2" s="13"/>
       <x:c r="N2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>攻击ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>攻击集合ID</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>组内顺序</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>攻击触发类型</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>冷却秒数</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>前摇秒数</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>有效秒数</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>基础伤害</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>投射物ID</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>打断笔势</x:v>
+      </x:c>
+      <x:c r="K3" s="221" t="str">
+        <x:v>打断开始秒数</x:v>
+      </x:c>
+      <x:c r="L3" s="221" t="str">
+        <x:v>打断结束秒数</x:v>
+      </x:c>
+      <x:c r="M3" s="221" t="str">
+        <x:v>效果组ID</x:v>
+      </x:c>
+      <x:c r="N3" s="222" t="str">
+        <x:v>选择权重</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>attackId</x:v>
@@ -2904,7 +3088,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65c7f4b0780c4184"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0521f9236bf64fa7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2956,6 +3140,41 @@
       <x:c r="J2" s="13"/>
       <x:c r="K2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>投射物ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>移动模式ID</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>飞行速度</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>投射物寿命秒数</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>基础伤害</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>可切断</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>可反弹</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>交互要求架势</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>命中半径</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>投射物资源键</x:v>
+      </x:c>
+      <x:c r="K3" s="222" t="str">
+        <x:v>特效键</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>projectileId</x:v>
@@ -3169,7 +3388,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cf18eb674a1419a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4e2eb0d1d5c4acf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3215,6 +3434,35 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>状态效果ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>状态类型</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>状态持续秒数</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>最大层数</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>效果强度</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>跳动间隔</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>刷新策略</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>特效键</x:v>
+      </x:c>
+      <x:c r="I3" s="222" t="str">
+        <x:v>文案键</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>buffId</x:v>
@@ -3433,7 +3681,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ef8c2eceab748b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R715604f2dd5547ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3485,6 +3733,41 @@
       <x:c r="J2" s="13"/>
       <x:c r="K2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>技能ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>名称文案键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>技能触发类型</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>释放要求架势</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>能量消耗</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>冷却秒数</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>笔势类型</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>输入窗口秒数</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>技能效果组</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>图标资源键</x:v>
+      </x:c>
+      <x:c r="K3" s="222" t="str">
+        <x:v>文案键</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>skillId</x:v>
@@ -3638,7 +3921,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7684439396044599"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd62afe365d214299"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3690,6 +3973,41 @@
       <x:c r="J2" s="13"/>
       <x:c r="K2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>效果组ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>组内顺序</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>效果类型</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>目标类型</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>主参数</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>次参数</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>效果持续秒数</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>状态效果ID</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>特效键</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>音频键</x:v>
+      </x:c>
+      <x:c r="K3" s="222" t="str">
+        <x:v>执行条件</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>effectGroupId</x:v>
@@ -4520,7 +4838,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff881f2adbd14334"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa839517e1c24195"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4575,6 +4893,44 @@
       <x:c r="K2" s="13"/>
       <x:c r="L2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>关卡ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>名称文案键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>场景资源键</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>背景资源键</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>时限秒数</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>下一关ID</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>奖励表ID</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>一星分数</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>二星分数</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>三星分数</x:v>
+      </x:c>
+      <x:c r="K3" s="221" t="str">
+        <x:v>教程ID</x:v>
+      </x:c>
+      <x:c r="L3" s="222" t="str">
+        <x:v>Boss敌人ID</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>levelId</x:v>
@@ -4728,7 +5084,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra07d87effbfe4e5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc90f9a33ff5494b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4774,6 +5130,35 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>波次ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>所属关卡ID</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>组内顺序</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>开始条件</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>开始延迟秒数</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>结束条件</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>结束延迟秒数</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>背景音乐键</x:v>
+      </x:c>
+      <x:c r="I3" s="222" t="str">
+        <x:v>最大存活数</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>waveId</x:v>
@@ -5282,7 +5667,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4fb5f56c93c49dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34d8543c41142ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5328,6 +5713,35 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>出生点ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>适用关卡ID</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>归一化X</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>归一化Y</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>路线层级</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>X随机偏移</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>Y随机偏移</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>初始朝向</x:v>
+      </x:c>
+      <x:c r="I3" s="222" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>spawnPointId</x:v>
@@ -5488,7 +5902,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f2d4467ab14bc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a286d2d87cb4c75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5531,6 +5945,32 @@
       <x:c r="G2" s="13"/>
       <x:c r="H2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>修饰器ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>名称文案键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>生命倍率</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>敌人伤害倍率</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>速度倍率</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>得分倍率</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>染色色值</x:v>
+      </x:c>
+      <x:c r="H3" s="222" t="str">
+        <x:v>附加状态ID</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>modifierId</x:v>
@@ -5614,7 +6054,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73f89f7100b740ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R830259a0c7634284"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5657,6 +6097,32 @@
       <x:c r="G2" s="13"/>
       <x:c r="H2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>配置键</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>值类型</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>整数值</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>小数值</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>文本值</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>布尔值</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>单位</x:v>
+      </x:c>
+      <x:c r="H3" s="222" t="str">
+        <x:v>参数说明</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>key</x:v>
@@ -5713,7 +6179,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.7-sample</x:v>
+        <x:v>0.6.8-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -6655,7 +7121,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a3589943bd54126"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4198224c6b5b4e1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6701,6 +7167,35 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>出生条目ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>所属波次ID</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>出生时刻秒数</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>敌人ID</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>出生数量</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>出生间隔秒数</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>出生点ID</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>出生队形</x:v>
+      </x:c>
+      <x:c r="I3" s="222" t="str">
+        <x:v>修饰器ID</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>spawnId</x:v>
@@ -7757,7 +8252,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2de1cc8a7449a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06207dddc465489b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7809,6 +8304,41 @@
       <x:c r="J2" s="13"/>
       <x:c r="K2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>Boss阶段ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>Boss敌人ID</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>组内顺序</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>进入生命比例</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>退出生命比例</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>阶段移动模式</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>阶段攻击集合</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>阶段防御规则</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>阶段弱点规则</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>入场效果组</x:v>
+      </x:c>
+      <x:c r="K3" s="222" t="str">
+        <x:v>阶段文案键</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>bossPhaseId</x:v>
@@ -7956,7 +8486,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R445807d47b5644a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55fb7d5d39b94cf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7996,6 +8526,29 @@
       <x:c r="F2" s="13"/>
       <x:c r="G2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>奖励表ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>组内顺序</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>奖励条件类型</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>奖励条件值</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>奖励类型</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>奖励对象ID</x:v>
+      </x:c>
+      <x:c r="G3" s="222" t="str">
+        <x:v>奖励数量</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>rewardTableId</x:v>
@@ -8172,7 +8725,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R114b977ab7104bdb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R407e61bfcd174a3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8218,6 +8771,35 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>教程ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>组内顺序</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>教程触发事件</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>阻断战斗推进</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>最短展示秒数</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>教程完成事件</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>文案键</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>高亮目标</x:v>
+      </x:c>
+      <x:c r="I3" s="222" t="str">
+        <x:v>笔势类型</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>tutorialId</x:v>
@@ -8491,7 +9073,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e1b340e53f24b1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59c5ec6c1e2d4893"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8522,6 +9104,20 @@
       <x:c r="C2" s="13"/>
       <x:c r="D2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>文案键</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>简体中文</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>英文</x:v>
+      </x:c>
+      <x:c r="D3" s="222" t="str">
+        <x:v>使用场景</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>textKey</x:v>
@@ -9411,7 +10007,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71a31bdecac749b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R729aa4eb239c45a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9454,6 +10050,32 @@
       <x:c r="G2" s="13"/>
       <x:c r="H2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>音频事件键</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>音频资源键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>音频分类</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>音量</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>最低音调</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>最高音调</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>最大并发数</x:v>
+      </x:c>
+      <x:c r="H3" s="222" t="str">
+        <x:v>冷却秒数</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>audioKey</x:v>
@@ -9934,7 +10556,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re59fbbe76e0844a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R532dbac6c0244c0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9974,6 +10596,29 @@
       <x:c r="F2" s="13"/>
       <x:c r="G2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>特效事件键</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>特效资源键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>特效寿命秒数</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>池预热数量</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>跟随目标</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>排序层</x:v>
+      </x:c>
+      <x:c r="G3" s="222" t="str">
+        <x:v>层内顺序</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>vfxKey</x:v>
@@ -10901,7 +11546,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95265f875b444a53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56548be9a04e486c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10935,6 +11580,23 @@
       <x:c r="D2" s="13"/>
       <x:c r="E2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>资源键</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>资源类型</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>审查路径</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>MVP必需</x:v>
+      </x:c>
+      <x:c r="E3" s="222" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>assetKey</x:v>
@@ -12273,7 +12935,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcffed01b6db149bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0aee00469ab74ea4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12304,6 +12966,20 @@
       <x:c r="C2" s="13"/>
       <x:c r="D2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>枚举类型</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>枚举值</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>枚举显示名</x:v>
+      </x:c>
+      <x:c r="D3" s="222" t="str">
+        <x:v>枚举说明</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>enumType</x:v>
@@ -13697,7 +14373,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3baf6da4ea2a4c2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d7ac17c3cfb4451"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13715,7 +14391,7 @@
     <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="21" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="62" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -13746,6 +14422,38 @@
       <x:c r="I2" s="13"/>
       <x:c r="J2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>所属Sheet</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>英文字段名</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>数据类型</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>是否必填</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>默认值</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>最小值</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>最大值</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>枚举类型</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>外键目标</x:v>
+      </x:c>
+      <x:c r="J3" s="222" t="str">
+        <x:v>中文字段说明</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>sheet</x:v>
@@ -13791,13 +14499,13 @@
       <x:c r="D5" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E5" s="35" t="str"/>
+      <x:c r="E5" s="35"/>
       <x:c r="F5" s="35"/>
       <x:c r="G5" s="35"/>
-      <x:c r="H5" s="35" t="str"/>
-      <x:c r="I5" s="35" t="str"/>
+      <x:c r="H5" s="35"/>
+      <x:c r="I5" s="35"/>
       <x:c r="J5" s="35" t="str">
-        <x:v>Global 表的 key 字段</x:v>
+        <x:v>配置键：全局参数的稳定英文键；代码和配置查询均以此键定位，发布后不得复用。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -13813,15 +14521,15 @@
       <x:c r="D6" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E6" s="35" t="str"/>
+      <x:c r="E6" s="35"/>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35"/>
       <x:c r="H6" s="35" t="str">
         <x:v>ValueType</x:v>
       </x:c>
-      <x:c r="I6" s="35" t="str"/>
+      <x:c r="I6" s="35"/>
       <x:c r="J6" s="35" t="str">
-        <x:v>Global 表的 valueType 字段</x:v>
+        <x:v>值类型：指定当前全局参数实际使用的值列，只允许登记在ValueType枚举中的类型。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -13837,13 +14545,13 @@
       <x:c r="D7" s="35" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="E7" s="35" t="str"/>
+      <x:c r="E7" s="35"/>
       <x:c r="F7" s="35"/>
       <x:c r="G7" s="35"/>
-      <x:c r="H7" s="35" t="str"/>
-      <x:c r="I7" s="35" t="str"/>
+      <x:c r="H7" s="35"/>
+      <x:c r="I7" s="35"/>
       <x:c r="J7" s="35" t="str">
-        <x:v>Global 表的 intValue 字段</x:v>
+        <x:v>整数值：当值类型为int时读取的整数；其他值类型下必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -13859,13 +14567,13 @@
       <x:c r="D8" s="35" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="E8" s="35" t="str"/>
+      <x:c r="E8" s="35"/>
       <x:c r="F8" s="35"/>
       <x:c r="G8" s="35"/>
-      <x:c r="H8" s="35" t="str"/>
-      <x:c r="I8" s="35" t="str"/>
+      <x:c r="H8" s="35"/>
+      <x:c r="I8" s="35"/>
       <x:c r="J8" s="35" t="str">
-        <x:v>Global 表的 floatValue 字段</x:v>
+        <x:v>小数值：当值类型为float时读取的小数；其他值类型下必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -13881,13 +14589,13 @@
       <x:c r="D9" s="35" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="E9" s="35" t="str"/>
+      <x:c r="E9" s="35"/>
       <x:c r="F9" s="35"/>
       <x:c r="G9" s="35"/>
-      <x:c r="H9" s="35" t="str"/>
-      <x:c r="I9" s="35" t="str"/>
+      <x:c r="H9" s="35"/>
+      <x:c r="I9" s="35"/>
       <x:c r="J9" s="35" t="str">
-        <x:v>Global 表的 stringValue 字段</x:v>
+        <x:v>文本值：当值类型为string时读取的文本；其他值类型下必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -13903,13 +14611,13 @@
       <x:c r="D10" s="35" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="E10" s="35" t="str"/>
+      <x:c r="E10" s="35"/>
       <x:c r="F10" s="35"/>
       <x:c r="G10" s="35"/>
-      <x:c r="H10" s="35" t="str"/>
-      <x:c r="I10" s="35" t="str"/>
+      <x:c r="H10" s="35"/>
+      <x:c r="I10" s="35"/>
       <x:c r="J10" s="35" t="str">
-        <x:v>Global 表的 boolValue 字段</x:v>
+        <x:v>布尔值：当值类型为bool时读取的真假值；其他值类型下必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -13925,13 +14633,13 @@
       <x:c r="D11" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E11" s="35" t="str"/>
+      <x:c r="E11" s="35"/>
       <x:c r="F11" s="35"/>
       <x:c r="G11" s="35"/>
-      <x:c r="H11" s="35" t="str"/>
-      <x:c r="I11" s="35" t="str"/>
+      <x:c r="H11" s="35"/>
+      <x:c r="I11" s="35"/>
       <x:c r="J11" s="35" t="str">
-        <x:v>Global 表的 unit 字段</x:v>
+        <x:v>单位：标明参数的量纲或解释口径，例如秒、参考像素、数量、比例或版本。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -13947,13 +14655,13 @@
       <x:c r="D12" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E12" s="35" t="str"/>
+      <x:c r="E12" s="35"/>
       <x:c r="F12" s="35"/>
       <x:c r="G12" s="35"/>
-      <x:c r="H12" s="35" t="str"/>
-      <x:c r="I12" s="35" t="str"/>
+      <x:c r="H12" s="35"/>
+      <x:c r="I12" s="35"/>
       <x:c r="J12" s="35" t="str">
-        <x:v>Global 表的 description 字段</x:v>
+        <x:v>参数说明：说明该全局配置键控制的系统行为和使用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -13969,13 +14677,13 @@
       <x:c r="D13" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E13" s="35" t="str"/>
+      <x:c r="E13" s="35"/>
       <x:c r="F13" s="35"/>
       <x:c r="G13" s="35"/>
-      <x:c r="H13" s="35" t="str"/>
-      <x:c r="I13" s="35" t="str"/>
+      <x:c r="H13" s="35"/>
+      <x:c r="I13" s="35"/>
       <x:c r="J13" s="35" t="str">
-        <x:v>玩家稳定ID</x:v>
+        <x:v>玩家ID：玩家定义的稳定主键，用于跨表引用和运行时索引。</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -13991,15 +14699,15 @@
       <x:c r="D14" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E14" s="35" t="str"/>
+      <x:c r="E14" s="35"/>
       <x:c r="F14" s="35"/>
       <x:c r="G14" s="35"/>
-      <x:c r="H14" s="35" t="str"/>
+      <x:c r="H14" s="35"/>
       <x:c r="I14" s="35" t="str">
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J14" s="35" t="str">
-        <x:v>显示名称文案键</x:v>
+        <x:v>名称文案键：引用Texts.textKey取得本地化显示名称，不直接填写玩家可见文字。</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -14015,15 +14723,15 @@
       <x:c r="D15" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E15" s="35" t="str"/>
+      <x:c r="E15" s="35"/>
       <x:c r="F15" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="35"/>
-      <x:c r="H15" s="35" t="str"/>
-      <x:c r="I15" s="35" t="str"/>
+      <x:c r="H15" s="35"/>
+      <x:c r="I15" s="35"/>
       <x:c r="J15" s="35" t="str">
-        <x:v>最大生命值</x:v>
+        <x:v>最大生命值：实体满状态时可拥有的生命值上限；生命值降至零时进入死亡流程。</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -14039,15 +14747,15 @@
       <x:c r="D16" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E16" s="35" t="str"/>
+      <x:c r="E16" s="35"/>
       <x:c r="F16" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G16" s="35"/>
-      <x:c r="H16" s="35" t="str"/>
-      <x:c r="I16" s="35" t="str"/>
+      <x:c r="H16" s="35"/>
+      <x:c r="I16" s="35"/>
       <x:c r="J16" s="35" t="str">
-        <x:v>最大能量</x:v>
+        <x:v>最大能量：玩家可储存的能量上限，获得能量时不得超过该值。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -14063,15 +14771,15 @@
       <x:c r="D17" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E17" s="35" t="str"/>
+      <x:c r="E17" s="35"/>
       <x:c r="F17" s="35"/>
       <x:c r="G17" s="35"/>
-      <x:c r="H17" s="35" t="str"/>
+      <x:c r="H17" s="35"/>
       <x:c r="I17" s="35" t="str">
         <x:v>Stances.stanceId</x:v>
       </x:c>
       <x:c r="J17" s="35" t="str">
-        <x:v>Players 表的 defaultStanceId 字段</x:v>
+        <x:v>默认架势：引用Stances.stanceId，指定玩家进入战斗时采用的初始架势。</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -14087,15 +14795,15 @@
       <x:c r="D18" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E18" s="35" t="str"/>
+      <x:c r="E18" s="35"/>
       <x:c r="F18" s="35"/>
       <x:c r="G18" s="35"/>
-      <x:c r="H18" s="35" t="str"/>
+      <x:c r="H18" s="35"/>
       <x:c r="I18" s="35" t="str">
         <x:v>Skills.skillId</x:v>
       </x:c>
       <x:c r="J18" s="35" t="str">
-        <x:v>Players 表的 ultimateSkillId 字段</x:v>
+        <x:v>终极技能：引用Skills.skillId，指定玩家能量满足条件后可释放的终极技能。</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -14111,13 +14819,13 @@
       <x:c r="D19" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E19" s="35" t="str"/>
+      <x:c r="E19" s="35"/>
       <x:c r="F19" s="35"/>
       <x:c r="G19" s="35"/>
-      <x:c r="H19" s="35" t="str"/>
-      <x:c r="I19" s="35" t="str"/>
+      <x:c r="H19" s="35"/>
+      <x:c r="I19" s="35"/>
       <x:c r="J19" s="35" t="str">
-        <x:v>Players 表的 hitInvulnSec 字段</x:v>
+        <x:v>受击无敌秒数：玩家受到一次有效伤害后忽略后续伤害的非负时间窗口，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -14133,15 +14841,15 @@
       <x:c r="D20" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E20" s="35" t="str"/>
+      <x:c r="E20" s="35"/>
       <x:c r="F20" s="35"/>
       <x:c r="G20" s="35"/>
-      <x:c r="H20" s="35" t="str"/>
+      <x:c r="H20" s="35"/>
       <x:c r="I20" s="35" t="str">
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J20" s="35" t="str">
-        <x:v>Unity资源注册键</x:v>
+        <x:v>角色资源键：引用AssetManifest.assetKey，并由Unity AssetRegistry解析为主角Sprite或Prefab。</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -14157,13 +14865,13 @@
       <x:c r="D21" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E21" s="35" t="str"/>
+      <x:c r="E21" s="35"/>
       <x:c r="F21" s="35"/>
       <x:c r="G21" s="35"/>
-      <x:c r="H21" s="35" t="str"/>
-      <x:c r="I21" s="35" t="str"/>
+      <x:c r="H21" s="35"/>
+      <x:c r="I21" s="35"/>
       <x:c r="J21" s="35" t="str">
-        <x:v>Stances 表的 stanceId 字段</x:v>
+        <x:v>架势ID：架势定义的稳定主键，用于玩家状态、技能和投射物规则引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -14179,15 +14887,15 @@
       <x:c r="D22" s="35" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="E22" s="35" t="str"/>
+      <x:c r="E22" s="35"/>
       <x:c r="F22" s="35"/>
       <x:c r="G22" s="35"/>
-      <x:c r="H22" s="35" t="str"/>
+      <x:c r="H22" s="35"/>
       <x:c r="I22" s="35" t="str">
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J22" s="35" t="str">
-        <x:v>显示名称文案键</x:v>
+        <x:v>名称文案键：引用Texts.textKey取得本地化显示名称，不直接填写玩家可见文字。</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -14206,12 +14914,12 @@
       <x:c r="E23" s="35"/>
       <x:c r="F23" s="35"/>
       <x:c r="G23" s="35"/>
-      <x:c r="H23" s="35" t="str"/>
+      <x:c r="H23" s="35"/>
       <x:c r="I23" s="35" t="str">
         <x:v>DamageFormulas.formulaId</x:v>
       </x:c>
       <x:c r="J23" s="35" t="str">
-        <x:v>架势使用的伤害公式外键</x:v>
+        <x:v>伤害公式：引用DamageFormulas.formulaId，指定该架势使用的基础伤害计算参数组。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -14235,7 +14943,7 @@
       <x:c r="H24" s="35"/>
       <x:c r="I24" s="35"/>
       <x:c r="J24" s="35" t="str">
-        <x:v>Stances 表的 damageMultiplier 字段</x:v>
+        <x:v>架势伤害倍率：使用该架势计算玩家伤害时应用的基础乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -14257,7 +14965,7 @@
       <x:c r="H25" s="35"/>
       <x:c r="I25" s="35"/>
       <x:c r="J25" s="35" t="str">
-        <x:v>Stances 表的 ghostDamageMultiplier 字段</x:v>
+        <x:v>幽魂伤害倍率：该架势攻击幽魂类目标时应用的额外伤害乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -14279,7 +14987,7 @@
       <x:c r="H26" s="35"/>
       <x:c r="I26" s="35"/>
       <x:c r="J26" s="35" t="str">
-        <x:v>Stances 表的 projectileCutMultiplier 字段</x:v>
+        <x:v>切弹倍率：该架势与可交互投射物接触时使用的切断能力倍率。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -14301,7 +15009,7 @@
       <x:c r="H27" s="35"/>
       <x:c r="I27" s="35"/>
       <x:c r="J27" s="35" t="str">
-        <x:v>Stances 表的 strokeWidthRefPx 字段</x:v>
+        <x:v>笔迹宽度：1920×1080参考分辨率下的基础笔迹宽度，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -14323,7 +15031,7 @@
       <x:c r="H28" s="35"/>
       <x:c r="I28" s="35"/>
       <x:c r="J28" s="35" t="str">
-        <x:v>Stances 表的 switchCooldownSec 字段</x:v>
+        <x:v>切换冷却秒数：两次架势切换之间必须等待的最短时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -14347,7 +15055,7 @@
         <x:v>SkillEffects.effectGroupId</x:v>
       </x:c>
       <x:c r="J29" s="35" t="str">
-        <x:v>Stances 表的 onSwitchEffectGroupId 字段</x:v>
+        <x:v>切换效果组：引用SkillEffects.effectGroupId，切入该架势时按顺序执行对应效果链。</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -14371,7 +15079,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J30" s="35" t="str">
-        <x:v>Unity资源注册键</x:v>
+        <x:v>架势图标资源键：引用AssetManifest.assetKey，并由Unity AssetRegistry解析为架势图标。</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -14393,7 +15101,7 @@
       <x:c r="H31" s="35"/>
       <x:c r="I31" s="35"/>
       <x:c r="J31" s="35" t="str">
-        <x:v>手势规则稳定ID</x:v>
+        <x:v>笔势规则ID：笔势识别规则的稳定主键，用于采样、分类和命中参数查询。</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -14417,7 +15125,7 @@
       </x:c>
       <x:c r="I32" s="35"/>
       <x:c r="J32" s="35" t="str">
-        <x:v>StrokeRules 表的 gestureType 字段</x:v>
+        <x:v>笔势类型：指定该规则或交互要求的手势类别，取值必须登记在GestureType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -14439,7 +15147,7 @@
       <x:c r="H33" s="35"/>
       <x:c r="I33" s="35"/>
       <x:c r="J33" s="35" t="str">
-        <x:v>StrokeRules 表的 minPointDistanceRefPx 字段</x:v>
+        <x:v>最小采样间距：相邻采样点必须达到的最小距离，单位为参考像素，用于抑制高频抖动点。</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -14461,7 +15169,7 @@
       <x:c r="H34" s="35"/>
       <x:c r="I34" s="35"/>
       <x:c r="J34" s="35" t="str">
-        <x:v>StrokeRules 表的 maxStrokeLengthRefPx 字段</x:v>
+        <x:v>最大笔迹长度：单次笔迹允许保留的最大累计长度，单位为参考像素，超出部分会被裁剪。</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -14483,7 +15191,7 @@
       <x:c r="H35" s="35"/>
       <x:c r="I35" s="35"/>
       <x:c r="J35" s="35" t="str">
-        <x:v>StrokeRules 表的 rdpEpsilonRefPx 字段</x:v>
+        <x:v>简化容差：RDP路径简化允许的最大偏差，单位为参考像素；数值越大保留点越少。</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -14509,7 +15217,7 @@
       <x:c r="H36" s="35"/>
       <x:c r="I36" s="35"/>
       <x:c r="J36" s="35" t="str">
-        <x:v>StrokeRules 表的 maxPointCount 字段</x:v>
+        <x:v>最大点数：单次笔迹处理和缓存允许保留的采样点数量上限。</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -14531,7 +15239,7 @@
       <x:c r="H37" s="35"/>
       <x:c r="I37" s="35"/>
       <x:c r="J37" s="35" t="str">
-        <x:v>StrokeRules 表的 minLengthRefPx 字段</x:v>
+        <x:v>最小有效长度：笔势被判定为有效前必须达到的最小路径长度，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -14557,7 +15265,7 @@
       <x:c r="H38" s="35"/>
       <x:c r="I38" s="35"/>
       <x:c r="J38" s="35" t="str">
-        <x:v>StrokeRules 表的 directionToleranceDeg 字段</x:v>
+        <x:v>方向容差角：横、竖或斜向笔势相对目标方向允许偏离的最大角度，单位为度。</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -14579,7 +15287,7 @@
       <x:c r="H39" s="35"/>
       <x:c r="I39" s="35"/>
       <x:c r="J39" s="35" t="str">
-        <x:v>StrokeRules 表的 closeDistanceRefPx 字段</x:v>
+        <x:v>闭合距离：首尾点距离不超过该参考像素值时可视为闭合笔势；不适用时填0。</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -14601,7 +15309,7 @@
       <x:c r="H40" s="35"/>
       <x:c r="I40" s="35"/>
       <x:c r="J40" s="35" t="str">
-        <x:v>StrokeRules 表的 minAreaRefPx2 字段</x:v>
+        <x:v>最小包围面积：闭合笔势必须覆盖的最小参考像素平方面积，用于过滤过小圆形。</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -14623,7 +15331,7 @@
       <x:c r="H41" s="35"/>
       <x:c r="I41" s="35"/>
       <x:c r="J41" s="35" t="str">
-        <x:v>StrokeRules 表的 minArcCurvature 字段</x:v>
+        <x:v>最小弧线曲率：弧形笔势必须达到的无量纲曲率阈值；不适用时填0。</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -14647,7 +15355,7 @@
       <x:c r="H42" s="35"/>
       <x:c r="I42" s="35"/>
       <x:c r="J42" s="35" t="str">
-        <x:v>StrokeRules 表的 chargeHoldSec 字段</x:v>
+        <x:v>蓄力时长：按住输入达到蓄力笔势所需的最短时间，单位为秒；不适用时填0。</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -14671,7 +15379,7 @@
       <x:c r="H43" s="35"/>
       <x:c r="I43" s="35"/>
       <x:c r="J43" s="35" t="str">
-        <x:v>StrokeRules 表的 hitRadiusRefPx 字段</x:v>
+        <x:v>命中半径：围绕笔迹或投射物中心参与碰撞查询的半径，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -14693,7 +15401,7 @@
       <x:c r="H44" s="35"/>
       <x:c r="I44" s="35"/>
       <x:c r="J44" s="35" t="str">
-        <x:v>伤害公式稳定ID</x:v>
+        <x:v>公式ID：伤害公式参数组的稳定主键，供架势和战斗规则引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -14717,7 +15425,7 @@
       <x:c r="H45" s="35"/>
       <x:c r="I45" s="35"/>
       <x:c r="J45" s="35" t="str">
-        <x:v>DamageFormulas 表的 baseDamage 字段</x:v>
+        <x:v>基础伤害：进入倍率、暴击、弱点和连击计算前的基础伤害值。</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -14743,7 +15451,7 @@
       <x:c r="H46" s="35"/>
       <x:c r="I46" s="35"/>
       <x:c r="J46" s="35" t="str">
-        <x:v>DamageFormulas 表的 criticalChance 字段</x:v>
+        <x:v>暴击概率：单次命中触发暴击的0到1概率。</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -14767,7 +15475,7 @@
       <x:c r="H47" s="35"/>
       <x:c r="I47" s="35"/>
       <x:c r="J47" s="35" t="str">
-        <x:v>DamageFormulas 表的 criticalMultiplier 字段</x:v>
+        <x:v>暴击倍率：暴击成立时应用于伤害的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -14789,7 +15497,7 @@
       <x:c r="H48" s="35"/>
       <x:c r="I48" s="35"/>
       <x:c r="J48" s="35" t="str">
-        <x:v>DamageFormulas 表的 weakpointMultiplier 字段</x:v>
+        <x:v>弱点倍率：命中有效弱点窗口时应用于伤害的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -14811,7 +15519,7 @@
       <x:c r="H49" s="35"/>
       <x:c r="I49" s="35"/>
       <x:c r="J49" s="35" t="str">
-        <x:v>DamageFormulas 表的 wrongDirectionMultiplier 字段</x:v>
+        <x:v>错误方向倍率：笔势方向不符合目标要求时应用的伤害乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -14833,7 +15541,7 @@
       <x:c r="H50" s="35"/>
       <x:c r="I50" s="35"/>
       <x:c r="J50" s="35" t="str">
-        <x:v>DamageFormulas 表的 comboStep 字段</x:v>
+        <x:v>连击步进倍率：每增加一层有效连击时追加的伤害倍率增量。</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -14855,7 +15563,7 @@
       <x:c r="H51" s="35"/>
       <x:c r="I51" s="35"/>
       <x:c r="J51" s="35" t="str">
-        <x:v>DamageFormulas 表的 comboMaxMultiplier 字段</x:v>
+        <x:v>连击倍率上限：连击系统允许达到的总伤害倍率上限。</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -14877,7 +15585,7 @@
       <x:c r="H52" s="35"/>
       <x:c r="I52" s="35"/>
       <x:c r="J52" s="35" t="str">
-        <x:v>DamageFormulas 表的 energyPerHit 字段</x:v>
+        <x:v>每击能量：每次有效命中基础获得的玩家能量值。</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -14899,7 +15607,7 @@
       <x:c r="H53" s="35"/>
       <x:c r="I53" s="35"/>
       <x:c r="J53" s="35" t="str">
-        <x:v>DamageFormulas 表的 scorePerHit 字段</x:v>
+        <x:v>每击得分：每次有效命中直接增加的基础分数。</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -14920,10 +15628,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G54" s="35"/>
-      <x:c r="H54" s="35" t="str"/>
-      <x:c r="I54" s="35" t="str"/>
+      <x:c r="H54" s="35"/>
+      <x:c r="I54" s="35"/>
       <x:c r="J54" s="35" t="str">
-        <x:v>每点最终原始伤害计入评分的系数</x:v>
+        <x:v>每伤害得分：每造成1点最终伤害追加的分数。</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -14945,7 +15653,7 @@
       <x:c r="H55" s="35"/>
       <x:c r="I55" s="35"/>
       <x:c r="J55" s="35" t="str">
-        <x:v>防御规则稳定ID</x:v>
+        <x:v>防御规则ID：防御规则的稳定主键，供敌人和Boss阶段引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -14967,7 +15675,7 @@
       <x:c r="H56" s="35"/>
       <x:c r="I56" s="35"/>
       <x:c r="J56" s="35" t="str">
-        <x:v>DefenseRules 表的 armorHp 字段</x:v>
+        <x:v>护甲生命值：目标初始护甲耐久；为0表示没有护甲层。</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -14991,7 +15699,7 @@
       </x:c>
       <x:c r="I57" s="35"/>
       <x:c r="J57" s="35" t="str">
-        <x:v>DefenseRules 表的 requiredGestureType 字段</x:v>
+        <x:v>要求笔势：破防或有效攻击要求的GestureType；Any表示不限制具体笔势。</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -15015,7 +15723,7 @@
         <x:v>Stances.stanceId</x:v>
       </x:c>
       <x:c r="J58" s="35" t="str">
-        <x:v>DefenseRules 表的 requiredStanceId 字段</x:v>
+        <x:v>破防要求架势：引用Stances.stanceId；留空表示任意架势都可满足防御规则。</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -15037,7 +15745,7 @@
       <x:c r="H59" s="35"/>
       <x:c r="I59" s="35"/>
       <x:c r="J59" s="35" t="str">
-        <x:v>DefenseRules 表的 breakDamageMultiplier 字段</x:v>
+        <x:v>破甲伤害倍率：护甲首次被击破时对该次伤害应用的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -15059,7 +15767,7 @@
       <x:c r="H60" s="35"/>
       <x:c r="I60" s="35"/>
       <x:c r="J60" s="35" t="str">
-        <x:v>DefenseRules 表的 wrongGestureDamageMultiplier 字段</x:v>
+        <x:v>错误笔势倍率：笔势不符合防御要求时应用的伤害乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -15081,7 +15789,7 @@
       <x:c r="H61" s="35"/>
       <x:c r="I61" s="35"/>
       <x:c r="J61" s="35" t="str">
-        <x:v>DefenseRules 表的 reflectDamage 字段</x:v>
+        <x:v>反伤值：触发该防御规则的反伤条件时返还给攻击方的固定伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -15105,7 +15813,7 @@
         <x:v>SkillEffects.effectGroupId</x:v>
       </x:c>
       <x:c r="J62" s="35" t="str">
-        <x:v>DefenseRules 表的 breakEffectGroupId 字段</x:v>
+        <x:v>破甲效果组：引用SkillEffects.effectGroupId，护甲首次归零时执行对应效果链。</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -15127,7 +15835,7 @@
       <x:c r="H63" s="35"/>
       <x:c r="I63" s="35"/>
       <x:c r="J63" s="35" t="str">
-        <x:v>弱点规则稳定ID</x:v>
+        <x:v>弱点规则ID：弱点窗口规则的稳定主键，供敌人和Boss阶段引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -15149,7 +15857,7 @@
       <x:c r="H64" s="35"/>
       <x:c r="I64" s="35"/>
       <x:c r="J64" s="35" t="str">
-        <x:v>WeakpointRules 表的 windowStartSec 字段</x:v>
+        <x:v>窗口开始秒数：相对攻击开始时刻，弱点进入有效状态的时间偏移，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -15171,7 +15879,7 @@
       <x:c r="H65" s="35"/>
       <x:c r="I65" s="35"/>
       <x:c r="J65" s="35" t="str">
-        <x:v>WeakpointRules 表的 windowEndSec 字段</x:v>
+        <x:v>窗口结束秒数：相对攻击开始时刻，弱点结束有效状态的时间偏移，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -15195,7 +15903,7 @@
       <x:c r="H66" s="35"/>
       <x:c r="I66" s="35"/>
       <x:c r="J66" s="35" t="str">
-        <x:v>WeakpointRules 表的 radiusRefPx 字段</x:v>
+        <x:v>弱点半径：弱点命中区域的半径，单位为参考像素；为0表示不创建弱点区域。</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -15219,7 +15927,7 @@
       <x:c r="H67" s="35"/>
       <x:c r="I67" s="35"/>
       <x:c r="J67" s="35" t="str">
-        <x:v>WeakpointRules 表的 damageMultiplier 字段</x:v>
+        <x:v>弱点伤害倍率：命中有效弱点窗口时对本次伤害应用的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -15241,7 +15949,7 @@
       <x:c r="H68" s="35"/>
       <x:c r="I68" s="35"/>
       <x:c r="J68" s="35" t="str">
-        <x:v>WeakpointRules 表的 interruptAttack 字段</x:v>
+        <x:v>是否打断攻击：命中有效弱点后是否立即中断敌人当前攻击。</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -15263,7 +15971,7 @@
       <x:c r="H69" s="35"/>
       <x:c r="I69" s="35"/>
       <x:c r="J69" s="35" t="str">
-        <x:v>WeakpointRules 表的 energyBonus 字段</x:v>
+        <x:v>额外能量：命中有效弱点时在常规能量奖励之外追加的能量。</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -15285,7 +15993,7 @@
       <x:c r="H70" s="35"/>
       <x:c r="I70" s="35"/>
       <x:c r="J70" s="35" t="str">
-        <x:v>WeakpointRules 表的 scoreBonus 字段</x:v>
+        <x:v>额外得分：命中有效弱点时在常规计分之外追加的分数。</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -15309,7 +16017,7 @@
         <x:v>VfxCues.vfxKey</x:v>
       </x:c>
       <x:c r="J71" s="35" t="str">
-        <x:v>特效事件键</x:v>
+        <x:v>特效键：引用VfxCues.vfxKey；留空表示该事件不播放额外特效。</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -15331,7 +16039,7 @@
       <x:c r="H72" s="35"/>
       <x:c r="I72" s="35"/>
       <x:c r="J72" s="35" t="str">
-        <x:v>移动策略配置ID</x:v>
+        <x:v>移动模式ID：移动策略参数组的稳定主键，供敌人、投射物和Boss阶段引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -15355,7 +16063,7 @@
       </x:c>
       <x:c r="I73" s="35"/>
       <x:c r="J73" s="35" t="str">
-        <x:v>MovePatterns 表的 patternType 字段</x:v>
+        <x:v>移动类型：选择代码已登记的移动策略类型，取值必须来自MovePatternType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -15377,7 +16085,7 @@
       <x:c r="H74" s="35"/>
       <x:c r="I74" s="35"/>
       <x:c r="J74" s="35" t="str">
-        <x:v>MovePatterns 表的 speedMultiplier 字段</x:v>
+        <x:v>速度倍率：对实体基础移动速度应用的乘数；1表示保持基础速度。</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -15399,7 +16107,7 @@
       <x:c r="H75" s="35"/>
       <x:c r="I75" s="35"/>
       <x:c r="J75" s="35" t="str">
-        <x:v>MovePatterns 表的 amplitudeRefPx 字段</x:v>
+        <x:v>振幅：摆动类移动相对主路径的最大偏移，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -15421,7 +16129,7 @@
       <x:c r="H76" s="35"/>
       <x:c r="I76" s="35"/>
       <x:c r="J76" s="35" t="str">
-        <x:v>MovePatterns 表的 frequency 字段</x:v>
+        <x:v>频率：周期移动每秒完成的循环次数；线性或不循环策略可填0。</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -15443,7 +16151,7 @@
       <x:c r="H77" s="35"/>
       <x:c r="I77" s="35"/>
       <x:c r="J77" s="35" t="str">
-        <x:v>MovePatterns 表的 startXNorm 字段</x:v>
+        <x:v>起点X比例：移动路径起点在Safe Area宽度中的归一化X坐标，范围0到1。</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -15465,7 +16173,7 @@
       <x:c r="H78" s="35"/>
       <x:c r="I78" s="35"/>
       <x:c r="J78" s="35" t="str">
-        <x:v>MovePatterns 表的 endXNorm 字段</x:v>
+        <x:v>终点X比例：移动路径终点在Safe Area宽度中的归一化X坐标，范围0到1。</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -15487,7 +16195,7 @@
       <x:c r="H79" s="35"/>
       <x:c r="I79" s="35"/>
       <x:c r="J79" s="35" t="str">
-        <x:v>MovePatterns 表的 startYNorm 字段</x:v>
+        <x:v>起点Y比例：移动路径起点在Safe Area高度中的归一化Y坐标，范围0到1。</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -15509,7 +16217,7 @@
       <x:c r="H80" s="35"/>
       <x:c r="I80" s="35"/>
       <x:c r="J80" s="35" t="str">
-        <x:v>MovePatterns 表的 endYNorm 字段</x:v>
+        <x:v>终点Y比例：移动路径终点在Safe Area高度中的归一化Y坐标，范围0到1。</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -15531,7 +16239,7 @@
       <x:c r="H81" s="35"/>
       <x:c r="I81" s="35"/>
       <x:c r="J81" s="35" t="str">
-        <x:v>MovePatterns 表的 loop 字段</x:v>
+        <x:v>是否循环：到达路径末端后是否从头继续执行该移动模式。</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -15553,7 +16261,7 @@
       <x:c r="H82" s="35"/>
       <x:c r="I82" s="35"/>
       <x:c r="J82" s="35" t="str">
-        <x:v>MovePatterns 表的 description 字段</x:v>
+        <x:v>移动说明：用中文概括该移动模式的路径方向、对象或设计用途。</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -15575,7 +16283,7 @@
       <x:c r="H83" s="35"/>
       <x:c r="I83" s="35"/>
       <x:c r="J83" s="35" t="str">
-        <x:v>敌人稳定ID</x:v>
+        <x:v>敌人ID：敌人定义的稳定主键，用于出生、Boss阶段和运行时实体配置。</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -15599,7 +16307,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J84" s="35" t="str">
-        <x:v>显示名称文案键</x:v>
+        <x:v>名称文案键：引用Texts.textKey取得本地化显示名称，不直接填写玩家可见文字。</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -15623,7 +16331,7 @@
       </x:c>
       <x:c r="I85" s="35"/>
       <x:c r="J85" s="35" t="str">
-        <x:v>Enemies 表的 tier 字段</x:v>
+        <x:v>敌人层级：区分普通、精英或Boss等内容层级，取值必须来自EnemyTier枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -15647,7 +16355,7 @@
       <x:c r="H86" s="35"/>
       <x:c r="I86" s="35"/>
       <x:c r="J86" s="35" t="str">
-        <x:v>最大生命值</x:v>
+        <x:v>最大生命值：实体满状态时可拥有的生命值上限；生命值降至零时进入死亡流程。</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -15671,7 +16379,7 @@
         <x:v>MovePatterns.movePatternId</x:v>
       </x:c>
       <x:c r="J87" s="35" t="str">
-        <x:v>移动策略配置ID</x:v>
+        <x:v>移动模式ID：引用MovePatterns.movePatternId，指定实体或投射物采用的移动策略参数。</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -15695,7 +16403,7 @@
       <x:c r="H88" s="35"/>
       <x:c r="I88" s="35"/>
       <x:c r="J88" s="35" t="str">
-        <x:v>Enemies 表的 moveSpeedRefPxSec 字段</x:v>
+        <x:v>移动速度：敌人的基础移动速度，单位为参考像素/秒，并受移动模式和修饰器倍率影响。</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -15717,7 +16425,7 @@
       <x:c r="H89" s="35"/>
       <x:c r="I89" s="35"/>
       <x:c r="J89" s="35" t="str">
-        <x:v>攻击集合分组ID</x:v>
+        <x:v>攻击集合ID：引用EnemyAttacks.attackSetId分组，指定该敌人可选择的攻击集合。</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -15741,7 +16449,7 @@
         <x:v>DefenseRules.defenseRuleId</x:v>
       </x:c>
       <x:c r="J90" s="35" t="str">
-        <x:v>防御规则稳定ID</x:v>
+        <x:v>防御规则ID：引用DefenseRules.defenseRuleId，指定该敌人的护甲和破防要求。</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -15765,7 +16473,7 @@
         <x:v>WeakpointRules.weakpointRuleId</x:v>
       </x:c>
       <x:c r="J91" s="35" t="str">
-        <x:v>弱点规则稳定ID</x:v>
+        <x:v>弱点规则ID：引用WeakpointRules.weakpointRuleId，指定该敌人的弱点窗口。</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -15789,7 +16497,7 @@
       </x:c>
       <x:c r="I92" s="35"/>
       <x:c r="J92" s="35" t="str">
-        <x:v>Enemies 表的 stanceVulnerability 字段</x:v>
+        <x:v>架势弱点：指定目标更容易受到哪类架势影响，取值必须来自StanceVulnerability枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -15813,7 +16521,7 @@
       <x:c r="H93" s="35"/>
       <x:c r="I93" s="35"/>
       <x:c r="J93" s="35" t="str">
-        <x:v>Enemies 表的 contactDamage 字段</x:v>
+        <x:v>接触伤害：敌人身体碰撞体实际接触玩家时造成的基础伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -15837,7 +16545,7 @@
       <x:c r="H94" s="35"/>
       <x:c r="I94" s="35"/>
       <x:c r="J94" s="35" t="str">
-        <x:v>击败基础得分</x:v>
+        <x:v>击败得分：该敌人被击败并被关卡接受后增加的基础分数。</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -15861,7 +16569,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J95" s="35" t="str">
-        <x:v>Unity资源注册键</x:v>
+        <x:v>敌人资源键：引用AssetManifest.assetKey，并由Unity AssetRegistry解析为敌人Sprite或Prefab。</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -15885,7 +16593,7 @@
       <x:c r="H96" s="35"/>
       <x:c r="I96" s="35"/>
       <x:c r="J96" s="35" t="str">
-        <x:v>对象池预热数量</x:v>
+        <x:v>池预热数量：进入会话时为该资源预先创建的对象数量，用于降低首次生成开销。</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -15907,7 +16615,7 @@
       <x:c r="H97" s="35"/>
       <x:c r="I97" s="35"/>
       <x:c r="J97" s="35" t="str">
-        <x:v>EnemyAttacks 表的 attackId 字段</x:v>
+        <x:v>攻击ID：敌人攻击定义的稳定主键。</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -15929,7 +16637,7 @@
       <x:c r="H98" s="35"/>
       <x:c r="I98" s="35"/>
       <x:c r="J98" s="35" t="str">
-        <x:v>攻击集合分组ID</x:v>
+        <x:v>攻击集合ID：把同组攻击条目组织成敌人或Boss阶段可选择的攻击集合。</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -15953,7 +16661,7 @@
       <x:c r="H99" s="35"/>
       <x:c r="I99" s="35"/>
       <x:c r="J99" s="35" t="str">
-        <x:v>组内执行/展示顺序，从1开始</x:v>
+        <x:v>组内顺序：同一分组内从1开始的稳定执行、选择或展示顺序。</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -15977,7 +16685,7 @@
       </x:c>
       <x:c r="I100" s="35"/>
       <x:c r="J100" s="35" t="str">
-        <x:v>EnemyAttacks 表的 triggerType 字段</x:v>
+        <x:v>攻击触发类型：指定攻击由冷却、距离、支援或生命阈值触发，取值来自AttackTriggerType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -16001,7 +16709,7 @@
       <x:c r="H101" s="35"/>
       <x:c r="I101" s="35"/>
       <x:c r="J101" s="35" t="str">
-        <x:v>冷却时间（秒）</x:v>
+        <x:v>冷却秒数：同一动作再次可用前必须等待的最短时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -16025,7 +16733,7 @@
       <x:c r="H102" s="35"/>
       <x:c r="I102" s="35"/>
       <x:c r="J102" s="35" t="str">
-        <x:v>攻击前摇（秒）</x:v>
+        <x:v>前摇秒数：攻击开始后到有效窗口开启前的预警时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -16049,7 +16757,7 @@
       <x:c r="H103" s="35"/>
       <x:c r="I103" s="35"/>
       <x:c r="J103" s="35" t="str">
-        <x:v>有效窗口（秒）</x:v>
+        <x:v>有效秒数：攻击进入可生效状态后持续的时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -16073,7 +16781,7 @@
       <x:c r="H104" s="35"/>
       <x:c r="I104" s="35"/>
       <x:c r="J104" s="35" t="str">
-        <x:v>造成的基础伤害</x:v>
+        <x:v>基础伤害：当前攻击或投射物命中合法目标时提交的基础伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -16097,7 +16805,7 @@
         <x:v>Projectiles.projectileId</x:v>
       </x:c>
       <x:c r="J105" s="35" t="str">
-        <x:v>弹幕稳定ID</x:v>
+        <x:v>投射物ID：引用Projectiles.projectileId；留空表示该攻击不生成投射物。</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -16121,7 +16829,7 @@
       </x:c>
       <x:c r="I106" s="35"/>
       <x:c r="J106" s="35" t="str">
-        <x:v>EnemyAttacks 表的 gestureInterruptType 字段</x:v>
+        <x:v>打断笔势：攻击前摇期间可打断该攻击的GestureType；Any表示任意有效笔势。</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -16143,7 +16851,7 @@
       <x:c r="H107" s="35"/>
       <x:c r="I107" s="35"/>
       <x:c r="J107" s="35" t="str">
-        <x:v>EnemyAttacks 表的 interruptStartSec 字段</x:v>
+        <x:v>打断开始秒数：相对攻击开始时刻，可被笔势打断的窗口起点，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -16165,7 +16873,7 @@
       <x:c r="H108" s="35"/>
       <x:c r="I108" s="35"/>
       <x:c r="J108" s="35" t="str">
-        <x:v>EnemyAttacks 表的 interruptEndSec 字段</x:v>
+        <x:v>打断结束秒数：相对攻击开始时刻，可被笔势打断的窗口终点，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -16189,7 +16897,7 @@
         <x:v>SkillEffects.effectGroupId</x:v>
       </x:c>
       <x:c r="J109" s="35" t="str">
-        <x:v>效果链分组ID</x:v>
+        <x:v>效果组ID：引用SkillEffects.effectGroupId，按order执行同组效果；留空表示没有附加效果。</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -16211,7 +16919,7 @@
       <x:c r="H110" s="35"/>
       <x:c r="I110" s="35"/>
       <x:c r="J110" s="35" t="str">
-        <x:v>EnemyAttacks 表的 weight 字段</x:v>
+        <x:v>选择权重：同一攻击集合中参与确定性加权选择的相对权重。</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -16233,7 +16941,7 @@
       <x:c r="H111" s="35"/>
       <x:c r="I111" s="35"/>
       <x:c r="J111" s="35" t="str">
-        <x:v>弹幕稳定ID</x:v>
+        <x:v>投射物ID：投射物定义的稳定主键，供敌人攻击配置引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -16257,7 +16965,7 @@
         <x:v>MovePatterns.movePatternId</x:v>
       </x:c>
       <x:c r="J112" s="35" t="str">
-        <x:v>移动策略配置ID</x:v>
+        <x:v>移动模式ID：引用MovePatterns.movePatternId，指定实体或投射物采用的移动策略参数。</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -16281,7 +16989,7 @@
       <x:c r="H113" s="35"/>
       <x:c r="I113" s="35"/>
       <x:c r="J113" s="35" t="str">
-        <x:v>Projectiles 表的 speedRefPxSec 字段</x:v>
+        <x:v>飞行速度：投射物在参考像素空间中的移动速度，单位为参考像素/秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -16305,7 +17013,7 @@
       <x:c r="H114" s="35"/>
       <x:c r="I114" s="35"/>
       <x:c r="J114" s="35" t="str">
-        <x:v>Projectiles 表的 lifeSec 字段</x:v>
+        <x:v>投射物寿命秒数：投射物生成后允许飞行的最长玩法时间，单位为秒，到期后回池。</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -16329,7 +17037,7 @@
       <x:c r="H115" s="35"/>
       <x:c r="I115" s="35"/>
       <x:c r="J115" s="35" t="str">
-        <x:v>造成的基础伤害</x:v>
+        <x:v>基础伤害：当前攻击或投射物命中合法目标时提交的基础伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -16351,7 +17059,7 @@
       <x:c r="H116" s="35"/>
       <x:c r="I116" s="35"/>
       <x:c r="J116" s="35" t="str">
-        <x:v>Projectiles 表的 cuttable 字段</x:v>
+        <x:v>可切断：是否允许有效画笔命中后直接切断并回收该投射物。</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -16373,7 +17081,7 @@
       <x:c r="H117" s="35"/>
       <x:c r="I117" s="35"/>
       <x:c r="J117" s="35" t="str">
-        <x:v>Projectiles 表的 reflectable 字段</x:v>
+        <x:v>可反弹：是否允许满足架势要求的画笔把投射物归属和方向反转。</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -16397,7 +17105,7 @@
         <x:v>Stances.stanceId</x:v>
       </x:c>
       <x:c r="J118" s="35" t="str">
-        <x:v>Projectiles 表的 requiredStanceId 字段</x:v>
+        <x:v>交互要求架势：引用Stances.stanceId；留空表示任意架势都可切断或反弹该投射物。</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -16421,7 +17129,7 @@
       <x:c r="H119" s="35"/>
       <x:c r="I119" s="35"/>
       <x:c r="J119" s="35" t="str">
-        <x:v>Projectiles 表的 hitRadiusRefPx 字段</x:v>
+        <x:v>命中半径：围绕笔迹或投射物中心参与碰撞查询的半径，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -16445,7 +17153,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J120" s="35" t="str">
-        <x:v>Unity资源注册键</x:v>
+        <x:v>投射物资源键：引用AssetManifest.assetKey，并由Unity AssetRegistry解析为投射物Sprite。</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -16469,7 +17177,7 @@
         <x:v>VfxCues.vfxKey</x:v>
       </x:c>
       <x:c r="J121" s="35" t="str">
-        <x:v>特效事件键</x:v>
+        <x:v>特效键：引用VfxCues.vfxKey；留空表示该事件不播放额外特效。</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -16491,7 +17199,7 @@
       <x:c r="H122" s="35"/>
       <x:c r="I122" s="35"/>
       <x:c r="J122" s="35" t="str">
-        <x:v>状态效果稳定ID</x:v>
+        <x:v>状态效果ID：状态效果定义的稳定主键，供技能效果和敌人修饰器引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -16515,7 +17223,7 @@
       </x:c>
       <x:c r="I123" s="35"/>
       <x:c r="J123" s="35" t="str">
-        <x:v>Buffs 表的 type 字段</x:v>
+        <x:v>状态类型：指定状态效果的行为类别，取值必须来自BuffType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -16539,7 +17247,7 @@
       <x:c r="H124" s="35"/>
       <x:c r="I124" s="35"/>
       <x:c r="J124" s="35" t="str">
-        <x:v>持续时间（秒）</x:v>
+        <x:v>状态持续秒数：状态效果保持有效的基础时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -16563,7 +17271,7 @@
       <x:c r="H125" s="35"/>
       <x:c r="I125" s="35"/>
       <x:c r="J125" s="35" t="str">
-        <x:v>Buffs 表的 maxStacks 字段</x:v>
+        <x:v>最大层数：同一状态效果在单个目标上允许累计的层数上限。</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -16587,7 +17295,7 @@
       <x:c r="H126" s="35"/>
       <x:c r="I126" s="35"/>
       <x:c r="J126" s="35" t="str">
-        <x:v>Buffs 表的 magnitude 字段</x:v>
+        <x:v>效果强度：状态效果的主要强度参数，具体含义由BuffType决定，例如减速比例或增伤比例。</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -16611,7 +17319,7 @@
       <x:c r="H127" s="35"/>
       <x:c r="I127" s="35"/>
       <x:c r="J127" s="35" t="str">
-        <x:v>Buffs 表的 tickSec 字段</x:v>
+        <x:v>跳动间隔：周期状态两次结算之间的时间，单位为秒；为0表示不按周期跳动。</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -16635,7 +17343,7 @@
       </x:c>
       <x:c r="I128" s="35"/>
       <x:c r="J128" s="35" t="str">
-        <x:v>Buffs 表的 refreshPolicy 字段</x:v>
+        <x:v>刷新策略：重复施加同一状态时采用的时长或层数处理方式，取值来自BuffRefreshPolicy枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -16659,7 +17367,7 @@
         <x:v>VfxCues.vfxKey</x:v>
       </x:c>
       <x:c r="J129" s="35" t="str">
-        <x:v>特效事件键</x:v>
+        <x:v>特效键：引用VfxCues.vfxKey；留空表示该事件不播放额外特效。</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -16683,7 +17391,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J130" s="35" t="str">
-        <x:v>文案键</x:v>
+        <x:v>文案键：引用Texts.textKey取得玩家可见的本地化文本。</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -16705,7 +17413,7 @@
       <x:c r="H131" s="35"/>
       <x:c r="I131" s="35"/>
       <x:c r="J131" s="35" t="str">
-        <x:v>技能稳定ID</x:v>
+        <x:v>技能ID：技能定义的稳定主键，供玩家、输入和进度系统引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -16729,7 +17437,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J132" s="35" t="str">
-        <x:v>显示名称文案键</x:v>
+        <x:v>名称文案键：引用Texts.textKey取得本地化显示名称，不直接填写玩家可见文字。</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -16753,7 +17461,7 @@
       </x:c>
       <x:c r="I133" s="35"/>
       <x:c r="J133" s="35" t="str">
-        <x:v>Skills 表的 triggerType 字段</x:v>
+        <x:v>技能触发类型：指定技能由被动、笔势或其他入口触发，取值来自SkillTriggerType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -16777,7 +17485,7 @@
         <x:v>Stances.stanceId</x:v>
       </x:c>
       <x:c r="J134" s="35" t="str">
-        <x:v>Skills 表的 requiredStanceId 字段</x:v>
+        <x:v>释放要求架势：引用Stances.stanceId；留空表示任意架势都可释放该技能。</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -16801,7 +17509,7 @@
       <x:c r="H135" s="35"/>
       <x:c r="I135" s="35"/>
       <x:c r="J135" s="35" t="str">
-        <x:v>Skills 表的 energyCost 字段</x:v>
+        <x:v>能量消耗：释放技能时需要扣除的玩家能量；被动技能通常为0。</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -16825,7 +17533,7 @@
       <x:c r="H136" s="35"/>
       <x:c r="I136" s="35"/>
       <x:c r="J136" s="35" t="str">
-        <x:v>冷却时间（秒）</x:v>
+        <x:v>冷却秒数：同一动作再次可用前必须等待的最短时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -16849,7 +17557,7 @@
       </x:c>
       <x:c r="I137" s="35"/>
       <x:c r="J137" s="35" t="str">
-        <x:v>Skills 表的 gestureType 字段</x:v>
+        <x:v>笔势类型：指定该规则或交互要求的手势类别，取值必须登记在GestureType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -16873,7 +17581,7 @@
       <x:c r="H138" s="35"/>
       <x:c r="I138" s="35"/>
       <x:c r="J138" s="35" t="str">
-        <x:v>Skills 表的 inputWindowSec 字段</x:v>
+        <x:v>输入窗口秒数：触发技能所需笔势允许完成的最长输入时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -16897,7 +17605,7 @@
         <x:v>SkillEffects.effectGroupId</x:v>
       </x:c>
       <x:c r="J139" s="35" t="str">
-        <x:v>效果链分组ID</x:v>
+        <x:v>技能效果组：引用SkillEffects.effectGroupId，指定释放技能时按order执行的效果链。</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -16921,7 +17629,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J140" s="35" t="str">
-        <x:v>Skills 表的 iconAssetKey 字段</x:v>
+        <x:v>图标资源键：引用AssetManifest.assetKey，指定技能在UI中使用的图标资源。</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -16945,7 +17653,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J141" s="35" t="str">
-        <x:v>文案键</x:v>
+        <x:v>文案键：引用Texts.textKey取得玩家可见的本地化文本。</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
@@ -16967,7 +17675,7 @@
       <x:c r="H142" s="35"/>
       <x:c r="I142" s="35"/>
       <x:c r="J142" s="35" t="str">
-        <x:v>效果链分组ID</x:v>
+        <x:v>效果组ID：把多条SkillEffects按order组织成可复用的有序效果链。</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
@@ -16991,7 +17699,7 @@
       <x:c r="H143" s="35"/>
       <x:c r="I143" s="35"/>
       <x:c r="J143" s="35" t="str">
-        <x:v>组内执行/展示顺序，从1开始</x:v>
+        <x:v>组内顺序：同一分组内从1开始的稳定执行、选择或展示顺序。</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -17015,7 +17723,7 @@
       </x:c>
       <x:c r="I144" s="35"/>
       <x:c r="J144" s="35" t="str">
-        <x:v>SkillEffects 表的 effectType 字段</x:v>
+        <x:v>效果类型：指定该效果行执行的规则类型，取值必须来自EffectType枚举并由代码注册。</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -17039,7 +17747,7 @@
       </x:c>
       <x:c r="I145" s="35"/>
       <x:c r="J145" s="35" t="str">
-        <x:v>SkillEffects 表的 targetType 字段</x:v>
+        <x:v>目标类型：指定效果作用对象的选择方式，取值必须来自TargetType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -17061,7 +17769,7 @@
       <x:c r="H146" s="35"/>
       <x:c r="I146" s="35"/>
       <x:c r="J146" s="35" t="str">
-        <x:v>SkillEffects 表的 value1 字段</x:v>
+        <x:v>主参数：效果类型定义的第一个数值参数；具体单位和含义由effectType决定。</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
@@ -17083,7 +17791,7 @@
       <x:c r="H147" s="35"/>
       <x:c r="I147" s="35"/>
       <x:c r="J147" s="35" t="str">
-        <x:v>SkillEffects 表的 value2 字段</x:v>
+        <x:v>次参数：效果类型定义的第二个数值参数；不需要时填0。</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -17107,7 +17815,7 @@
       <x:c r="H148" s="35"/>
       <x:c r="I148" s="35"/>
       <x:c r="J148" s="35" t="str">
-        <x:v>持续时间（秒）</x:v>
+        <x:v>效果持续秒数：该效果影响保持的时间，单位为秒；瞬时效果填0。</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -17131,7 +17839,7 @@
         <x:v>Buffs.buffId</x:v>
       </x:c>
       <x:c r="J149" s="35" t="str">
-        <x:v>状态效果稳定ID</x:v>
+        <x:v>状态效果ID：引用Buffs.buffId；仅需要施加状态的effectType填写，其他效果留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -17155,7 +17863,7 @@
         <x:v>VfxCues.vfxKey</x:v>
       </x:c>
       <x:c r="J150" s="35" t="str">
-        <x:v>特效事件键</x:v>
+        <x:v>特效键：引用VfxCues.vfxKey；留空表示该事件不播放额外特效。</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -17179,7 +17887,7 @@
         <x:v>AudioCues.audioKey</x:v>
       </x:c>
       <x:c r="J151" s="35" t="str">
-        <x:v>音频事件键</x:v>
+        <x:v>音频键：引用AudioCues.audioKey；留空表示该事件不播放额外音频。</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
@@ -17201,7 +17909,7 @@
       <x:c r="H152" s="35"/>
       <x:c r="I152" s="35"/>
       <x:c r="J152" s="35" t="str">
-        <x:v>SkillEffects 表的 condition 字段</x:v>
+        <x:v>执行条件：效果执行前检查的可选条件表达式；留空表示无额外条件。</x:v>
       </x:c>
     </x:row>
     <x:row r="153">
@@ -17223,7 +17931,7 @@
       <x:c r="H153" s="35"/>
       <x:c r="I153" s="35"/>
       <x:c r="J153" s="35" t="str">
-        <x:v>关卡稳定ID</x:v>
+        <x:v>关卡ID：关卡定义的稳定主键，供波次、出生点和进度系统引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
@@ -17247,7 +17955,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J154" s="35" t="str">
-        <x:v>显示名称文案键</x:v>
+        <x:v>名称文案键：引用Texts.textKey取得本地化显示名称，不直接填写玩家可见文字。</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
@@ -17271,7 +17979,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J155" s="35" t="str">
-        <x:v>Levels 表的 sceneKey 字段</x:v>
+        <x:v>场景资源键：引用AssetManifest.assetKey，指定承载该关卡的Unity场景。</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
@@ -17295,7 +18003,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J156" s="35" t="str">
-        <x:v>Levels 表的 backgroundAssetKey 字段</x:v>
+        <x:v>背景资源键：引用AssetManifest.assetKey，指定关卡使用的背景资源。</x:v>
       </x:c>
     </x:row>
     <x:row r="157">
@@ -17317,7 +18025,7 @@
       <x:c r="H157" s="35"/>
       <x:c r="I157" s="35"/>
       <x:c r="J157" s="35" t="str">
-        <x:v>Levels 表的 durationLimitSec 字段</x:v>
+        <x:v>时限秒数：关卡允许的最大玩法时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
@@ -17341,7 +18049,7 @@
         <x:v>Levels.levelId</x:v>
       </x:c>
       <x:c r="J158" s="35" t="str">
-        <x:v>Levels 表的 nextLevelId 字段</x:v>
+        <x:v>下一关ID：引用Levels.levelId；留空表示通关后没有自动可解锁的下一关。</x:v>
       </x:c>
     </x:row>
     <x:row r="159">
@@ -17365,7 +18073,7 @@
         <x:v>Rewards.rewardTableId</x:v>
       </x:c>
       <x:c r="J159" s="35" t="str">
-        <x:v>奖励表分组ID</x:v>
+        <x:v>奖励表ID：引用Rewards.rewardTableId分组，指定该关卡结算时评估的奖励集合。</x:v>
       </x:c>
     </x:row>
     <x:row r="160">
@@ -17389,7 +18097,7 @@
       <x:c r="H160" s="35"/>
       <x:c r="I160" s="35"/>
       <x:c r="J160" s="35" t="str">
-        <x:v>Levels 表的 starScore1 字段</x:v>
+        <x:v>一星分数：结算获得一星所需达到的最低分数。</x:v>
       </x:c>
     </x:row>
     <x:row r="161">
@@ -17413,7 +18121,7 @@
       <x:c r="H161" s="35"/>
       <x:c r="I161" s="35"/>
       <x:c r="J161" s="35" t="str">
-        <x:v>Levels 表的 starScore2 字段</x:v>
+        <x:v>二星分数：结算获得二星所需达到的最低分数，必须不低于一星门槛。</x:v>
       </x:c>
     </x:row>
     <x:row r="162">
@@ -17437,7 +18145,7 @@
       <x:c r="H162" s="35"/>
       <x:c r="I162" s="35"/>
       <x:c r="J162" s="35" t="str">
-        <x:v>Levels 表的 starScore3 字段</x:v>
+        <x:v>三星分数：结算获得三星所需达到的最低分数，必须不低于二星门槛。</x:v>
       </x:c>
     </x:row>
     <x:row r="163">
@@ -17461,7 +18169,7 @@
         <x:v>Tutorials.tutorialId</x:v>
       </x:c>
       <x:c r="J163" s="35" t="str">
-        <x:v>教程流程ID</x:v>
+        <x:v>教程ID：引用Tutorials.tutorialId分组，指定该关卡加载的教程流程。</x:v>
       </x:c>
     </x:row>
     <x:row r="164">
@@ -17485,7 +18193,7 @@
         <x:v>Enemies.enemyId</x:v>
       </x:c>
       <x:c r="J164" s="35" t="str">
-        <x:v>Levels 表的 bossEnemyId 字段</x:v>
+        <x:v>Boss敌人ID：引用Enemies.enemyId；留空表示该关卡不是Boss关。</x:v>
       </x:c>
     </x:row>
     <x:row r="165">
@@ -17507,7 +18215,7 @@
       <x:c r="H165" s="35"/>
       <x:c r="I165" s="35"/>
       <x:c r="J165" s="35" t="str">
-        <x:v>波次稳定ID</x:v>
+        <x:v>波次ID：波次定义的稳定主键，供出生计划引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="166">
@@ -17531,7 +18239,7 @@
         <x:v>Levels.levelId</x:v>
       </x:c>
       <x:c r="J166" s="35" t="str">
-        <x:v>关卡稳定ID</x:v>
+        <x:v>所属关卡ID：引用Levels.levelId，指定该波次归属的关卡。</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
@@ -17555,7 +18263,7 @@
       <x:c r="H167" s="35"/>
       <x:c r="I167" s="35"/>
       <x:c r="J167" s="35" t="str">
-        <x:v>组内执行/展示顺序，从1开始</x:v>
+        <x:v>组内顺序：同一分组内从1开始的稳定执行、选择或展示顺序。</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
@@ -17579,7 +18287,7 @@
       </x:c>
       <x:c r="I168" s="35"/>
       <x:c r="J168" s="35" t="str">
-        <x:v>Waves 表的 startTrigger 字段</x:v>
+        <x:v>开始条件：指定波次何时允许开始，取值必须来自WaveStartTrigger枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -17601,7 +18309,7 @@
       <x:c r="H169" s="35"/>
       <x:c r="I169" s="35"/>
       <x:c r="J169" s="35" t="str">
-        <x:v>Waves 表的 startDelaySec 字段</x:v>
+        <x:v>开始延迟秒数：开始条件成立后到波次正式开始的等待时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="170">
@@ -17625,7 +18333,7 @@
       </x:c>
       <x:c r="I170" s="35"/>
       <x:c r="J170" s="35" t="str">
-        <x:v>Waves 表的 endCondition 字段</x:v>
+        <x:v>结束条件：指定波次完成所需事实，取值必须来自WaveEndCondition枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -17647,7 +18355,7 @@
       <x:c r="H171" s="35"/>
       <x:c r="I171" s="35"/>
       <x:c r="J171" s="35" t="str">
-        <x:v>Waves 表的 endDelaySec 字段</x:v>
+        <x:v>结束延迟秒数：结束条件成立后到推进下一波的等待时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -17671,7 +18379,7 @@
         <x:v>AudioCues.audioKey</x:v>
       </x:c>
       <x:c r="J172" s="35" t="str">
-        <x:v>Waves 表的 musicKey 字段</x:v>
+        <x:v>背景音乐键：引用AudioCues.audioKey，指定该波次播放的背景音乐。</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -17695,7 +18403,7 @@
       <x:c r="H173" s="35"/>
       <x:c r="I173" s="35"/>
       <x:c r="J173" s="35" t="str">
-        <x:v>Waves 表的 maxAlive 字段</x:v>
+        <x:v>最大存活数：该波次允许同时处于活动状态的敌人数量上限。</x:v>
       </x:c>
     </x:row>
     <x:row r="174">
@@ -17717,7 +18425,7 @@
       <x:c r="H174" s="35"/>
       <x:c r="I174" s="35"/>
       <x:c r="J174" s="35" t="str">
-        <x:v>SpawnPoints 表的 spawnPointId 字段</x:v>
+        <x:v>出生点ID：出生点定义的稳定主键，供出生计划引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -17741,7 +18449,7 @@
         <x:v>Levels.levelId</x:v>
       </x:c>
       <x:c r="J175" s="35" t="str">
-        <x:v>关卡稳定ID</x:v>
+        <x:v>适用关卡ID：引用Levels.levelId；星号表示该出生点可供所有关卡使用。</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -17767,7 +18475,7 @@
       <x:c r="H176" s="35"/>
       <x:c r="I176" s="35"/>
       <x:c r="J176" s="35" t="str">
-        <x:v>Safe Area归一化X坐标</x:v>
+        <x:v>归一化X：出生点在Safe Area宽度中的X比例，0为左侧、1为右侧。</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -17793,7 +18501,7 @@
       <x:c r="H177" s="35"/>
       <x:c r="I177" s="35"/>
       <x:c r="J177" s="35" t="str">
-        <x:v>Safe Area归一化Y坐标</x:v>
+        <x:v>归一化Y：出生点在Safe Area高度中的Y比例，0为底部、1为顶部。</x:v>
       </x:c>
     </x:row>
     <x:row r="178">
@@ -17817,7 +18525,7 @@
       </x:c>
       <x:c r="I178" s="35"/>
       <x:c r="J178" s="35" t="str">
-        <x:v>SpawnPoints 表的 lane 字段</x:v>
+        <x:v>路线层级：指定出生点属于地面、空中或Boss等路线，取值来自SpawnLane枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="179">
@@ -17839,7 +18547,7 @@
       <x:c r="H179" s="35"/>
       <x:c r="I179" s="35"/>
       <x:c r="J179" s="35" t="str">
-        <x:v>SpawnPoints 表的 jitterX 字段</x:v>
+        <x:v>X随机偏移：出生时允许施加的最大横向归一化偏移量。</x:v>
       </x:c>
     </x:row>
     <x:row r="180">
@@ -17861,7 +18569,7 @@
       <x:c r="H180" s="35"/>
       <x:c r="I180" s="35"/>
       <x:c r="J180" s="35" t="str">
-        <x:v>SpawnPoints 表的 jitterY 字段</x:v>
+        <x:v>Y随机偏移：出生时允许施加的最大纵向归一化偏移量。</x:v>
       </x:c>
     </x:row>
     <x:row r="181">
@@ -17885,7 +18593,7 @@
       </x:c>
       <x:c r="I181" s="35"/>
       <x:c r="J181" s="35" t="str">
-        <x:v>SpawnPoints 表的 facing 字段</x:v>
+        <x:v>初始朝向：实体出生时的朝向，取值必须来自Facing枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -17907,7 +18615,7 @@
       <x:c r="H182" s="35"/>
       <x:c r="I182" s="35"/>
       <x:c r="J182" s="35" t="str">
-        <x:v>SpawnPoints 表的 notes 字段</x:v>
+        <x:v>备注：记录该出生点或资源条目的策划用途、来源或替换注意事项。</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -17929,7 +18637,7 @@
       <x:c r="H183" s="35"/>
       <x:c r="I183" s="35"/>
       <x:c r="J183" s="35" t="str">
-        <x:v>EnemyModifiers 表的 modifierId 字段</x:v>
+        <x:v>修饰器ID：敌人出生修饰器的稳定主键，供出生计划引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -17953,7 +18661,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J184" s="35" t="str">
-        <x:v>显示名称文案键</x:v>
+        <x:v>名称文案键：引用Texts.textKey取得本地化显示名称，不直接填写玩家可见文字。</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
@@ -17975,7 +18683,7 @@
       <x:c r="H185" s="35"/>
       <x:c r="I185" s="35"/>
       <x:c r="J185" s="35" t="str">
-        <x:v>EnemyModifiers 表的 hpMultiplier 字段</x:v>
+        <x:v>生命倍率：出生时对敌人最大生命值应用的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="186">
@@ -17999,7 +18707,7 @@
       <x:c r="H186" s="35"/>
       <x:c r="I186" s="35"/>
       <x:c r="J186" s="35" t="str">
-        <x:v>EnemyModifiers 表的 damageMultiplier 字段</x:v>
+        <x:v>敌人伤害倍率：出生时对敌人攻击和接触伤害应用的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -18021,7 +18729,7 @@
       <x:c r="H187" s="35"/>
       <x:c r="I187" s="35"/>
       <x:c r="J187" s="35" t="str">
-        <x:v>EnemyModifiers 表的 speedMultiplier 字段</x:v>
+        <x:v>速度倍率：对实体基础移动速度应用的乘数；1表示保持基础速度。</x:v>
       </x:c>
     </x:row>
     <x:row r="188">
@@ -18043,7 +18751,7 @@
       <x:c r="H188" s="35"/>
       <x:c r="I188" s="35"/>
       <x:c r="J188" s="35" t="str">
-        <x:v>EnemyModifiers 表的 scoreMultiplier 字段</x:v>
+        <x:v>得分倍率：击败带有该修饰器的敌人时对基础得分应用的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="189">
@@ -18065,7 +18773,7 @@
       <x:c r="H189" s="35"/>
       <x:c r="I189" s="35"/>
       <x:c r="J189" s="35" t="str">
-        <x:v>EnemyModifiers 表的 tintHex 字段</x:v>
+        <x:v>染色色值：敌人表现使用的十六进制颜色；不改变玩法属性。</x:v>
       </x:c>
     </x:row>
     <x:row r="190">
@@ -18089,7 +18797,7 @@
         <x:v>Buffs.buffId</x:v>
       </x:c>
       <x:c r="J190" s="35" t="str">
-        <x:v>EnemyModifiers 表的 extraBuffId 字段</x:v>
+        <x:v>附加状态ID：引用Buffs.buffId；留空表示出生时不附加额外状态。</x:v>
       </x:c>
     </x:row>
     <x:row r="191">
@@ -18111,7 +18819,7 @@
       <x:c r="H191" s="35"/>
       <x:c r="I191" s="35"/>
       <x:c r="J191" s="35" t="str">
-        <x:v>出生条目稳定ID</x:v>
+        <x:v>出生条目ID：单条出生计划的稳定主键。</x:v>
       </x:c>
     </x:row>
     <x:row r="192">
@@ -18135,7 +18843,7 @@
         <x:v>Waves.waveId</x:v>
       </x:c>
       <x:c r="J192" s="35" t="str">
-        <x:v>波次稳定ID</x:v>
+        <x:v>所属波次ID：引用Waves.waveId，指定该出生条目归属的波次。</x:v>
       </x:c>
     </x:row>
     <x:row r="193">
@@ -18157,7 +18865,7 @@
       <x:c r="H193" s="35"/>
       <x:c r="I193" s="35"/>
       <x:c r="J193" s="35" t="str">
-        <x:v>Spawns 表的 spawnTimeSec 字段</x:v>
+        <x:v>出生时刻秒数：相对所属波次开始时刻的第一次出生时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="194">
@@ -18181,7 +18889,7 @@
         <x:v>Enemies.enemyId</x:v>
       </x:c>
       <x:c r="J194" s="35" t="str">
-        <x:v>敌人稳定ID</x:v>
+        <x:v>敌人ID：引用Enemies.enemyId，指定该出生条目创建的敌人类型。</x:v>
       </x:c>
     </x:row>
     <x:row r="195">
@@ -18205,7 +18913,7 @@
       <x:c r="H195" s="35"/>
       <x:c r="I195" s="35"/>
       <x:c r="J195" s="35" t="str">
-        <x:v>Spawns 表的 count 字段</x:v>
+        <x:v>出生数量：该行计划连续生成的敌人总数。</x:v>
       </x:c>
     </x:row>
     <x:row r="196">
@@ -18229,7 +18937,7 @@
       <x:c r="H196" s="35"/>
       <x:c r="I196" s="35"/>
       <x:c r="J196" s="35" t="str">
-        <x:v>Spawns 表的 intervalSec 字段</x:v>
+        <x:v>出生间隔秒数：同一行多个敌人之间的生成间隔，单位为秒；单个敌人可填0。</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
@@ -18253,7 +18961,7 @@
         <x:v>SpawnPoints.spawnPointId</x:v>
       </x:c>
       <x:c r="J197" s="35" t="str">
-        <x:v>Spawns 表的 spawnPointId 字段</x:v>
+        <x:v>出生点ID：引用SpawnPoints.spawnPointId，指定敌人生成的位置规则。</x:v>
       </x:c>
     </x:row>
     <x:row r="198">
@@ -18277,7 +18985,7 @@
       </x:c>
       <x:c r="I198" s="35"/>
       <x:c r="J198" s="35" t="str">
-        <x:v>Spawns 表的 spawnPattern 字段</x:v>
+        <x:v>出生队形：同一出生条目采用的队形策略，取值必须来自SpawnPattern枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="199">
@@ -18301,7 +19009,7 @@
         <x:v>EnemyModifiers.modifierId</x:v>
       </x:c>
       <x:c r="J199" s="35" t="str">
-        <x:v>Spawns 表的 modifierId 字段</x:v>
+        <x:v>修饰器ID：引用EnemyModifiers.modifierId，指定出生时附加的数值修饰。</x:v>
       </x:c>
     </x:row>
     <x:row r="200">
@@ -18323,7 +19031,7 @@
       <x:c r="H200" s="35"/>
       <x:c r="I200" s="35"/>
       <x:c r="J200" s="35" t="str">
-        <x:v>BossPhases 表的 bossPhaseId 字段</x:v>
+        <x:v>Boss阶段ID：Boss阶段定义的稳定主键。</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
@@ -18347,7 +19055,7 @@
         <x:v>Enemies.enemyId</x:v>
       </x:c>
       <x:c r="J201" s="35" t="str">
-        <x:v>敌人稳定ID</x:v>
+        <x:v>Boss敌人ID：引用Enemies.enemyId，指定该阶段所属的Boss实体。</x:v>
       </x:c>
     </x:row>
     <x:row r="202">
@@ -18371,7 +19079,7 @@
       <x:c r="H202" s="35"/>
       <x:c r="I202" s="35"/>
       <x:c r="J202" s="35" t="str">
-        <x:v>组内执行/展示顺序，从1开始</x:v>
+        <x:v>组内顺序：同一分组内从1开始的稳定执行、选择或展示顺序。</x:v>
       </x:c>
     </x:row>
     <x:row r="203">
@@ -18397,7 +19105,7 @@
       <x:c r="H203" s="35"/>
       <x:c r="I203" s="35"/>
       <x:c r="J203" s="35" t="str">
-        <x:v>BossPhases 表的 enterHpRatio 字段</x:v>
+        <x:v>进入生命比例：Boss生命比例降到该上界时进入本阶段，范围0到1。</x:v>
       </x:c>
     </x:row>
     <x:row r="204">
@@ -18423,7 +19131,7 @@
       <x:c r="H204" s="35"/>
       <x:c r="I204" s="35"/>
       <x:c r="J204" s="35" t="str">
-        <x:v>BossPhases 表的 exitHpRatio 字段</x:v>
+        <x:v>退出生命比例：Boss生命比例降到该下界时退出本阶段，范围0到1。</x:v>
       </x:c>
     </x:row>
     <x:row r="205">
@@ -18447,7 +19155,7 @@
         <x:v>MovePatterns.movePatternId</x:v>
       </x:c>
       <x:c r="J205" s="35" t="str">
-        <x:v>BossPhases 表的 movementPatternId 字段</x:v>
+        <x:v>阶段移动模式：引用MovePatterns.movePatternId，指定Boss在该阶段使用的移动策略。</x:v>
       </x:c>
     </x:row>
     <x:row r="206">
@@ -18469,7 +19177,7 @@
       <x:c r="H206" s="35"/>
       <x:c r="I206" s="35"/>
       <x:c r="J206" s="35" t="str">
-        <x:v>攻击集合分组ID</x:v>
+        <x:v>阶段攻击集合：引用EnemyAttacks.attackSetId分组，指定Boss在该阶段使用的攻击集合。</x:v>
       </x:c>
     </x:row>
     <x:row r="207">
@@ -18493,7 +19201,7 @@
         <x:v>DefenseRules.defenseRuleId</x:v>
       </x:c>
       <x:c r="J207" s="35" t="str">
-        <x:v>防御规则稳定ID</x:v>
+        <x:v>阶段防御规则：引用DefenseRules.defenseRuleId，指定Boss在该阶段使用的防御规则。</x:v>
       </x:c>
     </x:row>
     <x:row r="208">
@@ -18517,7 +19225,7 @@
         <x:v>WeakpointRules.weakpointRuleId</x:v>
       </x:c>
       <x:c r="J208" s="35" t="str">
-        <x:v>弱点规则稳定ID</x:v>
+        <x:v>阶段弱点规则：引用WeakpointRules.weakpointRuleId，指定Boss在该阶段使用的弱点窗口。</x:v>
       </x:c>
     </x:row>
     <x:row r="209">
@@ -18541,7 +19249,7 @@
         <x:v>SkillEffects.effectGroupId</x:v>
       </x:c>
       <x:c r="J209" s="35" t="str">
-        <x:v>BossPhases 表的 onEnterEffectGroupId 字段</x:v>
+        <x:v>入场效果组：引用SkillEffects.effectGroupId，进入该Boss阶段时执行对应效果链。</x:v>
       </x:c>
     </x:row>
     <x:row r="210">
@@ -18565,7 +19273,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J210" s="35" t="str">
-        <x:v>BossPhases 表的 descriptionKey 字段</x:v>
+        <x:v>阶段文案键：引用Texts.textKey，取得该Boss阶段的本地化说明。</x:v>
       </x:c>
     </x:row>
     <x:row r="211">
@@ -18587,7 +19295,7 @@
       <x:c r="H211" s="35"/>
       <x:c r="I211" s="35"/>
       <x:c r="J211" s="35" t="str">
-        <x:v>奖励表分组ID</x:v>
+        <x:v>奖励表ID：把多条Rewards规则分组为关卡可引用的奖励集合。</x:v>
       </x:c>
     </x:row>
     <x:row r="212">
@@ -18611,7 +19319,7 @@
       <x:c r="H212" s="35"/>
       <x:c r="I212" s="35"/>
       <x:c r="J212" s="35" t="str">
-        <x:v>组内执行/展示顺序，从1开始</x:v>
+        <x:v>组内顺序：同一分组内从1开始的稳定执行、选择或展示顺序。</x:v>
       </x:c>
     </x:row>
     <x:row r="213">
@@ -18635,7 +19343,7 @@
       </x:c>
       <x:c r="I213" s="35"/>
       <x:c r="J213" s="35" t="str">
-        <x:v>Rewards 表的 conditionType 字段</x:v>
+        <x:v>奖励条件类型：指定奖励判定规则，取值必须来自RewardCondition枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="214">
@@ -18657,7 +19365,7 @@
       <x:c r="H214" s="35"/>
       <x:c r="I214" s="35"/>
       <x:c r="J214" s="35" t="str">
-        <x:v>Rewards 表的 conditionValue 字段</x:v>
+        <x:v>奖励条件值：按conditionType解释的条件参数，例如通关标记或最低星级。</x:v>
       </x:c>
     </x:row>
     <x:row r="215">
@@ -18681,7 +19389,7 @@
       </x:c>
       <x:c r="I215" s="35"/>
       <x:c r="J215" s="35" t="str">
-        <x:v>Rewards 表的 rewardType 字段</x:v>
+        <x:v>奖励类型：指定满足条件后发放的奖励类别，取值必须来自RewardType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="216">
@@ -18705,7 +19413,7 @@
         <x:v>conditional</x:v>
       </x:c>
       <x:c r="J216" s="35" t="str">
-        <x:v>Rewards 表的 rewardId 字段</x:v>
+        <x:v>奖励对象ID：按rewardType解释的奖励对象标识；解锁关卡时引用Levels.levelId。</x:v>
       </x:c>
     </x:row>
     <x:row r="217">
@@ -18727,7 +19435,7 @@
       <x:c r="H217" s="35"/>
       <x:c r="I217" s="35"/>
       <x:c r="J217" s="35" t="str">
-        <x:v>Rewards 表的 amount 字段</x:v>
+        <x:v>奖励数量：满足条件后发放或累计的奖励数量。</x:v>
       </x:c>
     </x:row>
     <x:row r="218">
@@ -18749,7 +19457,7 @@
       <x:c r="H218" s="35"/>
       <x:c r="I218" s="35"/>
       <x:c r="J218" s="35" t="str">
-        <x:v>教程流程ID</x:v>
+        <x:v>教程ID：把多条Tutorials步骤分组为关卡可引用的教程流程。</x:v>
       </x:c>
     </x:row>
     <x:row r="219">
@@ -18773,7 +19481,7 @@
       <x:c r="H219" s="35"/>
       <x:c r="I219" s="35"/>
       <x:c r="J219" s="35" t="str">
-        <x:v>组内执行/展示顺序，从1开始</x:v>
+        <x:v>组内顺序：同一分组内从1开始的稳定执行、选择或展示顺序。</x:v>
       </x:c>
     </x:row>
     <x:row r="220">
@@ -18795,7 +19503,7 @@
       <x:c r="H220" s="35"/>
       <x:c r="I220" s="35"/>
       <x:c r="J220" s="35" t="str">
-        <x:v>Tutorials 表的 triggerEvent 字段</x:v>
+        <x:v>教程触发事件：教程步骤开始等待的运行时事件协议名。</x:v>
       </x:c>
     </x:row>
     <x:row r="221">
@@ -18817,7 +19525,7 @@
       <x:c r="H221" s="35"/>
       <x:c r="I221" s="35"/>
       <x:c r="J221" s="35" t="str">
-        <x:v>Tutorials 表的 blockProgress 字段</x:v>
+        <x:v>阻断战斗推进：步骤显示期间是否暂停受教程门控制的战斗推进。</x:v>
       </x:c>
     </x:row>
     <x:row r="222">
@@ -18839,7 +19547,7 @@
       <x:c r="H222" s="35"/>
       <x:c r="I222" s="35"/>
       <x:c r="J222" s="35" t="str">
-        <x:v>Tutorials 表的 minDisplaySec 字段</x:v>
+        <x:v>最短展示秒数：教程步骤即使已满足完成条件也必须保持显示的最短时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="223">
@@ -18861,7 +19569,7 @@
       <x:c r="H223" s="35"/>
       <x:c r="I223" s="35"/>
       <x:c r="J223" s="35" t="str">
-        <x:v>Tutorials 表的 completeEvent 字段</x:v>
+        <x:v>教程完成事件：玩家完成本步骤所需发布的事件协议或带阈值事件表达式。</x:v>
       </x:c>
     </x:row>
     <x:row r="224">
@@ -18885,7 +19593,7 @@
         <x:v>Texts.textKey</x:v>
       </x:c>
       <x:c r="J224" s="35" t="str">
-        <x:v>文案键</x:v>
+        <x:v>文案键：引用Texts.textKey取得玩家可见的本地化文本。</x:v>
       </x:c>
     </x:row>
     <x:row r="225">
@@ -18907,7 +19615,7 @@
       <x:c r="H225" s="35"/>
       <x:c r="I225" s="35"/>
       <x:c r="J225" s="35" t="str">
-        <x:v>Tutorials 表的 highlightTarget 字段</x:v>
+        <x:v>高亮目标：教程遮罩需要突出显示的UI或战斗区域协议名。</x:v>
       </x:c>
     </x:row>
     <x:row r="226">
@@ -18931,7 +19639,7 @@
       </x:c>
       <x:c r="I226" s="35"/>
       <x:c r="J226" s="35" t="str">
-        <x:v>Tutorials 表的 gestureType 字段</x:v>
+        <x:v>笔势类型：指定该规则或交互要求的手势类别，取值必须登记在GestureType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="227">
@@ -18953,7 +19661,7 @@
       <x:c r="H227" s="35"/>
       <x:c r="I227" s="35"/>
       <x:c r="J227" s="35" t="str">
-        <x:v>文案键</x:v>
+        <x:v>文案键：本地化文案的稳定主键，供配置和UI引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="228">
@@ -18975,7 +19683,7 @@
       <x:c r="H228" s="35"/>
       <x:c r="I228" s="35"/>
       <x:c r="J228" s="35" t="str">
-        <x:v>Texts 表的 zhCN 字段</x:v>
+        <x:v>简体中文：该文案键对应的简体中文玩家可见文本。</x:v>
       </x:c>
     </x:row>
     <x:row r="229">
@@ -18997,7 +19705,7 @@
       <x:c r="H229" s="35"/>
       <x:c r="I229" s="35"/>
       <x:c r="J229" s="35" t="str">
-        <x:v>Texts 表的 enUS 字段</x:v>
+        <x:v>英文：该文案键对应的英文回退或本地化文本。</x:v>
       </x:c>
     </x:row>
     <x:row r="230">
@@ -19019,7 +19727,7 @@
       <x:c r="H230" s="35"/>
       <x:c r="I230" s="35"/>
       <x:c r="J230" s="35" t="str">
-        <x:v>Texts 表的 context 字段</x:v>
+        <x:v>使用场景：说明文案出现的位置或用途，便于翻译和字体覆盖审查。</x:v>
       </x:c>
     </x:row>
     <x:row r="231">
@@ -19041,7 +19749,7 @@
       <x:c r="H231" s="35"/>
       <x:c r="I231" s="35"/>
       <x:c r="J231" s="35" t="str">
-        <x:v>音频事件键</x:v>
+        <x:v>音频事件键：音频提示的稳定主键，供战斗、UI和反馈配置引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="232">
@@ -19065,7 +19773,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J232" s="35" t="str">
-        <x:v>Unity资源注册键</x:v>
+        <x:v>音频资源键：引用AssetManifest.assetKey，并由Unity AssetRegistry解析为AudioClip。</x:v>
       </x:c>
     </x:row>
     <x:row r="233">
@@ -19089,7 +19797,7 @@
       </x:c>
       <x:c r="I233" s="35"/>
       <x:c r="J233" s="35" t="str">
-        <x:v>AudioCues 表的 category 字段</x:v>
+        <x:v>音频分类：区分背景音乐、音效等通道类型，取值必须来自AudioCategory枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="234">
@@ -19115,7 +19823,7 @@
       <x:c r="H234" s="35"/>
       <x:c r="I234" s="35"/>
       <x:c r="J234" s="35" t="str">
-        <x:v>AudioCues 表的 volume 字段</x:v>
+        <x:v>音量：播放该音频时使用的0到1线性音量。</x:v>
       </x:c>
     </x:row>
     <x:row r="235">
@@ -19137,7 +19845,7 @@
       <x:c r="H235" s="35"/>
       <x:c r="I235" s="35"/>
       <x:c r="J235" s="35" t="str">
-        <x:v>AudioCues 表的 pitchMin 字段</x:v>
+        <x:v>最低音调：随机音调范围的下界；1表示原始音调。</x:v>
       </x:c>
     </x:row>
     <x:row r="236">
@@ -19159,7 +19867,7 @@
       <x:c r="H236" s="35"/>
       <x:c r="I236" s="35"/>
       <x:c r="J236" s="35" t="str">
-        <x:v>AudioCues 表的 pitchMax 字段</x:v>
+        <x:v>最高音调：随机音调范围的上界，必须不低于最低音调。</x:v>
       </x:c>
     </x:row>
     <x:row r="237">
@@ -19183,7 +19891,7 @@
       <x:c r="H237" s="35"/>
       <x:c r="I237" s="35"/>
       <x:c r="J237" s="35" t="str">
-        <x:v>AudioCues 表的 maxConcurrent 字段</x:v>
+        <x:v>最大并发数：该音频事件允许同时播放的实例数量上限。</x:v>
       </x:c>
     </x:row>
     <x:row r="238">
@@ -19207,7 +19915,7 @@
       <x:c r="H238" s="35"/>
       <x:c r="I238" s="35"/>
       <x:c r="J238" s="35" t="str">
-        <x:v>冷却时间（秒）</x:v>
+        <x:v>冷却秒数：同一动作再次可用前必须等待的最短时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="239">
@@ -19229,7 +19937,7 @@
       <x:c r="H239" s="35"/>
       <x:c r="I239" s="35"/>
       <x:c r="J239" s="35" t="str">
-        <x:v>特效事件键</x:v>
+        <x:v>特效事件键：特效提示的稳定主键，供技能、弱点和战斗反馈引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="240">
@@ -19253,7 +19961,7 @@
         <x:v>AssetManifest.assetKey</x:v>
       </x:c>
       <x:c r="J240" s="35" t="str">
-        <x:v>Unity资源注册键</x:v>
+        <x:v>特效资源键：引用AssetManifest.assetKey，并由Unity AssetRegistry解析为特效Prefab。</x:v>
       </x:c>
     </x:row>
     <x:row r="241">
@@ -19277,7 +19985,7 @@
       <x:c r="H241" s="35"/>
       <x:c r="I241" s="35"/>
       <x:c r="J241" s="35" t="str">
-        <x:v>VfxCues 表的 lifeSec 字段</x:v>
+        <x:v>特效寿命秒数：特效实例从播放到自动回池的非缩放时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="242">
@@ -19301,7 +20009,7 @@
       <x:c r="H242" s="35"/>
       <x:c r="I242" s="35"/>
       <x:c r="J242" s="35" t="str">
-        <x:v>对象池预热数量</x:v>
+        <x:v>池预热数量：进入会话时为该资源预先创建的对象数量，用于降低首次生成开销。</x:v>
       </x:c>
     </x:row>
     <x:row r="243">
@@ -19323,7 +20031,7 @@
       <x:c r="H243" s="35"/>
       <x:c r="I243" s="35"/>
       <x:c r="J243" s="35" t="str">
-        <x:v>VfxCues 表的 followTarget 字段</x:v>
+        <x:v>跟随目标：特效播放期间是否持续跟随目标；关闭时使用触发瞬间的位置快照。</x:v>
       </x:c>
     </x:row>
     <x:row r="244">
@@ -19345,7 +20053,7 @@
       <x:c r="H244" s="35"/>
       <x:c r="I244" s="35"/>
       <x:c r="J244" s="35" t="str">
-        <x:v>VfxCues 表的 sortingLayer 字段</x:v>
+        <x:v>排序层：SpriteRenderer或LineRenderer使用的Unity Sorting Layer名称。</x:v>
       </x:c>
     </x:row>
     <x:row r="245">
@@ -19367,7 +20075,7 @@
       <x:c r="H245" s="35"/>
       <x:c r="I245" s="35"/>
       <x:c r="J245" s="35" t="str">
-        <x:v>VfxCues 表的 sortingOrder 字段</x:v>
+        <x:v>层内顺序：在相同Sorting Layer内决定前后遮挡关系的整数顺序。</x:v>
       </x:c>
     </x:row>
     <x:row r="246">
@@ -19389,7 +20097,7 @@
       <x:c r="H246" s="35"/>
       <x:c r="I246" s="35"/>
       <x:c r="J246" s="35" t="str">
-        <x:v>Unity资源注册键</x:v>
+        <x:v>资源键：资源清单条目的稳定主键，供各配置表和Unity AssetRegistry共同引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="247">
@@ -19413,7 +20121,7 @@
       </x:c>
       <x:c r="I247" s="35"/>
       <x:c r="J247" s="35" t="str">
-        <x:v>AssetManifest 表的 assetType 字段</x:v>
+        <x:v>资源类型：指定资源键对应的Unity对象类型，取值必须来自AssetType枚举。</x:v>
       </x:c>
     </x:row>
     <x:row r="248">
@@ -19435,7 +20143,7 @@
       <x:c r="H248" s="35"/>
       <x:c r="I248" s="35"/>
       <x:c r="J248" s="35" t="str">
-        <x:v>AssetManifest 表的 addressOrPath 字段</x:v>
+        <x:v>审查路径：供作者工具和人工审查定位资源的工程路径；运行时仍通过AssetRegistry引用对象。</x:v>
       </x:c>
     </x:row>
     <x:row r="249">
@@ -19457,7 +20165,7 @@
       <x:c r="H249" s="35"/>
       <x:c r="I249" s="35"/>
       <x:c r="J249" s="35" t="str">
-        <x:v>AssetManifest 表的 requiredInMvp 字段</x:v>
+        <x:v>MVP必需：该资源是否属于MVP不可缺失的构建内容。</x:v>
       </x:c>
     </x:row>
     <x:row r="250">
@@ -19479,7 +20187,7 @@
       <x:c r="H250" s="35"/>
       <x:c r="I250" s="35"/>
       <x:c r="J250" s="35" t="str">
-        <x:v>AssetManifest 表的 notes 字段</x:v>
+        <x:v>备注：记录该出生点或资源条目的策划用途、来源或替换注意事项。</x:v>
       </x:c>
     </x:row>
     <x:row r="251">
@@ -19501,7 +20209,7 @@
       <x:c r="H251" s="35"/>
       <x:c r="I251" s="35"/>
       <x:c r="J251" s="35" t="str">
-        <x:v>Enums 表的 enumType 字段</x:v>
+        <x:v>枚举类型：枚举值所属的稳定类型名。</x:v>
       </x:c>
     </x:row>
     <x:row r="252">
@@ -19523,7 +20231,7 @@
       <x:c r="H252" s="35"/>
       <x:c r="I252" s="35"/>
       <x:c r="J252" s="35" t="str">
-        <x:v>Enums 表的 value 字段</x:v>
+        <x:v>枚举值：写入业务字段的稳定英文枚举值，必须与代码协议一致。</x:v>
       </x:c>
     </x:row>
     <x:row r="253">
@@ -19544,8 +20252,8 @@
       <x:c r="G253"/>
       <x:c r="H253"/>
       <x:c r="I253"/>
-      <x:c r="J253" t="str">
-        <x:v>Enums 表的 displayName 字段</x:v>
+      <x:c r="J253" s="34" t="str">
+        <x:v>枚举显示名：供配置编辑和审查使用的枚举名称，不作为玩家本地化文案。</x:v>
       </x:c>
     </x:row>
     <x:row r="254">
@@ -19566,8 +20274,8 @@
       <x:c r="G254"/>
       <x:c r="H254"/>
       <x:c r="I254"/>
-      <x:c r="J254" t="str">
-        <x:v>Enums 表的 description 字段</x:v>
+      <x:c r="J254" s="34" t="str">
+        <x:v>枚举说明：说明该枚举值的协议用途、约束或选择含义。</x:v>
       </x:c>
     </x:row>
     <x:row r="255">
@@ -19588,8 +20296,8 @@
       <x:c r="G255" s="132"/>
       <x:c r="H255" s="132"/>
       <x:c r="I255" s="132"/>
-      <x:c r="J255" s="132" t="str">
-        <x:v>反馈配置稳定ID。</x:v>
+      <x:c r="J255" s="203" t="str">
+        <x:v>反馈配置ID：战斗反馈档案的稳定主键，供命中、受击和死亡事件选择。</x:v>
       </x:c>
     </x:row>
     <x:row r="256">
@@ -19612,8 +20320,8 @@
       <x:c r="I256" s="137" t="str">
         <x:v>VfxCues.vfxKey</x:v>
       </x:c>
-      <x:c r="J256" s="137" t="str">
-        <x:v>反馈使用的特效提示外键。</x:v>
+      <x:c r="J256" s="204" t="str">
+        <x:v>反馈特效键：引用VfxCues.vfxKey，指定该战斗反馈必须播放的特效提示。</x:v>
       </x:c>
     </x:row>
     <x:row r="257">
@@ -19636,8 +20344,8 @@
       <x:c r="I257" s="132" t="str">
         <x:v>AudioCues.audioKey</x:v>
       </x:c>
-      <x:c r="J257" s="132" t="str">
-        <x:v>反馈使用的音频提示外键。</x:v>
+      <x:c r="J257" s="203" t="str">
+        <x:v>反馈音频键：引用AudioCues.audioKey，指定该战斗反馈必须播放的音频提示。</x:v>
       </x:c>
     </x:row>
     <x:row r="258">
@@ -19662,8 +20370,8 @@
       </x:c>
       <x:c r="H258" s="137"/>
       <x:c r="I258" s="137"/>
-      <x:c r="J258" s="137" t="str">
-        <x:v>反馈期间的玩法时间缩放；0表示完全停顿。</x:v>
+      <x:c r="J258" s="204" t="str">
+        <x:v>时间缩放：反馈期间玩法时间的缩放比例；0表示完全停顿，1表示正常速度。</x:v>
       </x:c>
     </x:row>
     <x:row r="259">
@@ -19688,8 +20396,8 @@
       </x:c>
       <x:c r="H259" s="132"/>
       <x:c r="I259" s="132"/>
-      <x:c r="J259" s="132" t="str">
-        <x:v>玩法时间缩放持续秒数，使用非缩放时间推进。</x:v>
+      <x:c r="J259" s="203" t="str">
+        <x:v>时间缩放秒数：时间缩放保持的非缩放时长，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="260">
@@ -19714,8 +20422,8 @@
       </x:c>
       <x:c r="H260" s="137"/>
       <x:c r="I260" s="137"/>
-      <x:c r="J260" s="137" t="str">
-        <x:v>目标白闪持续秒数。</x:v>
+      <x:c r="J260" s="204" t="str">
+        <x:v>闪白秒数：受击目标保持闪白表现的时间，单位为非缩放秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="261">
@@ -19740,8 +20448,8 @@
       </x:c>
       <x:c r="H261" s="132"/>
       <x:c r="I261" s="132"/>
-      <x:c r="J261" s="132" t="str">
-        <x:v>1920×1080参考分辨率下的震屏强度像素。</x:v>
+      <x:c r="J261" s="203" t="str">
+        <x:v>震屏强度：1920×1080参考分辨率下相机震动的最大位移，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="262">
@@ -19766,8 +20474,8 @@
       </x:c>
       <x:c r="H262" s="137"/>
       <x:c r="I262" s="137"/>
-      <x:c r="J262" s="137" t="str">
-        <x:v>震屏持续秒数。</x:v>
+      <x:c r="J262" s="204" t="str">
+        <x:v>震屏秒数：相机震动持续的非缩放时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="263">
@@ -19790,8 +20498,8 @@
         <x:v>FeedbackVibrationPattern</x:v>
       </x:c>
       <x:c r="I263" s="132"/>
-      <x:c r="J263" s="132" t="str">
-        <x:v>平台震动强度；可由用户总开关禁用。</x:v>
+      <x:c r="J263" s="203" t="str">
+        <x:v>震动档位：平台震动强度协议，取值来自FeedbackVibrationPattern枚举并受用户总开关控制。</x:v>
       </x:c>
     </x:row>
     <x:row r="264">
@@ -19812,8 +20520,8 @@
       <x:c r="G264" s="137"/>
       <x:c r="H264" s="137"/>
       <x:c r="I264" s="137"/>
-      <x:c r="J264" s="137" t="str">
-        <x:v>伤害数字颜色，格式为#RRGGBBAA。</x:v>
+      <x:c r="J264" s="204" t="str">
+        <x:v>伤害数字颜色：伤害数字使用的#RRGGBBAA十六进制颜色。</x:v>
       </x:c>
     </x:row>
     <x:row r="265">
@@ -19838,8 +20546,8 @@
       </x:c>
       <x:c r="H265" s="132"/>
       <x:c r="I265" s="132"/>
-      <x:c r="J265" s="132" t="str">
-        <x:v>1920×1080参考分辨率下的伤害数字字号。</x:v>
+      <x:c r="J265" s="203" t="str">
+        <x:v>伤害数字字号：1920×1080参考分辨率下的伤害数字字号。</x:v>
       </x:c>
     </x:row>
     <x:row r="266">
@@ -19864,8 +20572,8 @@
       </x:c>
       <x:c r="H266" s="137"/>
       <x:c r="I266" s="137"/>
-      <x:c r="J266" s="137" t="str">
-        <x:v>伤害数字存活秒数。</x:v>
+      <x:c r="J266" s="204" t="str">
+        <x:v>伤害数字寿命：伤害数字从出现到回池的非缩放时间，单位为秒。</x:v>
       </x:c>
     </x:row>
     <x:row r="267">
@@ -19890,8 +20598,8 @@
       </x:c>
       <x:c r="H267" s="132"/>
       <x:c r="I267" s="132"/>
-      <x:c r="J267" s="132" t="str">
-        <x:v>伤害数字生命周期内上浮的参考像素。</x:v>
+      <x:c r="J267" s="203" t="str">
+        <x:v>伤害数字上浮：伤害数字生命周期内向上移动的总距离，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="268">
@@ -19912,8 +20620,8 @@
       <x:c r="G268" s="137"/>
       <x:c r="H268" s="137"/>
       <x:c r="I268" s="137"/>
-      <x:c r="J268" s="137" t="str">
-        <x:v>反馈特效染色，格式为#RRGGBBAA。</x:v>
+      <x:c r="J268" s="204" t="str">
+        <x:v>特效染色：反馈特效使用的#RRGGBBAA十六进制乘色色值。</x:v>
       </x:c>
     </x:row>
     <x:row r="269">
@@ -19938,8 +20646,8 @@
       </x:c>
       <x:c r="H269" s="132"/>
       <x:c r="I269" s="132"/>
-      <x:c r="J269" s="132" t="str">
-        <x:v>1920×1080参考分辨率下的特效尺寸。</x:v>
+      <x:c r="J269" s="203" t="str">
+        <x:v>特效尺寸：1920×1080参考分辨率下反馈特效的目标显示尺寸。</x:v>
       </x:c>
     </x:row>
     <x:row r="270">
@@ -19960,8 +20668,8 @@
       <x:c r="G270" s="137"/>
       <x:c r="H270" s="137"/>
       <x:c r="I270" s="137"/>
-      <x:c r="J270" s="137" t="str">
-        <x:v>反馈配置用途说明。</x:v>
+      <x:c r="J270" s="204" t="str">
+        <x:v>反馈说明：概括该反馈档案对应的战斗事件和玩家感受目标。</x:v>
       </x:c>
     </x:row>
     <x:row r="271">
@@ -19984,8 +20692,8 @@
       <x:c r="I271" s="189" t="str">
         <x:v>StrokeTrailStyles.styleId</x:v>
       </x:c>
-      <x:c r="J271" s="189" t="str">
-        <x:v>架势选择的画笔表现样式外键。</x:v>
+      <x:c r="J271" s="205" t="str">
+        <x:v>画笔样式：引用StrokeTrailStyles.styleId，指定该架势的分层轨迹和电弧表现。</x:v>
       </x:c>
     </x:row>
     <x:row r="272">
@@ -20006,8 +20714,8 @@
       <x:c r="G272" s="189"/>
       <x:c r="H272" s="189"/>
       <x:c r="I272" s="189"/>
-      <x:c r="J272" s="189" t="str">
-        <x:v>画笔样式稳定ID。</x:v>
+      <x:c r="J272" s="205" t="str">
+        <x:v>样式ID：画笔轨迹样式的稳定主键，供Stances引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="273">
@@ -20028,8 +20736,8 @@
       <x:c r="G273" s="189"/>
       <x:c r="H273" s="189"/>
       <x:c r="I273" s="189"/>
-      <x:c r="J273" s="189" t="str">
-        <x:v>外层辉光颜色，格式为#RRGGBBAA。</x:v>
+      <x:c r="J273" s="205" t="str">
+        <x:v>外层颜色：轨迹外层辉光使用的#RRGGBBAA十六进制颜色。</x:v>
       </x:c>
     </x:row>
     <x:row r="274">
@@ -20050,8 +20758,8 @@
       <x:c r="G274" s="189"/>
       <x:c r="H274" s="189"/>
       <x:c r="I274" s="189"/>
-      <x:c r="J274" s="189" t="str">
-        <x:v>主体轨迹颜色，格式为#RRGGBBAA。</x:v>
+      <x:c r="J274" s="205" t="str">
+        <x:v>主体颜色：轨迹主体使用的#RRGGBBAA十六进制颜色。</x:v>
       </x:c>
     </x:row>
     <x:row r="275">
@@ -20072,8 +20780,8 @@
       <x:c r="G275" s="189"/>
       <x:c r="H275" s="189"/>
       <x:c r="I275" s="189"/>
-      <x:c r="J275" s="189" t="str">
-        <x:v>核心高光颜色，格式为#RRGGBBAA。</x:v>
+      <x:c r="J275" s="205" t="str">
+        <x:v>核心颜色：轨迹核心高光使用的#RRGGBBAA十六进制颜色。</x:v>
       </x:c>
     </x:row>
     <x:row r="276">
@@ -20098,8 +20806,8 @@
       </x:c>
       <x:c r="H276" s="189"/>
       <x:c r="I276" s="189"/>
-      <x:c r="J276" s="189" t="str">
-        <x:v>外层宽度相对架势基础笔宽的倍率。</x:v>
+      <x:c r="J276" s="205" t="str">
+        <x:v>外层宽度倍率：外层辉光宽度相对架势基础笔宽的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="277">
@@ -20124,8 +20832,8 @@
       </x:c>
       <x:c r="H277" s="189"/>
       <x:c r="I277" s="189"/>
-      <x:c r="J277" s="189" t="str">
-        <x:v>主体宽度相对架势基础笔宽的倍率。</x:v>
+      <x:c r="J277" s="205" t="str">
+        <x:v>主体宽度倍率：主体轨迹宽度相对架势基础笔宽的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="278">
@@ -20150,8 +20858,8 @@
       </x:c>
       <x:c r="H278" s="189"/>
       <x:c r="I278" s="189"/>
-      <x:c r="J278" s="189" t="str">
-        <x:v>核心宽度相对架势基础笔宽的倍率。</x:v>
+      <x:c r="J278" s="205" t="str">
+        <x:v>核心宽度倍率：核心高光宽度相对架势基础笔宽的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="279">
@@ -20172,8 +20880,8 @@
       <x:c r="G279" s="189"/>
       <x:c r="H279" s="189"/>
       <x:c r="I279" s="189"/>
-      <x:c r="J279" s="189" t="str">
-        <x:v>分支电弧颜色，格式为#RRGGBBAA。</x:v>
+      <x:c r="J279" s="205" t="str">
+        <x:v>分支颜色：分支电弧使用的#RRGGBBAA十六进制颜色。</x:v>
       </x:c>
     </x:row>
     <x:row r="280">
@@ -20198,8 +20906,8 @@
       </x:c>
       <x:c r="H280" s="189"/>
       <x:c r="I280" s="189"/>
-      <x:c r="J280" s="189" t="str">
-        <x:v>相邻分支电弧在参考路径上的目标间距。</x:v>
+      <x:c r="J280" s="205" t="str">
+        <x:v>分支间距：相邻分支沿主路径分布的目标间距，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="281">
@@ -20224,8 +20932,8 @@
       </x:c>
       <x:c r="H281" s="189"/>
       <x:c r="I281" s="189"/>
-      <x:c r="J281" s="189" t="str">
-        <x:v>分支电弧的参考像素长度。</x:v>
+      <x:c r="J281" s="205" t="str">
+        <x:v>分支长度：单条分支电弧的目标长度，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="282">
@@ -20250,8 +20958,8 @@
       </x:c>
       <x:c r="H282" s="189"/>
       <x:c r="I282" s="189"/>
-      <x:c r="J282" s="189" t="str">
-        <x:v>分支电弧折点的最大参考像素抖动。</x:v>
+      <x:c r="J282" s="205" t="str">
+        <x:v>分支抖动：分支折点允许偏离基准线的最大距离，单位为参考像素。</x:v>
       </x:c>
     </x:row>
     <x:row r="283">
@@ -20276,8 +20984,8 @@
       </x:c>
       <x:c r="H283" s="189"/>
       <x:c r="I283" s="189"/>
-      <x:c r="J283" s="189" t="str">
-        <x:v>分支宽度相对架势基础笔宽的倍率。</x:v>
+      <x:c r="J283" s="205" t="str">
+        <x:v>分支宽度倍率：分支电弧宽度相对架势基础笔宽的乘数。</x:v>
       </x:c>
     </x:row>
     <x:row r="284">
@@ -20302,8 +21010,8 @@
       </x:c>
       <x:c r="H284" s="189"/>
       <x:c r="I284" s="189"/>
-      <x:c r="J284" s="189" t="str">
-        <x:v>单条分支电弧的线段数量。</x:v>
+      <x:c r="J284" s="205" t="str">
+        <x:v>分支线段数：构成单条分支电弧的折线段数量。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20326,7 +21034,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0aabb4361c5145d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5592659899c4299"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20369,6 +21077,32 @@
       <x:c r="G2" s="13"/>
       <x:c r="H2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>玩家ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>名称文案键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>最大生命值</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>最大能量</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>默认架势</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>终极技能</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>受击无敌秒数</x:v>
+      </x:c>
+      <x:c r="H3" s="222" t="str">
+        <x:v>角色资源键</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>playerId</x:v>
@@ -20428,7 +21162,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4002b8104fa54564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd64f2401968f4d22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20494,6 +21228,56 @@
       <x:c r="N2" s="145"/>
       <x:c r="O2" s="145"/>
       <x:c r="P2" s="145"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>反馈配置ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>反馈特效键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>反馈音频键</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>时间缩放</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>时间缩放秒数</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>闪白秒数</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>震屏强度</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>震屏秒数</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>震动档位</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>伤害数字颜色</x:v>
+      </x:c>
+      <x:c r="K3" s="221" t="str">
+        <x:v>伤害数字字号</x:v>
+      </x:c>
+      <x:c r="L3" s="221" t="str">
+        <x:v>伤害数字寿命</x:v>
+      </x:c>
+      <x:c r="M3" s="221" t="str">
+        <x:v>伤害数字上浮</x:v>
+      </x:c>
+      <x:c r="N3" s="221" t="str">
+        <x:v>特效染色</x:v>
+      </x:c>
+      <x:c r="O3" s="221" t="str">
+        <x:v>特效尺寸</x:v>
+      </x:c>
+      <x:c r="P3" s="222" t="str">
+        <x:v>反馈说明</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
       <x:c r="A4" s="150" t="str">
@@ -20918,20 +21702,46 @@
       <x:c r="L2" s="177"/>
       <x:c r="M2" s="177"/>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3"/>
-      <x:c r="B3"/>
-      <x:c r="C3"/>
-      <x:c r="D3"/>
-      <x:c r="E3"/>
-      <x:c r="F3"/>
-      <x:c r="G3"/>
-      <x:c r="H3"/>
-      <x:c r="I3"/>
-      <x:c r="J3"/>
-      <x:c r="K3"/>
-      <x:c r="L3"/>
-      <x:c r="M3"/>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>样式ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>外层颜色</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>主体颜色</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>核心颜色</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>外层宽度倍率</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>主体宽度倍率</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>核心宽度倍率</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>分支颜色</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>分支间距</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>分支长度</x:v>
+      </x:c>
+      <x:c r="K3" s="221" t="str">
+        <x:v>分支抖动</x:v>
+      </x:c>
+      <x:c r="L3" s="221" t="str">
+        <x:v>分支宽度倍率</x:v>
+      </x:c>
+      <x:c r="M3" s="222" t="str">
+        <x:v>分支线段数</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="182" t="str">
@@ -21071,18 +21881,40 @@
       <x:c r="J2"/>
       <x:c r="K2"/>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3"/>
-      <x:c r="B3"/>
-      <x:c r="C3"/>
-      <x:c r="D3"/>
-      <x:c r="E3"/>
-      <x:c r="F3"/>
-      <x:c r="G3"/>
-      <x:c r="H3"/>
-      <x:c r="I3"/>
-      <x:c r="J3"/>
-      <x:c r="K3"/>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>架势ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>名称文案键</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>伤害公式</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>架势伤害倍率</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>幽魂伤害倍率</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>切弹倍率</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>笔迹宽度</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>切换冷却秒数</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>切换效果组</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>架势图标资源键</x:v>
+      </x:c>
+      <x:c r="K3" s="222" t="str">
+        <x:v>画笔样式</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
@@ -21196,7 +22028,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41f8d5a6bc043c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23c79ba441fb47eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21254,6 +22086,47 @@
       <x:c r="L2" s="13"/>
       <x:c r="M2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>笔势规则ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>笔势类型</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>最小采样间距</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>最大笔迹长度</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>简化容差</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>最大点数</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>最小有效长度</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>方向容差角</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>闭合距离</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>最小包围面积</x:v>
+      </x:c>
+      <x:c r="K3" s="221" t="str">
+        <x:v>最小弧线曲率</x:v>
+      </x:c>
+      <x:c r="L3" s="221" t="str">
+        <x:v>蓄力时长</x:v>
+      </x:c>
+      <x:c r="M3" s="222" t="str">
+        <x:v>命中半径</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>ruleId</x:v>
@@ -21594,7 +22467,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R825cf856ef7c4890"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc539224af5bb4bab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21644,6 +22517,41 @@
       <x:c r="I2" s="13"/>
       <x:c r="J2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>公式ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>基础伤害</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>暴击概率</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>暴击倍率</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>弱点倍率</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>错误方向倍率</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>连击步进倍率</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>连击倍率上限</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>每击能量</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>每击得分</x:v>
+      </x:c>
+      <x:c r="K3" s="222" t="str">
+        <x:v>每伤害得分</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>formulaId</x:v>
@@ -21791,7 +22699,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7ce3f330db4b7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R316d74ad46a54d82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21834,6 +22742,32 @@
       <x:c r="G2" s="13"/>
       <x:c r="H2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>防御规则ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>护甲生命值</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>要求笔势</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>破防要求架势</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>破甲伤害倍率</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>错误笔势倍率</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>反伤值</x:v>
+      </x:c>
+      <x:c r="H3" s="222" t="str">
+        <x:v>破甲效果组</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>defenseRuleId</x:v>
@@ -21970,7 +22904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10ab9fbff5894ffc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c7072a8b44d4059"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22016,6 +22950,35 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>弱点规则ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>窗口开始秒数</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>窗口结束秒数</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>弱点半径</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>弱点伤害倍率</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>是否打断攻击</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>额外能量</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>额外得分</x:v>
+      </x:c>
+      <x:c r="I3" s="222" t="str">
+        <x:v>特效键</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>weakpointRuleId</x:v>
@@ -22195,7 +23158,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b5be335053a4263"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44b08dcbe7f2417c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22247,6 +23210,41 @@
       <x:c r="J2" s="13"/>
       <x:c r="K2" s="13"/>
     </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="220" t="str">
+        <x:v>移动模式ID</x:v>
+      </x:c>
+      <x:c r="B3" s="221" t="str">
+        <x:v>移动类型</x:v>
+      </x:c>
+      <x:c r="C3" s="221" t="str">
+        <x:v>速度倍率</x:v>
+      </x:c>
+      <x:c r="D3" s="221" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="E3" s="221" t="str">
+        <x:v>频率</x:v>
+      </x:c>
+      <x:c r="F3" s="221" t="str">
+        <x:v>起点X比例</x:v>
+      </x:c>
+      <x:c r="G3" s="221" t="str">
+        <x:v>终点X比例</x:v>
+      </x:c>
+      <x:c r="H3" s="221" t="str">
+        <x:v>起点Y比例</x:v>
+      </x:c>
+      <x:c r="I3" s="221" t="str">
+        <x:v>终点Y比例</x:v>
+      </x:c>
+      <x:c r="J3" s="221" t="str">
+        <x:v>是否循环</x:v>
+      </x:c>
+      <x:c r="K3" s="222" t="str">
+        <x:v>移动说明</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
         <x:v>movePatternId</x:v>
@@ -22539,7 +23537,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1066ba924f70498c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ab7147f73f04cde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T699F: move charged stroke effect into particle prefab
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,37 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0d994e234f204509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rcf73312d6f0e418b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Ra3eb3ab098364194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R0e68ebf471ee477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R78557e40b6ec47d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rc35824a00083453c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R38efbc67439541a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R79bd1d68e904493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R939d2a5fecde4776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R6b5faf2752614513"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="R4706700d99c34793"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R1529f5df174c4efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R3dcc6767b9924b50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="Re226a78f2b8a42be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R2de9405744d449f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="Re00640125e734b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R5ace43e36af747f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Re49f80f4d7bc41c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R53727872fdd34dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="R640159f067324029"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rffed25b9c92e4070"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Ref872451606441ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Re5bd08291d1446bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R0763f32c23454f8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="R2b8418a9e04a4c30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R77f9faa9642c4605"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="R8fdddcfd8bce4e14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R03768efdc827409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Refb2912e273d4fb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="Re156a94b652a4091"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="Rb40b79303734445f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3c9b7c6cd74e4fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rd0ae8a87a9fe4220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rd3af204aeac64cb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R46f0965700114da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R7bd4847d1c2a45ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rdfe0914642ad4f77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Re3c45ae3cd404214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R2c22ff800c4e4af9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R136b69c9fb5246e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rce8e7e28ec974d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Reb9a077fa92b4b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rf1e99aceb2a649a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R39c61d02892d4b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R342df8f16ab04c76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Re834fef65ffb474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R8131efb5d9694db3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R4296fe5e856044e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R4023b22a25f14b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rb2ddb8ec9922445f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rc0765c2d78654edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rf6a6a9d184774356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rc6b0dce9beeb4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R3773c1c79c8f4f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rf51078e1a18b44db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rc34003afe0c94d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rf1efa655e64743a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rcd6458a39a404dab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R38b8668c4785411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rba888172d2e24fec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R6a847505c0574e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="Rf2dfb5f0218246b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1618,7 +1618,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.9-sample</x:v>
+        <x:v>0.6.10-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1789,7 +1789,7 @@
       </x:c>
       <x:c r="E18" s="89" t="n">
         <x:f>COUNTA('AssetManifest'!A5:A1000)</x:f>
-        <x:v>77</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="F18" s="92"/>
       <x:c r="G18" s="92"/>
@@ -2534,7 +2534,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0e863e1193c45c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e670471cad44548"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3128,7 +3128,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R403c48270ad34f95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12a2766f16dc4e35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3428,7 +3428,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e9f016cf8754eaf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6be53e8d75cb48f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3721,7 +3721,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re102328e7f1b41c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R913600137f174b74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3961,7 +3961,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf237a69225134119"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7166aeffe1384bb6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4878,7 +4878,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4985cb59e0a5474d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R469be6797f664805"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5124,7 +5124,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52c1664dfce74b07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc299c78962dc4304"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5707,7 +5707,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R630090a487f34419"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b08b210117841f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5942,7 +5942,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re20165884e944027"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4c99686cc6d41c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6094,7 +6094,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fe7f09b613944c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e42afe3bd3742ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6219,7 +6219,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.9-sample</x:v>
+        <x:v>0.6.10-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -7161,7 +7161,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R662b9679f79a43be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae51eb0e0dd04ce7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8292,7 +8292,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcdb1436b3be4e86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R689d669e40fc4536"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8526,7 +8526,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb669d6a17a7f431b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e589c1b09894d50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8765,7 +8765,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89b8f19f584d4364"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea59786a06bf4a4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9113,7 +9113,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0126e97ef9ee4757"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1062fd8db2b44afc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10047,7 +10047,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bf07fab66924d7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49b316d88e2545aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10596,7 +10596,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5af1f26f3ab441c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fea8c9c148c4501"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11586,7 +11586,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dbad347067c400b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re004a03f018646ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12963,6 +12963,23 @@
         <x:v>用户提供的十一帧怪物死亡爆炸动画</x:v>
       </x:c>
     </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>vfx_stroke_charge</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>Prefab</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>Assets/_Game/Art/VFX/vfx_stroke_charge.prefab</x:v>
+      </x:c>
+      <x:c r="D82" s="59" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>画笔停留蓄力的独立粒子特效Prefab；由StrokeTrailStyles选择。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -12975,7 +12992,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdccdda15938842be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64b016cefc9f4ccf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14413,7 +14430,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2006f9fb907c4803"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5756ca538ff946ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21054,6 +21071,30 @@
         <x:v>分支线段数：构成单条分支电弧的折线段数量。 配置约束：不得留空；有效范围2到8。</x:v>
       </x:c>
     </x:row>
+    <x:row r="285">
+      <x:c r="A285" t="str">
+        <x:v>StrokeTrailStyles</x:v>
+      </x:c>
+      <x:c r="B285" t="str">
+        <x:v>chargeVfxAssetKey</x:v>
+      </x:c>
+      <x:c r="C285" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D285" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E285"/>
+      <x:c r="F285"/>
+      <x:c r="G285"/>
+      <x:c r="H285"/>
+      <x:c r="I285" t="str">
+        <x:v>AssetManifest.assetKey</x:v>
+      </x:c>
+      <x:c r="J285" t="str">
+        <x:v>蓄力特效资源键：停留蓄力使用的独立粒子Prefab；换皮或新增样式只修改此引用。配置约束：不得留空；必须引用AssetManifest.assetKey的现有值，不存在时导出失败。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -21074,7 +21115,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00030b10506b4b76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9f244ca2fd84db1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21202,7 +21243,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87e0574349c345ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7eca228c9004755"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21706,6 +21747,7 @@
     <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="23" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="21" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="27" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -21727,7 +21769,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="177" t="str">
-        <x:v>画笔视觉样式。颜色、层宽与电弧参数全部来自配置；Prefab只保存分层组件引用。</x:v>
+        <x:v>画笔视觉样式。颜色、层宽、电弧参数与蓄力Prefab资源键全部来自配置；Prefab只保存组件和资源引用。</x:v>
       </x:c>
       <x:c r="B2" s="177"/>
       <x:c r="C2" s="177"/>
@@ -21782,6 +21824,9 @@
       <x:c r="M3" s="222" t="str">
         <x:v>分支线段数</x:v>
       </x:c>
+      <x:c r="N3" t="str">
+        <x:v>蓄力特效资源键</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="182" t="str">
@@ -21823,6 +21868,9 @@
       <x:c r="M4" s="182" t="str">
         <x:v>branchSegmentCount</x:v>
       </x:c>
+      <x:c r="N4" t="str">
+        <x:v>chargeVfxAssetKey</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="195" t="str">
@@ -21864,12 +21912,20 @@
       <x:c r="M5" s="197" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="N5" t="str">
+        <x:v>vfx_stroke_charge</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A2:M2"/>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="N5:N100">
+      <x:formula1>AssetManifest!$A$5:$A$200</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -22068,7 +22124,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89bb5db074244a07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fca08fd8cd34a2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22507,7 +22563,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R926c4ebfc90948d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde5c04832b7a42dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22739,7 +22795,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R923c885b5de64a63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcd2865d38e457d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22944,7 +23000,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2638fe3786914c54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6887f3ae89de4dba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23198,7 +23254,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R768d230d3de5454f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6987951557c496c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23577,7 +23633,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8887ea70e89e4742"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89695d6fa0fe489d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T699G: remove normal gesture shape gates
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,37 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3c9b7c6cd74e4fd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="Rd0ae8a87a9fe4220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Rd3af204aeac64cb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R46f0965700114da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R7bd4847d1c2a45ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Rdfe0914642ad4f77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Re3c45ae3cd404214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R2c22ff800c4e4af9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R136b69c9fb5246e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="Rce8e7e28ec974d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Reb9a077fa92b4b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Rf1e99aceb2a649a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R39c61d02892d4b6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R342df8f16ab04c76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Re834fef65ffb474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R8131efb5d9694db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R4296fe5e856044e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R4023b22a25f14b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="Rb2ddb8ec9922445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rc0765c2d78654edb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="Rf6a6a9d184774356"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Rc6b0dce9beeb4312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R3773c1c79c8f4f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="Rf51078e1a18b44db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rc34003afe0c94d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Rf1efa655e64743a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rcd6458a39a404dab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R38b8668c4785411d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rba888172d2e24fec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R6a847505c0574e85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="Rf2dfb5f0218246b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb808ba6218d64905"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R1fe077b669d44de9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Ra9b8a4a1604245b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R850888dfb0554124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R96a7c47cfb844aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Ra681538cb5c54ed2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rc584748d35074231"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Re09b89039a0e472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Rcb513993a447428a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R4c2d54153d0f4c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rc47e18f20d734b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R835bbdc727a54200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R117419a151b7484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R4fb39cc1102545c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R527e193ae0f54294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R2e6691cf4c5d4a5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R13079028b1744a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R12ec1c6a58644e24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R1453daeb78c74a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rd20849f06db14c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R569845c077ea4199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Ra4d20220dd814f0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R86ec583d466f449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R17556a55c4a24a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rfc02ed6d5b234eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Re3c73bb46aa24d3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Re98101307d694fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rbeb377880b25473b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rff83460f06b5469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="Raf654f200ff34f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="Rfc0366c87c8f4da8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1618,7 +1618,8 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>0.6.10-sample</x:v>
+        <x:f>'Global'!E6</x:f>
+        <x:v>0.6.11-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -2534,7 +2535,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e670471cad44548"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbbda562a9f0489d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2579,7 +2580,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>攻击集合由attackSetId分组，weight用于同一集合中的权重选择。</x:v>
+        <x:v>攻击集合由attackSetId分组；当前打断只要求在窗口内命中弱点，不要求指定笔势形状。</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -2754,7 +2755,7 @@
       </x:c>
       <x:c r="I6" s="35" t="str"/>
       <x:c r="J6" s="35" t="str">
-        <x:v>Horizontal</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="K6" s="72" t="n">
         <x:v>0.35</x:v>
@@ -2796,7 +2797,7 @@
       </x:c>
       <x:c r="I7" s="35" t="str"/>
       <x:c r="J7" s="35" t="str">
-        <x:v>Vertical</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="K7" s="72" t="n">
         <x:v>0.55</x:v>
@@ -2840,7 +2841,7 @@
         <x:v>proj_soul_shard</x:v>
       </x:c>
       <x:c r="J8" s="35" t="str">
-        <x:v>Arc</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="K8" s="72" t="n">
         <x:v>0.4</x:v>
@@ -2882,7 +2883,7 @@
       </x:c>
       <x:c r="I9" s="35" t="str"/>
       <x:c r="J9" s="35" t="str">
-        <x:v>Diagonal</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="K9" s="72" t="n">
         <x:v>0.2</x:v>
@@ -2924,7 +2925,7 @@
       </x:c>
       <x:c r="I10" s="35" t="str"/>
       <x:c r="J10" s="35" t="str">
-        <x:v>Circle</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="K10" s="72" t="n">
         <x:v>0.35</x:v>
@@ -3056,7 +3057,7 @@
         <x:v>proj_seal_wave</x:v>
       </x:c>
       <x:c r="J13" s="35" t="str">
-        <x:v>Horizontal</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="K13" s="72" t="n">
         <x:v>0.4</x:v>
@@ -3098,7 +3099,7 @@
       </x:c>
       <x:c r="I14" s="35" t="str"/>
       <x:c r="J14" s="35" t="str">
-        <x:v>Diagonal</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="K14" s="72" t="n">
         <x:v>0.55</x:v>
@@ -3128,7 +3129,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12a2766f16dc4e35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a991bebafbd4521"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3428,7 +3429,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6be53e8d75cb48f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f0eed6011234639"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3721,7 +3722,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R913600137f174b74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cbc5a6608b84b8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3898,7 +3899,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G6" s="35" t="str">
-        <x:v>Circle</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="H6" s="72" t="n">
         <x:v>1.8</x:v>
@@ -3961,7 +3962,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7166aeffe1384bb6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8aac50d0ca34a51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4878,7 +4879,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R469be6797f664805"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5c317f96c49442f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5124,7 +5125,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc299c78962dc4304"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc768420cfaad49d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5707,7 +5708,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b08b210117841f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc68a6b338b2c4adb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5942,7 +5943,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4c99686cc6d41c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc88ff251f1479c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6094,7 +6095,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e42afe3bd3742ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra552b3874b2e4684"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6219,7 +6220,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.10-sample</x:v>
+        <x:v>0.6.11-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -7161,7 +7162,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae51eb0e0dd04ce7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21dfc69dbb8a4f91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8292,7 +8293,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R689d669e40fc4536"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6505acb00af8434d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8526,7 +8527,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e589c1b09894d50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0572139783674e90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8765,7 +8766,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea59786a06bf4a4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f8237c9f8b491b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9113,7 +9114,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1062fd8db2b44afc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R995e4574131549aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9471,10 +9472,10 @@
         <x:v>text_skill_talisman_bind</x:v>
       </x:c>
       <x:c r="B26" s="35" t="str">
-        <x:v>缚妖圈</x:v>
+        <x:v>缚妖符</x:v>
       </x:c>
       <x:c r="C26" s="35" t="str">
-        <x:v>Demon Binding Circle</x:v>
+        <x:v>Demon Binding Talisman</x:v>
       </x:c>
       <x:c r="D26" s="35" t="str">
         <x:v>技能名</x:v>
@@ -9513,10 +9514,10 @@
         <x:v>text_skill_talisman_bind_desc</x:v>
       </x:c>
       <x:c r="B29" s="35" t="str">
-        <x:v>画出闭合符圈，定身圈内敌人</x:v>
+        <x:v>划过敌人，定身并造成符术伤害</x:v>
       </x:c>
       <x:c r="C29" s="35" t="str">
-        <x:v>Draw a closed circle to bind enemies</x:v>
+        <x:v>Swipe through enemies to bind and damage them</x:v>
       </x:c>
       <x:c r="D29" s="35" t="str">
         <x:v>技能说明</x:v>
@@ -9653,10 +9654,10 @@
         <x:v>text_boss_phase2</x:v>
       </x:c>
       <x:c r="B39" s="35" t="str">
-        <x:v>按方向斩开腹部封印</x:v>
+        <x:v>命中发光弱点，斩开腹部封印</x:v>
       </x:c>
       <x:c r="C39" s="35" t="str">
-        <x:v>Slash the seal in sequence</x:v>
+        <x:v>Hit the glowing weakpoint to break the abdominal seal</x:v>
       </x:c>
       <x:c r="D39" s="35" t="str">
         <x:v>Boss phase</x:v>
@@ -9667,10 +9668,10 @@
         <x:v>text_boss_phase3</x:v>
       </x:c>
       <x:c r="B40" s="35" t="str">
-        <x:v>斜斩打断冲撞，随后处决玄甲王</x:v>
+        <x:v>命中弱点打断冲撞，随后处决玄甲王</x:v>
       </x:c>
       <x:c r="C40" s="35" t="str">
-        <x:v>Interrupt the charge with a diagonal slash, then execute the Tomb King</x:v>
+        <x:v>Hit the weakpoint to interrupt the charge, then execute the Tomb King</x:v>
       </x:c>
       <x:c r="D40" s="35" t="str">
         <x:v>Boss phase</x:v>
@@ -10047,7 +10048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49b316d88e2545aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47f57bafd3f34e20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10596,7 +10597,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fea8c9c148c4501"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b07d5650ff44fbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11586,7 +11587,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re004a03f018646ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9b34398121c4bc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12992,7 +12993,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64b016cefc9f4ccf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6284ad8581754d2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14430,7 +14431,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5756ca538ff946ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radaf2c75e1194878"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21115,7 +21116,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9f244ca2fd84db1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6887a04982794d79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21243,7 +21244,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7eca228c9004755"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9071a235ec7e4f89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22124,7 +22125,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fca08fd8cd34a2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34749a95440b485f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22563,7 +22564,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde5c04832b7a42dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R346d634d4f2a4651"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22795,7 +22796,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcd2865d38e457d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb366903db6194ac8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22828,7 +22829,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>护甲、方向要求和破甲效果。空架势表示任意架势。</x:v>
+        <x:v>护甲、蓄力破防架势和破甲效果；普通战斗不要求方向或闭合形状。</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -22946,7 +22947,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C7" s="35" t="str">
-        <x:v>Horizontal</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str"/>
       <x:c r="E7" s="72" t="n">
@@ -22970,7 +22971,7 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="C8" s="35" t="str">
-        <x:v>Vertical</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="D8" s="35" t="str">
         <x:v>stance_blade</x:v>
@@ -23000,7 +23001,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6887f3ae89de4dba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35798f518e554d5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23254,7 +23255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6987951557c496c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a66fa13b07542a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23633,7 +23634,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89695d6fa0fe489d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aa277cd83d342f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T699H: add triangle slow gesture
</commit_message>
<xml_diff>
--- a/Design/Config/GameConfig.xlsx
+++ b/Design/Config/GameConfig.xlsx
@@ -2,37 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb808ba6218d64905"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R1fe077b669d44de9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="Ra9b8a4a1604245b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="R850888dfb0554124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="R96a7c47cfb844aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="Ra681538cb5c54ed2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="Rc584748d35074231"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="Re09b89039a0e472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="Rcb513993a447428a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R4c2d54153d0f4c5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rc47e18f20d734b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="R835bbdc727a54200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R117419a151b7484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R4fb39cc1102545c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="R527e193ae0f54294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R2e6691cf4c5d4a5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R13079028b1744a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="R12ec1c6a58644e24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R1453daeb78c74a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rd20849f06db14c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R569845c077ea4199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Ra4d20220dd814f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="R86ec583d466f449b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R17556a55c4a24a5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rfc02ed6d5b234eeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="Re3c73bb46aa24d3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Re98101307d694fd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="Rbeb377880b25473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Rff83460f06b5469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="Raf654f200ff34f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="Rfc0366c87c8f4da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd12fbc140e7f4713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global" sheetId="2" r:id="R6609af1a60a94fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="3" r:id="R979cf455e1254354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stances" sheetId="4" r:id="Ra9d077697e314e48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeRules" sheetId="5" r:id="Rd1a1771eb3034211"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DamageFormulas" sheetId="6" r:id="R239fe0117ee242b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefenseRules" sheetId="7" r:id="R4406718404834d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeakpointRules" sheetId="8" r:id="R35d1182d94d448ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MovePatterns" sheetId="9" r:id="R7dd6ad7237d24246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="10" r:id="R6a6c629ec7f246ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="11" r:id="Rd1aba417b9a5478b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projectiles" sheetId="12" r:id="Re64cce90eb9849d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buffs" sheetId="13" r:id="R37dc4877204c49c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="14" r:id="R63503ec4a20f4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillEffects" sheetId="15" r:id="Rf726f5b140be43bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="16" r:id="R2ffa66f9d9f04a4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waves" sheetId="17" r:id="R644360d30b904d74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPoints" sheetId="18" r:id="Rc097aefe6ada4ad0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyModifiers" sheetId="19" r:id="R8c0392dfa4064138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spawns" sheetId="20" r:id="Rbb2d979fe93c4a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="21" r:id="R7f11db2185f34300"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="22" r:id="Ra081941775ce4dc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="23" r:id="Rb3b449dc65eb482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texts" sheetId="24" r:id="R70c892e281cd4d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioCues" sheetId="25" r:id="Rf798175a02cf4740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VfxCues" sheetId="26" r:id="R77abb9f5f3cd4f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetManifest" sheetId="27" r:id="Rc13b03db0bb24bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="28" r:id="R47b3397cc03d45f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDictionary" sheetId="29" r:id="Raf1989d7f9654c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeedbackCues" sheetId="30" r:id="R3c15477bcd9c41df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrokeTrailStyles" sheetId="31" r:id="R5963fde67aa54c3c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,7 +116,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="35">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -268,8 +268,28 @@
         <x:fgColor rgb="FFEAF1F5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2D5B75"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB7DEED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="7">
     <x:border/>
     <x:border/>
     <x:border>
@@ -307,11 +327,25 @@
         <x:color rgb="FF9FBAD0"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="230">
+  <x:cellXfs count="243">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -883,6 +917,27 @@
     <x:xf numFmtId="0" fontId="5" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1603,7 +1658,7 @@
         <x:v>Schema版本</x:v>
       </x:c>
       <x:c r="B5" s="25" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Players</x:v>
@@ -1618,8 +1673,7 @@
         <x:v>内容版本</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:f>'Global'!E6</x:f>
-        <x:v>0.6.11-sample</x:v>
+        <x:v>0.7.0-sample</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Stances</x:v>
@@ -1686,7 +1740,7 @@
       </x:c>
       <x:c r="E11" s="107" t="n">
         <x:f>COUNTA('Skills'!A5:A1000)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F11" s="93"/>
       <x:c r="G11" s="93"/>
@@ -2535,7 +2589,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbbda562a9f0489d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40419accb68f4464"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3129,7 +3183,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a991bebafbd4521"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb60c1e94baf493e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3429,7 +3483,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f0eed6011234639"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4d85a5d61e84926"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3722,7 +3776,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cbc5a6608b84b8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4111b199883447e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3947,6 +4001,39 @@
         <x:v>text_skill_ultimate_desc</x:v>
       </x:c>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>skill_triangle_slow</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>text_buff_slow</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Gesture</x:v>
+      </x:c>
+      <x:c r="D8" t="str"/>
+      <x:c r="E8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Triangle</x:v>
+      </x:c>
+      <x:c r="H8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>fx_triangle_slow</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>icon_skill_talisman_bind</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>text_buff_slow</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -3962,7 +4049,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8aac50d0ca34a51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0bac2f0539f4a4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4872,6 +4959,37 @@
       <x:c r="J30"/>
       <x:c r="K30"/>
     </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>fx_triangle_slow</x:v>
+      </x:c>
+      <x:c r="B31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>ApplyBuff</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>AllEnemies</x:v>
+      </x:c>
+      <x:c r="E31" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G31" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>buff_slow_30</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>vfx_slow</x:v>
+      </x:c>
+      <x:c r="J31" t="str"/>
+      <x:c r="K31" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -4879,7 +4997,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5c317f96c49442f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12a872025f744c83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5125,7 +5243,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc768420cfaad49d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd79f1ff578da4f1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5708,7 +5826,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc68a6b338b2c4adb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab7ed4d8f60d47cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5943,7 +6061,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc88ff251f1479c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc20a209a74fe4e5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6095,7 +6213,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra552b3874b2e4684"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5be426cc274243d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6198,7 +6316,7 @@
         <x:v>int</x:v>
       </x:c>
       <x:c r="C5" s="68" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D5" s="35"/>
       <x:c r="E5" s="35"/>
@@ -6220,7 +6338,7 @@
       <x:c r="C6" s="68"/>
       <x:c r="D6" s="35"/>
       <x:c r="E6" s="35" t="str">
-        <x:v>0.6.11-sample</x:v>
+        <x:v>0.7.0-sample</x:v>
       </x:c>
       <x:c r="F6" s="35"/>
       <x:c r="G6" s="35" t="str">
@@ -7162,7 +7280,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21dfc69dbb8a4f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b5ee91467be4fa3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8293,7 +8411,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6505acb00af8434d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabd4de68175b4951"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8527,7 +8645,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0572139783674e90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570a98cc378c48ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8766,7 +8884,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f8237c9f8b491b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2b84dddf7a4339"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9114,7 +9232,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R995e4574131549aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra83d9f4db1294275"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10048,7 +10166,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47f57bafd3f34e20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc0d54415b464164"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10597,7 +10715,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b07d5650ff44fbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0d3c1a614341a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11587,7 +11705,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9b34398121c4bc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde53aac6aaff46b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12993,7 +13111,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6284ad8581754d2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re50e72169b974f1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13150,18 +13268,18 @@
         <x:v>要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A12" s="35" t="str">
-        <x:v>EnemyTier</x:v>
+        <x:v>GestureType</x:v>
       </x:c>
       <x:c r="B12" s="35" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Triangle</x:v>
       </x:c>
       <x:c r="C12" s="35" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Triangle</x:v>
       </x:c>
       <x:c r="D12" s="35" t="str">
-        <x:v>普通敌人层级；可被NormalEnemies目标筛选命中，不启用Boss阶段控制。</x:v>
+        <x:v>要求笔迹首尾近似闭合，并能由三个角点及三条直边拟合为三角形；闭合、面积、边偏差和角度阈值均读取StrokeRules。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -13169,13 +13287,13 @@
         <x:v>EnemyTier</x:v>
       </x:c>
       <x:c r="B13" s="35" t="str">
-        <x:v>Elite</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="C13" s="35" t="str">
-        <x:v>Elite</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="D13" s="35" t="str">
-        <x:v>精英敌人层级；仍属于非Boss目标并可被NormalEnemies筛选，但用于区分更高强度内容。</x:v>
+        <x:v>普通敌人层级；可被NormalEnemies目标筛选命中，不启用Boss阶段控制。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -13183,27 +13301,27 @@
         <x:v>EnemyTier</x:v>
       </x:c>
       <x:c r="B14" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Elite</x:v>
       </x:c>
       <x:c r="C14" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Elite</x:v>
       </x:c>
       <x:c r="D14" s="35" t="str">
-        <x:v>Boss层级；启用Boss身份校验、阶段配置和Boss专用目标/波次结束判断。</x:v>
+        <x:v>精英敌人层级；仍属于非Boss目标并可被NormalEnemies筛选，但用于区分更高强度内容。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="35" t="str">
-        <x:v>StanceVulnerability</x:v>
+        <x:v>EnemyTier</x:v>
       </x:c>
       <x:c r="B15" s="35" t="str">
-        <x:v>Any</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="C15" s="35" t="str">
-        <x:v>Any</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="D15" s="35" t="str">
-        <x:v>不声明特定架势弱点；当前运行时仅保存该分类，伤害仍由DamageFormulas和DefenseRules决定。</x:v>
+        <x:v>Boss层级；启用Boss身份校验、阶段配置和Boss专用目标/波次结束判断。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -13211,13 +13329,13 @@
         <x:v>StanceVulnerability</x:v>
       </x:c>
       <x:c r="B16" s="35" t="str">
-        <x:v>Blade</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="C16" s="35" t="str">
-        <x:v>Blade</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="D16" s="35" t="str">
-        <x:v>声明目标偏向受刀势克制；当前生产伤害链尚未读取此分类，单改该值不会改变伤害。</x:v>
+        <x:v>不声明特定架势弱点；当前运行时仅保存该分类，伤害仍由DamageFormulas和DefenseRules决定。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -13225,27 +13343,27 @@
         <x:v>StanceVulnerability</x:v>
       </x:c>
       <x:c r="B17" s="35" t="str">
-        <x:v>Talisman</x:v>
+        <x:v>Blade</x:v>
       </x:c>
       <x:c r="C17" s="35" t="str">
-        <x:v>Talisman</x:v>
+        <x:v>Blade</x:v>
       </x:c>
       <x:c r="D17" s="35" t="str">
-        <x:v>声明目标偏向受符势克制；当前生产伤害链尚未读取此分类，单改该值不会改变伤害。</x:v>
+        <x:v>声明目标偏向受刀势克制；当前生产伤害链尚未读取此分类，单改该值不会改变伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="35" t="str">
-        <x:v>MovePatternType</x:v>
+        <x:v>StanceVulnerability</x:v>
       </x:c>
       <x:c r="B18" s="35" t="str">
-        <x:v>Linear</x:v>
+        <x:v>Talisman</x:v>
       </x:c>
       <x:c r="C18" s="35" t="str">
-        <x:v>Linear</x:v>
+        <x:v>Talisman</x:v>
       </x:c>
       <x:c r="D18" s="35" t="str">
-        <x:v>按起点到终点的直线匀速插值移动，速度由敌人基础速度与speedMultiplier共同决定。</x:v>
+        <x:v>声明目标偏向受符势克制；当前生产伤害链尚未读取此分类，单改该值不会改变伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -13253,13 +13371,13 @@
         <x:v>MovePatternType</x:v>
       </x:c>
       <x:c r="B19" s="35" t="str">
-        <x:v>Sine</x:v>
+        <x:v>Linear</x:v>
       </x:c>
       <x:c r="C19" s="35" t="str">
-        <x:v>Sine</x:v>
+        <x:v>Linear</x:v>
       </x:c>
       <x:c r="D19" s="35" t="str">
-        <x:v>沿起点到终点推进，同时按amplitudeRefPx和frequency在垂直于主路径方向做正弦摆动。</x:v>
+        <x:v>按起点到终点的直线匀速插值移动，速度由敌人基础速度与speedMultiplier共同决定。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -13267,13 +13385,13 @@
         <x:v>MovePatternType</x:v>
       </x:c>
       <x:c r="B20" s="35" t="str">
-        <x:v>Dive</x:v>
+        <x:v>Sine</x:v>
       </x:c>
       <x:c r="C20" s="35" t="str">
-        <x:v>Dive</x:v>
+        <x:v>Sine</x:v>
       </x:c>
       <x:c r="D20" s="35" t="str">
-        <x:v>沿路径以前慢后快的下潜曲线推进，用于形成俯冲接近感。</x:v>
+        <x:v>沿起点到终点推进，同时按amplitudeRefPx和frequency在垂直于主路径方向做正弦摆动。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -13281,13 +13399,13 @@
         <x:v>MovePatternType</x:v>
       </x:c>
       <x:c r="B21" s="35" t="str">
-        <x:v>Hover</x:v>
+        <x:v>Dive</x:v>
       </x:c>
       <x:c r="C21" s="35" t="str">
-        <x:v>Hover</x:v>
+        <x:v>Dive</x:v>
       </x:c>
       <x:c r="D21" s="35" t="str">
-        <x:v>围绕配置起点按振幅和频率悬浮摆动，不持续推进到终点。</x:v>
+        <x:v>沿路径以前慢后快的下潜曲线推进，用于形成俯冲接近感。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -13295,27 +13413,27 @@
         <x:v>MovePatternType</x:v>
       </x:c>
       <x:c r="B22" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Hover</x:v>
       </x:c>
       <x:c r="C22" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Hover</x:v>
       </x:c>
       <x:c r="D22" s="35" t="str">
-        <x:v>按Boss专用往返曲线在配置区域移动，用于阶段战中的大体型目标。</x:v>
+        <x:v>围绕配置起点按振幅和频率悬浮摆动，不持续推进到终点。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="35" t="str">
-        <x:v>AttackTriggerType</x:v>
+        <x:v>MovePatternType</x:v>
       </x:c>
       <x:c r="B23" s="35" t="str">
-        <x:v>Cooldown</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="C23" s="35" t="str">
-        <x:v>Cooldown</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="D23" s="35" t="str">
-        <x:v>攻击冷却就绪时可参与选择；无距离、支援目标或生命阈值附加门槛。</x:v>
+        <x:v>按Boss专用往返曲线在配置区域移动，用于阶段战中的大体型目标。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -13323,13 +13441,13 @@
         <x:v>AttackTriggerType</x:v>
       </x:c>
       <x:c r="B24" s="35" t="str">
-        <x:v>Distance</x:v>
+        <x:v>Cooldown</x:v>
       </x:c>
       <x:c r="C24" s="35" t="str">
-        <x:v>Distance</x:v>
+        <x:v>Cooldown</x:v>
       </x:c>
       <x:c r="D24" s="35" t="str">
-        <x:v>目标进入攻击距离后可参与选择；无投射物时会生成冲撞类动作。</x:v>
+        <x:v>攻击冷却就绪时可参与选择；无距离、支援目标或生命阈值附加门槛。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -13337,13 +13455,13 @@
         <x:v>AttackTriggerType</x:v>
       </x:c>
       <x:c r="B25" s="35" t="str">
-        <x:v>Support</x:v>
+        <x:v>Distance</x:v>
       </x:c>
       <x:c r="C25" s="35" t="str">
-        <x:v>Support</x:v>
+        <x:v>Distance</x:v>
       </x:c>
       <x:c r="D25" s="35" t="str">
-        <x:v>存在合法友方支援目标时可参与选择；该类攻击不能配置直接伤害或投射物。</x:v>
+        <x:v>目标进入攻击距离后可参与选择；无投射物时会生成冲撞类动作。</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -13351,27 +13469,27 @@
         <x:v>AttackTriggerType</x:v>
       </x:c>
       <x:c r="B26" s="35" t="str">
-        <x:v>HpThreshold</x:v>
+        <x:v>Support</x:v>
       </x:c>
       <x:c r="C26" s="35" t="str">
-        <x:v>HpThreshold</x:v>
+        <x:v>Support</x:v>
       </x:c>
       <x:c r="D26" s="35" t="str">
-        <x:v>攻击者生命比例达到外部阶段阈值时可参与选择；无投射物时会生成冲撞类动作。</x:v>
+        <x:v>存在合法友方支援目标时可参与选择；该类攻击不能配置直接伤害或投射物。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="35" t="str">
-        <x:v>BuffType</x:v>
+        <x:v>AttackTriggerType</x:v>
       </x:c>
       <x:c r="B27" s="35" t="str">
-        <x:v>Slow</x:v>
+        <x:v>HpThreshold</x:v>
       </x:c>
       <x:c r="C27" s="35" t="str">
-        <x:v>Slow</x:v>
+        <x:v>HpThreshold</x:v>
       </x:c>
       <x:c r="D27" s="35" t="str">
-        <x:v>按1-magnitude×层数降低敌人移动倍率，最终倍率不会低于0。</x:v>
+        <x:v>攻击者生命比例达到外部阶段阈值时可参与选择；无投射物时会生成冲撞类动作。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
@@ -13379,13 +13497,13 @@
         <x:v>BuffType</x:v>
       </x:c>
       <x:c r="B28" s="35" t="str">
-        <x:v>Stun</x:v>
+        <x:v>Slow</x:v>
       </x:c>
       <x:c r="C28" s="35" t="str">
-        <x:v>Stun</x:v>
+        <x:v>Slow</x:v>
       </x:c>
       <x:c r="D28" s="35" t="str">
-        <x:v>使敌人进入限时眩晕状态并中断正常状态推进，到持续时间后恢复。</x:v>
+        <x:v>按1-magnitude×层数降低敌人移动倍率，最终倍率不会低于0。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -13393,13 +13511,13 @@
         <x:v>BuffType</x:v>
       </x:c>
       <x:c r="B29" s="35" t="str">
-        <x:v>DamageOverTime</x:v>
+        <x:v>Stun</x:v>
       </x:c>
       <x:c r="C29" s="35" t="str">
-        <x:v>DamageOverTime</x:v>
+        <x:v>Stun</x:v>
       </x:c>
       <x:c r="D29" s="35" t="str">
-        <x:v>周期伤害分类；当前运行时尚无按tickSec扣血的执行器，单独配置不会产生周期伤害。</x:v>
+        <x:v>使敌人进入限时眩晕状态并中断正常状态推进，到持续时间后恢复。</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
@@ -13407,13 +13525,13 @@
         <x:v>BuffType</x:v>
       </x:c>
       <x:c r="B30" s="35" t="str">
-        <x:v>Root</x:v>
+        <x:v>DamageOverTime</x:v>
       </x:c>
       <x:c r="C30" s="35" t="str">
-        <x:v>Root</x:v>
+        <x:v>DamageOverTime</x:v>
       </x:c>
       <x:c r="D30" s="35" t="str">
-        <x:v>定身分类；有效期间敌人保持IsRooted，生产移动适配器据此停止位置推进。</x:v>
+        <x:v>周期伤害分类；当前运行时尚无按tickSec扣血的执行器，单独配置不会产生周期伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -13421,27 +13539,27 @@
         <x:v>BuffType</x:v>
       </x:c>
       <x:c r="B31" s="35" t="str">
-        <x:v>DamageTaken</x:v>
+        <x:v>Root</x:v>
       </x:c>
       <x:c r="C31" s="35" t="str">
-        <x:v>DamageTaken</x:v>
+        <x:v>Root</x:v>
       </x:c>
       <x:c r="D31" s="35" t="str">
-        <x:v>按1+magnitude×层数提高目标受到的伤害倍率，可与其他伤害倍率相乘。</x:v>
+        <x:v>定身分类；有效期间敌人保持IsRooted，生产移动适配器据此停止位置推进。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="35" t="str">
-        <x:v>BuffRefreshPolicy</x:v>
+        <x:v>BuffType</x:v>
       </x:c>
       <x:c r="B32" s="35" t="str">
-        <x:v>Refresh</x:v>
+        <x:v>DamageTaken</x:v>
       </x:c>
       <x:c r="C32" s="35" t="str">
-        <x:v>Refresh</x:v>
+        <x:v>DamageTaken</x:v>
       </x:c>
       <x:c r="D32" s="35" t="str">
-        <x:v>重复施加同一Buff时保留当前层数，并从本次施加时刻重新计算到期时间。</x:v>
+        <x:v>按1+magnitude×层数提高目标受到的伤害倍率，可与其他伤害倍率相乘。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -13449,13 +13567,13 @@
         <x:v>BuffRefreshPolicy</x:v>
       </x:c>
       <x:c r="B33" s="35" t="str">
-        <x:v>Replace</x:v>
+        <x:v>Refresh</x:v>
       </x:c>
       <x:c r="C33" s="35" t="str">
-        <x:v>Replace</x:v>
+        <x:v>Refresh</x:v>
       </x:c>
       <x:c r="D33" s="35" t="str">
-        <x:v>重复施加同一Buff时替换旧实例、层数重置为1，并重新计算到期时间。</x:v>
+        <x:v>重复施加同一Buff时保留当前层数，并从本次施加时刻重新计算到期时间。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
@@ -13463,27 +13581,27 @@
         <x:v>BuffRefreshPolicy</x:v>
       </x:c>
       <x:c r="B34" s="35" t="str">
-        <x:v>AddStack</x:v>
+        <x:v>Replace</x:v>
       </x:c>
       <x:c r="C34" s="35" t="str">
-        <x:v>AddStack</x:v>
+        <x:v>Replace</x:v>
       </x:c>
       <x:c r="D34" s="35" t="str">
-        <x:v>重复施加同一Buff时增加1层但不超过maxStacks，同时重新计算到期时间。</x:v>
+        <x:v>重复施加同一Buff时替换旧实例、层数重置为1，并重新计算到期时间。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="35" t="str">
-        <x:v>SkillTriggerType</x:v>
+        <x:v>BuffRefreshPolicy</x:v>
       </x:c>
       <x:c r="B35" s="35" t="str">
-        <x:v>Passive</x:v>
+        <x:v>AddStack</x:v>
       </x:c>
       <x:c r="C35" s="35" t="str">
-        <x:v>Passive</x:v>
+        <x:v>AddStack</x:v>
       </x:c>
       <x:c r="D35" s="35" t="str">
-        <x:v>由系统事件或代码入口主动请求的被动技能；不要求笔势匹配，但仍经过架势、能量和冷却校验。</x:v>
+        <x:v>重复施加同一Buff时增加1层但不超过maxStacks，同时重新计算到期时间。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -13491,13 +13609,13 @@
         <x:v>SkillTriggerType</x:v>
       </x:c>
       <x:c r="B36" s="35" t="str">
-        <x:v>Gesture</x:v>
+        <x:v>Passive</x:v>
       </x:c>
       <x:c r="C36" s="35" t="str">
-        <x:v>Gesture</x:v>
+        <x:v>Passive</x:v>
       </x:c>
       <x:c r="D36" s="35" t="str">
-        <x:v>由普通笔势输入触发；必须在inputWindowSec内匹配gestureType后才可执行。</x:v>
+        <x:v>由系统事件或代码入口主动请求的被动技能；不要求笔势匹配，但仍经过架势、能量和冷却校验。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -13505,27 +13623,27 @@
         <x:v>SkillTriggerType</x:v>
       </x:c>
       <x:c r="B37" s="35" t="str">
-        <x:v>Ultimate</x:v>
+        <x:v>Gesture</x:v>
       </x:c>
       <x:c r="C37" s="35" t="str">
-        <x:v>Ultimate</x:v>
+        <x:v>Gesture</x:v>
       </x:c>
       <x:c r="D37" s="35" t="str">
-        <x:v>由终极技能入口触发；仍要求配置笔势，并同时校验能量、架势、输入窗和冷却。</x:v>
+        <x:v>由普通笔势输入触发；必须在inputWindowSec内匹配gestureType后才可执行。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="35" t="str">
-        <x:v>WaveStartTrigger</x:v>
+        <x:v>SkillTriggerType</x:v>
       </x:c>
       <x:c r="B38" s="35" t="str">
-        <x:v>LevelStart</x:v>
+        <x:v>Ultimate</x:v>
       </x:c>
       <x:c r="C38" s="35" t="str">
-        <x:v>LevelStart</x:v>
+        <x:v>Ultimate</x:v>
       </x:c>
       <x:c r="D38" s="35" t="str">
-        <x:v>以关卡开始时刻为计时零点，等待startDelaySec后启动；只允许第一波使用。</x:v>
+        <x:v>由终极技能入口触发；仍要求配置笔势，并同时校验能量、架势、输入窗和冷却。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
@@ -13533,13 +13651,13 @@
         <x:v>WaveStartTrigger</x:v>
       </x:c>
       <x:c r="B39" s="35" t="str">
-        <x:v>PreviousWaveEnd</x:v>
+        <x:v>LevelStart</x:v>
       </x:c>
       <x:c r="C39" s="35" t="str">
-        <x:v>PreviousWaveEnd</x:v>
+        <x:v>LevelStart</x:v>
       </x:c>
       <x:c r="D39" s="35" t="str">
-        <x:v>以上一波完成时刻为计时起点，等待startDelaySec后启动；第一波不可使用。</x:v>
+        <x:v>以关卡开始时刻为计时零点，等待startDelaySec后启动；只允许第一波使用。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
@@ -13547,13 +13665,13 @@
         <x:v>WaveStartTrigger</x:v>
       </x:c>
       <x:c r="B40" s="35" t="str">
-        <x:v>PlayerConfirmed</x:v>
+        <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="C40" s="35" t="str">
-        <x:v>PlayerConfirmed</x:v>
+        <x:v>PreviousWaveEnd</x:v>
       </x:c>
       <x:c r="D40" s="35" t="str">
-        <x:v>保持等待，收到玩家确认操作后再等待startDelaySec启动。</x:v>
+        <x:v>以上一波完成时刻为计时起点，等待startDelaySec后启动；第一波不可使用。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -13561,27 +13679,27 @@
         <x:v>WaveStartTrigger</x:v>
       </x:c>
       <x:c r="B41" s="35" t="str">
-        <x:v>TimeElapsed</x:v>
+        <x:v>PlayerConfirmed</x:v>
       </x:c>
       <x:c r="C41" s="35" t="str">
-        <x:v>TimeElapsed</x:v>
+        <x:v>PlayerConfirmed</x:v>
       </x:c>
       <x:c r="D41" s="35" t="str">
-        <x:v>以关卡开始时刻为计时零点，在累计时间达到startDelaySec后启动；若本波较晚才激活且时间已过则立即启动。</x:v>
+        <x:v>保持等待，收到玩家确认操作后再等待startDelaySec启动。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="35" t="str">
-        <x:v>WaveEndCondition</x:v>
+        <x:v>WaveStartTrigger</x:v>
       </x:c>
       <x:c r="B42" s="35" t="str">
-        <x:v>AllEnemiesDefeated</x:v>
+        <x:v>TimeElapsed</x:v>
       </x:c>
       <x:c r="C42" s="35" t="str">
-        <x:v>AllEnemiesDefeated</x:v>
+        <x:v>TimeElapsed</x:v>
       </x:c>
       <x:c r="D42" s="35" t="str">
-        <x:v>本波全部出生计划已发出且活动敌人数归零时满足结束条件。</x:v>
+        <x:v>以关卡开始时刻为计时零点，在累计时间达到startDelaySec后启动；若本波较晚才激活且时间已过则立即启动。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
@@ -13589,13 +13707,13 @@
         <x:v>WaveEndCondition</x:v>
       </x:c>
       <x:c r="B43" s="35" t="str">
-        <x:v>BossDefeated</x:v>
+        <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="C43" s="35" t="str">
-        <x:v>BossDefeated</x:v>
+        <x:v>AllEnemiesDefeated</x:v>
       </x:c>
       <x:c r="D43" s="35" t="str">
-        <x:v>关卡配置的Boss实体被击败时满足结束条件；该波必须实际生成该Boss。</x:v>
+        <x:v>本波全部出生计划已发出且活动敌人数归零时满足结束条件。</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
@@ -13603,13 +13721,13 @@
         <x:v>WaveEndCondition</x:v>
       </x:c>
       <x:c r="B44" s="35" t="str">
-        <x:v>TimeElapsed</x:v>
+        <x:v>BossDefeated</x:v>
       </x:c>
       <x:c r="C44" s="35" t="str">
-        <x:v>TimeElapsed</x:v>
+        <x:v>BossDefeated</x:v>
       </x:c>
       <x:c r="D44" s="35" t="str">
-        <x:v>本波运行时间达到endDelaySec时直接完成；此取值下endDelaySec是持续时长而非额外结束等待。</x:v>
+        <x:v>关卡配置的Boss实体被击败时满足结束条件；该波必须实际生成该Boss。</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
@@ -13617,27 +13735,27 @@
         <x:v>WaveEndCondition</x:v>
       </x:c>
       <x:c r="B45" s="35" t="str">
-        <x:v>PlayerConfirmed</x:v>
+        <x:v>TimeElapsed</x:v>
       </x:c>
       <x:c r="C45" s="35" t="str">
-        <x:v>PlayerConfirmed</x:v>
+        <x:v>TimeElapsed</x:v>
       </x:c>
       <x:c r="D45" s="35" t="str">
-        <x:v>本波运行期间收到玩家确认操作时满足条件，再等待endDelaySec后完成。</x:v>
+        <x:v>本波运行时间达到endDelaySec时直接完成；此取值下endDelaySec是持续时长而非额外结束等待。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="35" t="str">
-        <x:v>SpawnPattern</x:v>
+        <x:v>WaveEndCondition</x:v>
       </x:c>
       <x:c r="B46" s="35" t="str">
-        <x:v>Single</x:v>
+        <x:v>PlayerConfirmed</x:v>
       </x:c>
       <x:c r="C46" s="35" t="str">
-        <x:v>Single</x:v>
+        <x:v>PlayerConfirmed</x:v>
       </x:c>
       <x:c r="D46" s="35" t="str">
-        <x:v>同一出生条目的所有实例使用出生点中心，不应用jitterX或jitterY偏移。</x:v>
+        <x:v>本波运行期间收到玩家确认操作时满足条件，再等待endDelaySec后完成。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
@@ -13645,13 +13763,13 @@
         <x:v>SpawnPattern</x:v>
       </x:c>
       <x:c r="B47" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Single</x:v>
       </x:c>
       <x:c r="C47" s="35" t="str">
-        <x:v>Line</x:v>
+        <x:v>Single</x:v>
       </x:c>
       <x:c r="D47" s="35" t="str">
-        <x:v>在出生点的-jitterY到+jitterY范围内按实例顺序排成竖线，X保持中心值。</x:v>
+        <x:v>同一出生条目的所有实例使用出生点中心，不应用jitterX或jitterY偏移。</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
@@ -13659,13 +13777,13 @@
         <x:v>SpawnPattern</x:v>
       </x:c>
       <x:c r="B48" s="35" t="str">
-        <x:v>Scatter</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="C48" s="35" t="str">
-        <x:v>Scatter</x:v>
+        <x:v>Line</x:v>
       </x:c>
       <x:c r="D48" s="35" t="str">
-        <x:v>在±jitterX和±jitterY矩形内按spawnId与实例序号确定性散布，重开结果一致。</x:v>
+        <x:v>在出生点的-jitterY到+jitterY范围内按实例顺序排成竖线，X保持中心值。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
@@ -13673,27 +13791,27 @@
         <x:v>SpawnPattern</x:v>
       </x:c>
       <x:c r="B49" s="35" t="str">
-        <x:v>Stagger</x:v>
+        <x:v>Scatter</x:v>
       </x:c>
       <x:c r="C49" s="35" t="str">
-        <x:v>Stagger</x:v>
+        <x:v>Scatter</x:v>
       </x:c>
       <x:c r="D49" s="35" t="str">
-        <x:v>实例在左右、上下两个偏移端点之间交替出生，形成错位节奏。</x:v>
+        <x:v>在±jitterX和±jitterY矩形内按spawnId与实例序号确定性散布，重开结果一致。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="35" t="str">
-        <x:v>RewardCondition</x:v>
+        <x:v>SpawnPattern</x:v>
       </x:c>
       <x:c r="B50" s="35" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Stagger</x:v>
       </x:c>
       <x:c r="C50" s="35" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Stagger</x:v>
       </x:c>
       <x:c r="D50" s="35" t="str">
-        <x:v>关卡完成即满足；conditionValue必须填1，不额外要求星级或分数。</x:v>
+        <x:v>实例在左右、上下两个偏移端点之间交替出生，形成错位节奏。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
@@ -13701,13 +13819,13 @@
         <x:v>RewardCondition</x:v>
       </x:c>
       <x:c r="B51" s="35" t="str">
-        <x:v>StarAtLeast</x:v>
+        <x:v>Clear</x:v>
       </x:c>
       <x:c r="C51" s="35" t="str">
-        <x:v>StarAtLeast</x:v>
+        <x:v>Clear</x:v>
       </x:c>
       <x:c r="D51" s="35" t="str">
-        <x:v>结算星级达到conditionValue时满足；conditionValue只能为1、2或3。</x:v>
+        <x:v>关卡完成即满足；conditionValue必须填1，不额外要求星级或分数。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
@@ -13715,27 +13833,27 @@
         <x:v>RewardCondition</x:v>
       </x:c>
       <x:c r="B52" s="35" t="str">
-        <x:v>ScoreAtLeast</x:v>
+        <x:v>StarAtLeast</x:v>
       </x:c>
       <x:c r="C52" s="35" t="str">
-        <x:v>ScoreAtLeast</x:v>
+        <x:v>StarAtLeast</x:v>
       </x:c>
       <x:c r="D52" s="35" t="str">
-        <x:v>最终结算分数不低于conditionValue时满足；阈值必须为非负整数。</x:v>
+        <x:v>结算星级达到conditionValue时满足；conditionValue只能为1、2或3。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="35" t="str">
-        <x:v>RewardType</x:v>
+        <x:v>RewardCondition</x:v>
       </x:c>
       <x:c r="B53" s="35" t="str">
-        <x:v>UnlockLevel</x:v>
+        <x:v>ScoreAtLeast</x:v>
       </x:c>
       <x:c r="C53" s="35" t="str">
-        <x:v>UnlockLevel</x:v>
+        <x:v>ScoreAtLeast</x:v>
       </x:c>
       <x:c r="D53" s="35" t="str">
-        <x:v>解锁rewardId指定的Levels.levelId；amount必须为1。</x:v>
+        <x:v>最终结算分数不低于conditionValue时满足；阈值必须为非负整数。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
@@ -13743,13 +13861,13 @@
         <x:v>RewardType</x:v>
       </x:c>
       <x:c r="B54" s="35" t="str">
-        <x:v>UnlockFeature</x:v>
+        <x:v>UnlockLevel</x:v>
       </x:c>
       <x:c r="C54" s="35" t="str">
-        <x:v>UnlockFeature</x:v>
+        <x:v>UnlockLevel</x:v>
       </x:c>
       <x:c r="D54" s="35" t="str">
-        <x:v>解锁rewardId指定的feature_命名空间功能标记；amount必须为1。</x:v>
+        <x:v>解锁rewardId指定的Levels.levelId；amount必须为1。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
@@ -13757,27 +13875,27 @@
         <x:v>RewardType</x:v>
       </x:c>
       <x:c r="B55" s="35" t="str">
-        <x:v>ScoreToken</x:v>
+        <x:v>UnlockFeature</x:v>
       </x:c>
       <x:c r="C55" s="35" t="str">
-        <x:v>ScoreToken</x:v>
+        <x:v>UnlockFeature</x:v>
       </x:c>
       <x:c r="D55" s="35" t="str">
-        <x:v>向rewardId指定的token_命名空间计数累加amount，可用于局外累计资源。</x:v>
+        <x:v>解锁rewardId指定的feature_命名空间功能标记；amount必须为1。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="35" t="str">
-        <x:v>AssetType</x:v>
+        <x:v>RewardType</x:v>
       </x:c>
       <x:c r="B56" s="35" t="str">
-        <x:v>Sprite</x:v>
+        <x:v>ScoreToken</x:v>
       </x:c>
       <x:c r="C56" s="35" t="str">
-        <x:v>Sprite</x:v>
+        <x:v>ScoreToken</x:v>
       </x:c>
       <x:c r="D56" s="35" t="str">
-        <x:v>要求AssetRegistry中的对应对象为Sprite，用于静态图片、图标或精灵表现。</x:v>
+        <x:v>向rewardId指定的token_命名空间计数累加amount，可用于局外累计资源。</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
@@ -13785,13 +13903,13 @@
         <x:v>AssetType</x:v>
       </x:c>
       <x:c r="B57" s="35" t="str">
-        <x:v>Prefab</x:v>
+        <x:v>Sprite</x:v>
       </x:c>
       <x:c r="C57" s="35" t="str">
-        <x:v>Prefab</x:v>
+        <x:v>Sprite</x:v>
       </x:c>
       <x:c r="D57" s="35" t="str">
-        <x:v>要求AssetRegistry中的对应对象为Prefab，用于实例化角色、特效或其他GameObject。</x:v>
+        <x:v>要求AssetRegistry中的对应对象为Sprite，用于静态图片、图标或精灵表现。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
@@ -13799,13 +13917,13 @@
         <x:v>AssetType</x:v>
       </x:c>
       <x:c r="B58" s="35" t="str">
-        <x:v>AudioClip</x:v>
+        <x:v>Prefab</x:v>
       </x:c>
       <x:c r="C58" s="35" t="str">
-        <x:v>AudioClip</x:v>
+        <x:v>Prefab</x:v>
       </x:c>
       <x:c r="D58" s="35" t="str">
-        <x:v>要求AssetRegistry中的对应对象为AudioClip，供AudioCues播放。</x:v>
+        <x:v>要求AssetRegistry中的对应对象为Prefab，用于实例化角色、特效或其他GameObject。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
@@ -13813,13 +13931,13 @@
         <x:v>AssetType</x:v>
       </x:c>
       <x:c r="B59" s="35" t="str">
-        <x:v>Scene</x:v>
+        <x:v>AudioClip</x:v>
       </x:c>
       <x:c r="C59" s="35" t="str">
-        <x:v>Scene</x:v>
+        <x:v>AudioClip</x:v>
       </x:c>
       <x:c r="D59" s="35" t="str">
-        <x:v>要求AssetRegistry中的对应对象为SceneAsset，并在构建场景清单中可用。</x:v>
+        <x:v>要求AssetRegistry中的对应对象为AudioClip，供AudioCues播放。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
@@ -13827,13 +13945,13 @@
         <x:v>AssetType</x:v>
       </x:c>
       <x:c r="B60" s="35" t="str">
-        <x:v>Material</x:v>
+        <x:v>Scene</x:v>
       </x:c>
       <x:c r="C60" s="35" t="str">
-        <x:v>Material</x:v>
+        <x:v>Scene</x:v>
       </x:c>
       <x:c r="D60" s="35" t="str">
-        <x:v>要求AssetRegistry中的对应对象为Material，供渲染资源引用。</x:v>
+        <x:v>要求AssetRegistry中的对应对象为SceneAsset，并在构建场景清单中可用。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
@@ -13841,13 +13959,13 @@
         <x:v>AssetType</x:v>
       </x:c>
       <x:c r="B61" s="35" t="str">
-        <x:v>Font</x:v>
+        <x:v>Material</x:v>
       </x:c>
       <x:c r="C61" s="35" t="str">
-        <x:v>Font</x:v>
+        <x:v>Material</x:v>
       </x:c>
       <x:c r="D61" s="35" t="str">
-        <x:v>要求AssetRegistry中的对应对象为字体资源，供本地化UI使用。</x:v>
+        <x:v>要求AssetRegistry中的对应对象为Material，供渲染资源引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
@@ -13855,27 +13973,27 @@
         <x:v>AssetType</x:v>
       </x:c>
       <x:c r="B62" s="35" t="str">
-        <x:v>AnimationClip</x:v>
+        <x:v>Font</x:v>
       </x:c>
       <x:c r="C62" s="35" t="str">
-        <x:v>AnimationClip</x:v>
+        <x:v>Font</x:v>
       </x:c>
       <x:c r="D62" s="35" t="str">
-        <x:v>要求AssetRegistry中的对应对象为AnimationClip，供动画状态或表现流程使用。</x:v>
+        <x:v>要求AssetRegistry中的对应对象为字体资源，供本地化UI使用。</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="35" t="str">
-        <x:v>AudioCategory</x:v>
+        <x:v>AssetType</x:v>
       </x:c>
       <x:c r="B63" s="35" t="str">
-        <x:v>BGM</x:v>
+        <x:v>AnimationClip</x:v>
       </x:c>
       <x:c r="C63" s="35" t="str">
-        <x:v>BGM</x:v>
+        <x:v>AnimationClip</x:v>
       </x:c>
       <x:c r="D63" s="35" t="str">
-        <x:v>背景音乐通道；用于关卡或波次持续音乐，可由音乐切换逻辑替换。</x:v>
+        <x:v>要求AssetRegistry中的对应对象为AnimationClip，供动画状态或表现流程使用。</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
@@ -13883,13 +14001,13 @@
         <x:v>AudioCategory</x:v>
       </x:c>
       <x:c r="B64" s="35" t="str">
-        <x:v>SFX</x:v>
+        <x:v>BGM</x:v>
       </x:c>
       <x:c r="C64" s="35" t="str">
-        <x:v>SFX</x:v>
+        <x:v>BGM</x:v>
       </x:c>
       <x:c r="D64" s="35" t="str">
-        <x:v>战斗与环境音效通道；受同事件并发数和冷却限制。</x:v>
+        <x:v>背景音乐通道；用于关卡或波次持续音乐，可由音乐切换逻辑替换。</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
@@ -13897,27 +14015,27 @@
         <x:v>AudioCategory</x:v>
       </x:c>
       <x:c r="B65" s="35" t="str">
-        <x:v>UI</x:v>
+        <x:v>SFX</x:v>
       </x:c>
       <x:c r="C65" s="35" t="str">
-        <x:v>UI</x:v>
+        <x:v>SFX</x:v>
       </x:c>
       <x:c r="D65" s="35" t="str">
-        <x:v>界面交互音效通道；用于按钮、提示和结算等UI反馈。</x:v>
+        <x:v>战斗与环境音效通道；受同事件并发数和冷却限制。</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="35" t="str">
-        <x:v>EffectType</x:v>
+        <x:v>AudioCategory</x:v>
       </x:c>
       <x:c r="B66" s="35" t="str">
-        <x:v>Damage</x:v>
+        <x:v>UI</x:v>
       </x:c>
       <x:c r="C66" s="35" t="str">
-        <x:v>Damage</x:v>
+        <x:v>UI</x:v>
       </x:c>
       <x:c r="D66" s="35" t="str">
-        <x:v>对选中目标造成value1点直接伤害。</x:v>
+        <x:v>界面交互音效通道；用于按钮、提示和结算等UI反馈。</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
@@ -13925,13 +14043,13 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B67" s="35" t="str">
-        <x:v>ApplyBuff</x:v>
+        <x:v>Damage</x:v>
       </x:c>
       <x:c r="C67" s="35" t="str">
-        <x:v>ApplyBuff</x:v>
+        <x:v>Damage</x:v>
       </x:c>
       <x:c r="D67" s="35" t="str">
-        <x:v>向选中目标施加buffId；durationSec大于0时覆盖Buffs.durationSec。</x:v>
+        <x:v>对选中目标造成value1点直接伤害。</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
@@ -13939,13 +14057,13 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B68" s="35" t="str">
-        <x:v>RemoveArmor</x:v>
+        <x:v>ApplyBuff</x:v>
       </x:c>
       <x:c r="C68" s="35" t="str">
-        <x:v>RemoveArmor</x:v>
+        <x:v>ApplyBuff</x:v>
       </x:c>
       <x:c r="D68" s="35" t="str">
-        <x:v>移除选中目标value1点护甲，不直接扣除生命。</x:v>
+        <x:v>向选中目标施加buffId；durationSec大于0时覆盖Buffs.durationSec。</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
@@ -13953,13 +14071,13 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B69" s="35" t="str">
-        <x:v>Knockback</x:v>
+        <x:v>RemoveArmor</x:v>
       </x:c>
       <x:c r="C69" s="35" t="str">
-        <x:v>Knockback</x:v>
+        <x:v>RemoveArmor</x:v>
       </x:c>
       <x:c r="D69" s="35" t="str">
-        <x:v>使选中目标在durationSec内产生value1参考像素的击退意图。</x:v>
+        <x:v>移除选中目标value1点护甲，不直接扣除生命。</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
@@ -13967,13 +14085,13 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B70" s="35" t="str">
-        <x:v>RepeatStroke</x:v>
+        <x:v>Knockback</x:v>
       </x:c>
       <x:c r="C70" s="35" t="str">
-        <x:v>RepeatStroke</x:v>
+        <x:v>Knockback</x:v>
       </x:c>
       <x:c r="D70" s="35" t="str">
-        <x:v>以value1伤害倍率在value2秒后重复上一笔命中结果。</x:v>
+        <x:v>使选中目标在durationSec内产生value1参考像素的击退意图。</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
@@ -13981,13 +14099,13 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B71" s="35" t="str">
-        <x:v>TimeScale</x:v>
+        <x:v>RepeatStroke</x:v>
       </x:c>
       <x:c r="C71" s="35" t="str">
-        <x:v>TimeScale</x:v>
+        <x:v>RepeatStroke</x:v>
       </x:c>
       <x:c r="D71" s="35" t="str">
-        <x:v>把战斗时间倍率设为value1并保持durationSec；value1范围为(0,1]。</x:v>
+        <x:v>以value1伤害倍率在value2秒后重复上一笔命中结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
@@ -13995,13 +14113,13 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B72" s="35" t="str">
-        <x:v>ExecuteBelowHpRatio</x:v>
+        <x:v>TimeScale</x:v>
       </x:c>
       <x:c r="C72" s="35" t="str">
-        <x:v>ExecuteBelowHpRatio</x:v>
+        <x:v>TimeScale</x:v>
       </x:c>
       <x:c r="D72" s="35" t="str">
-        <x:v>当目标当前生命比例不高于value1时执行处决；value1范围为0到1。</x:v>
+        <x:v>把战斗时间倍率设为value1并保持durationSec；value1范围为(0,1]。</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
@@ -14009,13 +14127,13 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B73" s="35" t="str">
-        <x:v>DamageMultiplier</x:v>
+        <x:v>ExecuteBelowHpRatio</x:v>
       </x:c>
       <x:c r="C73" s="35" t="str">
-        <x:v>DamageMultiplier</x:v>
+        <x:v>ExecuteBelowHpRatio</x:v>
       </x:c>
       <x:c r="D73" s="35" t="str">
-        <x:v>把下一笔画的伤害倍率设为value1，value1必须大于0。</x:v>
+        <x:v>当目标当前生命比例不高于value1时执行处决；value1范围为0到1。</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
@@ -14023,27 +14141,27 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B74" s="35" t="str">
-        <x:v>IncrementCounter</x:v>
+        <x:v>DamageMultiplier</x:v>
       </x:c>
       <x:c r="C74" s="35" t="str">
-        <x:v>IncrementCounter</x:v>
+        <x:v>DamageMultiplier</x:v>
       </x:c>
       <x:c r="D74" s="35" t="str">
-        <x:v>给目标计数器增加value1，并以value2作为上限或触发阈值。</x:v>
+        <x:v>把下一笔画的伤害倍率设为value1，value1必须大于0。</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
       <x:c r="A75" s="35" t="str">
-        <x:v>TargetType</x:v>
+        <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B75" s="35" t="str">
-        <x:v>Target</x:v>
+        <x:v>IncrementCounter</x:v>
       </x:c>
       <x:c r="C75" s="35" t="str">
-        <x:v>Target</x:v>
+        <x:v>IncrementCounter</x:v>
       </x:c>
       <x:c r="D75" s="35" t="str">
-        <x:v>选择本次技能上下文中的主目标；无存活主目标时目标列表为空。</x:v>
+        <x:v>给目标计数器增加value1，并以value2作为上限或触发阈值。</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
@@ -14051,13 +14169,13 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B76" s="35" t="str">
-        <x:v>NextStroke</x:v>
+        <x:v>Target</x:v>
       </x:c>
       <x:c r="C76" s="35" t="str">
-        <x:v>NextStroke</x:v>
+        <x:v>Target</x:v>
       </x:c>
       <x:c r="D76" s="35" t="str">
-        <x:v>不选择当前实体，效果写入世界状态并作用于下一笔画。</x:v>
+        <x:v>选择本次技能上下文中的主目标；无存活主目标时目标列表为空。</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
@@ -14065,13 +14183,13 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B77" s="35" t="str">
-        <x:v>EnemiesInRadius</x:v>
+        <x:v>NextStroke</x:v>
       </x:c>
       <x:c r="C77" s="35" t="str">
-        <x:v>EnemiesInRadius</x:v>
+        <x:v>NextStroke</x:v>
       </x:c>
       <x:c r="D77" s="35" t="str">
-        <x:v>选择被运行时标记为处于效果半径内的全部存活敌人。</x:v>
+        <x:v>不选择当前实体，效果写入世界状态并作用于下一笔画。</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
@@ -14079,13 +14197,13 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B78" s="35" t="str">
-        <x:v>LastStrokeTargets</x:v>
+        <x:v>EnemiesInRadius</x:v>
       </x:c>
       <x:c r="C78" s="35" t="str">
-        <x:v>LastStrokeTargets</x:v>
+        <x:v>EnemiesInRadius</x:v>
       </x:c>
       <x:c r="D78" s="35" t="str">
-        <x:v>选择上一笔画实际命中的全部存活敌人。</x:v>
+        <x:v>选择被运行时标记为处于效果半径内的全部存活敌人。</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
@@ -14093,13 +14211,13 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B79" s="35" t="str">
-        <x:v>EnemiesInsideGesture</x:v>
+        <x:v>LastStrokeTargets</x:v>
       </x:c>
       <x:c r="C79" s="35" t="str">
-        <x:v>EnemiesInsideGesture</x:v>
+        <x:v>LastStrokeTargets</x:v>
       </x:c>
       <x:c r="D79" s="35" t="str">
-        <x:v>选择位于当前闭合笔势区域内的全部存活敌人。</x:v>
+        <x:v>选择上一笔画实际命中的全部存活敌人。</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
@@ -14107,13 +14225,13 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B80" s="35" t="str">
-        <x:v>Battle</x:v>
+        <x:v>EnemiesInsideGesture</x:v>
       </x:c>
       <x:c r="C80" s="35" t="str">
-        <x:v>Battle</x:v>
+        <x:v>EnemiesInsideGesture</x:v>
       </x:c>
       <x:c r="D80" s="35" t="str">
-        <x:v>不选择单体目标，效果直接作用于整个战斗世界。</x:v>
+        <x:v>选择位于当前闭合笔势区域内的全部存活敌人。</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
@@ -14121,13 +14239,13 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B81" s="35" t="str">
-        <x:v>AllEnemies</x:v>
+        <x:v>Battle</x:v>
       </x:c>
       <x:c r="C81" s="35" t="str">
-        <x:v>AllEnemies</x:v>
+        <x:v>Battle</x:v>
       </x:c>
       <x:c r="D81" s="35" t="str">
-        <x:v>选择当前全部存活敌人，包括普通、精英和Boss。</x:v>
+        <x:v>不选择单体目标，效果直接作用于整个战斗世界。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
@@ -14135,13 +14253,13 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B82" s="35" t="str">
-        <x:v>NormalEnemies</x:v>
+        <x:v>AllEnemies</x:v>
       </x:c>
       <x:c r="C82" s="35" t="str">
-        <x:v>NormalEnemies</x:v>
+        <x:v>AllEnemies</x:v>
       </x:c>
       <x:c r="D82" s="35" t="str">
-        <x:v>选择全部非Boss存活敌人，因此同时包含Normal与Elite。</x:v>
+        <x:v>选择当前全部存活敌人，包括普通、精英和Boss。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
@@ -14149,41 +14267,41 @@
         <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B83" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>NormalEnemies</x:v>
       </x:c>
       <x:c r="C83" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>NormalEnemies</x:v>
       </x:c>
       <x:c r="D83" s="35" t="str">
-        <x:v>只选择EnemyTier为Boss的存活敌人。</x:v>
+        <x:v>选择全部非Boss存活敌人，因此同时包含Normal与Elite。</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
       <x:c r="A84" s="35" t="str">
-        <x:v>EffectType</x:v>
+        <x:v>TargetType</x:v>
       </x:c>
       <x:c r="B84" s="35" t="str">
-        <x:v>PlayVfx</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="C84" s="35" t="str">
-        <x:v>PlayVfx</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="D84" s="35" t="str">
-        <x:v>不改变战斗数值，只按vfxKey在所选目标或世界范围播放特效。</x:v>
+        <x:v>只选择EnemyTier为Boss的存活敌人。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
       <x:c r="A85" s="35" t="str">
-        <x:v>ValueType</x:v>
+        <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B85" s="35" t="str">
-        <x:v>int</x:v>
+        <x:v>PlayVfx</x:v>
       </x:c>
       <x:c r="C85" s="35" t="str">
-        <x:v>int</x:v>
+        <x:v>PlayVfx</x:v>
       </x:c>
       <x:c r="D85" s="35" t="str">
-        <x:v>Global行从intValue读取整数，其他三个值列必须留空。</x:v>
+        <x:v>不改变战斗数值，只按vfxKey在所选目标或世界范围播放特效。</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
@@ -14191,13 +14309,13 @@
         <x:v>ValueType</x:v>
       </x:c>
       <x:c r="B86" s="35" t="str">
-        <x:v>float</x:v>
+        <x:v>int</x:v>
       </x:c>
       <x:c r="C86" s="35" t="str">
-        <x:v>float</x:v>
+        <x:v>int</x:v>
       </x:c>
       <x:c r="D86" s="35" t="str">
-        <x:v>Global行从floatValue读取浮点数，其他三个值列必须留空。</x:v>
+        <x:v>Global行从intValue读取整数，其他三个值列必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
@@ -14205,13 +14323,13 @@
         <x:v>ValueType</x:v>
       </x:c>
       <x:c r="B87" s="35" t="str">
-        <x:v>string</x:v>
+        <x:v>float</x:v>
       </x:c>
       <x:c r="C87" s="35" t="str">
-        <x:v>string</x:v>
+        <x:v>float</x:v>
       </x:c>
       <x:c r="D87" s="35" t="str">
-        <x:v>Global行从stringValue读取文本或稳定协议值，其他三个值列必须留空。</x:v>
+        <x:v>Global行从floatValue读取浮点数，其他三个值列必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
@@ -14219,27 +14337,27 @@
         <x:v>ValueType</x:v>
       </x:c>
       <x:c r="B88" s="35" t="str">
-        <x:v>bool</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="C88" s="35" t="str">
-        <x:v>bool</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="D88" s="35" t="str">
-        <x:v>Global行从boolValue读取真假开关，其他三个值列必须留空。</x:v>
+        <x:v>Global行从stringValue读取文本或稳定协议值，其他三个值列必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
       <x:c r="A89" s="35" t="str">
-        <x:v>SpawnLane</x:v>
+        <x:v>ValueType</x:v>
       </x:c>
       <x:c r="B89" s="35" t="str">
-        <x:v>Ground</x:v>
+        <x:v>bool</x:v>
       </x:c>
       <x:c r="C89" s="35" t="str">
-        <x:v>Ground</x:v>
+        <x:v>bool</x:v>
       </x:c>
       <x:c r="D89" s="35" t="str">
-        <x:v>地面出生通道标签；实际位置仍由normalizedX/Y决定，当前生产适配器不据此自动改变移动策略。</x:v>
+        <x:v>Global行从boolValue读取真假开关，其他三个值列必须留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
@@ -14247,13 +14365,13 @@
         <x:v>SpawnLane</x:v>
       </x:c>
       <x:c r="B90" s="35" t="str">
-        <x:v>Air</x:v>
+        <x:v>Ground</x:v>
       </x:c>
       <x:c r="C90" s="35" t="str">
-        <x:v>Air</x:v>
+        <x:v>Ground</x:v>
       </x:c>
       <x:c r="D90" s="35" t="str">
-        <x:v>空中出生通道标签；实际高度仍由normalizedY决定，当前生产适配器不据此自动赋予飞行能力。</x:v>
+        <x:v>地面出生通道标签；实际位置仍由normalizedX/Y决定，当前生产适配器不据此自动改变移动策略。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15" hidden="0" customHeight="1">
@@ -14261,27 +14379,27 @@
         <x:v>SpawnLane</x:v>
       </x:c>
       <x:c r="B91" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Air</x:v>
       </x:c>
       <x:c r="C91" s="35" t="str">
-        <x:v>Boss</x:v>
+        <x:v>Air</x:v>
       </x:c>
       <x:c r="D91" s="35" t="str">
-        <x:v>Boss出生通道标签；Boss身份仍由Enemies.tier、Levels.bossEnemyId和出生计划共同校验。</x:v>
+        <x:v>空中出生通道标签；实际高度仍由normalizedY决定，当前生产适配器不据此自动赋予飞行能力。</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="15" hidden="0" customHeight="1">
       <x:c r="A92" s="35" t="str">
-        <x:v>Facing</x:v>
+        <x:v>SpawnLane</x:v>
       </x:c>
       <x:c r="B92" s="35" t="str">
-        <x:v>Left</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="C92" s="35" t="str">
-        <x:v>Left</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="D92" s="35" t="str">
-        <x:v>声明实体出生时朝左；当前运行时会传递该值，但生产角色表现尚未据此自动翻转。</x:v>
+        <x:v>Boss出生通道标签；Boss身份仍由Enemies.tier、Levels.bossEnemyId和出生计划共同校验。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15" hidden="0" customHeight="1">
@@ -14289,27 +14407,27 @@
         <x:v>Facing</x:v>
       </x:c>
       <x:c r="B93" s="35" t="str">
-        <x:v>Right</x:v>
+        <x:v>Left</x:v>
       </x:c>
       <x:c r="C93" s="35" t="str">
-        <x:v>Right</x:v>
+        <x:v>Left</x:v>
       </x:c>
       <x:c r="D93" s="35" t="str">
-        <x:v>声明实体出生时朝右；当前运行时会传递该值，但生产角色表现尚未据此自动翻转。</x:v>
+        <x:v>声明实体出生时朝左；当前运行时会传递该值，但生产角色表现尚未据此自动翻转。</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="15" hidden="0" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>EffectType</x:v>
+        <x:v>Facing</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Heal</x:v>
+        <x:v>Right</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Heal</x:v>
+        <x:v>Right</x:v>
       </x:c>
       <x:c r="D94" s="34" t="str">
-        <x:v>为选中目标恢复value1点生命；目标接口负责上限和不可复活规则。</x:v>
+        <x:v>声明实体出生时朝右；当前运行时会传递该值，但生产角色表现尚未据此自动翻转。</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="15" hidden="0" customHeight="1">
@@ -14317,41 +14435,41 @@
         <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>ClearProjectiles</x:v>
+        <x:v>Heal</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>ClearProjectiles</x:v>
+        <x:v>Heal</x:v>
       </x:c>
       <x:c r="D95" s="34" t="str">
-        <x:v>清除当前世界中的敌方投射物，不影响已反弹为玩家阵营的投射物。</x:v>
+        <x:v>为选中目标恢复value1点生命；目标接口负责上限和不可复活规则。</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="15" hidden="0" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>BuffType</x:v>
+        <x:v>EffectType</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>DamageReduction</x:v>
+        <x:v>ClearProjectiles</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>DamageReduction</x:v>
+        <x:v>ClearProjectiles</x:v>
       </x:c>
       <x:c r="D96" s="34" t="str">
-        <x:v>按1-magnitude×层数降低目标受到的伤害倍率，结果钳制为不小于0。</x:v>
+        <x:v>清除当前世界中的敌方投射物，不影响已反弹为玩家阵营的投射物。</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="15" hidden="0" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>PoolExhaustionPolicy</x:v>
+        <x:v>BuffType</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Reject</x:v>
+        <x:v>DamageReduction</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Reject</x:v>
+        <x:v>DamageReduction</x:v>
       </x:c>
       <x:c r="D97" s="34" t="str">
-        <x:v>对象池达到活动容量时拒绝本次租用，不扩容、不回收仍在使用的对象。</x:v>
+        <x:v>按1-magnitude×层数降低目标受到的伤害倍率，结果钳制为不小于0。</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="15" hidden="0" customHeight="1">
@@ -14359,27 +14477,27 @@
         <x:v>PoolExhaustionPolicy</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>ReuseOldest</x:v>
+        <x:v>Reject</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>ReuseOldest</x:v>
+        <x:v>Reject</x:v>
       </x:c>
       <x:c r="D98" s="34" t="str">
-        <x:v>对象池达到活动容量时先完整回收最早的活动对象，再把该实例用于本次租用。</x:v>
+        <x:v>对象池达到活动容量时拒绝本次租用，不扩容、不回收仍在使用的对象。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="15" hidden="0" customHeight="1">
       <x:c r="A99" s="132" t="str">
-        <x:v>FeedbackVibrationPattern</x:v>
+        <x:v>PoolExhaustionPolicy</x:v>
       </x:c>
       <x:c r="B99" s="132" t="str">
-        <x:v>Off</x:v>
+        <x:v>ReuseOldest</x:v>
       </x:c>
       <x:c r="C99" s="132" t="str">
-        <x:v>关闭</x:v>
+        <x:v>ReuseOldest</x:v>
       </x:c>
       <x:c r="D99" s="203" t="str">
-        <x:v>不请求平台震动。</x:v>
+        <x:v>对象池达到活动容量时先完整回收最早的活动对象，再把该实例用于本次租用。</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="15" hidden="0" customHeight="1">
@@ -14387,13 +14505,13 @@
         <x:v>FeedbackVibrationPattern</x:v>
       </x:c>
       <x:c r="B100" s="137" t="str">
-        <x:v>Light</x:v>
+        <x:v>Off</x:v>
       </x:c>
       <x:c r="C100" s="137" t="str">
-        <x:v>轻震</x:v>
+        <x:v>关闭</x:v>
       </x:c>
       <x:c r="D100" s="204" t="str">
-        <x:v>请求轻量短震，适合普通命中等低强度反馈。</x:v>
+        <x:v>不请求平台震动。</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="15" hidden="0" customHeight="1">
@@ -14401,13 +14519,13 @@
         <x:v>FeedbackVibrationPattern</x:v>
       </x:c>
       <x:c r="B101" s="132" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Light</x:v>
       </x:c>
       <x:c r="C101" s="132" t="str">
-        <x:v>中震</x:v>
+        <x:v>轻震</x:v>
       </x:c>
       <x:c r="D101" s="203" t="str">
-        <x:v>请求中等震动，适合受击或较强技能反馈。</x:v>
+        <x:v>请求轻量短震，适合普通命中等低强度反馈。</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="15" hidden="0" customHeight="1">
@@ -14415,12 +14533,26 @@
         <x:v>FeedbackVibrationPattern</x:v>
       </x:c>
       <x:c r="B102" s="137" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C102" s="137" t="str">
+        <x:v>中震</x:v>
+      </x:c>
+      <x:c r="D102" s="204" t="str">
+        <x:v>请求中等震动，适合受击或较强技能反馈。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>FeedbackVibrationPattern</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
         <x:v>Heavy</x:v>
       </x:c>
-      <x:c r="C102" s="137" t="str">
+      <x:c r="C103" t="str">
         <x:v>重震</x:v>
       </x:c>
-      <x:c r="D102" s="204" t="str">
+      <x:c r="D103" t="str">
         <x:v>请求强震动，适合重击、Boss或重大结算反馈。</x:v>
       </x:c>
     </x:row>
@@ -14431,7 +14563,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radaf2c75e1194878"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f52abee47da46d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15183,7 +15315,7 @@
       </x:c>
       <x:c r="I32" s="35"/>
       <x:c r="J32" s="35" t="str">
-        <x:v>笔势类型：决定该笔势规则最终识别的输入类别；分类还会继续受到长度、方向、闭合、面积、曲率或蓄力阈值约束。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类。 配置约束：不得留空。</x:v>
+        <x:v>笔势类型：决定该笔势规则最终识别的输入类别；分类还会继续受到长度、方向、闭合、面积、曲率或蓄力阈值约束。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类；Triangle=要求首尾近似闭合且三条边、三个角点满足配置拟合阈值。 配置约束：不得留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -15367,7 +15499,7 @@
       <x:c r="H40" s="35"/>
       <x:c r="I40" s="35"/>
       <x:c r="J40" s="35" t="str">
-        <x:v>最小包围面积：闭合笔势必须覆盖的最小参考像素平方面积，用于过滤过小圆形。 参考像素以Global.reference_width/reference_height为设计空间，再映射到实际画面。 配置约束：不得留空。</x:v>
+        <x:v>最小包围面积：闭合形状必须覆盖的最小参考像素平方面积，用于过滤过小的圆形或三角形；不适用时填0。 参考像素以Global.reference_width/reference_height为设计空间，再映射到实际画面。 配置约束：不得留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -15757,7 +15889,7 @@
       </x:c>
       <x:c r="I57" s="35"/>
       <x:c r="J57" s="35" t="str">
-        <x:v>要求笔势：决定攻击护甲或触发有效破防所需的笔势；不匹配时改走wrongGestureDamageMultiplier和reflectDamage规则。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类。 配置约束：不得留空。</x:v>
+        <x:v>要求笔势：决定攻击护甲或触发有效破防所需的笔势；不匹配时改走wrongGestureDamageMultiplier和reflectDamage规则。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类；Triangle=要求首尾近似闭合且三条边、三个角点满足配置拟合阈值。 配置约束：不得留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -16887,7 +17019,7 @@
       </x:c>
       <x:c r="I106" s="35"/>
       <x:c r="J106" s="35" t="str">
-        <x:v>打断笔势：决定敌人攻击前摇期间允许哪类笔势打断；还必须命中interruptStartSec到interruptEndSec窗口。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类。 配置约束：不得留空。</x:v>
+        <x:v>打断笔势：决定敌人攻击前摇期间允许哪类笔势打断；还必须命中interruptStartSec到interruptEndSec窗口。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类；Triangle=要求首尾近似闭合且三条边、三个角点满足配置拟合阈值。 配置约束：不得留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="15" hidden="0" customHeight="1">
@@ -17615,7 +17747,7 @@
       </x:c>
       <x:c r="I137" s="35"/>
       <x:c r="J137" s="35" t="str">
-        <x:v>笔势类型：决定Gesture或Ultimate技能接受的笔势；Passive不依赖该笔势，但字段仍需填写有效协议值。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类。 配置约束：不得留空。</x:v>
+        <x:v>笔势类型：决定Gesture或Ultimate技能接受的笔势；Passive不依赖该笔势，但字段仍需填写有效协议值。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类；Triangle=要求首尾近似闭合且三条边、三个角点满足配置拟合阈值。 配置约束：不得留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="15" hidden="0" customHeight="1">
@@ -19697,7 +19829,7 @@
       </x:c>
       <x:c r="I226" s="35"/>
       <x:c r="J226" s="35" t="str">
-        <x:v>笔势类型：决定该教程步骤期望玩家完成的笔势；实际完成还要由completeEvent到达，不能只靠显示提示。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类。 配置约束：不得留空。</x:v>
+        <x:v>笔势类型：决定该教程步骤期望玩家完成的笔势；实际完成还要由completeEvent到达，不能只靠显示提示。 允许值及作用：Any=不限制具体笔势类别；Horizontal=要求笔迹主方向接近水平线；Vertical=要求笔迹主方向接近竖直线；Diagonal=要求笔迹主方向为斜线；Arc=要求笔迹形成达到minArcCurvature阈值的弧线，不要求首尾闭合；Circle=要求笔迹首尾距离和包围面积同时达到圆形规则，用于闭合环形输入；Charged=要求持续按住达到chargeHoldSec后释放的蓄力输入，不以普通直线方向分类；Triangle=要求首尾近似闭合且三条边、三个角点满足配置拟合阈值。 配置约束：不得留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="227" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -21094,6 +21226,80 @@
       </x:c>
       <x:c r="J285" t="str">
         <x:v>蓄力特效资源键：停留蓄力使用的独立粒子Prefab；换皮或新增样式只修改此引用。配置约束：不得留空；必须引用AssetManifest.assetKey的现有值，不存在时导出失败。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="15" hidden="0" customHeight="1">
+      <x:c r="A286" t="str">
+        <x:v>StrokeRules</x:v>
+      </x:c>
+      <x:c r="B286" t="str">
+        <x:v>shapeFitToleranceRefPx</x:v>
+      </x:c>
+      <x:c r="C286" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="D286" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E286" t="str"/>
+      <x:c r="F286" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G286"/>
+      <x:c r="H286" t="str"/>
+      <x:c r="I286" t="str"/>
+      <x:c r="J286" t="str">
+        <x:v>形状拟合容差：多边形形状识别时，处理后任一点到候选边的最大允许距离，单位为参考像素；Triangle用它容纳手绘抖动，0表示该规则不使用多边形拟合。 配置约束：不得留空；不得小于0。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="15" hidden="0" customHeight="1">
+      <x:c r="A287" t="str">
+        <x:v>StrokeRules</x:v>
+      </x:c>
+      <x:c r="B287" t="str">
+        <x:v>minCornerAngleDeg</x:v>
+      </x:c>
+      <x:c r="C287" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="D287" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="E287" t="str"/>
+      <x:c r="F287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G287" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="H287" t="str"/>
+      <x:c r="I287" t="str"/>
+      <x:c r="J287" t="str">
+        <x:v>最小角点角度：多边形形状识别时每个候选内角允许的最小角度，单位为度；Triangle中任一角小于该值时拒绝识别，0表示不使用角点门槛。 配置约束：不得留空；有效范围0到90。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="288" ht="15" hidden="0" customHeight="1">
+      <x:c r="A288" t="str">
+        <x:v>StrokeRules</x:v>
+      </x:c>
+      <x:c r="B288" t="str">
+        <x:v>onMatchSkillId</x:v>
+      </x:c>
+      <x:c r="C288" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D288" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="E288" t="str"/>
+      <x:c r="F288"/>
+      <x:c r="G288"/>
+      <x:c r="H288" t="str"/>
+      <x:c r="I288" t="str">
+        <x:v>Skills.skillId</x:v>
+      </x:c>
+      <x:c r="J288" t="str">
+        <x:v>命中后技能ID：该笔势成功分类后自动尝试释放的Skills.skillId；留空表示只执行普通笔画命中，不追加技能效果。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -21116,7 +21322,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6887a04982794d79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3685327362934f6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21244,7 +21450,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9071a235ec7e4f89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c9d9a277f55499d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22125,7 +22331,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34749a95440b485f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R788f4ddabe274df8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22147,6 +22353,9 @@
     <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="21.110000610351562" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -22165,6 +22374,9 @@
       <x:c r="K1" s="52"/>
       <x:c r="L1" s="52"/>
       <x:c r="M1" s="52"/>
+      <x:c r="N1"/>
+      <x:c r="O1"/>
+      <x:c r="P1"/>
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="13" t="str">
@@ -22182,6 +22394,9 @@
       <x:c r="K2" s="13"/>
       <x:c r="L2" s="13"/>
       <x:c r="M2" s="13"/>
+      <x:c r="N2"/>
+      <x:c r="O2"/>
+      <x:c r="P2"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="220" t="str">
@@ -22223,6 +22438,15 @@
       <x:c r="M3" s="222" t="str">
         <x:v>命中半径</x:v>
       </x:c>
+      <x:c r="N3" s="234" t="str">
+        <x:v>形状拟合容差</x:v>
+      </x:c>
+      <x:c r="O3" s="234" t="str">
+        <x:v>最小角点角度</x:v>
+      </x:c>
+      <x:c r="P3" s="234" t="str">
+        <x:v>命中后技能ID</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="58" t="str">
@@ -22264,6 +22488,15 @@
       <x:c r="M4" s="58" t="str">
         <x:v>hitRadiusRefPx</x:v>
       </x:c>
+      <x:c r="N4" s="238" t="str">
+        <x:v>shapeFitToleranceRefPx</x:v>
+      </x:c>
+      <x:c r="O4" s="238" t="str">
+        <x:v>minCornerAngleDeg</x:v>
+      </x:c>
+      <x:c r="P4" s="238" t="str">
+        <x:v>onMatchSkillId</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="35" t="str">
@@ -22305,6 +22538,13 @@
       <x:c r="M5" s="35" t="n">
         <x:v>18</x:v>
       </x:c>
+      <x:c r="N5" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O5" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P5" s="239" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="35" t="str">
@@ -22346,6 +22586,13 @@
       <x:c r="M6" s="35" t="n">
         <x:v>20</x:v>
       </x:c>
+      <x:c r="N6" s="242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O6" s="242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P6" s="240" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="35" t="str">
@@ -22387,6 +22634,13 @@
       <x:c r="M7" s="35" t="n">
         <x:v>20</x:v>
       </x:c>
+      <x:c r="N7" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O7" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P7" s="239" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="35" t="str">
@@ -22428,6 +22682,13 @@
       <x:c r="M8" s="35" t="n">
         <x:v>18</x:v>
       </x:c>
+      <x:c r="N8" s="242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O8" s="242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P8" s="240" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="35" t="str">
@@ -22469,6 +22730,13 @@
       <x:c r="M9" s="35" t="n">
         <x:v>24</x:v>
       </x:c>
+      <x:c r="N9" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O9" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P9" s="239" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="35" t="str">
@@ -22510,6 +22778,13 @@
       <x:c r="M10" s="35" t="n">
         <x:v>28</x:v>
       </x:c>
+      <x:c r="N10" s="242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O10" s="242" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P10" s="240" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="35" t="str">
@@ -22551,11 +22826,68 @@
       <x:c r="M11" s="35" t="n">
         <x:v>26</x:v>
       </x:c>
+      <x:c r="N11" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O11" s="241" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P11" s="239" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>stroke_triangle</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Triangle</x:v>
+      </x:c>
+      <x:c r="C12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D12" t="n">
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="E12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F12" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G12" t="n">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H12" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="I12" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="J12" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="K12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N12" s="242" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="O12" s="242" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="P12" s="240" t="str">
+        <x:v>skill_triangle_slow</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A2:M2"/>
+    <x:mergeCell ref="A1:P1"/>
+    <x:mergeCell ref="A2:P2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B5:B504">
@@ -22564,7 +22896,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R346d634d4f2a4651"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabfc856bf1394169"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22796,7 +23128,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb366903db6194ac8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb16bdee08de64733"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23001,7 +23333,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35798f518e554d5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refbdf41743ab46ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23255,7 +23587,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a66fa13b07542a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24471f8bd07b4786"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23634,7 +23966,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aa277cd83d342f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81825601e5a04133"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>